<commit_message>
Daily facility note collection 2026-09-13
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D576"/>
+  <dimension ref="A1:D665"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13088,6 +13088,1964 @@
         </is>
       </c>
     </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>9/1オーケー高槻赤大路店(大阪府高槻市)</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fOy</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>9/1 ライフ鎌倉梶原店</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fS5</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>9/3 サンディ吹田五月が丘店(大阪府吹田市)</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fPd</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>9/3改装 スーパーのアオキ直江津店(新潟県上越市)</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2v</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>9/3スギ薬局茜部南店(岐阜市)</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2N</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>9/4クックマート上西店（静岡県浜松市）</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7N</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>9/4(9/3プレ)スーパー生鮮館TAIGA桂子田店</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fZU</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>9/4改装 名古屋PARCO</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7c</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>9/4改装 メイチカ(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7g</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>9/4ウルフギャングステーキハウス名古屋店</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eZr</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>9/4 ゴジラ・ストア Nagoya</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fn6</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>9/4ロピア彦根ナフコ店</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fNK</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>(9/8ソフト)9/11そよら津桜橋(三重県津市)</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1bV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>9/9MARUAI BIG アクロスプラザ高砂店</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gbn</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>9/10改装 マルナカ檀紙店(香川県高松市)</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7X</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>9/10ザ・ビッグエクスプレスみよし店</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>9/10ファミリーマート中津川下野店</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g84</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>9/10とりせん田沼インター店(栃木県)</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9g</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>9/11スーパーマーケットバロー豊中島江店</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fXN</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>9/11ザ・ビッグ厚別店</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9V</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>9/16SANYO Style STORE PLUS イオンモール岡崎店</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fEw</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>9/17ロピア ムサシ新潟西店(新潟市)</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g6X</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>9/17明治屋自由が丘ストアー</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ga2</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>関東地方アイタウン魚津 2025年10月16日(木)開業！無印良品も出店へ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/43463</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>関東地方フォルテさくら氏家 2026年1月28日(水)開業！テナント随時更新中！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/43900</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>関東地方パークタワー川口本町 2026年秋完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26762</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>関東地方新宿駅西口地区に新駅ビル 2029年度開業予定！どのような建物に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/17061</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>関西地方BiVi二条 2024年8月末で一旦閉店し大規模改装！2025年6月20日(金)11時~開業！全26店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/33261</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>関東地方ベルク平塚田村店 2026年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47482</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>関東地方ヤオコー大宮市場店 2026年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48511</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>東北地方福島ピボット 2026年3月28日(土)開業！ロピアも出店！11店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/47552</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>関東地方自由が丘ミューズスクエア 2026年9月17日(木)開業！全59テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/23151</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>関西地方オークワ堺市駅前店 2025年8月30日(土)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/38273</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>中国地方そよら鳥取駅南 2026年10月上旬開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/49474</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>関東地方アトレ中野 2026年12月9日(水)開業！全73テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/27599</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>関東地方追浜駅前第2街区市街地再開発事業 2029年11月完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/32533</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>関東地方BLiX茅ヶ崎(ブリックス茅ヶ崎) 2025年11月27日(木)開業！テナント随時更新中！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/38752</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>九州地方メガセンタートライアル荒尾店 2025年2月11日(火)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/39634</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>中部地方加賀温泉駅前に大型商業施設計画！2029年度開業！アウトレットモールも？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/32477</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>関東地方和光市駅北口地区市街地再開発事業 2029年度完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/32817</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>北海道地方コープさっぽろ すながわ店 2026年9月10日(木)開業！無印良品も出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/48252</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>関西地方ケーズデンキ桜井店 2026年9月17日(木)開業予定！最新情報も！奈良県桜井市に関西ケーズデンキの店舗「ケーズデンキ桜井店」が2026年9月17日(木)開業予定！ケーズデンキの大型店舗が、新たに誕生する桜井複合商業施設へ出店！隣接地にはコーナンPROも新設！そんな、ケーズデンキ桜井店について、テナントや開...2026.09.12関西地方</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49275</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>東北地方スーパーセンタートライアル金ケ崎店 2026年9月16日(水)開業！15日(火)プレオープン！最新情報も！岩手県胆沢郡金ケ崎町にトライアルカンパニーの店舗「スーパーセンタートライアル金ケ崎店」が2026年9月16日(水)8：30グランドオープン！9月15日(火)10：00～19：00プレオープン！スーパーセンタートライアルが金ケ崎町に初出店！そ...2026.09.12東北地方</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/47232</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>ヤオコー／千葉県船橋市に「船橋薬円台店」9月15日オープン</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091116.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>バロー／名古屋市に「スーパーマーケットバロー矢田店」9月18日オープン</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091115.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>ベイシア／三心との連携1号店「岐南店」改装オープン、即食品強化・丸魚の販売継続</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091172.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>池袋パルコ／大規模リニューアル完了「ウルトラマンストア」など今秋15店舗オープン</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091176.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>仙台パルコ／秋冬リニューアルで新規含む16店舗オープン、PARCO2では飲食強化</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091175.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>あべのハルカス近鉄本店／10～11月、子ども服フロアの大規模リニューアル開始</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091114.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>コスモス薬品／福岡県・島根県に「ドラッグコスモス」計2店舗、27年4月新設</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0911012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>ビームス／原宿に「ビームス レコーズ／bPrビームス」9月19日オープン</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091113.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>フライングタイガー／池袋・サンシャインシティに10月16日新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091112.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>JR西日本／大阪駅にメーク直し・仕事・休憩に対応する駅ナカ空間オープン</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091118.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>成城石井／大阪府守口市に「京阪百貨店守口店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091141.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>オンデーズ／三重県4店舗目「OWNDAYS そよら津桜橋店」オープン</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091177.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>ケーズデンキ／宮城県名取市に「（仮称）新仙台南店（店舗面積5988.15m2）」27年3月23日新設</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0911011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>平和堂／「アルプラフーズマーケット富山掛尾」オープン、富山県に食品スーパー初出店</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091042.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>二子玉川ライズS.C.／今秋「マリークワント」「プリンセスタルト」など新規オープン</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091077.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>グランベリーパーク／秋リニューアルを実施、ラベンハムなど12店舗がオープン</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091045.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>DNP／グランスタ東京にブランド体験型店舗「＆found」今冬オープン</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091013.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>ヨドバシカメラ／東京・池袋に「リカーワールド ヨドバシ池袋店」9月19日オープン</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091044.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>まいばすけっと／神奈川県藤沢市に「湘南台駅西店」9月11日オープン</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091071.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>2026年09月13日</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>ニトリ／東京・神奈川の島忠2店舗にレディスアパレル「N+」9月11日オープン</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091072.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-14
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D665"/>
+  <dimension ref="A1:D754"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15046,6 +15046,1964 @@
         </is>
       </c>
     </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>9/1オーケー高槻赤大路店(大阪府高槻市)</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fOy</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>9/1 ライフ鎌倉梶原店</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fS5</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>9/3 サンディ吹田五月が丘店(大阪府吹田市)</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fPd</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>9/3改装 スーパーのアオキ直江津店(新潟県上越市)</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2v</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>9/3スギ薬局茜部南店(岐阜市)</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2N</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>9/4クックマート上西店（静岡県浜松市）</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7N</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>9/4(9/3プレ)スーパー生鮮館TAIGA桂子田店</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fZU</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>9/4改装 名古屋PARCO</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7c</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>9/4改装 メイチカ(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7g</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>9/4ウルフギャングステーキハウス名古屋店</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eZr</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>9/4 ゴジラ・ストア Nagoya</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fn6</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>9/4ロピア彦根ナフコ店</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fNK</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>(9/8ソフト)9/11そよら津桜橋(三重県津市)</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1bV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>9/9MARUAI BIG アクロスプラザ高砂店</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gbn</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>9/10改装 マルナカ檀紙店(香川県高松市)</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7X</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>9/10ザ・ビッグエクスプレスみよし店</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>9/10ファミリーマート中津川下野店</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g84</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>9/10とりせん田沼インター店(栃木県)</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9g</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>9/11スーパーマーケットバロー豊中島江店</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fXN</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>9/11ザ・ビッグ厚別店</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9V</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>9/16SANYO Style STORE PLUS イオンモール岡崎店</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fEw</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>9/17ロピア ムサシ新潟西店(新潟市)</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g6X</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>9/17明治屋自由が丘ストアー</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ga2</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>関東地方新松田駅北口地区市街地再開発事業 2030年初頭開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48018</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>関西地方コメリパワー平群店 2025年7月16日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39836</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>東北地方イオンスタイル山王 2025年3月20日(木)開業！無印良品も出店へ！全8テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/37974</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>関東地方前橋市野中町SC計画 2028年春開業！ベルクが出店へ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49033</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>九州地方天神大樹 イムズ跡地 2027年秋開業！どんな計画？テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/27165</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>関東地方三井アウトレットパーク木更津が第4期増床！2025年6月23日(月)開業！全33テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/37531</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>関東地方東京ドリームパーク 2026年3月27日(金)誕生！5千人収容ホールや商業施設 最新情報も！</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/32434</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>関東地方みなとみらい21中央地区60・61街区開発事業 2029年春開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36914</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>中部地方ニトリ焼津店 2025年6月27日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/41145</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>関東地方生鮮市場TOP栃木合戦場店 2026年8月1日(土)8時~開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47134</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>中部地方三島駅南口東街区Ａ地区市街地再開発事業 2027年竣工予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/25890</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>関西地方フレンドタウン守山 2025年11月28日(金)9時~開業！全12テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/25311</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>関東地方王子駅前地区市街地再開発事業 2034年度開業予定！商業施設も誕生！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47579</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>関東地方高崎駅東口栄町地区市街地再開発事業 2029年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/29079</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>関東地方東京ミッドタウン日本橋 2027年秋開業！コレド日本橋も大規模改装！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/17615</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>関東地方スーパーセンタートライアル深谷川本店 2026年4月29日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/44915</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>関東地方グラン8モール 2025年8月28日(木)より順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42179</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>関東地方イオンモール津田沼サウス 2026年3月18日(水)開業！全50店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/45209</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>関西地方ケーズデンキ桜井店 2026年9月17日(木)開業予定！最新情報も！奈良県桜井市に関西ケーズデンキの店舗「ケーズデンキ桜井店」が2026年9月17日(木)開業予定！ケーズデンキの大型店舗が、新たに誕生する桜井複合商業施設へ出店！隣接地にはコーナンPROも新設！そんな、ケーズデンキ桜井店について、テナントや開...2026.09.12関西地方</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49275</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>東北地方スーパーセンタートライアル金ケ崎店 2026年9月16日(水)開業！15日(火)プレオープン！最新情報も！岩手県胆沢郡金ケ崎町にトライアルカンパニーの店舗「スーパーセンタートライアル金ケ崎店」が2026年9月16日(水)8：30グランドオープン！9月15日(火)10：00～19：00プレオープン！スーパーセンタートライアルが金ケ崎町に初出店！そ...2026.09.12東北地方</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/47232</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>コスモス薬品／栃木県・大阪府に「ドラッグコスモス」計2店舗、27年4月新設</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0914011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>ジャック イン ザ ドーナツ／岡山市北区「イオンモール岡山店」9月18日オープン</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091473.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>ケーズデンキ／福岡県糟屋郡新宮町に「（仮称）福岡新宮店（店舗面積4015m2）」27年4月5日新設</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0914012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>牛カツ京都勝牛／京都市伏見区に「伏見稲荷大社前店」オープン、大鳥居正面に出店</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091444.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>ホットランド／「銀だこハイボール酒場 渋谷センター街店」9月15日オープン</t>
+        </is>
+      </c>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091413.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>ゴンチャ／大阪市北区「エキマルシェ大阪店」9月18日オープン</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091472.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>まいばすけっと／「高幡不動駅北口店」「東淵野辺3丁目店」9月18日同時オープン</t>
+        </is>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091446.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>ヤオコー／千葉県船橋市に「船橋薬円台店」9月15日オープン</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091116.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>バロー／名古屋市に「スーパーマーケットバロー矢田店」9月18日オープン</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091115.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>ベイシア／三心との連携1号店「岐南店」改装オープン、即食品強化・丸魚の販売継続</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091172.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>池袋パルコ／大規模リニューアル完了「ウルトラマンストア」など今秋15店舗オープン</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091176.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>仙台パルコ／秋冬リニューアルで新規含む16店舗オープン、PARCO2では飲食強化</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091175.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>あべのハルカス近鉄本店／10～11月、子ども服フロアの大規模リニューアル開始</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091114.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>コスモス薬品／福岡県・島根県に「ドラッグコスモス」計2店舗、27年4月新設</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0911012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>ビームス／原宿に「ビームス レコーズ／bPrビームス」9月19日オープン</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091113.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>フライングタイガー／池袋・サンシャインシティに10月16日新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091112.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>JR西日本／大阪駅にメーク直し・仕事・休憩に対応する駅ナカ空間オープン</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091118.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>成城石井／大阪府守口市に「京阪百貨店守口店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091141.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>オンデーズ／三重県4店舗目「OWNDAYS そよら津桜橋店」オープン</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091177.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>2026年09月14日</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>ケーズデンキ／宮城県名取市に「（仮称）新仙台南店（店舗面積5988.15m2）」27年3月23日新設</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0911011.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-15
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D754"/>
+  <dimension ref="A1:D854"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17004,6 +17004,2206 @@
         </is>
       </c>
     </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>MARE &amp; OYSTER エスパル仙台店</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>https://oysterbar.co.jp/shop/sendai-station-oysterbar-s-pal/</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>ヤオコー船橋薬円台店</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ggO</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>YANAKA COFFEE 柏高島屋ステーションモール店</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>https://www.takashimaya.co.jp/kashiwa/stemo/open_close/</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>TELA HAIR北越谷店</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>https://beauty.hotpepper.jp/slnH000824723/</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>melie beaute原宿店</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>https://beauty.hotpepper.jp/kr/slnH000822915/</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>Paw八王子店</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>https://lp.paw-fit.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>八王子焼肉 タマちゃん</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>https://yakiniku-carlos.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>LE CHOU CHOU -SWEETS＆DELI-</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr">
+        <is>
+          <t>https://hiltonodaiba.jp/plans/restaurants/7444</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>軽井沢 とりまち</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>https://store.tsite.jp/karuizawa/news/t-site/56506-1059460829.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>ケンタッキーフライドチキン武生楽市店</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>https://www.takefurakuichi.jp/shopguide.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>ドン・キホーテ岡山西大寺店</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>https://www.donki.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>買取大吉サニー加布里店</t>
+        </is>
+      </c>
+      <c r="D766" t="inlineStr">
+        <is>
+          <t>https://www.kaitori-daikichi.jp/list/gold/store/sunny-kafuri/</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>9/1オーケー高槻赤大路店(大阪府高槻市)</t>
+        </is>
+      </c>
+      <c r="D767" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fOy</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>9/1 ライフ鎌倉梶原店</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fS5</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>9/3 サンディ吹田五月が丘店(大阪府吹田市)</t>
+        </is>
+      </c>
+      <c r="D769" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fPd</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>9/3改装 スーパーのアオキ直江津店(新潟県上越市)</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2v</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>9/3スギ薬局茜部南店(岐阜市)</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2N</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>9/4クックマート上西店（静岡県浜松市）</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7N</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>9/4(9/3プレ)スーパー生鮮館TAIGA桂子田店</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fZU</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>9/4改装 名古屋PARCO</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7c</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>9/4改装 メイチカ(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7g</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>9/4ウルフギャングステーキハウス名古屋店</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eZr</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>9/4 ゴジラ・ストア Nagoya</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fn6</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>9/4ロピア彦根ナフコ店</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fNK</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>(9/8ソフト)9/11そよら津桜橋(三重県津市)</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1bV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>9/9MARUAI BIG アクロスプラザ高砂店</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gbn</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>9/10もとまちユニオン大船店</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gfg</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>9/10改装 マルナカ檀紙店(香川県高松市)</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7X</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>9/10ザ・ビッグエクスプレスみよし店</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>9/10ファミリーマート中津川下野店</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g84</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>9/10とりせん田沼インター店(栃木県)</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9g</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>9/10TOFROM YAESU TOWER(東京都)</t>
+        </is>
+      </c>
+      <c r="D786" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ged</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>9/10業務スーパー船場本町店</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gdW</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>9/10業務スーパー津山山北店(岡山県)</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ge1</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>9/10ラ・ムー飯塚花瀬店(福岡県)</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ge8</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>9/10マックスバリュ城栄店(長崎市)</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gel</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>9/11スーパーマーケットバロー豊中島江店</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fXN</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>9/11ザ・ビッグ厚別店</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9V</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>9/16SANYO Style STORE PLUS イオンモール岡崎店</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fEw</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>9/17ロピア ムサシ新潟西店(新潟市)</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g6X</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>関東地方品川駅西口地区A地区新築計画 2029年度竣工！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/24311</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>関東地方minanoba川口 2026年9月17日(金)開業！全10テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42094</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>九州地方遠賀川駅南商業店舗 2026年秋開業！ロピアが出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/48612</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>九州地方スーパーセンタートライアル飯塚庄内店 2025年1月29日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/39074</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>北海道地方【札幌駅・エスタ】北5西1・西2地区市街地再開発事業 2034年度開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/21614</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>中部地方富山市 桜木町地区市街地再開発事業 2032年度開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48025</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>関東地方パークタワー川口本町 2026年秋完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26762</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>九州地方アミュプラザ天神 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/48244</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>中部地方ミュープラット豊田市 2026年8月26日(水)開業！全7店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48621</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>北海道地方ケーズデンキ帯広店 2025年3月20日(木・祝)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/40212</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>関東地方ヤオコー板橋四葉店 2025年11月7日(金)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42113</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>関東地方セントラルガーデン月島 ザ タワー 2028年春完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26835</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>関東地方かすかべテラス 2025年6月10日(火)開業！コープみらいが出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/29383</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>関東地方アクロスプラザ鹿沼 2025年6月7日(土)開業！全5テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/41267</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>関東地方三井アウトレットパーク多摩南大沢 B街区が建て替えへ！2028年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42310</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>中部地方そよら飯田アップルロード 2025年7月18日(金)開業！全30店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/40463</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>関東地方ミナモニ有明 江東区有明1丁目計画 大和ハウスのマンションと商業施設に！2026年5月13日(水)9時~開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/35626</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>関西地方オトカリテ跡地にイオンモールの大型商業施設 2027年以降開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39391</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>東北地方スーパーセンタートライアル金ケ崎店 2026年9月16日(水)開業！15日(火)プレオープン！最新情報も！岩手県胆沢郡金ケ崎町にトライアルカンパニーの店舗「スーパーセンタートライアル金ケ崎店」が2026年9月16日(水)8：30グランドオープン！9月15日(火)10：00～19：00プレオープン！スーパーセンタートライアルが金ケ崎町に初出店！そ...2026.09.15東北地方</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/47232</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>関西地方ケーズデンキ桜井店 2026年9月17日(木)開業！最新情報も！奈良県桜井市に関西ケーズデンキの店舗「ケーズデンキ桜井店」が2026年9月17日(木)開業！ケーズデンキの大型店舗が、新たに誕生する桜井複合商業施設へ出店！隣接地にはコーナンPROも新設！そんな、ケーズデンキ桜井店について、テナントや開業日...2026.09.15関西地方</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49275</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>ヨドバシカメラ／「名鉄名古屋店」9月16日オープン、名鉄百貨店跡地に居ぬきで出店注目</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091544.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>明治屋／自由が丘ミューズスクエアに新店9月17日オープン、ギフト類・ワインも充実</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091571.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>ハンズ／自由が丘に4年ぶりの新店9月17日オープン、ギフト需要に対応</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091574.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>ららぽーと豊洲／9～10月8店舗新規・改装オープン、20周年記念でショップ別特典も</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>すし銚子丸／養殖魚メインの新業態「鮨Yasuke 潮彩 自由が丘店」9月17日オープン</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091572.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>三笠会館／自由が丘にイタリアンレストラン「AGIO」9月17日オープン、新メニュー導入</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091575.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>フォーシーズ／自由が丘ミューズスクエアに中華レストラン「香華園」9月17日オープン</t>
+        </is>
+      </c>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091573.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>カスミ／茨城県大洗町に「大洗店」9月18日オープン、セイブ食彩館大洗店を業態転換</t>
+        </is>
+      </c>
+      <c r="D842" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091542.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>クスリのアオキ／栃木県・新潟県・京都府に計3店舗、27年4～5月新設</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0915011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>CCC／スタバとの新業態3号店「SHARE LOUNGE 田町駅前」リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091577.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>ヤマダデンキ／群馬県太田市に「（仮称）Tecc LIFE SELECT太田高林店（店舗面積9364m2）」27年3月31日新設</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0915012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>自由が丘駅正面口／新ランドマーク「自由が丘ミューズスクエア」9月17日オープン注目</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091474.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>コスモス薬品／栃木県・大阪府に「ドラッグコスモス」計2店舗、27年4月新設</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0914011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>ジャック イン ザ ドーナツ／岡山市北区「イオンモール岡山店」9月18日オープン</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091473.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>ケーズデンキ／福岡県糟屋郡新宮町に「（仮称）福岡新宮店（店舗面積4015m2）」27年4月5日新設</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0914012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>まいばすけっと／「高幡不動駅北口店」「東淵野辺3丁目店」9月18日同時オープン</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091446.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>牛カツ京都勝牛／京都市伏見区に「伏見稲荷大社前店」オープン、大鳥居正面に出店</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091444.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>ホットランド／「銀だこハイボール酒場 渋谷センター街店」9月15日オープン</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091413.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>ゴンチャ／大阪市北区「エキマルシェ大阪店」9月18日オープン</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091472.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>2026年09月15日</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>ヤオコー／千葉県船橋市に「船橋薬円台店」9月15日オープン</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091116.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-16
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D854"/>
+  <dimension ref="A1:D954"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19204,6 +19204,2206 @@
         </is>
       </c>
     </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>トモズ 仙台一番町店</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>https://shop.tomods.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>元祖豚丼屋TONTON 山形大野目店</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>https://www.butadon-tonton.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>コメリハード＆グリーン酒田店</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>https://www.komeri.com/shop/storeSearch/StoreSelect.aspx?a_name=%E9%85%92%E7%94%B0%E5%B8%82&amp;p_code=06</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>すき家郡山富久山店</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>https://maps.sukiya.jp/jp/detail/396.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>カラオケCLUB DAM ピエロ諏訪店</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>https://karaokeclub.jp/shop/%E3%83%94%E3%82%A8%E3%83%AD%E8%AB%8F%E8%A8%AA%E5%BA%97/</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>9/16(9/15プレ)スーパーセンタートライアル金ケ崎店</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ghk</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>9/16エアウィーヴ FKDショッピングモール 宇都宮インターパーク店</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>https://airweave.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>ゆず庵 大宮本郷店</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>https://www.shabu-yuzuan.jp/shop/4224/</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>アエナ イオンモール羽生店</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>https://www.aena.co.jp/2023/02/13/4002/</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>Dr. Vranjes Kichijyoji</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>https://kichijoji.parco.jp/shop/detail/?cd=031620</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>おでんと釜たき飯 あおちょ 北千住店</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>https://buzzfoods.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>ラリック 玉川髙島屋店</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>https://jp.lalique.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>グランスタ東京 地下 丸の内改札内エリア</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>https://www.gransta.jp/news/info/marunouchi_sakarn/</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>PISOLA相模原小山店</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>https://pisola.jp/shop/sagamihara</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>アエナ イトーヨーカドー大船店</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>https://www.aena.co.jp/shop/</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>壱角家ジアウトレット湘南平塚店</t>
+        </is>
+      </c>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>https://gardengroup.co.jp/brand/ichikakuya/</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>すき家 7号新発田緑町店</t>
+        </is>
+      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>https://maps.sukiya.jp/jp/detail/6616.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>セブンイレブン大府吉田町６丁目</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>https://seven-eleven.areamarker.com/711map/info/565156?sej_nwshp=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>PLUSTA中津川</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>https://www.jr-plus.co.jp/store/239/</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>ヨドバシカメラ マルチメディア名鉄名古屋店</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>https://www.yodobashi.com/ec/support/news/260905336541/index.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>SANYO Style STORE PLUS イオンモール岡崎店</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr">
+        <is>
+          <t>https://store.sanyo-shokai.co.jp/blogs/news/baker-street-260916-sss-aeonmallokazaki</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>ウェルネス ハブ ストア ナゴヤ名古屋栄三越</t>
+        </is>
+      </c>
+      <c r="D876" t="inlineStr">
+        <is>
+          <t>https://www.mitsukoshi.mistore.jp/nagoya/event_calendar/renewal.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>9/18スーパーマーケットバロー矢田店</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ghC</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>サンドイッチハウス メルヘン ジェイアール京都伊勢丹店</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr">
+        <is>
+          <t>https://www.mistore.jp/store/kyoto/shops/foods/foods/shopnews_list/2026_b2shopnews8.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>ブルックス ブラザーズ ジェイアール京都伊勢丹店</t>
+        </is>
+      </c>
+      <c r="D879" t="inlineStr">
+        <is>
+          <t>https://www.mistore.jp/store/kyoto/event_calendar/irodorisai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>ムシベジプラスカフェ</t>
+        </is>
+      </c>
+      <c r="D880" t="inlineStr">
+        <is>
+          <t>https://www.tennoji-mio.co.jp/newshop?type=new</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>ファミリーマートESR尼崎／S店</t>
+        </is>
+      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>https://store.family.co.jp/new-open/points/81238</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>リンツ ショコラ ブティック 高松オルネ店</t>
+        </is>
+      </c>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>https://www.lindt.jp/contents/shop/5537/</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>Gente Selection 岩田屋本店</t>
+        </is>
+      </c>
+      <c r="D883" t="inlineStr">
+        <is>
+          <t>https://gentedimare.jp/news/news_20260902</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>9/1オーケー高槻赤大路店(大阪府高槻市)</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fOy</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>9/1 ライフ鎌倉梶原店</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fS5</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>9/3 サンディ吹田五月が丘店(大阪府吹田市)</t>
+        </is>
+      </c>
+      <c r="D886" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fPd</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>9/3改装 スーパーのアオキ直江津店(新潟県上越市)</t>
+        </is>
+      </c>
+      <c r="D887" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2v</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>9/3スギ薬局茜部南店(岐阜市)</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2N</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>9/4クックマート上西店（静岡県浜松市）</t>
+        </is>
+      </c>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7N</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>9/4(9/3プレ)スーパー生鮮館TAIGA桂子田店</t>
+        </is>
+      </c>
+      <c r="D890" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fZU</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>9/4改装 名古屋PARCO</t>
+        </is>
+      </c>
+      <c r="D891" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7c</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>9/4改装 メイチカ(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7g</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>9/4ウルフギャングステーキハウス名古屋店</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eZr</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>9/4 ゴジラ・ストア Nagoya</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fn6</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D909" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D910" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D911" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D912" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D913" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D914" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>関東地方みと好文テラス 2026年4月23日(木)開業！全11テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D915" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48066</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>関西地方うめきたグリーンプレイス 2025年3月21日(金)開業！全テナント20店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/24237</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>関東地方イオンタウン東浦和 2026年3月28日(土)開業！全22テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D917" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/29205</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>関東地方東京インテリア家具 八王子店が2026年6月5日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D918" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/46004</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>中国地方ハローズ宇部モール 2025年6月以降開業予定！ テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D919" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/42192</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>九州地方メガセンタートライアル荒尾店 2025年2月11日(火)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D920" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/39634</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>関東地方品川駅北口に新駅ビル 2031年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D921" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/33951</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>関東地方鎌倉梶原商業施設 2026年8月28日(金)より順次開業！ライフやカインズが出店！全4店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D922" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/43953</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>東北地方アネックスカワトク 2025年8月18日(月)で閉店 跡地はどうなる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D923" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/42658</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>九州地方ミーナ天神が建て替え検討！2030年代開業！どのような施設になる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D924" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/49546</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>関東地方ニトリ宇都宮インターパーク店 2025年6月20日(金)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D925" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/40136</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>関東地方プラウドタワー板橋 2027年秋開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D926" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26709</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>九州地方九州大学箱崎キャンパス跡地地区 2028年度より街びらき！商業施設も誕生！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D927" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/46612</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>九州地方新一日橋ショッピングセンター 2026年冬開業！30店舗が出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D928" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/45078</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>中部地方イオンスタイル黒埼 2025年3月18日(火)開業！全3テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D929" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/37860</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>中国地方ニトリ東岡山店 2025年12月5日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D930" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/42378</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>関西地方イオン五條店 跡地は複合施設と一体化へ！2029年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D931" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/43015</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>関東地方桜木駐車場用地活用事業 商業施設や結婚式場が2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D932" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/35670</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>中部地方イオンスタイル諏訪 2026年秋開業！テナントは？最新情報も！長野県諏訪郡下諏訪町の「イオン諏訪店」跡地に、イオンリテールの新商業施設「イオンスタイル諏訪」が2026年秋開業予定！平屋建ての「直営棟」と、2階建ての「専門店棟」のあわせて2棟が建設され、専門店棟の屋上には諏訪湖が望める展望デッキが設置さ...2026.09.16中部地方</t>
+        </is>
+      </c>
+      <c r="D933" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/36918</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>東北地方イオンモール伊達 2026年11月27日(金)9：00~開業！どのような施設に？テナント情報随時更新中！最新情報も！福島県伊達市にイオンモールの大型商業施設「イオンモール伊達」が2026年11月27日(金)9：00~グランドオープン！構想開始から実に31年！約17万㎡の広大な敷地に、核店舗「イオンスタイル伊達」をはじめ、東日本初となる大型アミューズメント...2026.09.16東北地方</t>
+        </is>
+      </c>
+      <c r="D934" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/17982</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>東京建物／川口市にNSC「ミナノバ」2号店オープン、2km商圏11万人の住宅地に出店注目</t>
+        </is>
+      </c>
+      <c r="D935" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091672.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>ヨドバシカメラ／体感できる売場で東海での認知度向上へ「名鉄名古屋店」オープン詳報</t>
+        </is>
+      </c>
+      <c r="D936" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091641.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>イオン／福島県に「イオンモール伊達」11月27日グランドオープン</t>
+        </is>
+      </c>
+      <c r="D937" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091620.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>イオンリテール／「イオンスタイル」をイオンモール伊達に11月27日オープン</t>
+        </is>
+      </c>
+      <c r="D938" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>オーケー／大阪8号店「長吉店」、9号店「下新庄店」27年2月オープン</t>
+        </is>
+      </c>
+      <c r="D939" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091618.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>ヤマダストアー／兵庫県宝塚市に「（仮称）宝塚市伊孑志計画（店舗面積3099m2）」27年3月1日新設</t>
+        </is>
+      </c>
+      <c r="D940" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0916011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>ドラッグストアモリ／宮城県仙台市に「（仮称）青葉区吉成店」27年3月28日新設</t>
+        </is>
+      </c>
+      <c r="D941" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0916012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>アットコスメストア／「京都河原町オーパ」に新店舗10月23日オープン、京都初出店</t>
+        </is>
+      </c>
+      <c r="D942" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091617.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>エコスグループ／栃木県小山市に「たいらや粟宮店」9月18日オープン</t>
+        </is>
+      </c>
+      <c r="D943" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091615.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>串カツ田中／津田沼駅北口エリアに「津田沼店」9月17日オープン</t>
+        </is>
+      </c>
+      <c r="D944" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091673.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>イオンモール福岡／コスメショップ「フルーツギャザリング」10月23日オープン</t>
+        </is>
+      </c>
+      <c r="D945" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091613.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>タワーレコード／渋谷に初の単独イベントスペース10月31日オープン</t>
+        </is>
+      </c>
+      <c r="D946" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091611.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>ヨドバシカメラ／「名鉄名古屋店」9月16日オープン、名鉄百貨店跡地に居ぬきで出店注目</t>
+        </is>
+      </c>
+      <c r="D947" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091544.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>明治屋／自由が丘ミューズスクエアに新店9月17日オープン、ギフト類・ワインも充実</t>
+        </is>
+      </c>
+      <c r="D948" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091571.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>ハンズ／自由が丘に4年ぶりの新店9月17日オープン、ギフト需要に対応</t>
+        </is>
+      </c>
+      <c r="D949" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091574.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>ららぽーと豊洲／9～10月8店舗新規・改装オープン、20周年記念でショップ別特典も</t>
+        </is>
+      </c>
+      <c r="D950" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>すし銚子丸／新業態「鮨Yasuke 潮彩 自由が丘店」9月17日オープン</t>
+        </is>
+      </c>
+      <c r="D951" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091572.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>三笠会館／自由が丘にイタリアンレストラン「AGIO」9月17日オープン、新メニュー導入</t>
+        </is>
+      </c>
+      <c r="D952" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091575.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>フォーシーズ／自由が丘ミューズスクエアに中華レストラン「香華園」9月17日オープン</t>
+        </is>
+      </c>
+      <c r="D953" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091573.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>2026年09月16日</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>カスミ／茨城県大洗町に「大洗店」9月18日オープン、セイブ食彩館大洗店を業態転換</t>
+        </is>
+      </c>
+      <c r="D954" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091542.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-17
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D954"/>
+  <dimension ref="A1:D1054"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21404,6 +21404,2206 @@
         </is>
       </c>
     </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>セブンイレブン伊勢崎中町店</t>
+        </is>
+      </c>
+      <c r="D955" t="inlineStr">
+        <is>
+          <t>https://ptj.sej.co.jp/arbeit/recruitment/jobfind-pc/job/All/1328787/</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>9/18カスミ大洗店(茨城県東茨城郡)</t>
+        </is>
+      </c>
+      <c r="D956" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1giA</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>資さんうどん児玉店</t>
+        </is>
+      </c>
+      <c r="D957" t="inlineStr">
+        <is>
+          <t>https://www.sukesanudon.com/map/page/4/</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>minanoba川口</t>
+        </is>
+      </c>
+      <c r="D958" t="inlineStr">
+        <is>
+          <t>https://minanoba-kawaguchi.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>鶏笑伊奈店</t>
+        </is>
+      </c>
+      <c r="D959" t="inlineStr">
+        <is>
+          <t>https://store.srsholdings.com/torisho/</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>pâtisserie BOSO SWEETS アトレ新浦安店</t>
+        </is>
+      </c>
+      <c r="D960" t="inlineStr">
+        <is>
+          <t>https://www.atre.co.jp/campaign/renewal/shin_urayasu/</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>串カツ田中津田沼店</t>
+        </is>
+      </c>
+      <c r="D961" t="inlineStr">
+        <is>
+          <t>https://restaurant.kushi-tanaka.com/detail/0248/</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>JIYUGAOKA MUSE SQUARE</t>
+        </is>
+      </c>
+      <c r="D962" t="inlineStr">
+        <is>
+          <t>https://jiyugaoka-muse-square.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>ジュエッテ玉川高島屋S・C店</t>
+        </is>
+      </c>
+      <c r="D963" t="inlineStr">
+        <is>
+          <t>https://www.takashimaya.co.jp/tamagawa/sc/new_shop/</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>NEWTRON</t>
+        </is>
+      </c>
+      <c r="D964" t="inlineStr">
+        <is>
+          <t>https://www.caretta.jp/shop/index/226</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>DESCENTE GINZA</t>
+        </is>
+      </c>
+      <c r="D965" t="inlineStr">
+        <is>
+          <t>https://store.descente.co.jp/descente/news/desginza260831/</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>ローソン上野御徒町</t>
+        </is>
+      </c>
+      <c r="D966" t="inlineStr">
+        <is>
+          <t>https://www.areamarker.com/lawson/info/388576</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>LUNA EARTHウィング上大岡店</t>
+        </is>
+      </c>
+      <c r="D967" t="inlineStr">
+        <is>
+          <t>https://endless-inc.jp/blogs/news/20260910</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>WithGreenジョイナス横浜店</t>
+        </is>
+      </c>
+      <c r="D968" t="inlineStr">
+        <is>
+          <t>https://www.sotetsu-joinus.com/pressrelease/10897</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>9/26ビッグ・エー春日部増富店</t>
+        </is>
+      </c>
+      <c r="D969" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gii</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>9/17明治屋自由が丘ストアー</t>
+        </is>
+      </c>
+      <c r="D970" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ga2</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>ローソン魚沼井口新田</t>
+        </is>
+      </c>
+      <c r="D971" t="inlineStr">
+        <is>
+          <t>https://www.areamarker.com/lawson/info/379790</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>9/17ロピア ムサシ新潟西店(新潟市)</t>
+        </is>
+      </c>
+      <c r="D972" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g6X</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>ローソン浜松砂山町</t>
+        </is>
+      </c>
+      <c r="D973" t="inlineStr">
+        <is>
+          <t>https://www.areamarker.com/lawson/info/387625</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>極味薬膳スープ 菜菜麻辣湯ららぽーと沼津店</t>
+        </is>
+      </c>
+      <c r="D974" t="inlineStr">
+        <is>
+          <t>https://mitsui-shopping-park.com/lalaport/numazu/openrenewal/index.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>すき家岡崎戸崎新町店</t>
+        </is>
+      </c>
+      <c r="D975" t="inlineStr">
+        <is>
+          <t>https://sukiya.jp/news/parts/news_store.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>ReDららぽーと愛知東郷店</t>
+        </is>
+      </c>
+      <c r="D976" t="inlineStr">
+        <is>
+          <t>https://mitsui-shopping-park.com/lalaport/togo/openrenewal/3612844.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>理容プラージュ長浜店</t>
+        </is>
+      </c>
+      <c r="D977" t="inlineStr">
+        <is>
+          <t>https://www.plage-bb.co.jp/barber/store/10842</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>パン工房カワ岸和田和泉店</t>
+        </is>
+      </c>
+      <c r="D978" t="inlineStr">
+        <is>
+          <t>https://bakery.e-kawa.co.jp/event/</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>ケーズデンキ桜井店</t>
+        </is>
+      </c>
+      <c r="D979" t="inlineStr">
+        <is>
+          <t>https://www.ksdenki.co.jp/store/detail/?prefectureCode=29&amp;code=4256</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>サンディ芦屋店</t>
+        </is>
+      </c>
+      <c r="D980" t="inlineStr">
+        <is>
+          <t>https://www.sundi.co.jp/shop/details-ashiya.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>アエナアルパーク店</t>
+        </is>
+      </c>
+      <c r="D981" t="inlineStr">
+        <is>
+          <t>https://www.aena.co.jp/2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>出雲ロフト</t>
+        </is>
+      </c>
+      <c r="D982" t="inlineStr">
+        <is>
+          <t>https://www.loft.co.jp/shop_list/detail.php?shop_id=671</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>9/17マックスバリュ長崎住吉店</t>
+        </is>
+      </c>
+      <c r="D983" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gia</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>9/1オーケー高槻赤大路店(大阪府高槻市)</t>
+        </is>
+      </c>
+      <c r="D984" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fOy</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>9/1 ライフ鎌倉梶原店</t>
+        </is>
+      </c>
+      <c r="D985" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fS5</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>9/3 サンディ吹田五月が丘店(大阪府吹田市)</t>
+        </is>
+      </c>
+      <c r="D986" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fPd</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>9/3改装 スーパーのアオキ直江津店(新潟県上越市)</t>
+        </is>
+      </c>
+      <c r="D987" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2v</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>9/3スギ薬局茜部南店(岐阜市)</t>
+        </is>
+      </c>
+      <c r="D988" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2N</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>9/4クックマート上西店（静岡県浜松市）</t>
+        </is>
+      </c>
+      <c r="D989" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7N</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>9/4(9/3プレ)スーパー生鮮館TAIGA桂子田店</t>
+        </is>
+      </c>
+      <c r="D990" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fZU</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>9/4改装 名古屋PARCO</t>
+        </is>
+      </c>
+      <c r="D991" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7c</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>9/4改装 メイチカ(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D992" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7g</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>9/4ウルフギャングステーキハウス名古屋店</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eZr</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>9/4 ゴジラ・ストア Nagoya</t>
+        </is>
+      </c>
+      <c r="D994" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fn6</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D995" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D996" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D998" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1000" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1001" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1004" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>関西地方フレスポ桜井が増床リニューアル！2026年3月6日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/43982</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>関西地方淀屋橋ステーションワン 2025年6月23日(月)に開業！テナント13店舗一覧！どのような建物に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1016" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/26225</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>中部地方ASTY岡崎 JR岡崎駅東口商業施設 2026年6月11日(木)10:00開業！7店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/43451</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>関東地方minanoba相模原（ミナノバ相模原） 2025年3月5日(水)開業！全11テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/35264</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>関西地方イオンタウン平野跡地に商業施設 2027年冬開業！ テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1019" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/42949</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>関東地方ベルク平塚田村店 2026年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1020" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47482</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>関西地方大阪・万博公園に大型アリーナや商業施設の再開発！2030年夏街びらき！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1021" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/33469</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>九州地方OHASHI HILL ゆめアール大橋跡地に2025年4月18日(金)先行開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/27364</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>関西地方イオンスタイル大津京 一旦閉店し建て替えて2028年開業！分譲マンションとの一体開発！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1023" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/35154</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>中部地方ニトリ鈴鹿中央通り店 2025年12月12日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1024" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/44303</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>関西地方六甲バター稲美工場跡地にマルアイが進出！2027年6月開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1025" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/43853</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>関西地方京都プロジェクト(仮称) 京都中央郵便局が建て替え！2029年度開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1026" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/22581</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>中部地方富士駅北口第一地区市街地再開発事業 2030年初頭開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1027" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/26250</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>関西地方そよら三田フラワータウン 2027年春開業！フローラ88 跡地 テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39680</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>北海道地方札幌4丁目プレイス 4PLA 2025年4月25日(金)から順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1029" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/32449</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>関東地方板橋駅西口地区市街地再開発事業 2029年10月完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1030" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26695</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>九州地方アクロスプラザ篠栗 2025年春グランドオープン！全10テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1031" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/38349</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>中部地方スーパーセンタートライアル本巣店 2026年7月22日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1032" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/45851</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>中部地方イオンスタイル諏訪 2026年秋開業！テナントは？最新情報も！長野県諏訪郡下諏訪町の「イオン諏訪店」跡地に、イオンリテールの新商業施設「イオンスタイル諏訪」が2026年秋開業予定！平屋建ての「直営棟」と、2階建ての「専門店棟」のあわせて2棟が建設され、専門店棟の屋上には諏訪湖が望める展望デッキが設置さ...2026.09.16中部地方</t>
+        </is>
+      </c>
+      <c r="D1033" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/36918</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>東北地方イオンモール伊達 2026年11月27日(金)9：00~開業！どのような施設に？テナント情報随時更新中！最新情報も！福島県伊達市にイオンモールの大型商業施設「イオンモール伊達」が2026年11月27日(金)9：00~グランドオープン！構想開始から実に31年！約17万㎡の広大な敷地に、核店舗「イオンスタイル伊達」をはじめ、東日本初となる大型アミューズメント...2026.09.16東北地方</t>
+        </is>
+      </c>
+      <c r="D1034" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/17982</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>マミーマート／「生鮮市場TOP！川口柳崎店」オープン、足元商圏のファミリー層狙う注目</t>
+        </is>
+      </c>
+      <c r="D1035" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091771.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>そごう広島店／コスメ売場をリニューアルし面積1.4倍に、フレグランス強化</t>
+        </is>
+      </c>
+      <c r="D1036" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091716.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>心斎橋パルコ／9～10月、セガの関西エリア初の旗艦店など3店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1037" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091721.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>コジマ×ビックカメラ／「minanoba川口店」オープン、子連れ客向け商品展開</t>
+        </is>
+      </c>
+      <c r="D1038" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091775.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>CCC／スタバとの複合店「SHARE LOUNGE 自由が丘ミューズスクエア」オープン</t>
+        </is>
+      </c>
+      <c r="D1039" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091776.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>アクタス／自由が丘にインテリアグリーンとカフェ複合の新業態店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1040" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091777.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>ライフ／大阪市中央区に「ビオラル淀屋橋ゲートタワー」12月2日オープン</t>
+        </is>
+      </c>
+      <c r="D1041" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091713.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>ドラッグストアモリ／山口県下松市に「下松美里町店」27年4月22日新設</t>
+        </is>
+      </c>
+      <c r="D1042" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0917012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>カインズ／リフォーム専門小型店「カインズリフォーム」小田急百貨店町田店にオープン</t>
+        </is>
+      </c>
+      <c r="D1043" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091714.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>パンチョ／新業態「ごちそうスープパスタ」東京・代々木に10月2日オープン</t>
+        </is>
+      </c>
+      <c r="D1044" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091718.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>コーナン商事／静岡県に「（仮称）コーナンPRO清水七ツ新屋店」27年3月24日新設</t>
+        </is>
+      </c>
+      <c r="D1045" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0917011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>東京建物／川口市にNSC「ミナノバ」2号店オープン、2km商圏11万人の住宅地に出店注目</t>
+        </is>
+      </c>
+      <c r="D1046" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091672.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>ヨドバシカメラ／体感できる売場で東海での認知度向上へ「名鉄名古屋店」オープン詳報</t>
+        </is>
+      </c>
+      <c r="D1047" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091641.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>イオン／福島県に「イオンモール伊達」11月27日グランドオープン</t>
+        </is>
+      </c>
+      <c r="D1048" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091620.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>イオンリテール／「イオンスタイル」をイオンモール伊達に11月27日オープン</t>
+        </is>
+      </c>
+      <c r="D1049" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>オーケー／大阪8号店「長吉店」、9号店「下新庄店」27年2月オープン</t>
+        </is>
+      </c>
+      <c r="D1050" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091618.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>ヤマダストアー／兵庫県宝塚市に「（仮称）宝塚市伊孑志計画（店舗面積3099m2）」27年3月1日新設</t>
+        </is>
+      </c>
+      <c r="D1051" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0916011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>ドラッグストアモリ／宮城県仙台市に「（仮称）青葉区吉成店」27年3月28日新設</t>
+        </is>
+      </c>
+      <c r="D1052" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0916012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>アットコスメストア／「京都河原町オーパ」に新店舗10月23日オープン、京都初出店</t>
+        </is>
+      </c>
+      <c r="D1053" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091617.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="inlineStr">
+        <is>
+          <t>2026年09月17日</t>
+        </is>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
+        <is>
+          <t>エコスグループ／栃木県小山市に「たいらや粟宮店」9月18日オープン</t>
+        </is>
+      </c>
+      <c r="D1054" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091615.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-18
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1054"/>
+  <dimension ref="A1:D1154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23604,6 +23604,2206 @@
         </is>
       </c>
     </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>9/18カスミ大洗店(茨城県東茨城郡)</t>
+        </is>
+      </c>
+      <c r="D1055" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1giA</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>9/18スーパーマーケットバロー矢田店</t>
+        </is>
+      </c>
+      <c r="D1056" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ghC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>9/1オーケー高槻赤大路店(大阪府高槻市)</t>
+        </is>
+      </c>
+      <c r="D1057" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fOy</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>9/1 ライフ鎌倉梶原店</t>
+        </is>
+      </c>
+      <c r="D1058" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fS5</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>9/3 サンディ吹田五月が丘店(大阪府吹田市)</t>
+        </is>
+      </c>
+      <c r="D1059" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fPd</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>9/3改装 スーパーのアオキ直江津店(新潟県上越市)</t>
+        </is>
+      </c>
+      <c r="D1060" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2v</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>9/3スギ薬局茜部南店(岐阜市)</t>
+        </is>
+      </c>
+      <c r="D1061" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2N</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>9/4クックマート上西店（静岡県浜松市）</t>
+        </is>
+      </c>
+      <c r="D1062" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7N</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>9/4(9/3プレ)スーパー生鮮館TAIGA桂子田店</t>
+        </is>
+      </c>
+      <c r="D1063" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fZU</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>9/4改装 名古屋PARCO</t>
+        </is>
+      </c>
+      <c r="D1064" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7c</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>9/4改装 メイチカ(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D1065" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7g</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>9/4ウルフギャングステーキハウス名古屋店</t>
+        </is>
+      </c>
+      <c r="D1066" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eZr</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>9/4 ゴジラ・ストア Nagoya</t>
+        </is>
+      </c>
+      <c r="D1067" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fn6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>9/4ロピア彦根ナフコ店</t>
+        </is>
+      </c>
+      <c r="D1068" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fNK</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>(9/8ソフト)9/11そよら津桜橋(三重県津市)</t>
+        </is>
+      </c>
+      <c r="D1069" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1bV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>9/9MARUAI BIG アクロスプラザ高砂店</t>
+        </is>
+      </c>
+      <c r="D1070" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gbn</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>9/10もとまちユニオン大船店</t>
+        </is>
+      </c>
+      <c r="D1071" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gfg</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>9/10改装 マルナカ檀紙店(香川県高松市)</t>
+        </is>
+      </c>
+      <c r="D1072" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7X</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>9/10ザ・ビッグエクスプレスみよし店</t>
+        </is>
+      </c>
+      <c r="D1073" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>9/10ファミリーマート中津川下野店</t>
+        </is>
+      </c>
+      <c r="D1074" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g84</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>9/10とりせん田沼インター店(栃木県)</t>
+        </is>
+      </c>
+      <c r="D1075" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9g</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>9/10TOFROM YAESU TOWER(東京都)</t>
+        </is>
+      </c>
+      <c r="D1076" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ged</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>9/10業務スーパー船場本町店</t>
+        </is>
+      </c>
+      <c r="D1077" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gdW</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>9/10業務スーパー津山山北店(岡山県)</t>
+        </is>
+      </c>
+      <c r="D1078" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ge1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>9/10ラ・ムー飯塚花瀬店(福岡県)</t>
+        </is>
+      </c>
+      <c r="D1079" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ge8</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>9/10マックスバリュ城栄店(長崎市)</t>
+        </is>
+      </c>
+      <c r="D1080" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gel</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>9/11スーパーマーケットバロー豊中島江店</t>
+        </is>
+      </c>
+      <c r="D1081" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fXN</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>9/11ザ・ビッグ厚別店</t>
+        </is>
+      </c>
+      <c r="D1082" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9V</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>9/15ヤオコー船橋薬円台店</t>
+        </is>
+      </c>
+      <c r="D1083" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ggO</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>9/16(9/15プレ)スーパーセンタートライアル金ケ崎店</t>
+        </is>
+      </c>
+      <c r="D1084" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ghk</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>9/16SANYO Style STORE PLUS イオンモール岡崎店</t>
+        </is>
+      </c>
+      <c r="D1085" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fEw</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>9/17ロピア ムサシ新潟西店(新潟市)</t>
+        </is>
+      </c>
+      <c r="D1086" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g6X</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>9/17明治屋自由が丘ストアー</t>
+        </is>
+      </c>
+      <c r="D1087" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ga2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>9/17マックスバリュ長崎住吉店</t>
+        </is>
+      </c>
+      <c r="D1088" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>9/26ビッグ・エー春日部増富店</t>
+        </is>
+      </c>
+      <c r="D1089" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gii</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D1090" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D1091" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D1092" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D1093" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D1094" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1095" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1096" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1097" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1098" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1099" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1100" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1101" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1102" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1103" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1104" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1105" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1106" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1107" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1108" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1109" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1110" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1111" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1112" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1113" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1114" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>九州地方LAプラザ ランドアーク島瀬 マックスバリュ佐世保島瀬店 2026年5月14日(木)9:00~開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1115" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/39475</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>中部地方イオンモール須坂 2025年10月3日(金)開業！全テナント166店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1116" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/11811</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>関西地方なんばアリーナ計画 2032年以降開業！商業施設も併設！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1117" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/48499</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>関東地方上板橋駅南口駅前東地区市街地再開発事業 2028年完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1118" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48931</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>関西地方ブライトステラ摂津千里丘 2027年春開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1119" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/16990</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>関東地方北青山三丁目地区市街地再開発事業 2029年完成！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1120" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/41322</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>関西地方コストコ箕面倉庫店 2027年夏開業！大阪府北部初出店！場所は？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1121" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/35667</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>東北地方スーパーセンタートライアル石巻店 2026年7月1日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1122" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/44362</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>中国地方岩国駅前南地区市街地再開発事業 2030年春以降開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1123" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/24871</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>関東地方マミーマート 見沼区東新井 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1124" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47301</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>関東地方ららテラス北綾瀬 北綾瀬駅前に2025年6月24日(火)開業！全テナント51店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1125" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26173</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>中部地方トライアルスマート西尾一色店 2026年3月25日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1126" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/44433</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>東北地方ニトリいわき店(仮称) 2026年9月開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1127" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/48631</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>九州地方三井アウトレットパーク福岡 2027年春開業！200店舗が出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1128" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/38113</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>関西地方ブランズタワー西宮 2027年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1129" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/23230</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>九州地方スーパーセンタートライアルうきは店 2026年11月下旬に開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1130" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/49325</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>関東地方赤坂トラストタワー 商業施設 2026年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1131" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/28300</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>関東地方イオンモール取手(仮称)2028年以降開業予定！どのような商業施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1132" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/22797</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>中部地方イオンスタイル諏訪 2026年秋開業！テナントは？最新情報も！長野県諏訪郡下諏訪町の「イオン諏訪店」跡地に、イオンリテールの新商業施設「イオンスタイル諏訪」が2026年秋開業予定！平屋建ての「直営棟」と、2階建ての「専門店棟」のあわせて2棟が建設され、専門店棟の屋上には諏訪湖が望める展望デッキが設置さ...2026.09.16中部地方</t>
+        </is>
+      </c>
+      <c r="D1133" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/36918</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>東北地方イオンモール伊達 2026年11月27日(金)9：00~開業！どのような施設に？テナント情報随時更新中！最新情報も！福島県伊達市にイオンモールの大型商業施設「イオンモール伊達」が2026年11月27日(金)9：00~グランドオープン！構想開始から実に31年！約17万㎡の広大な敷地に、核店舗「イオンスタイル伊達」をはじめ、東日本初となる大型アミューズメント...2026.09.16東北地方</t>
+        </is>
+      </c>
+      <c r="D1134" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/17982</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>イオンモール／京都・四条河原町「河原町オーパ」9月19日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1135" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091841.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>新宿マルイ アネックス／1階フロアを大幅リニューアル、多彩なコンテンツを集積</t>
+        </is>
+      </c>
+      <c r="D1136" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091744.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>カインズ／長野県上田市に「上田国分店」今秋オープン、農業資材・ペット用品充実</t>
+        </is>
+      </c>
+      <c r="D1137" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091873.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>有明ガーデン／「ペタリアフラワー」「チチカカ」新規オープン、国内外のニーズに対応</t>
+        </is>
+      </c>
+      <c r="D1138" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091871.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>ラルズ／札幌市「ビッグハウスウエスト」9月18日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1139" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091814.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>コーナン商事／兵庫県姫路市に「（仮称）コーナンPRO姫路飾磨店（店舗面積2089m2）」27年4月1日新設</t>
+        </is>
+      </c>
+      <c r="D1140" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0918012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>ゼビオ／富山県に「スーパースポーツゼビオ アクロスプラザ富山掛尾店」オープン</t>
+        </is>
+      </c>
+      <c r="D1141" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091877.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>クリエイトSD／群馬県太田市に「（仮称）太田本町店」27年3月30日新設</t>
+        </is>
+      </c>
+      <c r="D1142" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0918011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>ホームセンターバロー／愛知県に「プロサイトみよし店」10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D1143" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091879.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>DCM／奈良県にプロの職人向け専門店「ホダカ奈良橿原店」オープン</t>
+        </is>
+      </c>
+      <c r="D1144" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091878.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>イオンモール津田沼 South／イベントスペース「ハチステ supported by 明治安田」9月26日オープン</t>
+        </is>
+      </c>
+      <c r="D1145" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091813.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>ノジマ／埼玉県草加市に「草加セーモンプラザ店」オープン</t>
+        </is>
+      </c>
+      <c r="D1146" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091842.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>Zoff／長野県「イオン上田ショッピングセンター」に新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091874.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>松屋フーズ／東京・千葉に「すし松」9月下旬に2店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1148" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091875.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>ゴンチャ／神奈川県「イオンモール座間」に新店舗9月25日オープン</t>
+        </is>
+      </c>
+      <c r="D1149" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091876.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>マミーマート／「生鮮市場TOP！川口柳崎店」オープン、足元商圏のファミリー層狙う注目</t>
+        </is>
+      </c>
+      <c r="D1150" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091771.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>そごう広島店／コスメ売場をリニューアルし面積1.4倍に、フレグランス強化</t>
+        </is>
+      </c>
+      <c r="D1151" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091716.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>心斎橋パルコ／9～10月、セガの関西エリア初の旗艦店など3店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1152" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091721.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>コジマ×ビックカメラ／「minanoba川口店」オープン、子連れ客向け商品展開</t>
+        </is>
+      </c>
+      <c r="D1153" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091775.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>2026年09月18日</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>CCC／スタバとの複合店「SHARE LOUNGE 自由が丘ミューズスクエア」オープン</t>
+        </is>
+      </c>
+      <c r="D1154" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091776.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-19
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1154"/>
+  <dimension ref="A1:D1254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25804,6 +25804,2206 @@
         </is>
       </c>
     </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>9/1オーケー高槻赤大路店(大阪府高槻市)</t>
+        </is>
+      </c>
+      <c r="D1155" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fOy</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>9/1 ライフ鎌倉梶原店</t>
+        </is>
+      </c>
+      <c r="D1156" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fS5</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>9/3 サンディ吹田五月が丘店(大阪府吹田市)</t>
+        </is>
+      </c>
+      <c r="D1157" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fPd</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>9/3改装 スーパーのアオキ直江津店(新潟県上越市)</t>
+        </is>
+      </c>
+      <c r="D1158" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2v</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>9/3スギ薬局茜部南店(岐阜市)</t>
+        </is>
+      </c>
+      <c r="D1159" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2N</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>9/4クックマート上西店（静岡県浜松市）</t>
+        </is>
+      </c>
+      <c r="D1160" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7N</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>9/4(9/3プレ)スーパー生鮮館TAIGA桂子田店</t>
+        </is>
+      </c>
+      <c r="D1161" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fZU</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>9/4改装 名古屋PARCO</t>
+        </is>
+      </c>
+      <c r="D1162" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7c</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>9/4改装 メイチカ(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D1163" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7g</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>9/4ウルフギャングステーキハウス名古屋店</t>
+        </is>
+      </c>
+      <c r="D1164" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eZr</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>9/4 ゴジラ・ストア Nagoya</t>
+        </is>
+      </c>
+      <c r="D1165" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fn6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>9/4ロピア彦根ナフコ店</t>
+        </is>
+      </c>
+      <c r="D1166" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fNK</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>(9/8ソフト)9/11そよら津桜橋(三重県津市)</t>
+        </is>
+      </c>
+      <c r="D1167" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1bV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>9/9MARUAI BIG アクロスプラザ高砂店</t>
+        </is>
+      </c>
+      <c r="D1168" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gbn</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>9/10もとまちユニオン大船店</t>
+        </is>
+      </c>
+      <c r="D1169" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gfg</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>9/10改装 マルナカ檀紙店(香川県高松市)</t>
+        </is>
+      </c>
+      <c r="D1170" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7X</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>9/10ザ・ビッグエクスプレスみよし店</t>
+        </is>
+      </c>
+      <c r="D1171" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>9/10ファミリーマート中津川下野店</t>
+        </is>
+      </c>
+      <c r="D1172" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g84</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>9/10とりせん田沼インター店(栃木県)</t>
+        </is>
+      </c>
+      <c r="D1173" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9g</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>9/10TOFROM YAESU TOWER(東京都)</t>
+        </is>
+      </c>
+      <c r="D1174" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ged</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>9/10業務スーパー船場本町店</t>
+        </is>
+      </c>
+      <c r="D1175" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gdW</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>9/10業務スーパー津山山北店(岡山県)</t>
+        </is>
+      </c>
+      <c r="D1176" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ge1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>9/10ラ・ムー飯塚花瀬店(福岡県)</t>
+        </is>
+      </c>
+      <c r="D1177" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ge8</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>9/10マックスバリュ城栄店(長崎市)</t>
+        </is>
+      </c>
+      <c r="D1178" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gel</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>9/11スーパーマーケットバロー豊中島江店</t>
+        </is>
+      </c>
+      <c r="D1179" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fXN</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>9/11ザ・ビッグ厚別店</t>
+        </is>
+      </c>
+      <c r="D1180" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9V</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>9/15ヤオコー船橋薬円台店</t>
+        </is>
+      </c>
+      <c r="D1181" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ggO</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>9/16(9/15プレ)スーパーセンタートライアル金ケ崎店</t>
+        </is>
+      </c>
+      <c r="D1182" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ghk</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>9/16SANYO Style STORE PLUS イオンモール岡崎店</t>
+        </is>
+      </c>
+      <c r="D1183" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fEw</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>9/17ロピア ムサシ新潟西店(新潟市)</t>
+        </is>
+      </c>
+      <c r="D1184" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g6X</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>9/17明治屋自由が丘ストアー</t>
+        </is>
+      </c>
+      <c r="D1185" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ga2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>9/17マックスバリュ長崎住吉店</t>
+        </is>
+      </c>
+      <c r="D1186" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>9/18スーパーマーケットバロー矢田店</t>
+        </is>
+      </c>
+      <c r="D1187" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ghC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>9/18カスミ大洗店(茨城県東茨城郡)</t>
+        </is>
+      </c>
+      <c r="D1188" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1giA</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>9/26ビッグ・エー春日部増富店</t>
+        </is>
+      </c>
+      <c r="D1189" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gii</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D1190" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D1191" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D1192" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D1193" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D1194" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1195" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1196" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1197" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1198" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1199" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1200" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1200" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1201" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1201" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1202" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1202" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1203" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1203" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1204" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1204" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1205" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1206" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1207" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1208" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1209" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1210" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1211" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1212" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1213" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1214" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>中国地方広島駅ビル「minamoa（ミナモア）」2025年3月24日(月)開業！全220テナント公開！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1215" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/7700</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>九州地方ポートタウン門司港 AMAZING SPOT 2026年7月24日(金)開業！全9テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1216" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/48751</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>中部地方イチビル イチ＊ビル 2025年11月27日(木)~順次開業！全40店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1217" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/31747</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>中部地方富士駅北口第一地区市街地再開発事業 2030年初頭開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1218" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/26250</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>関東地方築地地区まちづくり事業 築地市場跡地 2030年代半ば開業！どのような施設になる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1219" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49238</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>関東地方イオン北浦和店 2025年9月30日(火)閉店 跡地はどうなる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1220" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/46169</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>中部地方三島駅南口東街区Ａ地区市街地再開発事業 2027年竣工予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1221" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/25890</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>関東地方イオン海老名店 2026年5月中旬で一旦閉店し建て替えへ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1222" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47523</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>関東地方取手駅西口A街区市街地再開発事業 2031年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1223" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/22823</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>中部地方デンソー池田工場跡地 日本エスコンが商業施設を計画！2027年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1224" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/39672</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>関東地方ケーズデンキ コーナン 桜井複合商業施設(仮称) 2026年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1225" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/45945</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>北海道地方札幌駅・パセオ跡地 高架下商業施設 2028年冬開業！200店舗が出店へ！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1226" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/43941</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>関西地方平和堂大久保店 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1227" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49605</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>関西地方GLION ARENA KOBE・TOTTEI PARKが 2025年4月4日(金)開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1228" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/33025</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>関東地方エキュート秋葉原 2025年4月7日(月)10時~開業！全24テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1229" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42906</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>関西地方そよら小野 2027年秋開業！イオン小野店跡地 21店舗が出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1230" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/43512</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>関東地方JR武蔵境駅東側開発 2028年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1231" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48480</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>関西地方フォレストモール泉南 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1232" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/48647</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>関西地方ケーズデンキ桜井店 2026年9月17日(木)開業！最新情報も！奈良県桜井市に関西ケーズデンキの店舗「ケーズデンキ桜井店」が2026年9月17日(木)開業！ケーズデンキの大型店舗が、新たに誕生する桜井複合商業施設へ出店！隣接地にはコーナンPROも新設！そんな、ケーズデンキ桜井店について、テナントや開業日...2026.09.19関西地方</t>
+        </is>
+      </c>
+      <c r="D1233" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49275</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>関東地方ニトリ川崎高津店(仮称) 2027年夏開業予定！最新情報も！神奈川県川崎市にニトリの店舗「ニトリ川崎高津店(仮称)」が2027年夏開業予定！県道9号線沿い、「ラウンドワン 高津店」跡地に出店する店舗となります！そんな、ニトリ川崎高津店について、テナントや開業日などを見ていきましょう！2026年1月2...2026.09.19関東地方</t>
+        </is>
+      </c>
+      <c r="D1234" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47017</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>イオンモール／京都・四条河原町「河原町オーパ」9月19日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1235" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091841.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>新宿マルイ アネックス／1階フロアを大幅リニューアル、多彩なコンテンツを集積</t>
+        </is>
+      </c>
+      <c r="D1236" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091744.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>カインズ／長野県上田市に「上田国分店」今秋オープン、農業資材・ペット用品充実</t>
+        </is>
+      </c>
+      <c r="D1237" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091873.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>有明ガーデン／「ペタリアフラワー」「チチカカ」新規オープン、国内外のニーズに対応</t>
+        </is>
+      </c>
+      <c r="D1238" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091871.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>ラルズ／札幌市「ビッグハウスウエスト」9月18日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1239" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091814.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>コーナン商事／兵庫県姫路市に「（仮称）コーナンPRO姫路飾磨店（店舗面積2089m2）」27年4月1日新設</t>
+        </is>
+      </c>
+      <c r="D1240" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0918012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>ゼビオ／富山県に「スーパースポーツゼビオ アクロスプラザ富山掛尾店」オープン</t>
+        </is>
+      </c>
+      <c r="D1241" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091877.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>クリエイトSD／群馬県太田市に「（仮称）太田本町店」27年3月30日新設</t>
+        </is>
+      </c>
+      <c r="D1242" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0918011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>ホームセンターバロー／愛知県に「プロサイトみよし店」10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D1243" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091879.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>DCM／奈良県にプロの職人向け専門店「ホダカ奈良橿原店」オープン</t>
+        </is>
+      </c>
+      <c r="D1244" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091878.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>イオンモール津田沼 South／イベントスペース「ハチステ supported by 明治安田」9月26日オープン</t>
+        </is>
+      </c>
+      <c r="D1245" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091813.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>ノジマ／埼玉県草加市に「草加セーモンプラザ店」オープン</t>
+        </is>
+      </c>
+      <c r="D1246" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091842.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>Zoff／長野県「イオン上田ショッピングセンター」に新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1247" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091874.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>松屋フーズ／東京・千葉に「すし松」9月下旬に2店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1248" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091875.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>ゴンチャ／神奈川県「イオンモール座間」に新店舗9月25日オープン</t>
+        </is>
+      </c>
+      <c r="D1249" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091876.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>マミーマート／「生鮮市場TOP！川口柳崎店」オープン、足元商圏のファミリー層狙う注目</t>
+        </is>
+      </c>
+      <c r="D1250" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091771.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>そごう広島店／コスメ売場をリニューアルし面積1.4倍に、フレグランス強化</t>
+        </is>
+      </c>
+      <c r="D1251" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091716.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>心斎橋パルコ／9～10月、セガの関西エリア初の旗艦店など3店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1252" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091721.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>コジマ×ビックカメラ／「minanoba川口店」オープン、子連れ客向け商品展開</t>
+        </is>
+      </c>
+      <c r="D1253" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091775.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr">
+        <is>
+          <t>2026年09月19日</t>
+        </is>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>CCC／スタバとの複合店「SHARE LOUNGE 自由が丘ミューズスクエア」オープン</t>
+        </is>
+      </c>
+      <c r="D1254" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091776.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-20
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1254"/>
+  <dimension ref="A1:D1320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28004,6 +28004,1458 @@
         </is>
       </c>
     </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D1255" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D1256" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D1257" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D1258" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D1259" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D1260" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1261" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1262" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1263" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1264" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1265" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1265" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1266" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1266" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1267" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1268" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1268" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1269" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1269" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1270" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1271" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1272" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1273" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1274" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1275" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1276" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1277" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1278" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1279" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1280" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>東北地方【電力ビル】一番町三丁目七番地区市街地再開発事業 2029年開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1281" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/31239</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>中国地方カミハチクロス 2027年度開業！アンダーズ広島が進出！商業施設も！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1282" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/27582</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>関東地方飯田橋駅東地区市街地再開発事業 2032年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1283" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/28149</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>関東地方minanoba川口 2026年9月17日(金)開業！全10テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1284" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42094</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>関東地方ハーモニーヒルズパーク入間 ベルクと屋上公園 2028年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1285" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/45967</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>関東地方平井テラス(プラウドタワー平井) 2025年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1286" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/19549</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>九州地方糸満市真栄里地区商業施設 2028年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1287" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/47815</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>関東地方ファスタ小岩 2026年3月17日(火)開業！テナント随時更新中！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1288" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/19980</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>中部地方マックスバリュ豊橋西幸町店 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1289" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48626</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>中国地方ニトリ東岡山店 2025年12月5日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1290" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/42378</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>関東地方グラン8モール 2025年8月28日(木)より順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1291" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42179</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>中国地方ケーズデンキ岩国店 2025年8月28日(木)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1292" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/42381</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>関東地方宮益坂地区市街地再開発事業 2031年秋完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1293" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/28157</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>関東地方高崎駅東口栄町地区市街地再開発事業 2029年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1294" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/29079</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>九州地方YAEYAMA GATE 石垣市役所跡地 2030年開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1295" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/33011</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>関東地方太田駅南口再開発 ベルクの複合商業施設 2026年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1296" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47305</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>関東地方立石駅南口西地区市街地再開発事業 2031年度完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1297" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/31932</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>関東地方みと好文テラス 2026年4月23日(木)開業！全11テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1298" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48066</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>関西地方ケーズデンキ桜井店 2026年9月17日(木)開業！最新情報も！奈良県桜井市に関西ケーズデンキの店舗「ケーズデンキ桜井店」が2026年9月17日(木)開業！ケーズデンキの大型店舗が、新たに誕生する桜井複合商業施設へ出店！隣接地にはコーナンPROも新設！そんな、ケーズデンキ桜井店について、テナントや開業日...2026.09.19関西地方</t>
+        </is>
+      </c>
+      <c r="D1299" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49275</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>関東地方ニトリ川崎高津店(仮称) 2027年夏開業予定！最新情報も！神奈川県川崎市にニトリの店舗「ニトリ川崎高津店(仮称)」が2027年夏開業予定！県道9号線沿い、「ラウンドワン 高津店」跡地に出店する店舗となります！そんな、ニトリ川崎高津店について、テナントや開業日などを見ていきましょう！2026年1月2...2026.09.19関東地方</t>
+        </is>
+      </c>
+      <c r="D1300" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47017</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>イオンモール／京都・四条河原町「河原町オーパ」9月19日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1301" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091841.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>新宿マルイ アネックス／1階フロアを大幅リニューアル、多彩なコンテンツを集積</t>
+        </is>
+      </c>
+      <c r="D1302" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091744.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>カインズ／長野県上田市に「上田国分店」今秋オープン、農業資材・ペット用品充実</t>
+        </is>
+      </c>
+      <c r="D1303" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091873.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>有明ガーデン／「ペタリアフラワー」「チチカカ」新規オープン、国内外のニーズに対応</t>
+        </is>
+      </c>
+      <c r="D1304" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091871.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>ラルズ／札幌市「ビッグハウスウエスト」9月18日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1305" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091814.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>コーナン商事／兵庫県姫路市に「（仮称）コーナンPRO姫路飾磨店（店舗面積2089m2）」27年4月1日新設</t>
+        </is>
+      </c>
+      <c r="D1306" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0918012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>ゼビオ／富山県に「スーパースポーツゼビオ アクロスプラザ富山掛尾店」オープン</t>
+        </is>
+      </c>
+      <c r="D1307" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091877.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>クリエイトSD／群馬県太田市に「（仮称）太田本町店」27年3月30日新設</t>
+        </is>
+      </c>
+      <c r="D1308" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0918011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>ホームセンターバロー／愛知県に「プロサイトみよし店」10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D1309" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091879.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>DCM／奈良県にプロの職人向け専門店「ホダカ奈良橿原店」オープン</t>
+        </is>
+      </c>
+      <c r="D1310" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091878.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>イオンモール津田沼 South／イベントスペース「ハチステ supported by 明治安田」9月26日オープン</t>
+        </is>
+      </c>
+      <c r="D1311" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091813.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>ノジマ／埼玉県草加市に「草加セーモンプラザ店」オープン</t>
+        </is>
+      </c>
+      <c r="D1312" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091842.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>Zoff／長野県「イオン上田ショッピングセンター」に新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1313" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091874.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>松屋フーズ／東京・千葉に「すし松」9月下旬に2店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1314" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091875.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>ゴンチャ／神奈川県「イオンモール座間」に新店舗9月25日オープン</t>
+        </is>
+      </c>
+      <c r="D1315" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091876.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>マミーマート／「生鮮市場TOP！川口柳崎店」オープン、足元商圏のファミリー層狙う注目</t>
+        </is>
+      </c>
+      <c r="D1316" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091771.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>そごう広島店／コスメ売場をリニューアルし面積1.4倍に、フレグランス強化</t>
+        </is>
+      </c>
+      <c r="D1317" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091716.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>心斎橋パルコ／9～10月、セガの関西エリア初の旗艦店など3店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1318" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091721.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr">
+        <is>
+          <t>コジマ×ビックカメラ／「minanoba川口店」オープン、子連れ客向け商品展開</t>
+        </is>
+      </c>
+      <c r="D1319" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091775.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr">
+        <is>
+          <t>2026年09月20日</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>CCC／スタバとの複合店「SHARE LOUNGE 自由が丘ミューズスクエア」オープン</t>
+        </is>
+      </c>
+      <c r="D1320" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091776.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-21
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1320"/>
+  <dimension ref="A1:D1380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29456,6 +29456,1326 @@
         </is>
       </c>
     </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1321" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1322" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1323" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1324" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1325" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1326" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1327" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1328" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1329" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1330" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1331" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1332" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1333" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1334" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1335" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1336" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1337" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1338" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1339" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1340" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr">
+        <is>
+          <t>関西地方イオンタウンあびこ駅前 2026年4月25日(土)開業！全18テナント一覧！</t>
+        </is>
+      </c>
+      <c r="D1341" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/42396</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>九州地方西日本シティビル 2026年7月21日(火)開業！全5テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1342" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/20689</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>関西地方針T・R・S（針テラス）イオンモールの商業施設へ！どのような施設になる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1343" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/48753</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>東北地方イオンスタイル山王 2025年3月20日(木)開業！無印良品も出店へ！全8テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1344" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/37974</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr">
+        <is>
+          <t>四国地方イオン坂出店 2024年2月29日(木)に閉店し建て替えへ！跡地はどうなる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1345" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/shikoku/34197</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr">
+        <is>
+          <t>関東地方みなとみらい21中央地区60・61街区開発事業 2029年春開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1346" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36914</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1347" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1347" t="inlineStr">
+        <is>
+          <t>関東地方新宿駅西南口開発計画(仮称)【北街区】 2040年代開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1347" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/24819</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1348" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1348" t="inlineStr">
+        <is>
+          <t>関東地方ケーズデンキ コーナン 桜井複合商業施設(仮称) 2026年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1348" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/45945</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1349" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1349" t="inlineStr">
+        <is>
+          <t>関東地方MARK IS 葛飾かなまち 2025年9月3日(水)開業！全テナント50店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1349" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/17267</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1350" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1350" t="inlineStr">
+        <is>
+          <t>中国地方ゆめモール山陽 2025年6月12日(木)開業！全14テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1350" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/35608</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1351" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1351" t="inlineStr">
+        <is>
+          <t>九州地方新一日橋ショッピングセンター 2026年冬開業！30店舗が出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1351" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/45078</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1352" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1352" t="inlineStr">
+        <is>
+          <t>東北地方スーパーセンタートライアル錦ケ丘店 2025年5月21日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1352" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/40364</t>
+        </is>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1353" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1353" t="inlineStr">
+        <is>
+          <t>関西地方GLION ARENA KOBE・TOTTEI PARKが 2025年4月4日(金)開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1353" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/33025</t>
+        </is>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1354" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1354" t="inlineStr">
+        <is>
+          <t>中国地方ケーズデンキ山口店(仮称) 2026年秋開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1354" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/44477</t>
+        </is>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1355" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1355" t="inlineStr">
+        <is>
+          <t>関東地方BASEGATE（ベースゲート）横浜関内 2026年3月19日(木)開業！全65店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1355" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/11753</t>
+        </is>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1356" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1356" t="inlineStr">
+        <is>
+          <t>関東地方ゆりストア百合丘本店 建て替え 2025年3月開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1356" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42337</t>
+        </is>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1357" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1357" t="inlineStr">
+        <is>
+          <t>関東地方ニトリふじみ野店 2026年10月開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1357" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48589</t>
+        </is>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1358" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1358" t="inlineStr">
+        <is>
+          <t>九州地方フレスポジャングルパークがリニューアル！2027年夏開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1358" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/42280</t>
+        </is>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1359" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1359" t="inlineStr">
+        <is>
+          <t>関東地方太田駅南口再開発 ベルクの複合商業施設 2026年秋開業！テナントは？最新情報も！群馬県太田市の太田駅南口の、旧ドン・キホーテ太田店跡地にて行われている再開発事業「太田駅南口第三地区第一種市街地再開発事業」の商業棟にベルクの複合商業施設が2026年秋開業！太田駅前に食品スーパーマーケットのベルクが初出店！（ベルク太田駅前...2026.09.21関東地方</t>
+        </is>
+      </c>
+      <c r="D1359" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47305</t>
+        </is>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1360" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1360" t="inlineStr">
+        <is>
+          <t>関東地方ベルク平塚田村店 2026年秋開業！テナントは？最新情報も！神奈川県平塚市の相模小学校跡地にベルクのスーパーマーケット「ベルク平塚田村店」が2026年秋開業！平塚市に食品スーパーマーケットのベルクが初出店！そんな、ベルク平塚田村店についてテナントや求人情報についていろいろ見ていきたいと思います。是非...2026.09.21関東地方</t>
+        </is>
+      </c>
+      <c r="D1360" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47482</t>
+        </is>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1361" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1361" t="inlineStr">
+        <is>
+          <t>イオンモール／京都・四条河原町「河原町オーパ」9月19日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1361" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091841.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1362" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1362" t="inlineStr">
+        <is>
+          <t>新宿マルイ アネックス／1階フロアを大幅リニューアル、多彩なコンテンツを集積</t>
+        </is>
+      </c>
+      <c r="D1362" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091744.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1363" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1363" t="inlineStr">
+        <is>
+          <t>カインズ／長野県上田市に「上田国分店」今秋オープン、農業資材・ペット用品充実</t>
+        </is>
+      </c>
+      <c r="D1363" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091873.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1364" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1364" t="inlineStr">
+        <is>
+          <t>有明ガーデン／「ペタリアフラワー」「チチカカ」新規オープン、国内外のニーズに対応</t>
+        </is>
+      </c>
+      <c r="D1364" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091871.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1365" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1365" t="inlineStr">
+        <is>
+          <t>ラルズ／札幌市「ビッグハウスウエスト」9月18日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1365" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091814.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1366" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1366" t="inlineStr">
+        <is>
+          <t>コーナン商事／兵庫県姫路市に「（仮称）コーナンPRO姫路飾磨店（店舗面積2089m2）」27年4月1日新設</t>
+        </is>
+      </c>
+      <c r="D1366" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0918012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1367" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1367" t="inlineStr">
+        <is>
+          <t>ゼビオ／富山県に「スーパースポーツゼビオ アクロスプラザ富山掛尾店」オープン</t>
+        </is>
+      </c>
+      <c r="D1367" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091877.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1368" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1368" t="inlineStr">
+        <is>
+          <t>クリエイトSD／群馬県太田市に「（仮称）太田本町店」27年3月30日新設</t>
+        </is>
+      </c>
+      <c r="D1368" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0918011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1369" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1369" t="inlineStr">
+        <is>
+          <t>ホームセンターバロー／愛知県に「プロサイトみよし店」10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D1369" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091879.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1370" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1370" t="inlineStr">
+        <is>
+          <t>DCM／奈良県にプロの職人向け専門店「ホダカ奈良橿原店」オープン</t>
+        </is>
+      </c>
+      <c r="D1370" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091878.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1371" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1371" t="inlineStr">
+        <is>
+          <t>イオンモール津田沼 South／イベントスペース「ハチステ supported by 明治安田」9月26日オープン</t>
+        </is>
+      </c>
+      <c r="D1371" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091813.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1372" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1372" t="inlineStr">
+        <is>
+          <t>ノジマ／埼玉県草加市に「草加セーモンプラザ店」オープン</t>
+        </is>
+      </c>
+      <c r="D1372" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091842.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1373" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1373" t="inlineStr">
+        <is>
+          <t>Zoff／長野県「イオン上田ショッピングセンター」に新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1373" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091874.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1374" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1374" t="inlineStr">
+        <is>
+          <t>松屋フーズ／東京・千葉に「すし松」9月下旬に2店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1374" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091875.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1375" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1375" t="inlineStr">
+        <is>
+          <t>ゴンチャ／神奈川県「イオンモール座間」に新店舗9月25日オープン</t>
+        </is>
+      </c>
+      <c r="D1375" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091876.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1376" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1376" t="inlineStr">
+        <is>
+          <t>マミーマート／「生鮮市場TOP！川口柳崎店」オープン、足元商圏のファミリー層狙う注目</t>
+        </is>
+      </c>
+      <c r="D1376" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091771.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1377" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1377" t="inlineStr">
+        <is>
+          <t>そごう広島店／コスメ売場をリニューアルし面積1.4倍に、フレグランス強化</t>
+        </is>
+      </c>
+      <c r="D1377" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091716.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1378" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1378" t="inlineStr">
+        <is>
+          <t>心斎橋パルコ／9～10月、セガの関西エリア初の旗艦店など3店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1378" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091721.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1379" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1379" t="inlineStr">
+        <is>
+          <t>コジマ×ビックカメラ／「minanoba川口店」オープン、子連れ客向け商品展開</t>
+        </is>
+      </c>
+      <c r="D1379" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091775.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="inlineStr">
+        <is>
+          <t>2026年09月21日</t>
+        </is>
+      </c>
+      <c r="B1380" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1380" t="inlineStr">
+        <is>
+          <t>CCC／スタバとの複合店「SHARE LOUNGE 自由が丘ミューズスクエア」オープン</t>
+        </is>
+      </c>
+      <c r="D1380" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091776.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-22
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1380"/>
+  <dimension ref="A1:D1447"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30776,6 +30776,1480 @@
         </is>
       </c>
     </row>
+    <row r="1381">
+      <c r="A1381" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1381" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1381" t="inlineStr">
+        <is>
+          <t>MY SUITCASE 札幌店</t>
+        </is>
+      </c>
+      <c r="D1381" t="inlineStr">
+        <is>
+          <t>https://repair-suitcase.com/shop/sapporo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1382" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1382" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D1382" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1383" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1383" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D1383" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1384" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1384" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D1384" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1385" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1385" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D1385" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1386" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D1386" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1387" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1387" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D1387" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1388" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1388" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1388" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1389" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1389" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1389" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1390" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1390" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1390" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1391" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1391" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1391" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1392" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1392" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1392" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1393" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1393" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1393" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1394" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1394" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1394" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1395" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1395" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1395" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1396" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1396" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1396" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1397" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1397" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1397" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1398" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1398" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1398" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1399" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1399" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1399" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1400" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1400" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1400" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1401" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1401" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1401" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1402" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1402" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1402" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1403" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1403" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1403" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1404" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1404" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1404" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1405" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1405" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1405" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1406" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1406" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1406" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1407" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1407" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1407" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1408" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1408" t="inlineStr">
+        <is>
+          <t>中部地方ライフガーデン中津川が2025年9月19日(金)より順次オープン！出店予定のテナントや場所を詳しく解説</t>
+        </is>
+      </c>
+      <c r="D1408" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/42932</t>
+        </is>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1409" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1409" t="inlineStr">
+        <is>
+          <t>関東地方HIBIYA CROSSPARK（日比谷クロスパーク）2029年春街びらき！2037年全体開業！どのような街に？</t>
+        </is>
+      </c>
+      <c r="D1409" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/24411</t>
+        </is>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1410" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1410" t="inlineStr">
+        <is>
+          <t>中部地方そよら津桜橋 イオン津SC跡地 2026年9月11日(金)開業！全テナント一覧！</t>
+        </is>
+      </c>
+      <c r="D1410" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/36891</t>
+        </is>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1411" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1411" t="inlineStr">
+        <is>
+          <t>四国地方湊町三丁目C街区市街地再開発事業 2028年度開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1411" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/shikoku/12204</t>
+        </is>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1412" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1412" t="inlineStr">
+        <is>
+          <t>関東地方霞が関・虎ノ門地区再開発ビル 2036年度開業予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1412" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47596</t>
+        </is>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1413" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1413" t="inlineStr">
+        <is>
+          <t>東北地方イオン仙台店 跡地に複合ビル建設へ 2029年度開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1413" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/40539</t>
+        </is>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1414" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1414" t="inlineStr">
+        <is>
+          <t>関東地方ベルク平塚田村店 2026年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1414" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47482</t>
+        </is>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1415" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1415" t="inlineStr">
+        <is>
+          <t>関東地方MARK IS 葛飾かなまち 2025年9月3日(水)開業！全テナント50店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1415" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/17267</t>
+        </is>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1416" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1416" t="inlineStr">
+        <is>
+          <t>関東地方ららテラス川口 2025年5月31日(土)開業！全94店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1416" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/33965</t>
+        </is>
+      </c>
+    </row>
+    <row r="1417">
+      <c r="A1417" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1417" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1417" t="inlineStr">
+        <is>
+          <t>関東地方W シティタワーズ 蕨駅西口地区市街地再開発事業 2027年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1417" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/16952</t>
+        </is>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1418" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1418" t="inlineStr">
+        <is>
+          <t>中部地方ベルク町田相原店 2026年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1418" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/47130</t>
+        </is>
+      </c>
+    </row>
+    <row r="1419">
+      <c r="A1419" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1419" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1419" t="inlineStr">
+        <is>
+          <t>中部地方トライアルスマート西尾一色店 2026年3月25日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1419" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/44433</t>
+        </is>
+      </c>
+    </row>
+    <row r="1420">
+      <c r="A1420" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1420" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1420" t="inlineStr">
+        <is>
+          <t>北海道地方MEGAドン・キホーテ北見店 イトーヨーカドー北見店跡地 2026年6月16日(火)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1420" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/36861</t>
+        </is>
+      </c>
+    </row>
+    <row r="1421">
+      <c r="A1421" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1421" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1421" t="inlineStr">
+        <is>
+          <t>中部地方イオンセントラルスクエア静岡 2026年3月6日(金)開業！アピタ静岡店跡地 全41店舗一覧！</t>
+        </is>
+      </c>
+      <c r="D1421" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/42340</t>
+        </is>
+      </c>
+    </row>
+    <row r="1422">
+      <c r="A1422" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1422" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1422" t="inlineStr">
+        <is>
+          <t>関東地方多磨駅前に三井不動産の大型商業施設 2029年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1422" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/37871</t>
+        </is>
+      </c>
+    </row>
+    <row r="1423">
+      <c r="A1423" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1423" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1423" t="inlineStr">
+        <is>
+          <t>関東地方明治安田新宿ビル 2026年11月下旬以降開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1423" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26240</t>
+        </is>
+      </c>
+    </row>
+    <row r="1424">
+      <c r="A1424" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1424" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1424" t="inlineStr">
+        <is>
+          <t>北海道地方tonarie（トナリエ）北広島 2025年3月15日(土)開業！全テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1424" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/21566</t>
+        </is>
+      </c>
+    </row>
+    <row r="1425">
+      <c r="A1425" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1425" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1425" t="inlineStr">
+        <is>
+          <t>関東地方イオン石岡店が建て替えへ！2028年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1425" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/45661</t>
+        </is>
+      </c>
+    </row>
+    <row r="1426">
+      <c r="A1426" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1426" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1426" t="inlineStr">
+        <is>
+          <t>関東地方大塚駅南口地区市街地再開発事業 2032年度完成予定！どのような施設に？最新情報も！東京都豊島区のJR山手線・都電荒川線「大塚駅」南口駅前に、東京建物・住友不動産が参画する超高層複合タワー「大塚駅南口地区市街地再開発事業」が2032年度に完成予定！JR大塚駅南口の駅前広場・サンモール大塚商店街入口一帯（約0.5ha）を一体...2026.09.22関東地方</t>
+        </is>
+      </c>
+      <c r="D1426" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49692</t>
+        </is>
+      </c>
+    </row>
+    <row r="1427">
+      <c r="A1427" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1427" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1427" t="inlineStr">
+        <is>
+          <t>関西地方スーパーセンタートライアル高砂曽根店が開業予定！最新情報も！兵庫県高砂市にトライアルカンパニーの店舗「スーパーセンタートライアル高砂曽根店」が開業予定！スーパーセンタートライアルが高砂市に初出店！そんな、スーパーセンタートライアル高砂曽根店について、テナントや開業日などを見ていきましょう！2026年...2026.09.22関西地方</t>
+        </is>
+      </c>
+      <c r="D1427" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49019</t>
+        </is>
+      </c>
+    </row>
+    <row r="1428">
+      <c r="A1428" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1428" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1428" t="inlineStr">
+        <is>
+          <t>イオンモール／京都・四条河原町「河原町オーパ」9月19日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1428" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091841.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1429">
+      <c r="A1429" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1429" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1429" t="inlineStr">
+        <is>
+          <t>新宿マルイ アネックス／1階フロアを大幅リニューアル、多彩なコンテンツを集積</t>
+        </is>
+      </c>
+      <c r="D1429" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091744.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1430">
+      <c r="A1430" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1430" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1430" t="inlineStr">
+        <is>
+          <t>カインズ／長野県上田市に「上田国分店」今秋オープン、農業資材・ペット用品充実</t>
+        </is>
+      </c>
+      <c r="D1430" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091873.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1431">
+      <c r="A1431" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1431" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1431" t="inlineStr">
+        <is>
+          <t>有明ガーデン／「ペタリアフラワー」「チチカカ」新規オープン、国内外のニーズに対応</t>
+        </is>
+      </c>
+      <c r="D1431" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091871.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1432">
+      <c r="A1432" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1432" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1432" t="inlineStr">
+        <is>
+          <t>ラルズ／札幌市「ビッグハウスウエスト」9月18日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1432" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091814.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1433">
+      <c r="A1433" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1433" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1433" t="inlineStr">
+        <is>
+          <t>コーナン商事／兵庫県姫路市に「（仮称）コーナンPRO姫路飾磨店（店舗面積2089m2）」27年4月1日新設</t>
+        </is>
+      </c>
+      <c r="D1433" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0918012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1434">
+      <c r="A1434" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1434" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1434" t="inlineStr">
+        <is>
+          <t>ゼビオ／富山県に「スーパースポーツゼビオ アクロスプラザ富山掛尾店」オープン</t>
+        </is>
+      </c>
+      <c r="D1434" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091877.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1435">
+      <c r="A1435" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1435" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1435" t="inlineStr">
+        <is>
+          <t>クリエイトSD／群馬県太田市に「（仮称）太田本町店」27年3月30日新設</t>
+        </is>
+      </c>
+      <c r="D1435" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0918011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1436">
+      <c r="A1436" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1436" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1436" t="inlineStr">
+        <is>
+          <t>ホームセンターバロー／愛知県に「プロサイトみよし店」10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D1436" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091879.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1437">
+      <c r="A1437" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1437" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1437" t="inlineStr">
+        <is>
+          <t>DCM／奈良県にプロの職人向け専門店「ホダカ奈良橿原店」オープン</t>
+        </is>
+      </c>
+      <c r="D1437" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091878.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1438">
+      <c r="A1438" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1438" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1438" t="inlineStr">
+        <is>
+          <t>イオンモール津田沼 South／イベントスペース「ハチステ supported by 明治安田」9月26日オープン</t>
+        </is>
+      </c>
+      <c r="D1438" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091813.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1439">
+      <c r="A1439" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1439" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1439" t="inlineStr">
+        <is>
+          <t>ノジマ／埼玉県草加市に「草加セーモンプラザ店」オープン</t>
+        </is>
+      </c>
+      <c r="D1439" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091842.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1440">
+      <c r="A1440" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1440" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1440" t="inlineStr">
+        <is>
+          <t>Zoff／長野県「イオン上田ショッピングセンター」に新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1440" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091874.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1441">
+      <c r="A1441" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1441" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1441" t="inlineStr">
+        <is>
+          <t>松屋フーズ／東京・千葉に「すし松」9月下旬に2店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1441" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091875.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1442">
+      <c r="A1442" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1442" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1442" t="inlineStr">
+        <is>
+          <t>ゴンチャ／神奈川県「イオンモール座間」に新店舗9月25日オープン</t>
+        </is>
+      </c>
+      <c r="D1442" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091876.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1443">
+      <c r="A1443" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1443" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1443" t="inlineStr">
+        <is>
+          <t>マミーマート／「生鮮市場TOP！川口柳崎店」オープン、足元商圏のファミリー層狙う注目</t>
+        </is>
+      </c>
+      <c r="D1443" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091771.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1444" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1444" t="inlineStr">
+        <is>
+          <t>そごう広島店／コスメ売場をリニューアルし面積1.4倍に、フレグランス強化</t>
+        </is>
+      </c>
+      <c r="D1444" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091716.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1445" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1445" t="inlineStr">
+        <is>
+          <t>心斎橋パルコ／9～10月、セガの関西エリア初の旗艦店など3店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1445" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091721.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1446">
+      <c r="A1446" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1446" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1446" t="inlineStr">
+        <is>
+          <t>コジマ×ビックカメラ／「minanoba川口店」オープン、子連れ客向け商品展開</t>
+        </is>
+      </c>
+      <c r="D1446" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091775.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" t="inlineStr">
+        <is>
+          <t>2026年09月22日</t>
+        </is>
+      </c>
+      <c r="B1447" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1447" t="inlineStr">
+        <is>
+          <t>CCC／スタバとの複合店「SHARE LOUNGE 自由が丘ミューズスクエア」オープン</t>
+        </is>
+      </c>
+      <c r="D1447" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091776.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-23
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1447"/>
+  <dimension ref="A1:D1518"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32250,6 +32250,1568 @@
         </is>
       </c>
     </row>
+    <row r="1448">
+      <c r="A1448" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1448" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1448" t="inlineStr">
+        <is>
+          <t>9/24カネスエ上ノ町店(愛知県春日井市)</t>
+        </is>
+      </c>
+      <c r="D1448" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gmT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1449">
+      <c r="A1449" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1449" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1449" t="inlineStr">
+        <is>
+          <t>はま寿司 岡崎戸崎新町店</t>
+        </is>
+      </c>
+      <c r="D1449" t="inlineStr">
+        <is>
+          <t>https://www.hama-sushi.co.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1450">
+      <c r="A1450" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1450" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1450" t="inlineStr">
+        <is>
+          <t>9/16ヤオマサ富水店(神奈川県小田原市)</t>
+        </is>
+      </c>
+      <c r="D1450" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gmA</t>
+        </is>
+      </c>
+    </row>
+    <row r="1451">
+      <c r="A1451" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1451" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1451" t="inlineStr">
+        <is>
+          <t>9/17 サンディ芦屋店</t>
+        </is>
+      </c>
+      <c r="D1451" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gaR</t>
+        </is>
+      </c>
+    </row>
+    <row r="1452">
+      <c r="A1452" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1452" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1452" t="inlineStr">
+        <is>
+          <t>9/19生鮮市場ダイイチ蒲田店(東京都大田区)</t>
+        </is>
+      </c>
+      <c r="D1452" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gmO</t>
+        </is>
+      </c>
+    </row>
+    <row r="1453">
+      <c r="A1453" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1453" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1453" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D1453" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="1454">
+      <c r="A1454" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1454" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1454" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D1454" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="1455">
+      <c r="A1455" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1455" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1455" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D1455" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1456" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1456" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D1456" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1457" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1457" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D1457" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1458" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1458" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D1458" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1459" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1459" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1459" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1460" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1460" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1460" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1461" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1461" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1461" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1462" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1462" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1462" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1463" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1463" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1463" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1464">
+      <c r="A1464" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1464" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1464" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1464" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1465" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1465" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1465" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1466">
+      <c r="A1466" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1466" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1466" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1466" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1467" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1467" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1467" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1468" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1468" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1468" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1469" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1469" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1469" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1470" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1470" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1470" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1471" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1471" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1471" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1472">
+      <c r="A1472" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1472" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1472" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1472" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1473">
+      <c r="A1473" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1473" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1473" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1473" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1474">
+      <c r="A1474" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1474" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1474" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1474" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1475">
+      <c r="A1475" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1475" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1475" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1475" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1476">
+      <c r="A1476" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1476" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1476" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1476" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1477">
+      <c r="A1477" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1477" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1477" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1477" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1478">
+      <c r="A1478" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1478" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1478" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1478" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1479">
+      <c r="A1479" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1479" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1479" t="inlineStr">
+        <is>
+          <t>関西地方神戸三宮TWINGATE（ツインゲート） 2028年春開業予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1479" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/25375</t>
+        </is>
+      </c>
+    </row>
+    <row r="1480">
+      <c r="A1480" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1480" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1480" t="inlineStr">
+        <is>
+          <t>中部地方ロピアモール滝ノ水 2026年5月21日(木)開業！全7テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1480" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48558</t>
+        </is>
+      </c>
+    </row>
+    <row r="1481">
+      <c r="A1481" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1481" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1481" t="inlineStr">
+        <is>
+          <t>関東地方SHIKANISHI Terrace 鹿西テラス(ベルクス足立鹿浜店) 2026年3月19日(木)~順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1481" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/31997</t>
+        </is>
+      </c>
+    </row>
+    <row r="1482">
+      <c r="A1482" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1482" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1482" t="inlineStr">
+        <is>
+          <t>関東地方ららテラス北綾瀬 北綾瀬駅前に2025年6月24日(火)開業！全テナント51店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1482" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26173</t>
+        </is>
+      </c>
+    </row>
+    <row r="1483">
+      <c r="A1483" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1483" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1483" t="inlineStr">
+        <is>
+          <t>関東地方霞が関・虎ノ門地区再開発ビル 2036年度開業予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1483" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47596</t>
+        </is>
+      </c>
+    </row>
+    <row r="1484">
+      <c r="A1484" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1484" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1484" t="inlineStr">
+        <is>
+          <t>中国地方スーパーセンタートライアル勝央店 2027年1月下旬に開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1484" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/47478</t>
+        </is>
+      </c>
+    </row>
+    <row r="1485">
+      <c r="A1485" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1485" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1485" t="inlineStr">
+        <is>
+          <t>九州地方レイリア春日原 2026年6月11日(木)開業！全10店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1485" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/38672</t>
+        </is>
+      </c>
+    </row>
+    <row r="1486">
+      <c r="A1486" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1486" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1486" t="inlineStr">
+        <is>
+          <t>関東地方大宮駅西口第3-A･D地区市街地再開発事業 2031年以降開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1486" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/16908</t>
+        </is>
+      </c>
+    </row>
+    <row r="1487">
+      <c r="A1487" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1487" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1487" t="inlineStr">
+        <is>
+          <t>関西地方大阪マルビル建替プロジェクト 商業施設 2030年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1487" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/41182</t>
+        </is>
+      </c>
+    </row>
+    <row r="1488">
+      <c r="A1488" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1488" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1488" t="inlineStr">
+        <is>
+          <t>中国地方スーパーセンタートライアル山口小郡店 2026年11月上旬開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1488" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/49136</t>
+        </is>
+      </c>
+    </row>
+    <row r="1489">
+      <c r="A1489" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1489" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1489" t="inlineStr">
+        <is>
+          <t>関東地方北小金駅南口東地区市街地再開発事業 2028年度完成 テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1489" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49735</t>
+        </is>
+      </c>
+    </row>
+    <row r="1490">
+      <c r="A1490" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1490" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1490" t="inlineStr">
+        <is>
+          <t>四国地方スーパーセンタートライアル三木店 2025年7月16日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1490" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/shikoku/41508</t>
+        </is>
+      </c>
+    </row>
+    <row r="1491">
+      <c r="A1491" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1491" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1491" t="inlineStr">
+        <is>
+          <t>中部地方富士モータースポーツフォレストテラス 2026年6月5日(金)先行開業！5店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1491" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/44714</t>
+        </is>
+      </c>
+    </row>
+    <row r="1492">
+      <c r="A1492" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1492" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1492" t="inlineStr">
+        <is>
+          <t>関西地方ヤマイチGARDEN桜井 マツゲンが出店！2025年11月21日(金)~順次開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1492" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39875</t>
+        </is>
+      </c>
+    </row>
+    <row r="1493">
+      <c r="A1493" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1493" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1493" t="inlineStr">
+        <is>
+          <t>関東地方JR武蔵境駅東側開発 2028年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1493" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48480</t>
+        </is>
+      </c>
+    </row>
+    <row r="1494">
+      <c r="A1494" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1494" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1494" t="inlineStr">
+        <is>
+          <t>関西地方豊中市立庄内さくら学園中学校跡地 複合商業施設 2028年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1494" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/46363</t>
+        </is>
+      </c>
+    </row>
+    <row r="1495">
+      <c r="A1495" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1495" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1495" t="inlineStr">
+        <is>
+          <t>関西地方ハローズ本多聞店 2026年6月24日(水)から順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1495" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/46204</t>
+        </is>
+      </c>
+    </row>
+    <row r="1496">
+      <c r="A1496" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1496" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1496" t="inlineStr">
+        <is>
+          <t>関東地方スーパーセンタートライアル山武成東店 2026年5月20日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1496" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/46150</t>
+        </is>
+      </c>
+    </row>
+    <row r="1497">
+      <c r="A1497" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1497" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1497" t="inlineStr">
+        <is>
+          <t>中部地方名古屋競馬場跡地に日本エスコンの複合商業施設 2029年開業予定！テナントは？最新情報も！愛知県名古屋市港区のあおなみ線「港北駅」東側に広がる旧名古屋競馬場跡地に、中部電力・日本エスコンなどが手掛ける大型複合商業施設「(仮称)名古屋競馬場跡地複合商業施設」が2029年頃に開業予定！バンテリンドーム約4個分（約20.7ha）におよ...2026.09.23中部地方</t>
+        </is>
+      </c>
+      <c r="D1497" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/49742</t>
+        </is>
+      </c>
+    </row>
+    <row r="1498">
+      <c r="A1498" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1498" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1498" t="inlineStr">
+        <is>
+          <t>関東地方上大岡C北地区第一種市街地再開発事業 2034年度完成予定！テナントは？最新情報も！神奈川県横浜市港南区の京急本線・横浜市営地下鉄ブルーライン「上大岡駅」西口駅前に、京浜急行電鉄・大林組が参画する超高層複合タワー「上大岡C北地区第一種市街地再開発事業」が2034年度完成予定！「富士ショッピングセンター」やパサージュ上大岡周...2026.09.23関東地方</t>
+        </is>
+      </c>
+      <c r="D1498" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49754</t>
+        </is>
+      </c>
+    </row>
+    <row r="1499">
+      <c r="A1499" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1499" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1499" t="inlineStr">
+        <is>
+          <t>イオンモール／京都・四条河原町「河原町オーパ」9月19日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1499" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091841.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1500">
+      <c r="A1500" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1500" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1500" t="inlineStr">
+        <is>
+          <t>新宿マルイ アネックス／1階フロアを大幅リニューアル、多彩なコンテンツを集積</t>
+        </is>
+      </c>
+      <c r="D1500" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091744.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1501">
+      <c r="A1501" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1501" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1501" t="inlineStr">
+        <is>
+          <t>カインズ／長野県上田市に「上田国分店」今秋オープン、農業資材・ペット用品充実</t>
+        </is>
+      </c>
+      <c r="D1501" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091873.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1502">
+      <c r="A1502" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1502" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1502" t="inlineStr">
+        <is>
+          <t>有明ガーデン／「ペタリアフラワー」「チチカカ」新規オープン、国内外のニーズに対応</t>
+        </is>
+      </c>
+      <c r="D1502" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091871.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1503">
+      <c r="A1503" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1503" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1503" t="inlineStr">
+        <is>
+          <t>ラルズ／札幌市「ビッグハウスウエスト」9月18日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1503" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091814.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1504">
+      <c r="A1504" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1504" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1504" t="inlineStr">
+        <is>
+          <t>コーナン商事／兵庫県姫路市に「（仮称）コーナンPRO姫路飾磨店（店舗面積2089m2）」27年4月1日新設</t>
+        </is>
+      </c>
+      <c r="D1504" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0918012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1505">
+      <c r="A1505" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1505" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1505" t="inlineStr">
+        <is>
+          <t>ゼビオ／富山県に「スーパースポーツゼビオ アクロスプラザ富山掛尾店」オープン</t>
+        </is>
+      </c>
+      <c r="D1505" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091877.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1506">
+      <c r="A1506" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1506" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1506" t="inlineStr">
+        <is>
+          <t>クリエイトSD／群馬県太田市に「（仮称）太田本町店」27年3月30日新設</t>
+        </is>
+      </c>
+      <c r="D1506" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0918011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1507">
+      <c r="A1507" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1507" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1507" t="inlineStr">
+        <is>
+          <t>ホームセンターバロー／愛知県に「プロサイトみよし店」10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D1507" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091879.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1508">
+      <c r="A1508" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1508" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1508" t="inlineStr">
+        <is>
+          <t>DCM／奈良県にプロの職人向け専門店「ホダカ奈良橿原店」オープン</t>
+        </is>
+      </c>
+      <c r="D1508" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091878.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1509">
+      <c r="A1509" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1509" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1509" t="inlineStr">
+        <is>
+          <t>イオンモール津田沼 South／イベントスペース「ハチステ supported by 明治安田」9月26日オープン</t>
+        </is>
+      </c>
+      <c r="D1509" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091813.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1510">
+      <c r="A1510" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1510" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1510" t="inlineStr">
+        <is>
+          <t>ノジマ／埼玉県草加市に「草加セーモンプラザ店」オープン</t>
+        </is>
+      </c>
+      <c r="D1510" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091842.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1511">
+      <c r="A1511" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1511" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1511" t="inlineStr">
+        <is>
+          <t>Zoff／長野県「イオン上田ショッピングセンター」に新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1511" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091874.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1512">
+      <c r="A1512" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1512" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1512" t="inlineStr">
+        <is>
+          <t>松屋フーズ／東京・千葉に「すし松」9月下旬に2店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1512" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091875.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1513">
+      <c r="A1513" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1513" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1513" t="inlineStr">
+        <is>
+          <t>ゴンチャ／神奈川県「イオンモール座間」に新店舗9月25日オープン</t>
+        </is>
+      </c>
+      <c r="D1513" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091876.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1514">
+      <c r="A1514" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1514" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1514" t="inlineStr">
+        <is>
+          <t>マミーマート／「生鮮市場TOP！川口柳崎店」オープン、足元商圏のファミリー層狙う注目</t>
+        </is>
+      </c>
+      <c r="D1514" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091771.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1515">
+      <c r="A1515" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1515" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1515" t="inlineStr">
+        <is>
+          <t>そごう広島店／コスメ売場をリニューアルし面積1.4倍に、フレグランス強化</t>
+        </is>
+      </c>
+      <c r="D1515" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091716.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1516">
+      <c r="A1516" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1516" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1516" t="inlineStr">
+        <is>
+          <t>心斎橋パルコ／9～10月、セガの関西エリア初の旗艦店など3店舗オープン</t>
+        </is>
+      </c>
+      <c r="D1516" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091721.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1517">
+      <c r="A1517" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1517" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1517" t="inlineStr">
+        <is>
+          <t>コジマ×ビックカメラ／「minanoba川口店」オープン、子連れ客向け商品展開</t>
+        </is>
+      </c>
+      <c r="D1517" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091775.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1518">
+      <c r="A1518" t="inlineStr">
+        <is>
+          <t>2026年09月23日</t>
+        </is>
+      </c>
+      <c r="B1518" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1518" t="inlineStr">
+        <is>
+          <t>CCC／スタバとの複合店「SHARE LOUNGE 自由が丘ミューズスクエア」オープン</t>
+        </is>
+      </c>
+      <c r="D1518" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091776.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-24
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1518"/>
+  <dimension ref="A1:D1592"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33812,6 +33812,1634 @@
         </is>
       </c>
     </row>
+    <row r="1519">
+      <c r="A1519" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1519" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1519" t="inlineStr">
+        <is>
+          <t>お好み焼 道とん堀 前橋荒牧店</t>
+        </is>
+      </c>
+      <c r="D1519" t="inlineStr">
+        <is>
+          <t>https://dohtonbori.com/shop/%E5%89%8D%E6%A9%8B%E8%8D%92%E5%B7%BB%E5%BA%97%E3%80%809%E6%9C%8824%E6%97%A5%E6%9C%A8open%EF%BC%81%EF%BC%81/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1520">
+      <c r="A1520" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1520" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1520" t="inlineStr">
+        <is>
+          <t>ヘアカラー専門店fufuファボーレ富山店</t>
+        </is>
+      </c>
+      <c r="D1520" t="inlineStr">
+        <is>
+          <t>https://fufucolor.com/shop-list/dtl/%E3%83%95%E3%82%A1%E3%83%9C%E3%83%BC%E3%83%AC%E5%AF%8C%E5%B1%B1%E5%BA%97/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1521">
+      <c r="A1521" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1521" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1521" t="inlineStr">
+        <is>
+          <t>Workman Colors 清水屋春日井店</t>
+        </is>
+      </c>
+      <c r="D1521" t="inlineStr">
+        <is>
+          <t>https://www.workman.co.jp/store/workman-colors-%E6%B8%85%E6%B0%B4%E5%B1%8B%E6%98%A5%E6%97%A5%E4%BA%95%E5%BA%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="1522">
+      <c r="A1522" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1522" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1522" t="inlineStr">
+        <is>
+          <t>9/24カネスエ上ノ町店(愛知県春日井市)</t>
+        </is>
+      </c>
+      <c r="D1522" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gmT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1523">
+      <c r="A1523" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1523" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1523" t="inlineStr">
+        <is>
+          <t>9/16ヤオマサ富水店(神奈川県小田原市)</t>
+        </is>
+      </c>
+      <c r="D1523" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gmA</t>
+        </is>
+      </c>
+    </row>
+    <row r="1524">
+      <c r="A1524" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1524" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1524" t="inlineStr">
+        <is>
+          <t>9/17 サンディ芦屋店</t>
+        </is>
+      </c>
+      <c r="D1524" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gaR</t>
+        </is>
+      </c>
+    </row>
+    <row r="1525">
+      <c r="A1525" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1525" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1525" t="inlineStr">
+        <is>
+          <t>9/19生鮮市場ダイイチ蒲田店(東京都大田区)</t>
+        </is>
+      </c>
+      <c r="D1525" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gmO</t>
+        </is>
+      </c>
+    </row>
+    <row r="1526">
+      <c r="A1526" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1526" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1526" t="inlineStr">
+        <is>
+          <t>9/26ビッグ・エー春日部増富店</t>
+        </is>
+      </c>
+      <c r="D1526" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gii</t>
+        </is>
+      </c>
+    </row>
+    <row r="1527">
+      <c r="A1527" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1527" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1527" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D1527" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="1528">
+      <c r="A1528" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1528" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1528" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D1528" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="1529">
+      <c r="A1529" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1529" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1529" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D1529" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1530">
+      <c r="A1530" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1530" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1530" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D1530" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="1531">
+      <c r="A1531" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1531" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1531" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D1531" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1532">
+      <c r="A1532" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1532" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1532" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D1532" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="1533">
+      <c r="A1533" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1533" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1533" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1533" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1534">
+      <c r="A1534" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1534" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1534" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1534" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1535">
+      <c r="A1535" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1535" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1535" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1535" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1536">
+      <c r="A1536" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1536" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1536" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1536" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1537">
+      <c r="A1537" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1537" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1537" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1537" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1538">
+      <c r="A1538" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1538" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1538" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1538" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1539">
+      <c r="A1539" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1539" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1539" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1539" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1540">
+      <c r="A1540" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1540" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1540" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1540" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1541">
+      <c r="A1541" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1541" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1541" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1541" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1542">
+      <c r="A1542" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1542" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1542" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1542" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1543">
+      <c r="A1543" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1543" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1543" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1543" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1544">
+      <c r="A1544" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1544" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1544" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1544" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1545">
+      <c r="A1545" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1545" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1545" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1545" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1546">
+      <c r="A1546" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1546" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1546" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1546" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1547">
+      <c r="A1547" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1547" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1547" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1547" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1548">
+      <c r="A1548" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1548" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1548" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1548" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1549">
+      <c r="A1549" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1549" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1549" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1549" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1550">
+      <c r="A1550" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1550" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1550" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1550" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1551">
+      <c r="A1551" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1551" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1551" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1551" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1552">
+      <c r="A1552" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1552" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1552" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1552" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1553">
+      <c r="A1553" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1553" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1553" t="inlineStr">
+        <is>
+          <t>関西地方イオン姫路店 2026年8月末で一旦閉店し建て替えへ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1553" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49763</t>
+        </is>
+      </c>
+    </row>
+    <row r="1554">
+      <c r="A1554" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1554" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1554" t="inlineStr">
+        <is>
+          <t>東北地方オルフィーカ美田園 2025年5月23日(金)より順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1554" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/39130</t>
+        </is>
+      </c>
+    </row>
+    <row r="1555">
+      <c r="A1555" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1555" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1555" t="inlineStr">
+        <is>
+          <t>中部地方名古屋駅 メイチカが大規模リニューアル！2026年9月4日(金)開業！全17店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1555" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/32948</t>
+        </is>
+      </c>
+    </row>
+    <row r="1556">
+      <c r="A1556" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1556" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1556" t="inlineStr">
+        <is>
+          <t>関西地方GLION ARENA KOBE・TOTTEI PARKが 2025年4月4日(金)開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1556" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/33025</t>
+        </is>
+      </c>
+    </row>
+    <row r="1557">
+      <c r="A1557" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1557" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1557" t="inlineStr">
+        <is>
+          <t>中部地方スーパーセンタートライアル・コメリパワー垂井店 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1557" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48537</t>
+        </is>
+      </c>
+    </row>
+    <row r="1558">
+      <c r="A1558" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1558" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1558" t="inlineStr">
+        <is>
+          <t>関西地方ハローズ洲本モール 2026年冬開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1558" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/42115</t>
+        </is>
+      </c>
+    </row>
+    <row r="1559">
+      <c r="A1559" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1559" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1559" t="inlineStr">
+        <is>
+          <t>中国地方ハローズ宇部モール 2025年6月以降開業予定！ テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1559" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/42192</t>
+        </is>
+      </c>
+    </row>
+    <row r="1560">
+      <c r="A1560" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1560" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1560" t="inlineStr">
+        <is>
+          <t>関東地方上板橋駅南口駅前東地区市街地再開発事業 2028年完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1560" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48931</t>
+        </is>
+      </c>
+    </row>
+    <row r="1561">
+      <c r="A1561" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1561" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1561" t="inlineStr">
+        <is>
+          <t>関東地方新松戸駅東側地区開発事業 2032年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1561" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/29149</t>
+        </is>
+      </c>
+    </row>
+    <row r="1562">
+      <c r="A1562" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1562" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1562" t="inlineStr">
+        <is>
+          <t>関東地方ヴィータモールせいせき 2025年10月31日(金)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1562" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/45333</t>
+        </is>
+      </c>
+    </row>
+    <row r="1563">
+      <c r="A1563" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1563" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1563" t="inlineStr">
+        <is>
+          <t>中部地方松本シェーナ 松本パルコ跡地に2026年6月30日(火)開業！ドンキが出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1563" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/45051</t>
+        </is>
+      </c>
+    </row>
+    <row r="1564">
+      <c r="A1564" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1564" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1564" t="inlineStr">
+        <is>
+          <t>関東地方ミナモニ有明 江東区有明1丁目計画 大和ハウスのマンションと商業施設に！2026年5月13日(水)9時~開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1564" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/35626</t>
+        </is>
+      </c>
+    </row>
+    <row r="1565">
+      <c r="A1565" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1565" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1565" t="inlineStr">
+        <is>
+          <t>関西地方フレスポ桜井が増床リニューアル！2026年3月6日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1565" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/43982</t>
+        </is>
+      </c>
+    </row>
+    <row r="1566">
+      <c r="A1566" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1566" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1566" t="inlineStr">
+        <is>
+          <t>中国地方カインズ日吉津店 2025年3月12日(水)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1566" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/34869</t>
+        </is>
+      </c>
+    </row>
+    <row r="1567">
+      <c r="A1567" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1567" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1567" t="inlineStr">
+        <is>
+          <t>中部地方能美市福島町 複合商業施設 2027年度以降開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1567" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/36955</t>
+        </is>
+      </c>
+    </row>
+    <row r="1568">
+      <c r="A1568" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1568" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1568" t="inlineStr">
+        <is>
+          <t>関東地方WORLD TOWER RESIDENCE 2026年12月完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1568" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/19463</t>
+        </is>
+      </c>
+    </row>
+    <row r="1569">
+      <c r="A1569" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1569" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1569" t="inlineStr">
+        <is>
+          <t>中部地方イオンタウン岐阜北方 2026年3月27日(金)開業！全24テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1569" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/16776</t>
+        </is>
+      </c>
+    </row>
+    <row r="1570">
+      <c r="A1570" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1570" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1570" t="inlineStr">
+        <is>
+          <t>関西地方キッピーテラス 三田駅前に2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1570" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/21864</t>
+        </is>
+      </c>
+    </row>
+    <row r="1571">
+      <c r="A1571" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1571" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1571" t="inlineStr">
+        <is>
+          <t>中部地方名古屋競馬場跡地に日本エスコンの複合商業施設 2029年開業予定！テナントは？最新情報も！愛知県名古屋市港区のあおなみ線「港北駅」東側に広がる旧名古屋競馬場跡地に、中部電力・日本エスコンなどが手掛ける大型複合商業施設「(仮称)名古屋競馬場跡地複合商業施設」が2029年頃に開業予定！バンテリンドーム約4個分（約20.7ha）におよ...2026.09.23中部地方</t>
+        </is>
+      </c>
+      <c r="D1571" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/49742</t>
+        </is>
+      </c>
+    </row>
+    <row r="1572">
+      <c r="A1572" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1572" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1572" t="inlineStr">
+        <is>
+          <t>関東地方上大岡C北地区第一種市街地再開発事業 2034年度完成予定！テナントは？最新情報も！神奈川県横浜市港南区の京急本線・横浜市営地下鉄ブルーライン「上大岡駅」西口駅前に、京浜急行電鉄・大林組が参画する超高層複合タワー「上大岡C北地区第一種市街地再開発事業」が2034年度完成予定！「富士ショッピングセンター」やパサージュ上大岡周...2026.09.23関東地方</t>
+        </is>
+      </c>
+      <c r="D1572" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49754</t>
+        </is>
+      </c>
+    </row>
+    <row r="1573">
+      <c r="A1573" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1573" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1573" t="inlineStr">
+        <is>
+          <t>セブンタウン小豆沢／新ブランド「コムリエ」に10月9日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1573" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1574">
+      <c r="A1574" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1574" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1574" t="inlineStr">
+        <is>
+          <t>東京ミッドタウン八重洲／今秋、タイ料理などグルメな3店舗をオープン</t>
+        </is>
+      </c>
+      <c r="D1574" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092413.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1575">
+      <c r="A1575" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1575" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1575" t="inlineStr">
+        <is>
+          <t>カインズ／神奈川県綾瀬市に「（仮称）綾瀬店（店舗面積7560m2）」27年3月29日新設</t>
+        </is>
+      </c>
+      <c r="D1575" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0924011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1576">
+      <c r="A1576" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1576" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1576" t="inlineStr">
+        <is>
+          <t>ベイシア／埼玉県「本庄早稲田ゲート店」9月25日リニューアルオープン、新商品充実</t>
+        </is>
+      </c>
+      <c r="D1576" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092479.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1577">
+      <c r="A1577" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1577" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1577" t="inlineStr">
+        <is>
+          <t>イズミ／福岡県行橋市の「ゆめタウン行橋」10月2日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1577" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092441.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1578">
+      <c r="A1578" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1578" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1578" t="inlineStr">
+        <is>
+          <t>まいばすけっと／東京都内に「平井駅前店」「百草園駅前店」9月25日同時オープン</t>
+        </is>
+      </c>
+      <c r="D1578" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092478.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1579">
+      <c r="A1579" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1579" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1579" t="inlineStr">
+        <is>
+          <t>オオゼキ／神奈川県「中央林間店」10月2日リニューアルオープン、生鮮・総菜強化</t>
+        </is>
+      </c>
+      <c r="D1579" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092475.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1580">
+      <c r="A1580" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1580" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1580" t="inlineStr">
+        <is>
+          <t>コメリ／大阪府内初のPRO業態「富田林店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D1580" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092477.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1581">
+      <c r="A1581" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1581" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1581" t="inlineStr">
+        <is>
+          <t>ゴンチャ／「南砂町ショッピングセンターSUNAMO」に新店舗10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D1581" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092476.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1582">
+      <c r="A1582" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1582" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1582" t="inlineStr">
+        <is>
+          <t>プロント／「日本橋三井タワー店」10月19日オープン</t>
+        </is>
+      </c>
+      <c r="D1582" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092411.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1583">
+      <c r="A1583" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1583" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1583" t="inlineStr">
+        <is>
+          <t>クリエイトSD／千葉県柏市に「柏船戸店」27年4月18日新設</t>
+        </is>
+      </c>
+      <c r="D1583" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0924012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1584">
+      <c r="A1584" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1584" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1584" t="inlineStr">
+        <is>
+          <t>クリスプサラダワークス／東京都渋谷区に「CIRCLES渋谷店」9月30日オープン</t>
+        </is>
+      </c>
+      <c r="D1584" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092474.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1585">
+      <c r="A1585" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1585" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1585" t="inlineStr">
+        <is>
+          <t>ゴディバ／関西初の新スタイル導入店舗「なんばCITY店」9月30日オープン</t>
+        </is>
+      </c>
+      <c r="D1585" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092473.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1586">
+      <c r="A1586" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1586" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1586" t="inlineStr">
+        <is>
+          <t>イオンモール／京都・四条河原町「河原町オーパ」9月19日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1586" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091841.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1587">
+      <c r="A1587" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1587" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1587" t="inlineStr">
+        <is>
+          <t>新宿マルイ アネックス／1階フロアを大幅リニューアル、多彩なコンテンツを集積</t>
+        </is>
+      </c>
+      <c r="D1587" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091744.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1588">
+      <c r="A1588" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1588" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1588" t="inlineStr">
+        <is>
+          <t>カインズ／長野県上田市に「上田国分店」今秋オープン、農業資材・ペット用品充実</t>
+        </is>
+      </c>
+      <c r="D1588" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091873.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1589">
+      <c r="A1589" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1589" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1589" t="inlineStr">
+        <is>
+          <t>有明ガーデン／「ペタリアフラワー」「チチカカ」新規オープン、国内外のニーズに対応</t>
+        </is>
+      </c>
+      <c r="D1589" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091871.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1590">
+      <c r="A1590" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1590" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1590" t="inlineStr">
+        <is>
+          <t>ラルズ／札幌市「ビッグハウスウエスト」9月18日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1590" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091814.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1591">
+      <c r="A1591" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1591" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1591" t="inlineStr">
+        <is>
+          <t>コーナン商事／兵庫県姫路市に「（仮称）コーナンPRO姫路飾磨店（店舗面積2089m2）」27年4月1日新設</t>
+        </is>
+      </c>
+      <c r="D1591" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0918012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1592">
+      <c r="A1592" t="inlineStr">
+        <is>
+          <t>2026年09月24日</t>
+        </is>
+      </c>
+      <c r="B1592" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1592" t="inlineStr">
+        <is>
+          <t>ゼビオ／富山県に「スーパースポーツゼビオ アクロスプラザ富山掛尾店」オープン</t>
+        </is>
+      </c>
+      <c r="D1592" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091877.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-25
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1592"/>
+  <dimension ref="A1:D1664"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35440,6 +35440,1590 @@
         </is>
       </c>
     </row>
+    <row r="1593">
+      <c r="A1593" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1593" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1593" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D1593" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="1594">
+      <c r="A1594" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1594" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1594" t="inlineStr">
+        <is>
+          <t>9/16ヤオマサ富水店(神奈川県小田原市)</t>
+        </is>
+      </c>
+      <c r="D1594" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gmA</t>
+        </is>
+      </c>
+    </row>
+    <row r="1595">
+      <c r="A1595" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1595" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1595" t="inlineStr">
+        <is>
+          <t>9/17 サンディ芦屋店</t>
+        </is>
+      </c>
+      <c r="D1595" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gaR</t>
+        </is>
+      </c>
+    </row>
+    <row r="1596">
+      <c r="A1596" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1596" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1596" t="inlineStr">
+        <is>
+          <t>9/19生鮮市場ダイイチ蒲田店(東京都大田区)</t>
+        </is>
+      </c>
+      <c r="D1596" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gmO</t>
+        </is>
+      </c>
+    </row>
+    <row r="1597">
+      <c r="A1597" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1597" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1597" t="inlineStr">
+        <is>
+          <t>9/24カネスエ上ノ町店(愛知県春日井市)</t>
+        </is>
+      </c>
+      <c r="D1597" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gmT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1598">
+      <c r="A1598" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1598" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1598" t="inlineStr">
+        <is>
+          <t>9/26ビッグ・エー春日部増富店</t>
+        </is>
+      </c>
+      <c r="D1598" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gii</t>
+        </is>
+      </c>
+    </row>
+    <row r="1599">
+      <c r="A1599" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1599" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1599" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D1599" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="1600">
+      <c r="A1600" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1600" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1600" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D1600" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="1601">
+      <c r="A1601" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1601" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1601" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D1601" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1602">
+      <c r="A1602" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1602" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1602" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D1602" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="1603">
+      <c r="A1603" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1603" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1603" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D1603" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1604">
+      <c r="A1604" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1604" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1604" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D1604" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="1605">
+      <c r="A1605" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1605" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1605" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1605" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1606">
+      <c r="A1606" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1606" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1606" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1606" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1607">
+      <c r="A1607" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1607" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1607" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1607" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1608">
+      <c r="A1608" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1608" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1608" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1608" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1609">
+      <c r="A1609" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1609" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1609" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1609" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1610">
+      <c r="A1610" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1610" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1610" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1610" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1611">
+      <c r="A1611" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1611" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1611" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1611" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1612">
+      <c r="A1612" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1612" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1612" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1612" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1613">
+      <c r="A1613" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1613" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1613" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1613" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1614">
+      <c r="A1614" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1614" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1614" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1614" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1615">
+      <c r="A1615" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1615" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1615" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1615" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1616">
+      <c r="A1616" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1616" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1616" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1616" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1617">
+      <c r="A1617" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1617" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1617" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1617" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1618">
+      <c r="A1618" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1618" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1618" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1618" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1619">
+      <c r="A1619" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1619" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1619" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1619" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1620">
+      <c r="A1620" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1620" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1620" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1620" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1621">
+      <c r="A1621" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1621" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1621" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1621" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1622">
+      <c r="A1622" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1622" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1622" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1622" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1623">
+      <c r="A1623" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1623" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1623" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1623" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1624">
+      <c r="A1624" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1624" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1624" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1624" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1625">
+      <c r="A1625" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1625" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1625" t="inlineStr">
+        <is>
+          <t>九州地方スプリングガーデン御代志2025年3月24日(月)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1625" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/36931</t>
+        </is>
+      </c>
+    </row>
+    <row r="1626">
+      <c r="A1626" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1626" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1626" t="inlineStr">
+        <is>
+          <t>関東地方東武曳舟駅前地区市街地再開発事業 2032年開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1626" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48112</t>
+        </is>
+      </c>
+    </row>
+    <row r="1627">
+      <c r="A1627" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1627" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1627" t="inlineStr">
+        <is>
+          <t>東北地方イオンスタイル八戸沼館 2025年4月25日(金)開業！全テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1627" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/42366</t>
+        </is>
+      </c>
+    </row>
+    <row r="1628">
+      <c r="A1628" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1628" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1628" t="inlineStr">
+        <is>
+          <t>関西地方ひらら光善寺 2023年12月9日(土)開業！全18テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1628" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/21577</t>
+        </is>
+      </c>
+    </row>
+    <row r="1629">
+      <c r="A1629" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1629" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1629" t="inlineStr">
+        <is>
+          <t>関東地方イオンスタイル大宮西 2027年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1629" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48705</t>
+        </is>
+      </c>
+    </row>
+    <row r="1630">
+      <c r="A1630" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1630" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1630" t="inlineStr">
+        <is>
+          <t>九州地方スーパーセンタートライアル加納店 2025年4月29日(火・祝)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1630" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/40580</t>
+        </is>
+      </c>
+    </row>
+    <row r="1631">
+      <c r="A1631" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1631" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1631" t="inlineStr">
+        <is>
+          <t>関東地方ニトリモール東八三鷹 2028年開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1631" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/44873</t>
+        </is>
+      </c>
+    </row>
+    <row r="1632">
+      <c r="A1632" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1632" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1632" t="inlineStr">
+        <is>
+          <t>関西地方イオンスタイル大津京 一旦閉店し建て替えて2028年開業！分譲マンションとの一体開発！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1632" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/35154</t>
+        </is>
+      </c>
+    </row>
+    <row r="1633">
+      <c r="A1633" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1633" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1633" t="inlineStr">
+        <is>
+          <t>東北地方イオン土崎港店跡地 2026年2月28日閉店 跡地はどうなる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1633" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/45956</t>
+        </is>
+      </c>
+    </row>
+    <row r="1634">
+      <c r="A1634" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1634" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1634" t="inlineStr">
+        <is>
+          <t>関東地方道玄坂二丁目南地区市街地再開発事業 2027年春開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1634" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/23396</t>
+        </is>
+      </c>
+    </row>
+    <row r="1635">
+      <c r="A1635" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1635" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1635" t="inlineStr">
+        <is>
+          <t>関東地方BASEGATE（ベースゲート）横浜関内 2026年3月19日(木)開業！全65店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1635" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/11753</t>
+        </is>
+      </c>
+    </row>
+    <row r="1636">
+      <c r="A1636" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1636" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1636" t="inlineStr">
+        <is>
+          <t>関西地方平和堂岸辺店 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1636" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49465</t>
+        </is>
+      </c>
+    </row>
+    <row r="1637">
+      <c r="A1637" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1637" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1637" t="inlineStr">
+        <is>
+          <t>東北地方イオンモール仙台上杉 2025年10月8日(水)開業！全テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1637" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/2380</t>
+        </is>
+      </c>
+    </row>
+    <row r="1638">
+      <c r="A1638" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1638" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1638" t="inlineStr">
+        <is>
+          <t>関東地方カインズ伊勢崎境保泉店 2028年春開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1638" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47795</t>
+        </is>
+      </c>
+    </row>
+    <row r="1639">
+      <c r="A1639" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1639" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1639" t="inlineStr">
+        <is>
+          <t>関東地方グラン8モール 2025年8月28日(木)より順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1639" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42179</t>
+        </is>
+      </c>
+    </row>
+    <row r="1640">
+      <c r="A1640" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1640" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1640" t="inlineStr">
+        <is>
+          <t>関東地方そよら入曽駅前 2025年3月21日(金)開業！全テナント10店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1640" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/22304</t>
+        </is>
+      </c>
+    </row>
+    <row r="1641">
+      <c r="A1641" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1641" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1641" t="inlineStr">
+        <is>
+          <t>関東地方カスミ赤羽神谷店 2026年1月23日(金)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1641" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42132</t>
+        </is>
+      </c>
+    </row>
+    <row r="1642">
+      <c r="A1642" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1642" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1642" t="inlineStr">
+        <is>
+          <t>関東地方築地地区まちづくり事業 築地市場跡地 2030年代半ば開業！どのような施設になる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1642" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49238</t>
+        </is>
+      </c>
+    </row>
+    <row r="1643">
+      <c r="A1643" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1643" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1643" t="inlineStr">
+        <is>
+          <t>関西地方イオン姫路店 2026年8月末で一旦閉店し建て替えへ！テナントは？最新情報も！兵庫県姫路市増位本町のイオンリテールの商業施設「イオン姫路店（旧サティ姫路店）」が2026年8月31日にいったん閉店し、既存建物を解体した上で、新たな商業施設に建て替わる計画が明らかになりました！1979年の開業から約47年にわたり親しまれ...2026.09.25関西地方</t>
+        </is>
+      </c>
+      <c r="D1643" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49763</t>
+        </is>
+      </c>
+    </row>
+    <row r="1644">
+      <c r="A1644" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1644" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1644" t="inlineStr">
+        <is>
+          <t>東北地方イオン相馬店 建て替え 2027年夏開業！テナントは？最新情報も！福島県相馬市馬場野の国道6号沿いに、イオン東北が手掛ける新たな地域密着型商業施設「イオン相馬店（建て替え再建）」が2027年開業！1989年の開業以来、相双エリアの中核商業施設として親しまれ、2022年3月の地震被害を乗り越えて全面建て替え...2026.09.24東北地方</t>
+        </is>
+      </c>
+      <c r="D1644" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/49770</t>
+        </is>
+      </c>
+    </row>
+    <row r="1645">
+      <c r="A1645" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1645" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1645" t="inlineStr">
+        <is>
+          <t>ハンズ新宿店／9月30日リニューアルオープン、自販機型サンプリング機を初導入</t>
+        </is>
+      </c>
+      <c r="D1645" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092512.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1646">
+      <c r="A1646" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1646" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1646" t="inlineStr">
+        <is>
+          <t>フレスタ／生鮮市場ベジタ店跡地に「ワークマンプラス」など3店舗10月以降オープン</t>
+        </is>
+      </c>
+      <c r="D1646" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092576.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1647">
+      <c r="A1647" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1647" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1647" t="inlineStr">
+        <is>
+          <t>ピソラ／熊本県に「PISOLA熊本嘉島店」10月21日オープン、九州地方に初出店</t>
+        </is>
+      </c>
+      <c r="D1647" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092541.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1648">
+      <c r="A1648" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1648" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1648" t="inlineStr">
+        <is>
+          <t>富澤商店／神奈川県に「ダイナシティ小田原店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D1648" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092575.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1649">
+      <c r="A1649" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1649" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1649" t="inlineStr">
+        <is>
+          <t>そごう横浜店／地下2階の酒売場9月30日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1649" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1650">
+      <c r="A1650" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1650" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1650" t="inlineStr">
+        <is>
+          <t>大黒天物産／熊本県山鹿市に「（仮称）ラ・ムー山鹿店」27年4月20日新設</t>
+        </is>
+      </c>
+      <c r="D1650" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0925012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1651">
+      <c r="A1651" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1651" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1651" t="inlineStr">
+        <is>
+          <t>ブルボン／大丸東京店にコンセプトストア期間限定オープン、10月21日から</t>
+        </is>
+      </c>
+      <c r="D1651" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092511.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1652">
+      <c r="A1652" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1652" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1652" t="inlineStr">
+        <is>
+          <t>サブウェイ／横浜市に「コーナン港北インター店」10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D1652" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092514.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1653">
+      <c r="A1653" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1653" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1653" t="inlineStr">
+        <is>
+          <t>薬王堂／群馬県伊勢崎市に「伊勢崎東店」27年4月18日新設</t>
+        </is>
+      </c>
+      <c r="D1653" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0925011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1654">
+      <c r="A1654" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1654" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1654" t="inlineStr">
+        <is>
+          <t>日販／図書館内の無人ショップ「TOSHOP」八王子に10月3日オープン</t>
+        </is>
+      </c>
+      <c r="D1654" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092577.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1655">
+      <c r="A1655" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1655" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1655" t="inlineStr">
+        <is>
+          <t>クリスプサラダワークス／東京都品川区に「大崎ニューシティ店」10月6日オープン</t>
+        </is>
+      </c>
+      <c r="D1655" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092574.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1656">
+      <c r="A1656" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1656" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1656" t="inlineStr">
+        <is>
+          <t>セブンタウン小豆沢／新ブランド「コムリエ」に10月9日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1656" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1657">
+      <c r="A1657" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1657" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1657" t="inlineStr">
+        <is>
+          <t>東京ミッドタウン八重洲／今秋、タイ料理などグルメな3店舗をオープン</t>
+        </is>
+      </c>
+      <c r="D1657" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092413.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1658">
+      <c r="A1658" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1658" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1658" t="inlineStr">
+        <is>
+          <t>カインズ／神奈川県綾瀬市に「（仮称）綾瀬店（店舗面積7560m2）」27年3月29日新設</t>
+        </is>
+      </c>
+      <c r="D1658" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0924011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1659">
+      <c r="A1659" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1659" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1659" t="inlineStr">
+        <is>
+          <t>ベイシア／埼玉県「本庄早稲田ゲート店」9月25日リニューアルオープン、新商品充実</t>
+        </is>
+      </c>
+      <c r="D1659" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092479.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1660">
+      <c r="A1660" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1660" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1660" t="inlineStr">
+        <is>
+          <t>イズミ／福岡県行橋市の「ゆめタウン行橋」10月2日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1660" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092441.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1661">
+      <c r="A1661" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1661" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1661" t="inlineStr">
+        <is>
+          <t>まいばすけっと／東京都内に「平井駅前店」「百草園駅前店」9月25日同時オープン</t>
+        </is>
+      </c>
+      <c r="D1661" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092478.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1662">
+      <c r="A1662" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1662" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1662" t="inlineStr">
+        <is>
+          <t>オオゼキ／神奈川県「中央林間店」10月2日リニューアルオープン、生鮮・総菜強化</t>
+        </is>
+      </c>
+      <c r="D1662" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092475.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1663">
+      <c r="A1663" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1663" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1663" t="inlineStr">
+        <is>
+          <t>コメリ／大阪府内初のPRO業態「富田林店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D1663" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092477.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1664">
+      <c r="A1664" t="inlineStr">
+        <is>
+          <t>2026年09月25日</t>
+        </is>
+      </c>
+      <c r="B1664" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1664" t="inlineStr">
+        <is>
+          <t>ゴンチャ／「南砂町ショッピングセンターSUNAMO」に新店舗10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D1664" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092476.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-26
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1664"/>
+  <dimension ref="A1:D1737"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37024,6 +37024,1612 @@
         </is>
       </c>
     </row>
+    <row r="1665">
+      <c r="A1665" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1665" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1665" t="inlineStr">
+        <is>
+          <t>9/26ビッグ・エー春日部増富店</t>
+        </is>
+      </c>
+      <c r="D1665" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gii</t>
+        </is>
+      </c>
+    </row>
+    <row r="1666">
+      <c r="A1666" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1666" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1666" t="inlineStr">
+        <is>
+          <t>9/26三杉屋天六店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D1666" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gpn</t>
+        </is>
+      </c>
+    </row>
+    <row r="1667">
+      <c r="A1667" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1667" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1667" t="inlineStr">
+        <is>
+          <t>9/16ヤオマサ富水店(神奈川県小田原市)</t>
+        </is>
+      </c>
+      <c r="D1667" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gmA</t>
+        </is>
+      </c>
+    </row>
+    <row r="1668">
+      <c r="A1668" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1668" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1668" t="inlineStr">
+        <is>
+          <t>9/17 サンディ芦屋店</t>
+        </is>
+      </c>
+      <c r="D1668" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gaR</t>
+        </is>
+      </c>
+    </row>
+    <row r="1669">
+      <c r="A1669" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1669" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1669" t="inlineStr">
+        <is>
+          <t>9/19生鮮市場ダイイチ蒲田店(東京都大田区)</t>
+        </is>
+      </c>
+      <c r="D1669" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gmO</t>
+        </is>
+      </c>
+    </row>
+    <row r="1670">
+      <c r="A1670" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1670" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1670" t="inlineStr">
+        <is>
+          <t>9/24カネスエ上ノ町店(愛知県春日井市)</t>
+        </is>
+      </c>
+      <c r="D1670" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gmT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1671">
+      <c r="A1671" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1671" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1671" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D1671" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="1672">
+      <c r="A1672" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1672" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1672" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D1672" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="1673">
+      <c r="A1673" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1673" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1673" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D1673" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="1674">
+      <c r="A1674" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1674" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1674" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D1674" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1675">
+      <c r="A1675" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1675" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1675" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D1675" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="1676">
+      <c r="A1676" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1676" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1676" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D1676" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1677">
+      <c r="A1677" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1677" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1677" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D1677" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="1678">
+      <c r="A1678" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1678" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1678" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1678" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1679">
+      <c r="A1679" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1679" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1679" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1679" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1680">
+      <c r="A1680" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1680" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1680" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1680" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1681">
+      <c r="A1681" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1681" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1681" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1681" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1682">
+      <c r="A1682" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1682" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1682" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1682" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1683">
+      <c r="A1683" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1683" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1683" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1683" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1684">
+      <c r="A1684" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1684" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1684" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1684" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1685">
+      <c r="A1685" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1685" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1685" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1685" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1686">
+      <c r="A1686" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1686" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1686" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1686" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1687">
+      <c r="A1687" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1687" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1687" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1687" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1688">
+      <c r="A1688" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1688" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1688" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1688" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1689">
+      <c r="A1689" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1689" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1689" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1689" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1690">
+      <c r="A1690" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1690" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1690" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1690" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1691">
+      <c r="A1691" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1691" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1691" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1691" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1692">
+      <c r="A1692" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1692" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1692" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1692" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1693">
+      <c r="A1693" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1693" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1693" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1693" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1694">
+      <c r="A1694" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1694" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1694" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1694" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1695">
+      <c r="A1695" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1695" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1695" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1695" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1696">
+      <c r="A1696" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1696" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1696" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1696" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1697">
+      <c r="A1697" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1697" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1697" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1697" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1698">
+      <c r="A1698" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1698" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1698" t="inlineStr">
+        <is>
+          <t>中部地方ニトリ鈴鹿中央通り店 2025年12月12日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1698" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/44303</t>
+        </is>
+      </c>
+    </row>
+    <row r="1699">
+      <c r="A1699" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1699" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1699" t="inlineStr">
+        <is>
+          <t>関東地方スーパーセンタートライアル鹿沼店 2025年10月1日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1699" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/41441</t>
+        </is>
+      </c>
+    </row>
+    <row r="1700">
+      <c r="A1700" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1700" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1700" t="inlineStr">
+        <is>
+          <t>中部地方イオンスタイル黒埼 2025年3月18日(火)開業！全3テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1700" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/37860</t>
+        </is>
+      </c>
+    </row>
+    <row r="1701">
+      <c r="A1701" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1701" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1701" t="inlineStr">
+        <is>
+          <t>中国地方ハローズ西岐波店 2026年8月6日(木)開業！全4テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1701" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/48261</t>
+        </is>
+      </c>
+    </row>
+    <row r="1702">
+      <c r="A1702" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1702" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1702" t="inlineStr">
+        <is>
+          <t>関西地方アークスクエア茨木 2025年5月21日(水)より順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1702" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/21729</t>
+        </is>
+      </c>
+    </row>
+    <row r="1703">
+      <c r="A1703" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1703" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1703" t="inlineStr">
+        <is>
+          <t>関東地方トーチタワー 地上385mの日本一高いビルが2028年度竣工！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1703" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/15125</t>
+        </is>
+      </c>
+    </row>
+    <row r="1704">
+      <c r="A1704" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1704" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1704" t="inlineStr">
+        <is>
+          <t>中部地方新潟市東区中木戸商業施設(仮称) 2027年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1704" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/47439</t>
+        </is>
+      </c>
+    </row>
+    <row r="1705">
+      <c r="A1705" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1705" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1705" t="inlineStr">
+        <is>
+          <t>関東地方ONO CROSS プラウドタワー相模大野クロス 2026年1月23日(金)より順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1705" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/35191</t>
+        </is>
+      </c>
+    </row>
+    <row r="1706">
+      <c r="A1706" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1706" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1706" t="inlineStr">
+        <is>
+          <t>関東地方中山駅南口地区市街地再開発事業 2029年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1706" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26880</t>
+        </is>
+      </c>
+    </row>
+    <row r="1707">
+      <c r="A1707" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1707" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1707" t="inlineStr">
+        <is>
+          <t>関東地方アクロスプラザ北柏 2026年4月1日(水)より順次開業！全19テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1707" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/35911</t>
+        </is>
+      </c>
+    </row>
+    <row r="1708">
+      <c r="A1708" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1708" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1708" t="inlineStr">
+        <is>
+          <t>関東地方minanoba相模原（ミナノバ相模原） 2025年3月5日(水)開業！全11テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1708" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/35264</t>
+        </is>
+      </c>
+    </row>
+    <row r="1709">
+      <c r="A1709" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1709" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1709" t="inlineStr">
+        <is>
+          <t>北海道地方ヤマダデンキテックランドNew恵庭店 2025年2月28日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1709" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/40074</t>
+        </is>
+      </c>
+    </row>
+    <row r="1710">
+      <c r="A1710" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1710" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1710" t="inlineStr">
+        <is>
+          <t>関東地方秋葉原UDX アキバイチが2026年1月23日(金) 閉店 2026年冬リニューアル開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1710" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/46578</t>
+        </is>
+      </c>
+    </row>
+    <row r="1711">
+      <c r="A1711" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1711" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1711" t="inlineStr">
+        <is>
+          <t>関東地方三河島駅前北地区市街地再開発事業 2031年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1711" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26830</t>
+        </is>
+      </c>
+    </row>
+    <row r="1712">
+      <c r="A1712" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1712" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1712" t="inlineStr">
+        <is>
+          <t>中国地方カミハチクロス 2027年度開業！アンダーズ広島が進出！商業施設も！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1712" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/27582</t>
+        </is>
+      </c>
+    </row>
+    <row r="1713">
+      <c r="A1713" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1713" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1713" t="inlineStr">
+        <is>
+          <t>中部地方星が丘ボウル跡地プロジェクト 商業施設 2027年春 第1期開業 28年春全面開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1713" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/41720</t>
+        </is>
+      </c>
+    </row>
+    <row r="1714">
+      <c r="A1714" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1714" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1714" t="inlineStr">
+        <is>
+          <t>関東地方イオン北浦和店 2025年9月30日(火)閉店 跡地はどうなる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1714" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/46169</t>
+        </is>
+      </c>
+    </row>
+    <row r="1715">
+      <c r="A1715" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1715" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1715" t="inlineStr">
+        <is>
+          <t>関東地方関内駅前港町地区市街地再開発事業 2031年開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1715" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/17590</t>
+        </is>
+      </c>
+    </row>
+    <row r="1716">
+      <c r="A1716" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1716" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1716" t="inlineStr">
+        <is>
+          <t>関東地方新綱島MICCA 2026年10月28日(水)開業！21店舗が出店！テナントは？最新情報も！神奈川県横浜市港北区の東急新横浜線「新綱島駅」前に、歴史的古民家と木造商業施設が融合した新施設「新綱島MICCA（シンツナシマ ミッカ）」が2026年10月28日（水）にグランドオープン！正式オープン日が2026年10月28日（水）に決定！...2026.09.26関東地方</t>
+        </is>
+      </c>
+      <c r="D1716" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49470</t>
+        </is>
+      </c>
+    </row>
+    <row r="1717">
+      <c r="A1717" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1717" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1717" t="inlineStr">
+        <is>
+          <t>関西地方ヤマダデンキ テックランド堺南島店 2027年冬に開業予定！大阪府堺市に「ヤマダデンキ テックランド 堺南島店(仮称)」が2027年冬に開業予定！ヤマダ電機の中では大型店舗となります！そんな、ヤマダデンキ テックランド堺南島店について、テナントや開業日などを見ていきましょう！2026年4月13日　公...2026.09.26関西地方</t>
+        </is>
+      </c>
+      <c r="D1717" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/48191</t>
+        </is>
+      </c>
+    </row>
+    <row r="1718">
+      <c r="A1718" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1718" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1718" t="inlineStr">
+        <is>
+          <t>ハンズ新宿店／9月30日リニューアルオープン、自販機型サンプリング機を初導入</t>
+        </is>
+      </c>
+      <c r="D1718" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092512.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1719">
+      <c r="A1719" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1719" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1719" t="inlineStr">
+        <is>
+          <t>フレスタ／生鮮市場ベジタ店跡地に「ワークマンプラス」など3店舗10月以降オープン</t>
+        </is>
+      </c>
+      <c r="D1719" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092576.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1720">
+      <c r="A1720" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1720" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1720" t="inlineStr">
+        <is>
+          <t>ピソラ／熊本県に「PISOLA熊本嘉島店」10月21日オープン、九州地方に初出店</t>
+        </is>
+      </c>
+      <c r="D1720" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092541.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1721">
+      <c r="A1721" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1721" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1721" t="inlineStr">
+        <is>
+          <t>富澤商店／神奈川県に「ダイナシティ小田原店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D1721" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092575.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1722">
+      <c r="A1722" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1722" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1722" t="inlineStr">
+        <is>
+          <t>そごう横浜店／地下2階の酒売場9月30日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1722" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1723">
+      <c r="A1723" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1723" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1723" t="inlineStr">
+        <is>
+          <t>大黒天物産／熊本県山鹿市に「（仮称）ラ・ムー山鹿店」27年4月20日新設</t>
+        </is>
+      </c>
+      <c r="D1723" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0925012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1724">
+      <c r="A1724" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1724" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1724" t="inlineStr">
+        <is>
+          <t>ブルボン／大丸東京店にコンセプトストア期間限定オープン、10月21日から</t>
+        </is>
+      </c>
+      <c r="D1724" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092511.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1725">
+      <c r="A1725" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1725" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1725" t="inlineStr">
+        <is>
+          <t>サブウェイ／横浜市に「コーナン港北インター店」10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D1725" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092514.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1726">
+      <c r="A1726" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1726" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1726" t="inlineStr">
+        <is>
+          <t>薬王堂／群馬県伊勢崎市に「伊勢崎東店」27年4月18日新設</t>
+        </is>
+      </c>
+      <c r="D1726" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0925011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1727">
+      <c r="A1727" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1727" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1727" t="inlineStr">
+        <is>
+          <t>日販／図書館内の無人ショップ「TOSHOP」八王子に10月3日オープン</t>
+        </is>
+      </c>
+      <c r="D1727" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092577.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1728">
+      <c r="A1728" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1728" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1728" t="inlineStr">
+        <is>
+          <t>クリスプサラダワークス／東京都品川区に「大崎ニューシティ店」10月6日オープン</t>
+        </is>
+      </c>
+      <c r="D1728" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092574.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1729">
+      <c r="A1729" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1729" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1729" t="inlineStr">
+        <is>
+          <t>セブンタウン小豆沢／新ブランド「コムリエ」に10月9日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1729" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1730">
+      <c r="A1730" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1730" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1730" t="inlineStr">
+        <is>
+          <t>東京ミッドタウン八重洲／今秋、タイ料理などグルメな3店舗をオープン</t>
+        </is>
+      </c>
+      <c r="D1730" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092413.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1731">
+      <c r="A1731" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1731" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1731" t="inlineStr">
+        <is>
+          <t>カインズ／神奈川県綾瀬市に「（仮称）綾瀬店（店舗面積7560m2）」27年3月29日新設</t>
+        </is>
+      </c>
+      <c r="D1731" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0924011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1732">
+      <c r="A1732" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1732" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1732" t="inlineStr">
+        <is>
+          <t>ベイシア／埼玉県「本庄早稲田ゲート店」9月25日リニューアルオープン、新商品充実</t>
+        </is>
+      </c>
+      <c r="D1732" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092479.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1733">
+      <c r="A1733" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1733" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1733" t="inlineStr">
+        <is>
+          <t>イズミ／福岡県行橋市の「ゆめタウン行橋」10月2日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1733" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092441.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1734">
+      <c r="A1734" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1734" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1734" t="inlineStr">
+        <is>
+          <t>まいばすけっと／東京都内に「平井駅前店」「百草園駅前店」9月25日同時オープン</t>
+        </is>
+      </c>
+      <c r="D1734" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092478.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1735">
+      <c r="A1735" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1735" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1735" t="inlineStr">
+        <is>
+          <t>オオゼキ／神奈川県「中央林間店」10月2日リニューアルオープン、生鮮・総菜強化</t>
+        </is>
+      </c>
+      <c r="D1735" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092475.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1736">
+      <c r="A1736" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1736" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1736" t="inlineStr">
+        <is>
+          <t>コメリ／大阪府内初のPRO業態「富田林店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D1736" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092477.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1737">
+      <c r="A1737" t="inlineStr">
+        <is>
+          <t>2026年09月26日</t>
+        </is>
+      </c>
+      <c r="B1737" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1737" t="inlineStr">
+        <is>
+          <t>ゴンチャ／「南砂町ショッピングセンターSUNAMO」に新店舗10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D1737" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092476.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-27
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1737"/>
+  <dimension ref="A1:D1813"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38630,6 +38630,1678 @@
         </is>
       </c>
     </row>
+    <row r="1738">
+      <c r="A1738" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1738" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1738" t="inlineStr">
+        <is>
+          <t>新渡戸記念館 READYFOR</t>
+        </is>
+      </c>
+      <c r="D1738" t="inlineStr">
+        <is>
+          <t>https://www.nitobe.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1739">
+      <c r="A1739" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1739" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1739" t="inlineStr">
+        <is>
+          <t>PLUS SQUARED プラススクエアード</t>
+        </is>
+      </c>
+      <c r="D1739" t="inlineStr">
+        <is>
+          <t>https://plusmania.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1740">
+      <c r="A1740" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1740" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1740" t="inlineStr">
+        <is>
+          <t>JPCスポーツ教室 小倉店</t>
+        </is>
+      </c>
+      <c r="D1740" t="inlineStr">
+        <is>
+          <t>https://jpc-sports.com/kokura/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1741">
+      <c r="A1741" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1741" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1741" t="inlineStr">
+        <is>
+          <t>9/16ヤオマサ富水店(神奈川県小田原市)</t>
+        </is>
+      </c>
+      <c r="D1741" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gmA</t>
+        </is>
+      </c>
+    </row>
+    <row r="1742">
+      <c r="A1742" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1742" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1742" t="inlineStr">
+        <is>
+          <t>9/17 サンディ芦屋店</t>
+        </is>
+      </c>
+      <c r="D1742" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gaR</t>
+        </is>
+      </c>
+    </row>
+    <row r="1743">
+      <c r="A1743" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1743" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1743" t="inlineStr">
+        <is>
+          <t>9/19生鮮市場ダイイチ蒲田店(東京都大田区)</t>
+        </is>
+      </c>
+      <c r="D1743" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gmO</t>
+        </is>
+      </c>
+    </row>
+    <row r="1744">
+      <c r="A1744" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1744" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1744" t="inlineStr">
+        <is>
+          <t>9/24カネスエ上ノ町店(愛知県春日井市)</t>
+        </is>
+      </c>
+      <c r="D1744" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gmT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1745">
+      <c r="A1745" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1745" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1745" t="inlineStr">
+        <is>
+          <t>9/26ビッグ・エー春日部増富店</t>
+        </is>
+      </c>
+      <c r="D1745" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gii</t>
+        </is>
+      </c>
+    </row>
+    <row r="1746">
+      <c r="A1746" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1746" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1746" t="inlineStr">
+        <is>
+          <t>9/26三杉屋天六店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D1746" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gpn</t>
+        </is>
+      </c>
+    </row>
+    <row r="1747">
+      <c r="A1747" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1747" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1747" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D1747" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="1748">
+      <c r="A1748" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1748" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1748" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D1748" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="1749">
+      <c r="A1749" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1749" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1749" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D1749" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="1750">
+      <c r="A1750" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1750" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1750" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D1750" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1751">
+      <c r="A1751" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1751" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1751" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D1751" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="1752">
+      <c r="A1752" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1752" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1752" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D1752" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1753">
+      <c r="A1753" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1753" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1753" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D1753" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="1754">
+      <c r="A1754" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1754" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1754" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1754" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1755">
+      <c r="A1755" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1755" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1755" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1755" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1756">
+      <c r="A1756" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1756" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1756" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1756" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1757">
+      <c r="A1757" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1757" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1757" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1757" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1758">
+      <c r="A1758" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1758" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1758" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1758" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1759">
+      <c r="A1759" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1759" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1759" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1759" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1760">
+      <c r="A1760" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1760" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1760" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1760" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1761">
+      <c r="A1761" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1761" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1761" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1761" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1762">
+      <c r="A1762" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1762" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1762" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1762" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1763">
+      <c r="A1763" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1763" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1763" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1763" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1764">
+      <c r="A1764" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1764" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1764" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1764" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1765">
+      <c r="A1765" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1765" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1765" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1765" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1766">
+      <c r="A1766" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1766" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1766" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1766" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1767">
+      <c r="A1767" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1767" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1767" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1767" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1768">
+      <c r="A1768" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1768" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1768" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1768" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1769">
+      <c r="A1769" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1769" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1769" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1769" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1770">
+      <c r="A1770" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1770" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1770" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1770" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1771">
+      <c r="A1771" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1771" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1771" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1771" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1772">
+      <c r="A1772" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1772" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1772" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1772" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1773">
+      <c r="A1773" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1773" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1773" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1773" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1774">
+      <c r="A1774" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1774" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1774" t="inlineStr">
+        <is>
+          <t>関東地方川崎アリーナシティプロジェクト 2030年10月開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1774" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/33041</t>
+        </is>
+      </c>
+    </row>
+    <row r="1775">
+      <c r="A1775" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1775" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1775" t="inlineStr">
+        <is>
+          <t>関東地方アクアゲートヴィレッジ(旧:木更津ゲートウェイ・ヴィレッジ) 2027年度以降開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1775" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/18709</t>
+        </is>
+      </c>
+    </row>
+    <row r="1776">
+      <c r="A1776" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1776" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1776" t="inlineStr">
+        <is>
+          <t>関東地方WORLD TOWER RESIDENCE 2026年12月完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1776" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/19463</t>
+        </is>
+      </c>
+    </row>
+    <row r="1777">
+      <c r="A1777" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1777" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1777" t="inlineStr">
+        <is>
+          <t>関東地方アクロスプラザ宇都宮インターパーク 2025年10月3日(木)10時~順次開業！全5テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1777" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/39701</t>
+        </is>
+      </c>
+    </row>
+    <row r="1778">
+      <c r="A1778" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1778" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1778" t="inlineStr">
+        <is>
+          <t>関東地方関内駅前港町地区市街地再開発事業 2031年開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1778" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/17590</t>
+        </is>
+      </c>
+    </row>
+    <row r="1779">
+      <c r="A1779" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1779" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1779" t="inlineStr">
+        <is>
+          <t>中部地方スーパーセンタートライアル掛川店 2025年7月23日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1779" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/43118</t>
+        </is>
+      </c>
+    </row>
+    <row r="1780">
+      <c r="A1780" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1780" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1780" t="inlineStr">
+        <is>
+          <t>関東地方南小岩七丁目地区市街地再開発事業 2030年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1780" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/19966</t>
+        </is>
+      </c>
+    </row>
+    <row r="1781">
+      <c r="A1781" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1781" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1781" t="inlineStr">
+        <is>
+          <t>中国地方リベモール深川 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1781" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/48520</t>
+        </is>
+      </c>
+    </row>
+    <row r="1782">
+      <c r="A1782" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1782" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1782" t="inlineStr">
+        <is>
+          <t>関東地方虎ノ門アルセアタワー 2025年2月竣工！11店舗が出店！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1782" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26017</t>
+        </is>
+      </c>
+    </row>
+    <row r="1783">
+      <c r="A1783" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1783" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1783" t="inlineStr">
+        <is>
+          <t>関東地方ニトリふじみ野店 2026年10月開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1783" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48589</t>
+        </is>
+      </c>
+    </row>
+    <row r="1784">
+      <c r="A1784" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1784" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1784" t="inlineStr">
+        <is>
+          <t>関東地方高崎駅東口栄町地区市街地再開発事業 2029年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1784" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/29079</t>
+        </is>
+      </c>
+    </row>
+    <row r="1785">
+      <c r="A1785" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1785" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1785" t="inlineStr">
+        <is>
+          <t>中部地方イチビル イチ＊ビル 2025年11月27日(木)~順次開業！全40店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1785" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/31747</t>
+        </is>
+      </c>
+    </row>
+    <row r="1786">
+      <c r="A1786" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1786" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1786" t="inlineStr">
+        <is>
+          <t>九州地方OHASHI HILL ゆめアール大橋跡地に2025年4月18日(金)先行開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1786" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/27364</t>
+        </is>
+      </c>
+    </row>
+    <row r="1787">
+      <c r="A1787" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1787" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1787" t="inlineStr">
+        <is>
+          <t>北海道地方札幌4丁目プレイス 4PLA 2025年4月25日(金)から順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1787" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/32449</t>
+        </is>
+      </c>
+    </row>
+    <row r="1788">
+      <c r="A1788" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1788" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1788" t="inlineStr">
+        <is>
+          <t>九州地方スーパーセンタートライアル上毛店 2025年7月23日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1788" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/40427</t>
+        </is>
+      </c>
+    </row>
+    <row r="1789">
+      <c r="A1789" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1789" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1789" t="inlineStr">
+        <is>
+          <t>関東地方コープ幕張駅北口店 2025年2月25日(火)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1789" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/39459</t>
+        </is>
+      </c>
+    </row>
+    <row r="1790">
+      <c r="A1790" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1790" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1790" t="inlineStr">
+        <is>
+          <t>東北地方イオンスタイル八戸沼館 2025年4月25日(金)開業！全テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1790" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/42366</t>
+        </is>
+      </c>
+    </row>
+    <row r="1791">
+      <c r="A1791" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1791" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1791" t="inlineStr">
+        <is>
+          <t>北海道地方アーバンネット札幌リンクタワー 2026年9月1日(火)より順次開業！全10テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1791" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/22779</t>
+        </is>
+      </c>
+    </row>
+    <row r="1792">
+      <c r="A1792" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1792" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1792" t="inlineStr">
+        <is>
+          <t>関東地方新綱島MICCA 2026年10月28日(水)開業！21店舗が出店！テナントは？最新情報も！神奈川県横浜市港北区の東急新横浜線「新綱島駅」前に、歴史的古民家と木造商業施設が融合した新施設「新綱島MICCA（シンツナシマ ミッカ）」が2026年10月28日（水）にグランドオープン！正式オープン日が2026年10月28日（水）に決定！...2026.09.26関東地方</t>
+        </is>
+      </c>
+      <c r="D1792" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49470</t>
+        </is>
+      </c>
+    </row>
+    <row r="1793">
+      <c r="A1793" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1793" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1793" t="inlineStr">
+        <is>
+          <t>関西地方ヤマダデンキ テックランド堺南島店 2027年冬に開業予定！大阪府堺市に「ヤマダデンキ テックランド 堺南島店(仮称)」が2027年冬に開業予定！ヤマダ電機の中では大型店舗となります！そんな、ヤマダデンキ テックランド堺南島店について、テナントや開業日などを見ていきましょう！2026年4月13日　公...2026.09.26関西地方</t>
+        </is>
+      </c>
+      <c r="D1793" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/48191</t>
+        </is>
+      </c>
+    </row>
+    <row r="1794">
+      <c r="A1794" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1794" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1794" t="inlineStr">
+        <is>
+          <t>ハンズ新宿店／9月30日リニューアルオープン、自販機型サンプリング機を初導入</t>
+        </is>
+      </c>
+      <c r="D1794" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092512.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1795">
+      <c r="A1795" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1795" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1795" t="inlineStr">
+        <is>
+          <t>フレスタ／生鮮市場ベジタ店跡地に「ワークマンプラス」など3店舗10月以降オープン</t>
+        </is>
+      </c>
+      <c r="D1795" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092576.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1796">
+      <c r="A1796" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1796" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1796" t="inlineStr">
+        <is>
+          <t>ピソラ／熊本県に「PISOLA熊本嘉島店」10月21日オープン、九州地方に初出店</t>
+        </is>
+      </c>
+      <c r="D1796" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092541.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1797">
+      <c r="A1797" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1797" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1797" t="inlineStr">
+        <is>
+          <t>富澤商店／神奈川県に「ダイナシティ小田原店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D1797" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092575.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1798">
+      <c r="A1798" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1798" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1798" t="inlineStr">
+        <is>
+          <t>そごう横浜店／地下2階の酒売場9月30日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1798" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1799">
+      <c r="A1799" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1799" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1799" t="inlineStr">
+        <is>
+          <t>大黒天物産／熊本県山鹿市に「（仮称）ラ・ムー山鹿店」27年4月20日新設</t>
+        </is>
+      </c>
+      <c r="D1799" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0925012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1800">
+      <c r="A1800" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1800" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1800" t="inlineStr">
+        <is>
+          <t>ブルボン／大丸東京店にコンセプトストア期間限定オープン、10月21日から</t>
+        </is>
+      </c>
+      <c r="D1800" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092511.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1801">
+      <c r="A1801" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1801" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1801" t="inlineStr">
+        <is>
+          <t>サブウェイ／横浜市に「コーナン港北インター店」10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D1801" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092514.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1802">
+      <c r="A1802" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1802" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1802" t="inlineStr">
+        <is>
+          <t>薬王堂／群馬県伊勢崎市に「伊勢崎東店」27年4月18日新設</t>
+        </is>
+      </c>
+      <c r="D1802" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0925011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1803">
+      <c r="A1803" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1803" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1803" t="inlineStr">
+        <is>
+          <t>日販／図書館内の無人ショップ「TOSHOP」八王子に10月3日オープン</t>
+        </is>
+      </c>
+      <c r="D1803" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092577.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1804">
+      <c r="A1804" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1804" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1804" t="inlineStr">
+        <is>
+          <t>クリスプサラダワークス／東京都品川区に「大崎ニューシティ店」10月6日オープン</t>
+        </is>
+      </c>
+      <c r="D1804" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092574.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1805">
+      <c r="A1805" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1805" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1805" t="inlineStr">
+        <is>
+          <t>セブンタウン小豆沢／新ブランド「コムリエ」に10月9日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1805" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1806">
+      <c r="A1806" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1806" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1806" t="inlineStr">
+        <is>
+          <t>東京ミッドタウン八重洲／今秋、タイ料理などグルメな3店舗をオープン</t>
+        </is>
+      </c>
+      <c r="D1806" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092413.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1807">
+      <c r="A1807" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1807" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1807" t="inlineStr">
+        <is>
+          <t>カインズ／神奈川県綾瀬市に「（仮称）綾瀬店（店舗面積7560m2）」27年3月29日新設</t>
+        </is>
+      </c>
+      <c r="D1807" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0924011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1808">
+      <c r="A1808" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1808" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1808" t="inlineStr">
+        <is>
+          <t>ベイシア／埼玉県「本庄早稲田ゲート店」9月25日リニューアルオープン、新商品充実</t>
+        </is>
+      </c>
+      <c r="D1808" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092479.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1809">
+      <c r="A1809" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1809" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1809" t="inlineStr">
+        <is>
+          <t>イズミ／福岡県行橋市の「ゆめタウン行橋」10月2日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1809" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092441.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1810">
+      <c r="A1810" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1810" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1810" t="inlineStr">
+        <is>
+          <t>まいばすけっと／東京都内に「平井駅前店」「百草園駅前店」9月25日同時オープン</t>
+        </is>
+      </c>
+      <c r="D1810" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092478.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1811">
+      <c r="A1811" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1811" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1811" t="inlineStr">
+        <is>
+          <t>オオゼキ／神奈川県「中央林間店」10月2日リニューアルオープン、生鮮・総菜強化</t>
+        </is>
+      </c>
+      <c r="D1811" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092475.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1812">
+      <c r="A1812" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1812" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1812" t="inlineStr">
+        <is>
+          <t>コメリ／大阪府内初のPRO業態「富田林店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D1812" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092477.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1813">
+      <c r="A1813" t="inlineStr">
+        <is>
+          <t>2026年09月27日</t>
+        </is>
+      </c>
+      <c r="B1813" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1813" t="inlineStr">
+        <is>
+          <t>ゴンチャ／「南砂町ショッピングセンターSUNAMO」に新店舗10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D1813" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092476.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-28
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1813"/>
+  <dimension ref="A1:D1853"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40302,6 +40302,886 @@
         </is>
       </c>
     </row>
+    <row r="1814">
+      <c r="A1814" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1814" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1814" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1814" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1815">
+      <c r="A1815" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1815" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1815" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1815" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1816">
+      <c r="A1816" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1816" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1816" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1816" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1817">
+      <c r="A1817" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1817" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1817" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1817" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1818">
+      <c r="A1818" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1818" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1818" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1818" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1819">
+      <c r="A1819" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1819" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1819" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1819" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1820">
+      <c r="A1820" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1820" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1820" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1820" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1821">
+      <c r="A1821" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1821" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1821" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1821" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1822">
+      <c r="A1822" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1822" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1822" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1822" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1823">
+      <c r="A1823" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1823" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1823" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1823" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1824">
+      <c r="A1824" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1824" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1824" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1824" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1825">
+      <c r="A1825" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1825" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1825" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1825" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1826">
+      <c r="A1826" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1826" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1826" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1826" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1827">
+      <c r="A1827" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1827" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1827" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1827" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1828">
+      <c r="A1828" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1828" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1828" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1828" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1829">
+      <c r="A1829" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1829" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1829" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1829" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1830">
+      <c r="A1830" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1830" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1830" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1830" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1831">
+      <c r="A1831" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1831" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1831" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1831" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1832">
+      <c r="A1832" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1832" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1832" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1832" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1833">
+      <c r="A1833" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1833" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1833" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1833" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1834">
+      <c r="A1834" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1834" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1834" t="inlineStr">
+        <is>
+          <t>ミーナ津田沼／10月16日リニューアル、飲食ゾーン「しんつだぬま食堂」オープン</t>
+        </is>
+      </c>
+      <c r="D1834" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092873.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1835">
+      <c r="A1835" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1835" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1835" t="inlineStr">
+        <is>
+          <t>東急／古民家を活用した複合施設「新綱島ミッカ」10月28日グランドオープン</t>
+        </is>
+      </c>
+      <c r="D1835" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092875.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1836">
+      <c r="A1836" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1836" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1836" t="inlineStr">
+        <is>
+          <t>JR博多シティ／福岡市「アミュプラザ天神」来春オープン、ヴィオロを順次改装</t>
+        </is>
+      </c>
+      <c r="D1836" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092874.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1837">
+      <c r="A1837" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1837" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1837" t="inlineStr">
+        <is>
+          <t>ローソン／「ハッピーローソンタウン日野高幡台店」近くにオンライン診療受診施設を開設</t>
+        </is>
+      </c>
+      <c r="D1837" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1838">
+      <c r="A1838" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1838" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1838" t="inlineStr">
+        <is>
+          <t>マックスバリュ東海／愛知県豊橋市に「（仮称）マックスバリュ豊橋西幸町店（店舗面積4344m2）」27年4月1日新設</t>
+        </is>
+      </c>
+      <c r="D1838" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0928012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1839">
+      <c r="A1839" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1839" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1839" t="inlineStr">
+        <is>
+          <t>エディオン／北海道の「旭川永山店」10月16日移転オープン</t>
+        </is>
+      </c>
+      <c r="D1839" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092815.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1840">
+      <c r="A1840" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1840" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1840" t="inlineStr">
+        <is>
+          <t>Salomon／東京都「サロモンストア 吉祥寺店」10月2日オープン、ナイキ跡地に出店</t>
+        </is>
+      </c>
+      <c r="D1840" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092877.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1841">
+      <c r="A1841" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1841" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1841" t="inlineStr">
+        <is>
+          <t>コロワイド／岐阜県に「大戸屋ごはん処 多治見店」オープン</t>
+        </is>
+      </c>
+      <c r="D1841" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092876.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1842">
+      <c r="A1842" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1842" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1842" t="inlineStr">
+        <is>
+          <t>まいばすけっと／神奈川県川崎市「日進町市電通り店」10月30日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1842" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092842.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1843">
+      <c r="A1843" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1843" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1843" t="inlineStr">
+        <is>
+          <t>ワッツ／福岡市中央区に「ワッツウィズ 今川マックスバリュエクスプレス店」オープン</t>
+        </is>
+      </c>
+      <c r="D1843" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092841.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1844">
+      <c r="A1844" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1844" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1844" t="inlineStr">
+        <is>
+          <t>ハンズ新宿店／9月30日リニューアルオープン、自販機型サンプリング機を初導入</t>
+        </is>
+      </c>
+      <c r="D1844" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092512.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1845">
+      <c r="A1845" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1845" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1845" t="inlineStr">
+        <is>
+          <t>フレスタ／生鮮市場ベジタ店跡地に「ワークマンプラス」など3店舗10月以降オープン</t>
+        </is>
+      </c>
+      <c r="D1845" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092576.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1846">
+      <c r="A1846" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1846" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1846" t="inlineStr">
+        <is>
+          <t>ピソラ／熊本県に「PISOLA熊本嘉島店」10月21日オープン、九州地方に初出店</t>
+        </is>
+      </c>
+      <c r="D1846" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092541.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1847">
+      <c r="A1847" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1847" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1847" t="inlineStr">
+        <is>
+          <t>富澤商店／神奈川県に「ダイナシティ小田原店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D1847" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092575.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1848">
+      <c r="A1848" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1848" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1848" t="inlineStr">
+        <is>
+          <t>そごう横浜店／地下2階の酒売場9月30日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D1848" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1849">
+      <c r="A1849" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1849" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1849" t="inlineStr">
+        <is>
+          <t>大黒天物産／熊本県山鹿市に「（仮称）ラ・ムー山鹿店」27年4月20日新設</t>
+        </is>
+      </c>
+      <c r="D1849" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0925012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1850">
+      <c r="A1850" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1850" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1850" t="inlineStr">
+        <is>
+          <t>ブルボン／大丸東京店にコンセプトストア期間限定オープン、10月21日から</t>
+        </is>
+      </c>
+      <c r="D1850" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092511.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1851">
+      <c r="A1851" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1851" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1851" t="inlineStr">
+        <is>
+          <t>サブウェイ／横浜市に「コーナン港北インター店」10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D1851" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092514.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1852">
+      <c r="A1852" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1852" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1852" t="inlineStr">
+        <is>
+          <t>薬王堂／群馬県伊勢崎市に「伊勢崎東店」27年4月18日新設</t>
+        </is>
+      </c>
+      <c r="D1852" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0925011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1853">
+      <c r="A1853" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1853" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1853" t="inlineStr">
+        <is>
+          <t>日販／図書館内の無人ショップ「TOSHOP」八王子に10月3日オープン</t>
+        </is>
+      </c>
+      <c r="D1853" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092577.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-29
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1853"/>
+  <dimension ref="A1:D1913"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41182,6 +41182,1326 @@
         </is>
       </c>
     </row>
+    <row r="1854">
+      <c r="A1854" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1854" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1854" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1854" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1855">
+      <c r="A1855" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1855" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1855" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1855" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1856">
+      <c r="A1856" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1856" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1856" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1856" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1857">
+      <c r="A1857" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1857" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1857" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1857" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1858">
+      <c r="A1858" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1858" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1858" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1858" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1859">
+      <c r="A1859" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1859" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1859" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1859" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1860">
+      <c r="A1860" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1860" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1860" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1860" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1861">
+      <c r="A1861" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1861" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1861" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1861" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1862">
+      <c r="A1862" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1862" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1862" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1862" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1863">
+      <c r="A1863" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1863" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1863" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1863" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1864">
+      <c r="A1864" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1864" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1864" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1864" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1865">
+      <c r="A1865" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1865" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1865" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1865" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1866">
+      <c r="A1866" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1866" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1866" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1866" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1867">
+      <c r="A1867" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1867" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1867" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1867" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1868">
+      <c r="A1868" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1868" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1868" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1868" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1869">
+      <c r="A1869" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1869" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1869" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1869" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1870">
+      <c r="A1870" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1870" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1870" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1870" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1871">
+      <c r="A1871" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1871" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1871" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1871" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1872">
+      <c r="A1872" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1872" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1872" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1872" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1873">
+      <c r="A1873" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1873" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1873" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1873" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1874">
+      <c r="A1874" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1874" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1874" t="inlineStr">
+        <is>
+          <t>中部地方コストコが山梨県初出店！南アルプス市に出店へ！2025年4月11日(金)開業予定！場所は？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1874" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/26058</t>
+        </is>
+      </c>
+    </row>
+    <row r="1875">
+      <c r="A1875" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1875" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1875" t="inlineStr">
+        <is>
+          <t>関西地方イオン京橋店跡地 将来的に再開発へ！2028年以降開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1875" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/16733</t>
+        </is>
+      </c>
+    </row>
+    <row r="1876">
+      <c r="A1876" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1876" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1876" t="inlineStr">
+        <is>
+          <t>東北地方滝沢チャグチャグモール いとく滝沢店は2026年4月17日(金)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1876" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/31250</t>
+        </is>
+      </c>
+    </row>
+    <row r="1877">
+      <c r="A1877" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1877" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1877" t="inlineStr">
+        <is>
+          <t>九州地方天神大樹 イムズ跡地 2027年秋開業！どんな計画？テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1877" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/27165</t>
+        </is>
+      </c>
+    </row>
+    <row r="1878">
+      <c r="A1878" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1878" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1878" t="inlineStr">
+        <is>
+          <t>中部地方アスナル金山 2036年3月閉店！当初計画の再開発の内容は？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1878" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/45176</t>
+        </is>
+      </c>
+    </row>
+    <row r="1879">
+      <c r="A1879" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1879" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1879" t="inlineStr">
+        <is>
+          <t>東北地方イオンタウン外旭川 秋田市に開業予定！どのような商業施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1879" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/24596</t>
+        </is>
+      </c>
+    </row>
+    <row r="1880">
+      <c r="A1880" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1880" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1880" t="inlineStr">
+        <is>
+          <t>関西地方京都城陽プレミアム・アウトレット 2028年以降開業！150店舗が出店予定！どのような商業施設に？</t>
+        </is>
+      </c>
+      <c r="D1880" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/10189</t>
+        </is>
+      </c>
+    </row>
+    <row r="1881">
+      <c r="A1881" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1881" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1881" t="inlineStr">
+        <is>
+          <t>北海道地方ヤマダデンキ Tecc LIFE SELECT札幌北33条店 2025年11月28日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1881" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/40915</t>
+        </is>
+      </c>
+    </row>
+    <row r="1882">
+      <c r="A1882" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1882" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1882" t="inlineStr">
+        <is>
+          <t>中国地方スーパーセンタートライアル勝央店 2027年1月下旬に開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1882" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/47478</t>
+        </is>
+      </c>
+    </row>
+    <row r="1883">
+      <c r="A1883" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1883" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1883" t="inlineStr">
+        <is>
+          <t>関東地方高崎駅東口栄町地区市街地再開発事業 2029年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1883" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/29079</t>
+        </is>
+      </c>
+    </row>
+    <row r="1884">
+      <c r="A1884" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1884" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1884" t="inlineStr">
+        <is>
+          <t>北海道地方ケーズデンキ帯広店 2025年3月20日(木・祝)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1884" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/40212</t>
+        </is>
+      </c>
+    </row>
+    <row r="1885">
+      <c r="A1885" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1885" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1885" t="inlineStr">
+        <is>
+          <t>関東地方ミナモニ有明 江東区有明1丁目計画 大和ハウスのマンションと商業施設に！2026年5月13日(水)9時~開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1885" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/35626</t>
+        </is>
+      </c>
+    </row>
+    <row r="1886">
+      <c r="A1886" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1886" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1886" t="inlineStr">
+        <is>
+          <t>関東地方東京インテリア家具 八王子店が2026年6月5日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1886" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/46004</t>
+        </is>
+      </c>
+    </row>
+    <row r="1887">
+      <c r="A1887" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1887" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1887" t="inlineStr">
+        <is>
+          <t>関東地方武蔵小金井駅北口駅前東地区市街地再開発事業 2030年1月完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1887" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48940</t>
+        </is>
+      </c>
+    </row>
+    <row r="1888">
+      <c r="A1888" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1888" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1888" t="inlineStr">
+        <is>
+          <t>関東地方Beisia Foods Park 伊勢崎境保泉店 2028年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1888" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47770</t>
+        </is>
+      </c>
+    </row>
+    <row r="1889">
+      <c r="A1889" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1889" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1889" t="inlineStr">
+        <is>
+          <t>九州地方スーパーセンタートライアル阿蘇店 2026年11月中旬に開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1889" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/48550</t>
+        </is>
+      </c>
+    </row>
+    <row r="1890">
+      <c r="A1890" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1890" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1890" t="inlineStr">
+        <is>
+          <t>関東地方みなとみらい21中央地区60・61街区開発事業 2029年春開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1890" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36914</t>
+        </is>
+      </c>
+    </row>
+    <row r="1891">
+      <c r="A1891" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1891" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1891" t="inlineStr">
+        <is>
+          <t>関東地方イオンスタイル大宮西 2027年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1891" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48705</t>
+        </is>
+      </c>
+    </row>
+    <row r="1892">
+      <c r="A1892" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1892" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1892" t="inlineStr">
+        <is>
+          <t>関東地方松戸駅 新駅ビルに商業施設 2027年春開業！テナントは？最新情報も！千葉県松戸市のJR松戸駅の駅直結型複合ビル「松戸駅 新駅ビル商業施設(仮称)」が2027年春開業！松戸駅線路上空に地上6階建ての新たな駅ビルが建設中！東西自由通路が幅14mへ大幅拡幅されるとともに、新公衆トイレ新設や改札切り替え、西口エスカ...2026.09.29関東地方</t>
+        </is>
+      </c>
+      <c r="D1892" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/29225</t>
+        </is>
+      </c>
+    </row>
+    <row r="1893">
+      <c r="A1893" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1893" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1893" t="inlineStr">
+        <is>
+          <t>中国地方岡山ゲートプレイス プラウドタワー岡山 2027年3月20日(土)開業！テナントは？最新情報も！岡山県岡山市北区に再開発複合ビル「OKAYAMA GATE PLACE（オカヤマゲートプレイス）」が2027年3月20日(土)にグランドオープン！正式施設名称が「OKAYAMA GATE PLACE」に決定！野村不動産の分譲マンション「プラ...2026.09.29中国地方</t>
+        </is>
+      </c>
+      <c r="D1893" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/16944</t>
+        </is>
+      </c>
+    </row>
+    <row r="1894">
+      <c r="A1894" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1894" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1894" t="inlineStr">
+        <is>
+          <t>コープみらい／東京都に「コープ小川駅前店」10月6日オープン、年商15.9億円を計画</t>
+        </is>
+      </c>
+      <c r="D1894" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092941.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1895">
+      <c r="A1895" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1895" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1895" t="inlineStr">
+        <is>
+          <t>しまむら／京都市四条河原町に新旗艦店29年オープン、7階建ての商業ビルを計画</t>
+        </is>
+      </c>
+      <c r="D1895" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092976.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1896">
+      <c r="A1896" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1896" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1896" t="inlineStr">
+        <is>
+          <t>マルト／福島県いわき市に「（仮称）いわきスマートタウン計画（店舗面積2813m2）」27年4月20日新設</t>
+        </is>
+      </c>
+      <c r="D1896" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0929013.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1897">
+      <c r="A1897" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1897" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1897" t="inlineStr">
+        <is>
+          <t>ツルハ／北海道江別市に「（仮称）ツルハドラッグ野幌若葉町店」27年4月18日新設</t>
+        </is>
+      </c>
+      <c r="D1897" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0929012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1898">
+      <c r="A1898" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1898" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1898" t="inlineStr">
+        <is>
+          <t>国分首都圏／横浜市に酒類専門店「EXIVIN そごう横浜店」オープン、500品目を展開</t>
+        </is>
+      </c>
+      <c r="D1898" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092943.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1899">
+      <c r="A1899" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1899" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1899" t="inlineStr">
+        <is>
+          <t>まいばすけっと／都内に「永福4丁目店」「国立中1丁目店」10月2日オープン</t>
+        </is>
+      </c>
+      <c r="D1899" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092974.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1900">
+      <c r="A1900" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1900" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1900" t="inlineStr">
+        <is>
+          <t>相鉄ライフ三ツ境／10月30日に開業40周年、ポイントプレゼント企画も</t>
+        </is>
+      </c>
+      <c r="D1900" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092912.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1901">
+      <c r="A1901" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1901" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1901" t="inlineStr">
+        <is>
+          <t>三井アウトレットパーク仙台港／事業延長が決定</t>
+        </is>
+      </c>
+      <c r="D1901" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092914.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1902">
+      <c r="A1902" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1902" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1902" t="inlineStr">
+        <is>
+          <t>大黒屋／高級腕時計専門店「中野ブロードウェイ店」9月30日オープン</t>
+        </is>
+      </c>
+      <c r="D1902" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092911.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1903">
+      <c r="A1903" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1903" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1903" t="inlineStr">
+        <is>
+          <t>ノジマ／千葉県「イオン新松戸」に新店舗10月2日オープン</t>
+        </is>
+      </c>
+      <c r="D1903" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092973.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1904">
+      <c r="A1904" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1904" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1904" t="inlineStr">
+        <is>
+          <t>イオンファンタジー／愛知県春日井市に「クレーン横丁 極」10月7日東海初オープン</t>
+        </is>
+      </c>
+      <c r="D1904" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092972.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1905">
+      <c r="A1905" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1905" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1905" t="inlineStr">
+        <is>
+          <t>ホットランド／「厚切りとんかつ よし平 仙台中央店」9月30日オープン、宮城3店舗目</t>
+        </is>
+      </c>
+      <c r="D1905" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092971.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1906">
+      <c r="A1906" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1906" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1906" t="inlineStr">
+        <is>
+          <t>ミーナ津田沼／10月16日リニューアル、飲食ゾーン「しんつだぬま食堂」オープン</t>
+        </is>
+      </c>
+      <c r="D1906" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092873.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1907">
+      <c r="A1907" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1907" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1907" t="inlineStr">
+        <is>
+          <t>東急／古民家を活用した複合施設「新綱島ミッカ」10月28日グランドオープン</t>
+        </is>
+      </c>
+      <c r="D1907" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092875.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1908">
+      <c r="A1908" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1908" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1908" t="inlineStr">
+        <is>
+          <t>JR博多シティ／福岡市「アミュプラザ天神」来春オープン、ヴィオロを順次改装</t>
+        </is>
+      </c>
+      <c r="D1908" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092874.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1909">
+      <c r="A1909" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1909" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1909" t="inlineStr">
+        <is>
+          <t>ローソン／「ハッピーローソンタウン日野高幡台店」近くにオンライン診療受診施設を開設</t>
+        </is>
+      </c>
+      <c r="D1909" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1910">
+      <c r="A1910" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1910" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1910" t="inlineStr">
+        <is>
+          <t>マックスバリュ東海／愛知県豊橋市に「（仮称）マックスバリュ豊橋西幸町店（店舗面積4344m2）」27年4月1日新設</t>
+        </is>
+      </c>
+      <c r="D1910" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0928012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1911">
+      <c r="A1911" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1911" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1911" t="inlineStr">
+        <is>
+          <t>エディオン／北海道の「旭川永山店」10月16日移転オープン</t>
+        </is>
+      </c>
+      <c r="D1911" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092815.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1912">
+      <c r="A1912" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1912" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1912" t="inlineStr">
+        <is>
+          <t>Salomon／東京都「サロモンストア 吉祥寺店」10月2日オープン、ナイキ跡地に出店</t>
+        </is>
+      </c>
+      <c r="D1912" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092877.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1913">
+      <c r="A1913" t="inlineStr">
+        <is>
+          <t>2026年09月29日</t>
+        </is>
+      </c>
+      <c r="B1913" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1913" t="inlineStr">
+        <is>
+          <t>コロワイド／岐阜県に「大戸屋ごはん処 多治見店」オープン</t>
+        </is>
+      </c>
+      <c r="D1913" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092876.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-30
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1913"/>
+  <dimension ref="A1:D1981"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42502,6 +42502,1502 @@
         </is>
       </c>
     </row>
+    <row r="1914">
+      <c r="A1914" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1914" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1914" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D1914" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="1915">
+      <c r="A1915" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1915" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1915" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D1915" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="1916">
+      <c r="A1916" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1916" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1916" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D1916" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="1917">
+      <c r="A1917" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1917" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1917" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D1917" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1918">
+      <c r="A1918" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1918" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1918" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D1918" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="1919">
+      <c r="A1919" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1919" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1919" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D1919" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="1920">
+      <c r="A1920" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1920" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1920" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D1920" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1921">
+      <c r="A1921" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1921" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C1921" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D1921" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="1922">
+      <c r="A1922" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1922" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1922" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1922" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1923">
+      <c r="A1923" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1923" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1923" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1923" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1924">
+      <c r="A1924" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1924" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1924" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1924" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1925">
+      <c r="A1925" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1925" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1925" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1925" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1926">
+      <c r="A1926" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1926" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1926" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1926" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1927">
+      <c r="A1927" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1927" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1927" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1927" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1928">
+      <c r="A1928" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1928" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1928" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1928" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1929">
+      <c r="A1929" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1929" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1929" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1929" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1930">
+      <c r="A1930" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1930" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1930" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1930" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1931">
+      <c r="A1931" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1931" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1931" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1931" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1932">
+      <c r="A1932" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1932" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1932" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1932" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1933">
+      <c r="A1933" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1933" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1933" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1933" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1934">
+      <c r="A1934" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1934" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1934" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1934" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1935">
+      <c r="A1935" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1935" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1935" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1935" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1936">
+      <c r="A1936" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1936" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1936" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1936" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1937">
+      <c r="A1937" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1937" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1937" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1937" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1938">
+      <c r="A1938" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1938" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1938" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1938" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1939">
+      <c r="A1939" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1939" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1939" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1939" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1940">
+      <c r="A1940" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1940" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1940" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1940" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1941">
+      <c r="A1941" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1941" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1941" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1941" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1942">
+      <c r="A1942" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1942" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1942" t="inlineStr">
+        <is>
+          <t>東北地方ニトリいわき店(仮称) 2026年9月開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1942" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/48631</t>
+        </is>
+      </c>
+    </row>
+    <row r="1943">
+      <c r="A1943" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1943" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1943" t="inlineStr">
+        <is>
+          <t>中部地方ニトリ焼津店 2025年6月27日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1943" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/41145</t>
+        </is>
+      </c>
+    </row>
+    <row r="1944">
+      <c r="A1944" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1944" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1944" t="inlineStr">
+        <is>
+          <t>東北地方【電力ビル】一番町三丁目七番地区市街地再開発事業 2029年開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1944" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/31239</t>
+        </is>
+      </c>
+    </row>
+    <row r="1945">
+      <c r="A1945" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1945" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1945" t="inlineStr">
+        <is>
+          <t>関西地方泉ケ丘駅前活性化計画 計画再始動！商業施設は2028年度開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1945" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/23983</t>
+        </is>
+      </c>
+    </row>
+    <row r="1946">
+      <c r="A1946" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1946" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1946" t="inlineStr">
+        <is>
+          <t>関東地方アクロスプラザ宇都宮インターパーク 2025年10月3日(木)10時~順次開業！全5テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1946" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/39701</t>
+        </is>
+      </c>
+    </row>
+    <row r="1947">
+      <c r="A1947" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1947" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1947" t="inlineStr">
+        <is>
+          <t>東北地方ヨークベニマル岩沼店 リニューアルオープン 2025年11月28日(金)9時~開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1947" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/38131</t>
+        </is>
+      </c>
+    </row>
+    <row r="1948">
+      <c r="A1948" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1948" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1948" t="inlineStr">
+        <is>
+          <t>関西地方アスモ大和郡山跡地 複合商業施設 2028年度開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1948" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/46357</t>
+        </is>
+      </c>
+    </row>
+    <row r="1949">
+      <c r="A1949" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1949" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1949" t="inlineStr">
+        <is>
+          <t>九州地方スーパーセンタートライアル八代古閑浜店 2026年6月10日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1949" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/45102</t>
+        </is>
+      </c>
+    </row>
+    <row r="1950">
+      <c r="A1950" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1950" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1950" t="inlineStr">
+        <is>
+          <t>北海道地方コメリパワー恵庭店 2025年3月21日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1950" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/40058</t>
+        </is>
+      </c>
+    </row>
+    <row r="1951">
+      <c r="A1951" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1951" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1951" t="inlineStr">
+        <is>
+          <t>関東地方宮益坂地区市街地再開発事業 2031年秋完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1951" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/28157</t>
+        </is>
+      </c>
+    </row>
+    <row r="1952">
+      <c r="A1952" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1952" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1952" t="inlineStr">
+        <is>
+          <t>関東地方神宮外苑地区市街地再開発事業 2030年より街びらき！2038年完成！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1952" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/33186</t>
+        </is>
+      </c>
+    </row>
+    <row r="1953">
+      <c r="A1953" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1953" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1953" t="inlineStr">
+        <is>
+          <t>東北地方イオンタウン三沢 2031年以降開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1953" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/47877</t>
+        </is>
+      </c>
+    </row>
+    <row r="1954">
+      <c r="A1954" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1954" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1954" t="inlineStr">
+        <is>
+          <t>九州地方トライアルスマート東長崎店 2025年8月20日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1954" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/42038</t>
+        </is>
+      </c>
+    </row>
+    <row r="1955">
+      <c r="A1955" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1955" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1955" t="inlineStr">
+        <is>
+          <t>関東地方(仮称)小杉町一丁目計画 武蔵小杉駅北口 タワマンと商業施設に！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1955" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/35200</t>
+        </is>
+      </c>
+    </row>
+    <row r="1956">
+      <c r="A1956" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1956" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1956" t="inlineStr">
+        <is>
+          <t>関西地方Kubota field(クボタフィールド) 2032年以降開業予定！クボタららアリーナや商業施設が誕生！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1956" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49228</t>
+        </is>
+      </c>
+    </row>
+    <row r="1957">
+      <c r="A1957" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1957" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1957" t="inlineStr">
+        <is>
+          <t>関東地方ビバタウン沼田再開発 ベルクが出店 2025年7月23日(水)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1957" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/40309</t>
+        </is>
+      </c>
+    </row>
+    <row r="1958">
+      <c r="A1958" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1958" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1958" t="inlineStr">
+        <is>
+          <t>中国地方カインズ日吉津店 2025年3月12日(水)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1958" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/34869</t>
+        </is>
+      </c>
+    </row>
+    <row r="1959">
+      <c r="A1959" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1959" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1959" t="inlineStr">
+        <is>
+          <t>九州地方遠賀川駅南商業店舗 2026年秋開業！ロピアが出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D1959" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/48612</t>
+        </is>
+      </c>
+    </row>
+    <row r="1960">
+      <c r="A1960" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1960" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1960" t="inlineStr">
+        <is>
+          <t>関西地方イオンタウン堺水賀池 2027年冬開業！30店舗が出店！テナントは？最新情報も！大阪府堺市中区深井の水賀池公園のプロジェクト「水賀池公園整備事業」において、イオンタウン堺水賀池が2027年冬開業！イオンタウン公式リリースが発表！深井駅徒歩3分、水賀池公園に「イオンタウン堺水賀池」が誕生！敷地面積約1.46万㎡・地上2階...2026.09.30関西地方</t>
+        </is>
+      </c>
+      <c r="D1960" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/45734</t>
+        </is>
+      </c>
+    </row>
+    <row r="1961">
+      <c r="A1961" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1961" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C1961" t="inlineStr">
+        <is>
+          <t>関東地方JR武蔵境駅東側開発 2028年開業！テナントは？最新情報も！東京都武蔵野市のJR武蔵境駅東側エリアに、JR東日本による駅直結複合ビル「（仮称）武蔵境駅東側駅ビル」が2028年度冬に開業！JR東日本が「（仮称）武蔵境駅東側駅ビル」の建設工事に2026年10月より本格着手！地上9階建て・延床約6,000...2026.09.30関東地方</t>
+        </is>
+      </c>
+      <c r="D1961" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48480</t>
+        </is>
+      </c>
+    </row>
+    <row r="1962">
+      <c r="A1962" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1962" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1962" t="inlineStr">
+        <is>
+          <t>イオンリテール／「そよらつくば学園の森」10月25日オープン、バーガーキング・ダイソーなど出店</t>
+        </is>
+      </c>
+      <c r="D1962" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093016.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1963">
+      <c r="A1963" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1963" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1963" t="inlineStr">
+        <is>
+          <t>JR東日本／神奈川県「逗子駅ビル」の建設工事を開始、28年春に商業施設オープン</t>
+        </is>
+      </c>
+      <c r="D1963" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093074.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1964">
+      <c r="A1964" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1964" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1964" t="inlineStr">
+        <is>
+          <t>新宿マルイ／PLAZAの新業態「プラザ トーキョープラス」11月20日オープン</t>
+        </is>
+      </c>
+      <c r="D1964" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093076.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1965">
+      <c r="A1965" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1965" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1965" t="inlineStr">
+        <is>
+          <t>大丸梅田店／「太陽ノ塔」「堂島ロール」の新業態など新規5店舗が12月1日オープン</t>
+        </is>
+      </c>
+      <c r="D1965" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093077.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1966">
+      <c r="A1966" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1966" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1966" t="inlineStr">
+        <is>
+          <t>コーナン商事／鹿児島県に初出店「コーナンPRO 鹿児島東開店」オープン</t>
+        </is>
+      </c>
+      <c r="D1966" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093072.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1967">
+      <c r="A1967" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1967" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1967" t="inlineStr">
+        <is>
+          <t>東京インテリア家具／栃木県小山市に「（仮称）マックス小山店」27年4月27日新設</t>
+        </is>
+      </c>
+      <c r="D1967" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0930012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1968">
+      <c r="A1968" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1968" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1968" t="inlineStr">
+        <is>
+          <t>クリエイトSD／茨城県つくば市に「つくば市学園の森商業施設」27年4月13日新設</t>
+        </is>
+      </c>
+      <c r="D1968" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0930011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1969">
+      <c r="A1969" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1969" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1969" t="inlineStr">
+        <is>
+          <t>ビームス／香川・金刀比羅宮表参道に「ビームス ジャパン 琴平」10月31日オープン</t>
+        </is>
+      </c>
+      <c r="D1969" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093073.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1970">
+      <c r="A1970" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1970" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1970" t="inlineStr">
+        <is>
+          <t>レデイ薬局／愛媛県松山市に調剤薬局「レデイ薬局 南斎院店」10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D1970" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1971">
+      <c r="A1971" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1971" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1971" t="inlineStr">
+        <is>
+          <t>猿田彦珈琲／「京都高島屋 S.C.T8」に新店舗10月2日オープン</t>
+        </is>
+      </c>
+      <c r="D1971" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093071.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1972">
+      <c r="A1972" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1972" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1972" t="inlineStr">
+        <is>
+          <t>コロワイド／福島初出店「チーズガーデン イオンモール伊達店」11月27日オープン</t>
+        </is>
+      </c>
+      <c r="D1972" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093075.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1973">
+      <c r="A1973" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1973" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1973" t="inlineStr">
+        <is>
+          <t>串カツ田中／滋賀県大津市に「膳所店」オープン、膳所駅から徒歩3分</t>
+        </is>
+      </c>
+      <c r="D1973" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093041.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1974">
+      <c r="A1974" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1974" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1974" t="inlineStr">
+        <is>
+          <t>コープみらい／東京都に「コープ小川駅前店」10月6日オープン、年商15.9億円を計画</t>
+        </is>
+      </c>
+      <c r="D1974" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092941.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1975">
+      <c r="A1975" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1975" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1975" t="inlineStr">
+        <is>
+          <t>しまむら／京都市四条河原町に新旗艦店29年オープン、7階建ての商業ビルを計画</t>
+        </is>
+      </c>
+      <c r="D1975" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092976.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1976">
+      <c r="A1976" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1976" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1976" t="inlineStr">
+        <is>
+          <t>マルト／福島県いわき市に「（仮称）いわきスマートタウン計画（店舗面積2813m2）」27年4月20日新設</t>
+        </is>
+      </c>
+      <c r="D1976" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0929013.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1977">
+      <c r="A1977" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1977" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1977" t="inlineStr">
+        <is>
+          <t>ツルハ／北海道江別市に「（仮称）ツルハドラッグ野幌若葉町店」27年4月18日新設</t>
+        </is>
+      </c>
+      <c r="D1977" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0929012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1978">
+      <c r="A1978" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1978" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1978" t="inlineStr">
+        <is>
+          <t>国分首都圏／横浜市に酒類専門店「EXIVIN そごう横浜店」オープン、500品目を展開</t>
+        </is>
+      </c>
+      <c r="D1978" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092943.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1979">
+      <c r="A1979" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1979" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1979" t="inlineStr">
+        <is>
+          <t>まいばすけっと／都内に「永福4丁目店」「国立中1丁目店」10月2日オープン</t>
+        </is>
+      </c>
+      <c r="D1979" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092974.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1980">
+      <c r="A1980" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1980" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1980" t="inlineStr">
+        <is>
+          <t>相鉄ライフ三ツ境／10月30日に開業40周年、ポイントプレゼント企画も</t>
+        </is>
+      </c>
+      <c r="D1980" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092912.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1981">
+      <c r="A1981" t="inlineStr">
+        <is>
+          <t>2026年09月30日</t>
+        </is>
+      </c>
+      <c r="B1981" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C1981" t="inlineStr">
+        <is>
+          <t>三井アウトレットパーク仙台港／事業延長が決定</t>
+        </is>
+      </c>
+      <c r="D1981" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092914.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-01
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1981"/>
+  <dimension ref="A1:D2041"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43998,6 +43998,1326 @@
         </is>
       </c>
     </row>
+    <row r="1982">
+      <c r="A1982" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1982" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1982" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1982" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1983">
+      <c r="A1983" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1983" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1983" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1983" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1984">
+      <c r="A1984" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1984" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1984" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1984" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1985">
+      <c r="A1985" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1985" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1985" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1985" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1986">
+      <c r="A1986" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1986" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1986" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1986" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1987">
+      <c r="A1987" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1987" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1987" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1987" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1988">
+      <c r="A1988" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1988" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1988" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1988" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1989">
+      <c r="A1989" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1989" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1989" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1989" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1990">
+      <c r="A1990" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1990" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1990" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D1990" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1991">
+      <c r="A1991" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1991" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1991" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1991" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1992">
+      <c r="A1992" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1992" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1992" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D1992" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1993">
+      <c r="A1993" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1993" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1993" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D1993" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1994">
+      <c r="A1994" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1994" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1994" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D1994" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1995">
+      <c r="A1995" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1995" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1995" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D1995" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1996">
+      <c r="A1996" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1996" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1996" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1996" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1997">
+      <c r="A1997" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1997" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1997" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D1997" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1998">
+      <c r="A1998" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1998" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1998" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D1998" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="1999">
+      <c r="A1999" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B1999" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C1999" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D1999" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2000">
+      <c r="A2000" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2000" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2000" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2000" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2001">
+      <c r="A2001" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2001" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2001" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2001" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2002">
+      <c r="A2002" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2002" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2002" t="inlineStr">
+        <is>
+          <t>九州地方天神ビジネスセンターII 2026年8月4日(火)開業！全16テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2002" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/41150</t>
+        </is>
+      </c>
+    </row>
+    <row r="2003">
+      <c r="A2003" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2003" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2003" t="inlineStr">
+        <is>
+          <t>関西地方コメリパワー平群店 2025年7月16日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2003" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39836</t>
+        </is>
+      </c>
+    </row>
+    <row r="2004">
+      <c r="A2004" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2004" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2004" t="inlineStr">
+        <is>
+          <t>関東地方イオン海老名店 2026年5月中旬で一旦閉店し建て替えへ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2004" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47523</t>
+        </is>
+      </c>
+    </row>
+    <row r="2005">
+      <c r="A2005" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2005" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2005" t="inlineStr">
+        <is>
+          <t>北海道地方札幌4丁目プレイス 4PLA 2025年4月25日(金)から順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2005" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/32449</t>
+        </is>
+      </c>
+    </row>
+    <row r="2006">
+      <c r="A2006" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2006" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2006" t="inlineStr">
+        <is>
+          <t>関東地方そよらリーフシティ市川 2026年3月28日(土)開業！全8テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2006" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36718</t>
+        </is>
+      </c>
+    </row>
+    <row r="2007">
+      <c r="A2007" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2007" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2007" t="inlineStr">
+        <is>
+          <t>九州地方イオン熊本中央店 2025年2月28日(金)に閉店し建て替えへ！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2007" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/39651</t>
+        </is>
+      </c>
+    </row>
+    <row r="2008">
+      <c r="A2008" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2008" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2008" t="inlineStr">
+        <is>
+          <t>関東地方ヤオコーまるひろ上尾SC 2025年9月12日(金)開業！全テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2008" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42379</t>
+        </is>
+      </c>
+    </row>
+    <row r="2009">
+      <c r="A2009" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2009" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2009" t="inlineStr">
+        <is>
+          <t>関東地方フォルテさくら氏家 2026年1月28日(水)開業！テナント随時更新中！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2009" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/43900</t>
+        </is>
+      </c>
+    </row>
+    <row r="2010">
+      <c r="A2010" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2010" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2010" t="inlineStr">
+        <is>
+          <t>九州地方トライアルスマート小倉熊谷店 2026年12月初旬に開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2010" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/48785</t>
+        </is>
+      </c>
+    </row>
+    <row r="2011">
+      <c r="A2011" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2011" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2011" t="inlineStr">
+        <is>
+          <t>関東地方北千住駅前地区市街地再開発事業 2031年度開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2011" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/32865</t>
+        </is>
+      </c>
+    </row>
+    <row r="2012">
+      <c r="A2012" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2012" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2012" t="inlineStr">
+        <is>
+          <t>関東地方川崎市千年商業施設計画 ノジマが出店へ 2029年初頭開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2012" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42082</t>
+        </is>
+      </c>
+    </row>
+    <row r="2013">
+      <c r="A2013" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2013" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2013" t="inlineStr">
+        <is>
+          <t>関東地方新小岩駅南口地区市街地再開発事業 2032年度完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2013" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/21403</t>
+        </is>
+      </c>
+    </row>
+    <row r="2014">
+      <c r="A2014" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2014" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2014" t="inlineStr">
+        <is>
+          <t>東北地方イオンタウン三沢 2031年以降開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2014" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/47877</t>
+        </is>
+      </c>
+    </row>
+    <row r="2015">
+      <c r="A2015" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2015" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2015" t="inlineStr">
+        <is>
+          <t>関西地方イオン京橋店跡地 将来的に再開発へ！2028年以降開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2015" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/16733</t>
+        </is>
+      </c>
+    </row>
+    <row r="2016">
+      <c r="A2016" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2016" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2016" t="inlineStr">
+        <is>
+          <t>九州地方スプリングガーデン御代志2025年3月24日(月)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2016" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/36931</t>
+        </is>
+      </c>
+    </row>
+    <row r="2017">
+      <c r="A2017" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2017" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2017" t="inlineStr">
+        <is>
+          <t>中部地方掛川市結縁寺物販店舗 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2017" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/49478</t>
+        </is>
+      </c>
+    </row>
+    <row r="2018">
+      <c r="A2018" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2018" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2018" t="inlineStr">
+        <is>
+          <t>関東地方トーチタワー 地上385mの日本一高いビルが2028年度竣工！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2018" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/15125</t>
+        </is>
+      </c>
+    </row>
+    <row r="2019">
+      <c r="A2019" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2019" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2019" t="inlineStr">
+        <is>
+          <t>関東地方ニトリ川崎高津店(仮称) 2027年夏開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2019" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47017</t>
+        </is>
+      </c>
+    </row>
+    <row r="2020">
+      <c r="A2020" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2020" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2020" t="inlineStr">
+        <is>
+          <t>関西地方イオンタウン堺水賀池 2027年冬開業！30店舗が出店！テナントは？最新情報も！大阪府堺市中区深井の水賀池公園のプロジェクト「水賀池公園整備事業」において、イオンタウン堺水賀池が2027年冬開業！イオンタウン公式リリースが発表！深井駅徒歩3分、水賀池公園に「イオンタウン堺水賀池」が誕生！敷地面積約1.46万㎡・地上2階...2026.09.30関西地方</t>
+        </is>
+      </c>
+      <c r="D2020" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/45734</t>
+        </is>
+      </c>
+    </row>
+    <row r="2021">
+      <c r="A2021" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2021" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2021" t="inlineStr">
+        <is>
+          <t>関東地方JR武蔵境駅東側開発 2028年開業！テナントは？最新情報も！東京都武蔵野市のJR武蔵境駅東側エリアに、JR東日本による駅直結複合ビル「（仮称）武蔵境駅東側駅ビル」が2028年度冬に開業！JR東日本が「（仮称）武蔵境駅東側駅ビル」の建設工事に2026年10月より本格着手！地上9階建て・延床約6,000...2026.09.30関東地方</t>
+        </is>
+      </c>
+      <c r="D2021" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48480</t>
+        </is>
+      </c>
+    </row>
+    <row r="2022">
+      <c r="A2022" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2022" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2022" t="inlineStr">
+        <is>
+          <t>JR東日本／商業・ホテル複合「武蔵境駅東側駅ビル」28年度冬オープン</t>
+        </is>
+      </c>
+      <c r="D2022" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100175.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2023">
+      <c r="A2023" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2023" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2023" t="inlineStr">
+        <is>
+          <t>オーケーほか／東京都北区に「（仮称）北区豊島四丁目SC計画（店舗面積2670m2）」27年3月23日新設</t>
+        </is>
+      </c>
+      <c r="D2023" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1001011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2024">
+      <c r="A2024" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2024" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2024" t="inlineStr">
+        <is>
+          <t>しまむら／東京都練馬区に「（仮称）ファッションセンターしまむら中村南店」27年3月29日新設</t>
+        </is>
+      </c>
+      <c r="D2024" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1001012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2025">
+      <c r="A2025" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2025" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2025" t="inlineStr">
+        <is>
+          <t>東京ソラマチ／10月以降「Eggs ’n Things」など新規6店舗オープン</t>
+        </is>
+      </c>
+      <c r="D2025" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100176.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2026">
+      <c r="A2026" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2026" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2026" t="inlineStr">
+        <is>
+          <t>ユニクロ／「ゆめタウン光の森店」10月9日リニューアルオープン、熊本県最大店舗に</t>
+        </is>
+      </c>
+      <c r="D2026" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100115.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2027">
+      <c r="A2027" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2027" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2027" t="inlineStr">
+        <is>
+          <t>中部薬品／富山県氷見市に「V・drug氷見栄薬局」10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D2027" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100111.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2028">
+      <c r="A2028" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2028" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2028" t="inlineStr">
+        <is>
+          <t>大丸京都店／「白い恋人」ISHIYAのギフト向けスイーツブランド新規オープン</t>
+        </is>
+      </c>
+      <c r="D2028" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100173.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2029">
+      <c r="A2029" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2029" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2029" t="inlineStr">
+        <is>
+          <t>イオンリテール／「そよらつくば学園の森」10月25日オープン、バーガーキング・ダイソーなど出店</t>
+        </is>
+      </c>
+      <c r="D2029" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093016.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2030">
+      <c r="A2030" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2030" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2030" t="inlineStr">
+        <is>
+          <t>JR東日本／神奈川県「逗子駅ビル」の建設工事を開始、28年春に商業施設オープン</t>
+        </is>
+      </c>
+      <c r="D2030" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093074.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2031">
+      <c r="A2031" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2031" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2031" t="inlineStr">
+        <is>
+          <t>新宿マルイ／PLAZAの新業態「プラザ トーキョープラス」11月20日オープン</t>
+        </is>
+      </c>
+      <c r="D2031" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093076.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2032">
+      <c r="A2032" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2032" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2032" t="inlineStr">
+        <is>
+          <t>大丸梅田店／「太陽ノ塔」「堂島ロール」の新業態など新規5店舗が12月1日オープン</t>
+        </is>
+      </c>
+      <c r="D2032" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093077.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2033">
+      <c r="A2033" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2033" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2033" t="inlineStr">
+        <is>
+          <t>コーナン商事／鹿児島県に初出店「コーナンPRO 鹿児島東開店」オープン</t>
+        </is>
+      </c>
+      <c r="D2033" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093072.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2034">
+      <c r="A2034" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2034" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2034" t="inlineStr">
+        <is>
+          <t>東京インテリア家具／栃木県小山市に「（仮称）マックス小山店」27年4月27日新設</t>
+        </is>
+      </c>
+      <c r="D2034" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0930012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2035">
+      <c r="A2035" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2035" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2035" t="inlineStr">
+        <is>
+          <t>クリエイトSD／茨城県つくば市に「つくば市学園の森商業施設」27年4月13日新設</t>
+        </is>
+      </c>
+      <c r="D2035" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0930011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2036">
+      <c r="A2036" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2036" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2036" t="inlineStr">
+        <is>
+          <t>ビームス／香川・金刀比羅宮表参道に「ビームス ジャパン 琴平」10月31日オープン</t>
+        </is>
+      </c>
+      <c r="D2036" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093073.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2037">
+      <c r="A2037" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2037" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2037" t="inlineStr">
+        <is>
+          <t>レデイ薬局／愛媛県松山市に調剤薬局「レデイ薬局 南斎院店」10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D2037" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2038">
+      <c r="A2038" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2038" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2038" t="inlineStr">
+        <is>
+          <t>猿田彦珈琲／「京都高島屋 S.C.T8」に新店舗10月2日オープン</t>
+        </is>
+      </c>
+      <c r="D2038" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093071.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2039">
+      <c r="A2039" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2039" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2039" t="inlineStr">
+        <is>
+          <t>コロワイド／福島初出店「チーズガーデン イオンモール伊達店」11月27日オープン</t>
+        </is>
+      </c>
+      <c r="D2039" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093075.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2040">
+      <c r="A2040" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2040" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2040" t="inlineStr">
+        <is>
+          <t>串カツ田中／滋賀県大津市に「膳所店」オープン、膳所駅から徒歩3分</t>
+        </is>
+      </c>
+      <c r="D2040" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s093041.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2041">
+      <c r="A2041" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2041" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2041" t="inlineStr">
+        <is>
+          <t>三井アウトレットパーク仙台港／事業延長が決定</t>
+        </is>
+      </c>
+      <c r="D2041" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s092914.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-02
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2041"/>
+  <dimension ref="A1:D2110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45318,6 +45318,1524 @@
         </is>
       </c>
     </row>
+    <row r="2042">
+      <c r="A2042" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2042" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2042" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D2042" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="2043">
+      <c r="A2043" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2043" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2043" t="inlineStr">
+        <is>
+          <t>10/8成城石井京阪百貨店守口店(大阪府守口市)</t>
+        </is>
+      </c>
+      <c r="D2043" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gtA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2044">
+      <c r="A2044" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2044" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2044" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D2044" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="2045">
+      <c r="A2045" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2045" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2045" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D2045" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2046">
+      <c r="A2046" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2046" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2046" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D2046" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="2047">
+      <c r="A2047" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2047" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2047" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D2047" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2048">
+      <c r="A2048" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2048" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2048" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D2048" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="2049">
+      <c r="A2049" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2049" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2049" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D2049" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2050">
+      <c r="A2050" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2050" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2050" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D2050" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="2051">
+      <c r="A2051" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2051" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2051" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2051" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2052">
+      <c r="A2052" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2052" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2052" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2052" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2053">
+      <c r="A2053" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2053" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2053" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2053" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2054">
+      <c r="A2054" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2054" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2054" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2054" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2055">
+      <c r="A2055" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2055" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2055" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2055" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2056">
+      <c r="A2056" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2056" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2056" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2056" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2057">
+      <c r="A2057" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2057" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2057" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2057" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2058">
+      <c r="A2058" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2058" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2058" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2058" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2059">
+      <c r="A2059" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2059" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2059" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2059" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2060">
+      <c r="A2060" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2060" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2060" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2060" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2061">
+      <c r="A2061" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2061" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2061" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2061" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2062">
+      <c r="A2062" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2062" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2062" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2062" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2063">
+      <c r="A2063" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2063" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2063" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2063" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2064">
+      <c r="A2064" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2064" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2064" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2064" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2065">
+      <c r="A2065" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2065" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2065" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2065" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2066">
+      <c r="A2066" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2066" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2066" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2066" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2067">
+      <c r="A2067" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2067" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2067" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2067" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2068">
+      <c r="A2068" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2068" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2068" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2068" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2069">
+      <c r="A2069" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2069" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2069" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2069" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2070">
+      <c r="A2070" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2070" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2070" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2070" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2071">
+      <c r="A2071" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2071" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2071" t="inlineStr">
+        <is>
+          <t>中国地方コープ総社東 2026年7月17日(金)開業！テナント随時更新中！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2071" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/48269</t>
+        </is>
+      </c>
+    </row>
+    <row r="2072">
+      <c r="A2072" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2072" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2072" t="inlineStr">
+        <is>
+          <t>関西地方ハローズ本多聞店 2026年6月24日(水)から順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2072" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/46204</t>
+        </is>
+      </c>
+    </row>
+    <row r="2073">
+      <c r="A2073" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2073" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2073" t="inlineStr">
+        <is>
+          <t>中国地方カミハチクロス 2027年度開業！アンダーズ広島が進出！商業施設も！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2073" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/27582</t>
+        </is>
+      </c>
+    </row>
+    <row r="2074">
+      <c r="A2074" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2074" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2074" t="inlineStr">
+        <is>
+          <t>関東地方minanoba川口 2026年9月17日(金)開業！全10テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2074" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42094</t>
+        </is>
+      </c>
+    </row>
+    <row r="2075">
+      <c r="A2075" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2075" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2075" t="inlineStr">
+        <is>
+          <t>関西地方高島屋堺店跡地にHiViE堺東が2027年春全体開業！ライフが出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2075" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/41410</t>
+        </is>
+      </c>
+    </row>
+    <row r="2076">
+      <c r="A2076" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2076" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2076" t="inlineStr">
+        <is>
+          <t>関東地方三井アウトレットパーク多摩南大沢 B街区が建て替えへ！2028年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2076" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42310</t>
+        </is>
+      </c>
+    </row>
+    <row r="2077">
+      <c r="A2077" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2077" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2077" t="inlineStr">
+        <is>
+          <t>中部地方富士モータースポーツフォレストテラス 2026年6月5日(金)先行開業！5店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2077" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/44714</t>
+        </is>
+      </c>
+    </row>
+    <row r="2078">
+      <c r="A2078" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2078" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2078" t="inlineStr">
+        <is>
+          <t>関西地方平和堂岸辺店 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2078" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49465</t>
+        </is>
+      </c>
+    </row>
+    <row r="2079">
+      <c r="A2079" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2079" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2079" t="inlineStr">
+        <is>
+          <t>関東地方TAIRAYA与野店 与野フード建て替え 2025年4月24日(木)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2079" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/37854</t>
+        </is>
+      </c>
+    </row>
+    <row r="2080">
+      <c r="A2080" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2080" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2080" t="inlineStr">
+        <is>
+          <t>関西地方アクロスプラザ和泉観音寺 2026年11月開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2080" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/47867</t>
+        </is>
+      </c>
+    </row>
+    <row r="2081">
+      <c r="A2081" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2081" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2081" t="inlineStr">
+        <is>
+          <t>関東地方横須賀・若松町1丁目地区市街地再開発事業 2030年春開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2081" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47566</t>
+        </is>
+      </c>
+    </row>
+    <row r="2082">
+      <c r="A2082" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2082" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2082" t="inlineStr">
+        <is>
+          <t>中部地方新潟市東区中木戸商業施設(仮称) 2027年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2082" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/47439</t>
+        </is>
+      </c>
+    </row>
+    <row r="2083">
+      <c r="A2083" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2083" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2083" t="inlineStr">
+        <is>
+          <t>東北地方【電力ビル】一番町三丁目七番地区市街地再開発事業 2029年開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2083" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/31239</t>
+        </is>
+      </c>
+    </row>
+    <row r="2084">
+      <c r="A2084" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2084" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2084" t="inlineStr">
+        <is>
+          <t>関西地方グラングリーン大阪 2025年3月21日(金)南館開業！テナントは？どのような街に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2084" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/4448</t>
+        </is>
+      </c>
+    </row>
+    <row r="2085">
+      <c r="A2085" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2085" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2085" t="inlineStr">
+        <is>
+          <t>東北地方東松島市赤井にヨークベニマルの大型商業施設 2028年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2085" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/33547</t>
+        </is>
+      </c>
+    </row>
+    <row r="2086">
+      <c r="A2086" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2086" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2086" t="inlineStr">
+        <is>
+          <t>関東地方COMMONS TACHIKAWA TACHIHIが2025年7月30日(水)より順次開業！全テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2086" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/44255</t>
+        </is>
+      </c>
+    </row>
+    <row r="2087">
+      <c r="A2087" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2087" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2087" t="inlineStr">
+        <is>
+          <t>北海道地方tonarie（トナリエ）北広島 2025年3月15日(土)開業！全テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2087" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/21566</t>
+        </is>
+      </c>
+    </row>
+    <row r="2088">
+      <c r="A2088" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2088" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2088" t="inlineStr">
+        <is>
+          <t>関東地方スーパーセンタートライアル深谷川本店 2026年4月29日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2088" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/44915</t>
+        </is>
+      </c>
+    </row>
+    <row r="2089">
+      <c r="A2089" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2089" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2089" t="inlineStr">
+        <is>
+          <t>関西地方イオンタウン堺水賀池 2027年冬開業！30店舗が出店！テナントは？最新情報も！大阪府堺市中区深井の水賀池公園のプロジェクト「水賀池公園整備事業」において、イオンタウン堺水賀池が2027年冬開業！イオンタウン公式リリースが発表！深井駅徒歩3分、水賀池公園に「イオンタウン堺水賀池」が誕生！敷地面積約1.46万㎡・地上2階...2026.09.30関西地方</t>
+        </is>
+      </c>
+      <c r="D2089" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/45734</t>
+        </is>
+      </c>
+    </row>
+    <row r="2090">
+      <c r="A2090" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2090" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2090" t="inlineStr">
+        <is>
+          <t>関東地方JR武蔵境駅東側開発 2028年開業！テナントは？最新情報も！東京都武蔵野市のJR武蔵境駅東側エリアに、JR東日本による駅直結複合ビル「（仮称）武蔵境駅東側駅ビル」が2028年度冬に開業！JR東日本が「（仮称）武蔵境駅東側駅ビル」の建設工事に2026年10月より本格着手！地上9階建て・延床約6,000...2026.09.30関東地方</t>
+        </is>
+      </c>
+      <c r="D2090" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48480</t>
+        </is>
+      </c>
+    </row>
+    <row r="2091">
+      <c r="A2091" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2091" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2091" t="inlineStr">
+        <is>
+          <t>平和堂／平松社長「富山県でドミナント強化、富山掛尾店の滑り出し好調」注目</t>
+        </is>
+      </c>
+      <c r="D2091" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100214.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2092">
+      <c r="A2092" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2092" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2092" t="inlineStr">
+        <is>
+          <t>イオンリテール／イオン諏訪店跡地に「イオンスタイル」10月21日オープン</t>
+        </is>
+      </c>
+      <c r="D2092" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100278.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2093">
+      <c r="A2093" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2093" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2093" t="inlineStr">
+        <is>
+          <t>ユニクロ京都／西日本初登場の「UNIQLO COFFEE」導入、地元コラボTシャツも登場</t>
+        </is>
+      </c>
+      <c r="D2093" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100275.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2094">
+      <c r="A2094" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2094" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2094" t="inlineStr">
+        <is>
+          <t>大阪屋ショップ／愛知県2店舗目「日進店」オープン、鮮魚・魚総菜に注力</t>
+        </is>
+      </c>
+      <c r="D2094" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100271.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2095">
+      <c r="A2095" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2095" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2095" t="inlineStr">
+        <is>
+          <t>ジーユー／熊本県「ゆめタウン光の森」に10月9日移転・増床オープン</t>
+        </is>
+      </c>
+      <c r="D2095" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100211.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2096">
+      <c r="A2096" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2096" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2096" t="inlineStr">
+        <is>
+          <t>ヨークベニマル／福島県南相馬市に「ヨークベニマル原町西店衣料館」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2096" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100219.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2097">
+      <c r="A2097" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2097" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2097" t="inlineStr">
+        <is>
+          <t>ロイヤルホームセンター／京都府城陽市に「ロイヤルプロ城陽インター（店舗面積2400m2）」27年5月21日新設</t>
+        </is>
+      </c>
+      <c r="D2097" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1002011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2098">
+      <c r="A2098" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2098" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2098" t="inlineStr">
+        <is>
+          <t>コスモス薬品／群馬県渋川市に「ドラッグコスモス阿久津店」27年9月30日新設</t>
+        </is>
+      </c>
+      <c r="D2098" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1002012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2099">
+      <c r="A2099" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2099" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2099" t="inlineStr">
+        <is>
+          <t>ビームス／新宿区に初のスポーツコンセプトストア10月12日オープン</t>
+        </is>
+      </c>
+      <c r="D2099" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100276.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2100">
+      <c r="A2100" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2100" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2100" t="inlineStr">
+        <is>
+          <t>西鉄ストア／福岡市城南区「レガネット七隈」リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D2100" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100272.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2101">
+      <c r="A2101" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2101" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2101" t="inlineStr">
+        <is>
+          <t>キルフェボン／東京・新宿「明治安田新宿ビル」に新店舗11月28日オープン</t>
+        </is>
+      </c>
+      <c r="D2101" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100274.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2102">
+      <c r="A2102" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2102" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2102" t="inlineStr">
+        <is>
+          <t>ミスターマックス／広島県福山市に「MrMax Select福山店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D2102" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100283.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2103">
+      <c r="A2103" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2103" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2103" t="inlineStr">
+        <is>
+          <t>ストライプ／「AMERICAN HOLIC 京王モール店」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2103" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100215.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2104">
+      <c r="A2104" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2104" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2104" t="inlineStr">
+        <is>
+          <t>フランフラン／ルミネエスト新宿に10月9日新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D2104" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100216.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2105">
+      <c r="A2105" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2105" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2105" t="inlineStr">
+        <is>
+          <t>メガネスーパー／「イオンモール松本」「ゆめタウン三豊」にコンタクトレンズ専門店10月3日オープン</t>
+        </is>
+      </c>
+      <c r="D2105" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100279.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2106">
+      <c r="A2106" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2106" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2106" t="inlineStr">
+        <is>
+          <t>物語コーポレーション／「丸源ラーメン イオンモール甲府昭和店」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2106" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100273.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2107">
+      <c r="A2107" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2107" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2107" t="inlineStr">
+        <is>
+          <t>JR東日本／商業・ホテル複合「武蔵境駅東側駅ビル」28年度冬オープン</t>
+        </is>
+      </c>
+      <c r="D2107" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100175.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2108">
+      <c r="A2108" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2108" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2108" t="inlineStr">
+        <is>
+          <t>オーケーほか／東京都北区に「（仮称）北区豊島四丁目SC計画（店舗面積2670m2）」27年3月23日新設</t>
+        </is>
+      </c>
+      <c r="D2108" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1001011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2109">
+      <c r="A2109" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2109" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2109" t="inlineStr">
+        <is>
+          <t>しまむら／東京都練馬区に「（仮称）ファッションセンターしまむら中村南店」27年3月29日新設</t>
+        </is>
+      </c>
+      <c r="D2109" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1001012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2110">
+      <c r="A2110" t="inlineStr">
+        <is>
+          <t>2026年10月02日</t>
+        </is>
+      </c>
+      <c r="B2110" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2110" t="inlineStr">
+        <is>
+          <t>東京ソラマチ／10月以降「Eggs ’n Things」など新規6店舗オープン</t>
+        </is>
+      </c>
+      <c r="D2110" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100176.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-03
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2110"/>
+  <dimension ref="A1:D2182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46836,6 +46836,1590 @@
         </is>
       </c>
     </row>
+    <row r="2111">
+      <c r="A2111" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2111" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2111" t="inlineStr">
+        <is>
+          <t>10/21イオンスタイル諏訪(長野県諏訪市)</t>
+        </is>
+      </c>
+      <c r="D2111" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1abH</t>
+        </is>
+      </c>
+    </row>
+    <row r="2112">
+      <c r="A2112" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2112" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2112" t="inlineStr">
+        <is>
+          <t>もち吉大津店</t>
+        </is>
+      </c>
+      <c r="D2112" t="inlineStr">
+        <is>
+          <t>https://www.mochikichi.co.jp/shop/info</t>
+        </is>
+      </c>
+    </row>
+    <row r="2113">
+      <c r="A2113" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2113" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2113" t="inlineStr">
+        <is>
+          <t>ラーメン荘 地球規模で考えろ サン</t>
+        </is>
+      </c>
+      <c r="D2113" t="inlineStr">
+        <is>
+          <t>https://than.co.jp/brands/%E3%83%A9%E3%83%BC%E3%83%A1%E3%83%B3%E8%8D%98-%E5%9C%B0%E7%90%83%E8%A6%8F%E6%A8%A1%E3%81%A7%E8%80%83%E3%81%88%E3%82%8D/</t>
+        </is>
+      </c>
+    </row>
+    <row r="2114">
+      <c r="A2114" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2114" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2114" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D2114" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="2115">
+      <c r="A2115" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2115" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2115" t="inlineStr">
+        <is>
+          <t>10/8成城石井京阪百貨店守口店(大阪府)</t>
+        </is>
+      </c>
+      <c r="D2115" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gtA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2116">
+      <c r="A2116" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2116" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2116" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D2116" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="2117">
+      <c r="A2117" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2117" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2117" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D2117" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2118">
+      <c r="A2118" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2118" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2118" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D2118" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="2119">
+      <c r="A2119" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2119" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2119" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D2119" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2120">
+      <c r="A2120" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2120" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2120" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D2120" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="2121">
+      <c r="A2121" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2121" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2121" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D2121" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2122">
+      <c r="A2122" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2122" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2122" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D2122" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="2123">
+      <c r="A2123" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2123" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2123" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2123" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2124">
+      <c r="A2124" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2124" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2124" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2124" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2125">
+      <c r="A2125" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2125" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2125" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2125" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2126">
+      <c r="A2126" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2126" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2126" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2126" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2127">
+      <c r="A2127" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2127" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2127" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2127" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2128">
+      <c r="A2128" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2128" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2128" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2128" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2129">
+      <c r="A2129" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2129" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2129" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2129" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2130">
+      <c r="A2130" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2130" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2130" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2130" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2131">
+      <c r="A2131" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2131" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2131" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2131" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2132">
+      <c r="A2132" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2132" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2132" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2132" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2133">
+      <c r="A2133" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2133" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2133" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2133" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2134">
+      <c r="A2134" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2134" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2134" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2134" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2135">
+      <c r="A2135" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2135" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2135" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2135" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2136">
+      <c r="A2136" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2136" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2136" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2136" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2137">
+      <c r="A2137" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2137" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2137" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2137" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2138">
+      <c r="A2138" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2138" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2138" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2138" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2139">
+      <c r="A2139" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2139" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2139" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2139" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2140">
+      <c r="A2140" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2140" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2140" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2140" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2141">
+      <c r="A2141" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2141" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2141" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2141" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2142">
+      <c r="A2142" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2142" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2142" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2142" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2143">
+      <c r="A2143" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2143" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2143" t="inlineStr">
+        <is>
+          <t>九州地方ゆめモール那珂川 2026年2月20日(金)~順次開業！全20店舗一覧！</t>
+        </is>
+      </c>
+      <c r="D2143" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/31176</t>
+        </is>
+      </c>
+    </row>
+    <row r="2144">
+      <c r="A2144" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2144" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2144" t="inlineStr">
+        <is>
+          <t>北海道地方【札幌西武跡地】北4⻄3地区市街地再開発事業 2028年夏開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2144" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/17705</t>
+        </is>
+      </c>
+    </row>
+    <row r="2145">
+      <c r="A2145" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2145" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2145" t="inlineStr">
+        <is>
+          <t>九州地方スーパーセンタートライアル鹿屋上野町店 2025年7月9日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2145" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/41750</t>
+        </is>
+      </c>
+    </row>
+    <row r="2146">
+      <c r="A2146" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2146" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2146" t="inlineStr">
+        <is>
+          <t>関西地方南紀の台 よってって広場 2025年3月18日(火)9時~開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2146" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39105</t>
+        </is>
+      </c>
+    </row>
+    <row r="2147">
+      <c r="A2147" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2147" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2147" t="inlineStr">
+        <is>
+          <t>北海道地方SAPPORO ONE サッポロワン 大通西4南地区市街地再開発事業 2029年8月完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2147" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/26256</t>
+        </is>
+      </c>
+    </row>
+    <row r="2148">
+      <c r="A2148" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2148" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2148" t="inlineStr">
+        <is>
+          <t>関東地方ザ・パークハウス 赤羽台タワー＆レジデンス 2028年10月完成予定！商業施設も誕生 最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2148" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/39853</t>
+        </is>
+      </c>
+    </row>
+    <row r="2149">
+      <c r="A2149" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2149" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2149" t="inlineStr">
+        <is>
+          <t>関東地方豊洲セイルパーク 2025年7月24日~順次開業！全21テナント一覧 最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2149" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/18680</t>
+        </is>
+      </c>
+    </row>
+    <row r="2150">
+      <c r="A2150" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2150" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2150" t="inlineStr">
+        <is>
+          <t>関西地方ヤマダストアー宝塚店 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2150" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/48714</t>
+        </is>
+      </c>
+    </row>
+    <row r="2151">
+      <c r="A2151" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2151" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2151" t="inlineStr">
+        <is>
+          <t>関東地方石神井公園駅南口西地区市街地再開発事業 2028年春完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2151" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26815</t>
+        </is>
+      </c>
+    </row>
+    <row r="2152">
+      <c r="A2152" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2152" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2152" t="inlineStr">
+        <is>
+          <t>関東地方HIBIYA CROSSPARK（日比谷クロスパーク）2029年春街びらき！2037年全体開業！どのような街に？</t>
+        </is>
+      </c>
+      <c r="D2152" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/24411</t>
+        </is>
+      </c>
+    </row>
+    <row r="2153">
+      <c r="A2153" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2153" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2153" t="inlineStr">
+        <is>
+          <t>東北地方イオンスタイル山王 2025年3月20日(木)開業！無印良品も出店へ！全8テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2153" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/37974</t>
+        </is>
+      </c>
+    </row>
+    <row r="2154">
+      <c r="A2154" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2154" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2154" t="inlineStr">
+        <is>
+          <t>関東地方JR小岩駅北口地区再開発事業 2027年春完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2154" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/20970</t>
+        </is>
+      </c>
+    </row>
+    <row r="2155">
+      <c r="A2155" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2155" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2155" t="inlineStr">
+        <is>
+          <t>関東地方品川駅北口に新駅ビル 2031年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2155" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/33951</t>
+        </is>
+      </c>
+    </row>
+    <row r="2156">
+      <c r="A2156" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2156" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2156" t="inlineStr">
+        <is>
+          <t>関東地方みと好文テラス 2026年4月23日(木)開業！全11テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2156" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48066</t>
+        </is>
+      </c>
+    </row>
+    <row r="2157">
+      <c r="A2157" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2157" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2157" t="inlineStr">
+        <is>
+          <t>九州地方OHASHI HILL ゆめアール大橋跡地に2025年4月18日(金)先行開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2157" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/27364</t>
+        </is>
+      </c>
+    </row>
+    <row r="2158">
+      <c r="A2158" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2158" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2158" t="inlineStr">
+        <is>
+          <t>関東地方大宮駅西口第3-A･D地区市街地再開発事業 2031年以降開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2158" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/16908</t>
+        </is>
+      </c>
+    </row>
+    <row r="2159">
+      <c r="A2159" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2159" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2159" t="inlineStr">
+        <is>
+          <t>東北地方イオンスタイル八戸沼館 2025年4月25日(金)開業！全テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2159" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/42366</t>
+        </is>
+      </c>
+    </row>
+    <row r="2160">
+      <c r="A2160" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2160" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2160" t="inlineStr">
+        <is>
+          <t>関西地方レイクウェル堅田 2025年10月31日(金)より順次開業！全4テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2160" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/42148</t>
+        </is>
+      </c>
+    </row>
+    <row r="2161">
+      <c r="A2161" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2161" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2161" t="inlineStr">
+        <is>
+          <t>東北地方ケーズデンキ新仙台南店 2027年春に開業予定！最新情報も！宮城県名取市にデンコードーの店舗「ケーズデンキ新仙台南店(仮称)」が2027年春に開業予定！ケーズデンキの中では大型店舗となります。そんな、ケーズデンキ新仙台南店について、テナントや開業日などを見ていきましょう！2026年10月3日　公開ケ...2026.10.03東北地方</t>
+        </is>
+      </c>
+      <c r="D2161" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/49847</t>
+        </is>
+      </c>
+    </row>
+    <row r="2162">
+      <c r="A2162" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2162" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2162" t="inlineStr">
+        <is>
+          <t>中部地方スーパーセンタートライアル名古屋みなと店 2026年11月開業予定！最新情報も！愛知県名古屋市港区にトライアルカンパニーの店舗「スーパーセンタートライアル名古屋みなと店」が2026年11月開業予定！スーパーセンタートライアルが名古屋市港区に2店舗目の出店！そんな、スーパーセンタートライアル名古屋みなと店について、テナン...2026.10.03中部地方</t>
+        </is>
+      </c>
+      <c r="D2162" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48009</t>
+        </is>
+      </c>
+    </row>
+    <row r="2163">
+      <c r="A2163" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2163" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2163" t="inlineStr">
+        <is>
+          <t>平和堂／平松社長「富山県でドミナント強化、富山掛尾店の滑り出し好調」注目</t>
+        </is>
+      </c>
+      <c r="D2163" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100214.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2164">
+      <c r="A2164" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2164" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2164" t="inlineStr">
+        <is>
+          <t>イオンリテール／イオン諏訪店跡地に「イオンスタイル」10月21日オープン</t>
+        </is>
+      </c>
+      <c r="D2164" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100278.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2165">
+      <c r="A2165" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2165" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2165" t="inlineStr">
+        <is>
+          <t>ユニクロ京都／西日本初登場の「UNIQLO COFFEE」導入、地元コラボTシャツも登場</t>
+        </is>
+      </c>
+      <c r="D2165" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100275.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2166">
+      <c r="A2166" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2166" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2166" t="inlineStr">
+        <is>
+          <t>大阪屋ショップ／愛知県2店舗目「日進店」オープン、鮮魚・魚総菜に注力</t>
+        </is>
+      </c>
+      <c r="D2166" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100271.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2167">
+      <c r="A2167" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2167" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2167" t="inlineStr">
+        <is>
+          <t>ジーユー／熊本県「ゆめタウン光の森」に10月9日移転・増床オープン</t>
+        </is>
+      </c>
+      <c r="D2167" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100211.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2168">
+      <c r="A2168" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2168" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2168" t="inlineStr">
+        <is>
+          <t>ヨークベニマル／福島県南相馬市に「ヨークベニマル原町西店衣料館」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2168" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100219.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2169">
+      <c r="A2169" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2169" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2169" t="inlineStr">
+        <is>
+          <t>ロイヤルホームセンター／京都府城陽市に「ロイヤルプロ城陽インター（店舗面積2400m2）」27年5月21日新設</t>
+        </is>
+      </c>
+      <c r="D2169" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1002011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2170">
+      <c r="A2170" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2170" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2170" t="inlineStr">
+        <is>
+          <t>コスモス薬品／群馬県渋川市に「ドラッグコスモス阿久津店」27年9月30日新設</t>
+        </is>
+      </c>
+      <c r="D2170" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1002012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2171">
+      <c r="A2171" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2171" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2171" t="inlineStr">
+        <is>
+          <t>ビームス／新宿区に初のスポーツコンセプトストア10月12日オープン</t>
+        </is>
+      </c>
+      <c r="D2171" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100276.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2172">
+      <c r="A2172" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2172" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2172" t="inlineStr">
+        <is>
+          <t>西鉄ストア／福岡市城南区「レガネット七隈」リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D2172" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100272.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2173">
+      <c r="A2173" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2173" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2173" t="inlineStr">
+        <is>
+          <t>キルフェボン／東京・新宿「明治安田新宿ビル」に新店舗11月28日オープン</t>
+        </is>
+      </c>
+      <c r="D2173" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100274.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2174">
+      <c r="A2174" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2174" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2174" t="inlineStr">
+        <is>
+          <t>ミスターマックス／広島県福山市に「MrMax Select福山店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D2174" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100283.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2175">
+      <c r="A2175" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2175" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2175" t="inlineStr">
+        <is>
+          <t>ストライプ／「AMERICAN HOLIC 京王モール店」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2175" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100215.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2176">
+      <c r="A2176" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2176" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2176" t="inlineStr">
+        <is>
+          <t>フランフラン／ルミネエスト新宿に10月9日新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D2176" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100216.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2177">
+      <c r="A2177" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2177" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2177" t="inlineStr">
+        <is>
+          <t>メガネスーパー／「イオンモール松本」「ゆめタウン三豊」にコンタクトレンズ専門店10月3日オープン</t>
+        </is>
+      </c>
+      <c r="D2177" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100279.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2178">
+      <c r="A2178" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2178" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2178" t="inlineStr">
+        <is>
+          <t>物語コーポレーション／「丸源ラーメン イオンモール甲府昭和店」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2178" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100273.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2179">
+      <c r="A2179" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2179" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2179" t="inlineStr">
+        <is>
+          <t>JR東日本／商業・ホテル複合「武蔵境駅東側駅ビル」28年度冬オープン</t>
+        </is>
+      </c>
+      <c r="D2179" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100175.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2180">
+      <c r="A2180" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2180" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2180" t="inlineStr">
+        <is>
+          <t>オーケーほか／東京都北区に「（仮称）北区豊島四丁目SC計画（店舗面積2670m2）」27年3月23日新設</t>
+        </is>
+      </c>
+      <c r="D2180" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1001011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2181">
+      <c r="A2181" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2181" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2181" t="inlineStr">
+        <is>
+          <t>しまむら／東京都練馬区に「（仮称）ファッションセンターしまむら中村南店」27年3月29日新設</t>
+        </is>
+      </c>
+      <c r="D2181" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1001012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2182">
+      <c r="A2182" t="inlineStr">
+        <is>
+          <t>2026年10月03日</t>
+        </is>
+      </c>
+      <c r="B2182" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2182" t="inlineStr">
+        <is>
+          <t>東京ソラマチ／10月以降「Eggs ’n Things」など新規6店舗オープン</t>
+        </is>
+      </c>
+      <c r="D2182" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100176.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-04
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2182"/>
+  <dimension ref="A1:D2254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48420,6 +48420,1590 @@
         </is>
       </c>
     </row>
+    <row r="2183">
+      <c r="A2183" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2183" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2183" t="inlineStr">
+        <is>
+          <t>https://www.uniqlo.com/jp/ja/contents/corp/press-release/2026/10/26100211_store.html</t>
+        </is>
+      </c>
+      <c r="D2183" t="inlineStr">
+        <is>
+          <t>https://www.uniqlo.com/jp/ja/contents/corp/press-release/2026/10/26100211_store.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2184">
+      <c r="A2184" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2184" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2184" t="inlineStr">
+        <is>
+          <t>10/8MrMax Select福山店(広島県福山市)</t>
+        </is>
+      </c>
+      <c r="D2184" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gv0</t>
+        </is>
+      </c>
+    </row>
+    <row r="2185">
+      <c r="A2185" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2185" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2185" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D2185" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="2186">
+      <c r="A2186" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2186" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2186" t="inlineStr">
+        <is>
+          <t>10/8成城石井京阪百貨店守口店(大阪府守口市)</t>
+        </is>
+      </c>
+      <c r="D2186" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gtA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2187">
+      <c r="A2187" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2187" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2187" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D2187" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="2188">
+      <c r="A2188" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2188" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2188" t="inlineStr">
+        <is>
+          <t>10/21イオンスタイル諏訪(長野県諏訪市)</t>
+        </is>
+      </c>
+      <c r="D2188" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1abH</t>
+        </is>
+      </c>
+    </row>
+    <row r="2189">
+      <c r="A2189" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2189" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2189" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D2189" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2190">
+      <c r="A2190" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2190" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2190" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D2190" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="2191">
+      <c r="A2191" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2191" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2191" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D2191" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2192">
+      <c r="A2192" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2192" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2192" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D2192" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="2193">
+      <c r="A2193" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2193" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2193" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D2193" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2194">
+      <c r="A2194" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2194" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2194" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D2194" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="2195">
+      <c r="A2195" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2195" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2195" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2195" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2196">
+      <c r="A2196" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2196" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2196" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2196" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2197">
+      <c r="A2197" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2197" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2197" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2197" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2198">
+      <c r="A2198" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2198" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2198" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2198" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2199">
+      <c r="A2199" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2199" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2199" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2199" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2200">
+      <c r="A2200" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2200" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2200" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2200" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2201">
+      <c r="A2201" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2201" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2201" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2201" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2202">
+      <c r="A2202" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2202" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2202" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2202" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2203">
+      <c r="A2203" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2203" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2203" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2203" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2204">
+      <c r="A2204" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2204" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2204" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2204" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2205">
+      <c r="A2205" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2205" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2205" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2205" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2206">
+      <c r="A2206" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2206" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2206" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2206" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2207">
+      <c r="A2207" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2207" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2207" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2207" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2208">
+      <c r="A2208" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2208" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2208" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2208" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2209">
+      <c r="A2209" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2209" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2209" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2209" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2210">
+      <c r="A2210" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2210" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2210" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2210" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2211">
+      <c r="A2211" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2211" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2211" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2211" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2212">
+      <c r="A2212" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2212" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2212" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2212" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2213">
+      <c r="A2213" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2213" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2213" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2213" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2214">
+      <c r="A2214" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2214" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2214" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2214" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2215">
+      <c r="A2215" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2215" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2215" t="inlineStr">
+        <is>
+          <t>関東地方石神井公園駅南口西地区市街地再開発事業 2028年春完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2215" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26815</t>
+        </is>
+      </c>
+    </row>
+    <row r="2216">
+      <c r="A2216" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2216" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2216" t="inlineStr">
+        <is>
+          <t>関東地方W シティタワーズ 蕨駅西口地区市街地再開発事業 2027年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2216" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/16952</t>
+        </is>
+      </c>
+    </row>
+    <row r="2217">
+      <c r="A2217" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2217" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2217" t="inlineStr">
+        <is>
+          <t>関東地方みなとみらい21中央地区60・61街区開発事業 2029年春開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2217" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36914</t>
+        </is>
+      </c>
+    </row>
+    <row r="2218">
+      <c r="A2218" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2218" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2218" t="inlineStr">
+        <is>
+          <t>関東地方ゆりストア百合丘本店 建て替え 2025年3月開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2218" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42337</t>
+        </is>
+      </c>
+    </row>
+    <row r="2219">
+      <c r="A2219" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2219" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2219" t="inlineStr">
+        <is>
+          <t>関東地方JR小岩駅北口地区再開発事業 2027年春完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2219" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/20970</t>
+        </is>
+      </c>
+    </row>
+    <row r="2220">
+      <c r="A2220" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2220" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2220" t="inlineStr">
+        <is>
+          <t>九州地方佐賀玉屋本館 建て替えて2028年～29年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2220" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/43066</t>
+        </is>
+      </c>
+    </row>
+    <row r="2221">
+      <c r="A2221" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2221" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2221" t="inlineStr">
+        <is>
+          <t>関東地方ケーズデンキ コーナン 桜井複合商業施設(仮称) 2026年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2221" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/45945</t>
+        </is>
+      </c>
+    </row>
+    <row r="2222">
+      <c r="A2222" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2222" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2222" t="inlineStr">
+        <is>
+          <t>関東地方松戸駅 新駅ビルに商業施設 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2222" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/29225</t>
+        </is>
+      </c>
+    </row>
+    <row r="2223">
+      <c r="A2223" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2223" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2223" t="inlineStr">
+        <is>
+          <t>東北地方いろは蔵パーク 2025年3月27日(木)開業！無印良品が出店へ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2223" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/38677</t>
+        </is>
+      </c>
+    </row>
+    <row r="2224">
+      <c r="A2224" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2224" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2224" t="inlineStr">
+        <is>
+          <t>関西地方オークワ堺市駅前店 2025年8月30日(土)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2224" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/38273</t>
+        </is>
+      </c>
+    </row>
+    <row r="2225">
+      <c r="A2225" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2225" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2225" t="inlineStr">
+        <is>
+          <t>関西地方iyouTown（アイユータウン）須磨 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2225" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/43508</t>
+        </is>
+      </c>
+    </row>
+    <row r="2226">
+      <c r="A2226" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2226" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2226" t="inlineStr">
+        <is>
+          <t>関東地方TOCビル 建て替えて2027年竣工！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2226" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/23255</t>
+        </is>
+      </c>
+    </row>
+    <row r="2227">
+      <c r="A2227" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2227" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2227" t="inlineStr">
+        <is>
+          <t>関東地方渋谷二丁目西地区市街地再開発事業 2029年度竣工予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2227" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/24394</t>
+        </is>
+      </c>
+    </row>
+    <row r="2228">
+      <c r="A2228" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2228" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2228" t="inlineStr">
+        <is>
+          <t>関東地方ららテラス川口 2025年5月31日(土)開業！全94店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2228" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/33965</t>
+        </is>
+      </c>
+    </row>
+    <row r="2229">
+      <c r="A2229" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2229" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2229" t="inlineStr">
+        <is>
+          <t>関東地方BASEGATE（ベースゲート）横浜関内 2026年3月19日(木)開業！全65店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2229" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/11753</t>
+        </is>
+      </c>
+    </row>
+    <row r="2230">
+      <c r="A2230" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2230" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2230" t="inlineStr">
+        <is>
+          <t>北海道地方札幌4丁目プレイス 4PLA 2025年4月25日(金)から順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2230" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/32449</t>
+        </is>
+      </c>
+    </row>
+    <row r="2231">
+      <c r="A2231" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2231" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2231" t="inlineStr">
+        <is>
+          <t>関東地方福生駅西口地区市街地再開発事業 2027年春完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2231" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36735</t>
+        </is>
+      </c>
+    </row>
+    <row r="2232">
+      <c r="A2232" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2232" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2232" t="inlineStr">
+        <is>
+          <t>中部地方福井駅前南通り地区市街地再開発事業 2027年より順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2232" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/43036</t>
+        </is>
+      </c>
+    </row>
+    <row r="2233">
+      <c r="A2233" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2233" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2233" t="inlineStr">
+        <is>
+          <t>四国地方フジ三町店 イヨテツスポーツセンター跡地 2028年開業！テナントは？最新情報も！愛媛県松山市三町の「イヨテツスポーツセンター」跡地に、株式会社フジによる新たな商業施設「フジ三町店（仮称）」が2028年ごろ開業予定！県内唯一のアイススケート場や屋外プールとして約60年にわたり親しまれた「イヨテツスポーツセンター」跡地を中...2026.10.04四国地方</t>
+        </is>
+      </c>
+      <c r="D2233" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/shikoku/49886</t>
+        </is>
+      </c>
+    </row>
+    <row r="2234">
+      <c r="A2234" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2234" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2234" t="inlineStr">
+        <is>
+          <t>関東地方湯島三丁目地区市街地再開発事業 2035年度完成予定！どのような施設に？最新情報も！東京都文京区湯島に、地上40階建ての超高層ランドマーク複合ビル「湯島三丁目地区市街地再開発事業」が2035年度に完成予定！東京メトロ千代田線「湯島駅」直結！高さ約170m・延床面積約11万㎡の超高層タワーが誕生！低層階の商業ゾーンをはじめ、...2026.10.04関東地方</t>
+        </is>
+      </c>
+      <c r="D2234" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49878</t>
+        </is>
+      </c>
+    </row>
+    <row r="2235">
+      <c r="A2235" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2235" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2235" t="inlineStr">
+        <is>
+          <t>平和堂／平松社長「富山県でドミナント強化、富山掛尾店の滑り出し好調」注目</t>
+        </is>
+      </c>
+      <c r="D2235" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100214.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2236">
+      <c r="A2236" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2236" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2236" t="inlineStr">
+        <is>
+          <t>イオンリテール／イオン諏訪店跡地に「イオンスタイル」10月21日オープン</t>
+        </is>
+      </c>
+      <c r="D2236" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100278.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2237">
+      <c r="A2237" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2237" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2237" t="inlineStr">
+        <is>
+          <t>ユニクロ京都／西日本初登場の「UNIQLO COFFEE」導入、地元コラボTシャツも登場</t>
+        </is>
+      </c>
+      <c r="D2237" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100275.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2238">
+      <c r="A2238" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2238" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2238" t="inlineStr">
+        <is>
+          <t>大阪屋ショップ／愛知県2店舗目「日進店」オープン、鮮魚・魚総菜に注力</t>
+        </is>
+      </c>
+      <c r="D2238" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100271.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2239">
+      <c r="A2239" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2239" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2239" t="inlineStr">
+        <is>
+          <t>ジーユー／熊本県「ゆめタウン光の森」に10月9日移転・増床オープン</t>
+        </is>
+      </c>
+      <c r="D2239" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100211.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2240">
+      <c r="A2240" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2240" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2240" t="inlineStr">
+        <is>
+          <t>ヨークベニマル／福島県南相馬市に「ヨークベニマル原町西店衣料館」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2240" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100219.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2241">
+      <c r="A2241" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2241" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2241" t="inlineStr">
+        <is>
+          <t>ロイヤルホームセンター／京都府城陽市に「ロイヤルプロ城陽インター（店舗面積2400m2）」27年5月21日新設</t>
+        </is>
+      </c>
+      <c r="D2241" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1002011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2242">
+      <c r="A2242" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2242" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2242" t="inlineStr">
+        <is>
+          <t>コスモス薬品／群馬県渋川市に「ドラッグコスモス阿久津店」27年9月30日新設</t>
+        </is>
+      </c>
+      <c r="D2242" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1002012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2243">
+      <c r="A2243" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2243" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2243" t="inlineStr">
+        <is>
+          <t>ビームス／新宿区に初のスポーツコンセプトストア10月12日オープン</t>
+        </is>
+      </c>
+      <c r="D2243" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100276.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2244">
+      <c r="A2244" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2244" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2244" t="inlineStr">
+        <is>
+          <t>西鉄ストア／福岡市城南区「レガネット七隈」リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D2244" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100272.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2245">
+      <c r="A2245" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2245" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2245" t="inlineStr">
+        <is>
+          <t>キルフェボン／東京・新宿「明治安田新宿ビル」に新店舗11月28日オープン</t>
+        </is>
+      </c>
+      <c r="D2245" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100274.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2246">
+      <c r="A2246" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2246" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2246" t="inlineStr">
+        <is>
+          <t>ミスターマックス／広島県福山市に「MrMax Select福山店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D2246" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100283.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2247">
+      <c r="A2247" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2247" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2247" t="inlineStr">
+        <is>
+          <t>ストライプ／「AMERICAN HOLIC 京王モール店」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2247" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100215.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2248">
+      <c r="A2248" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2248" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2248" t="inlineStr">
+        <is>
+          <t>フランフラン／ルミネエスト新宿に10月9日新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D2248" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100216.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2249">
+      <c r="A2249" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2249" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2249" t="inlineStr">
+        <is>
+          <t>メガネスーパー／「イオンモール松本」「ゆめタウン三豊」にコンタクトレンズ専門店10月3日オープン</t>
+        </is>
+      </c>
+      <c r="D2249" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100279.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2250">
+      <c r="A2250" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2250" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2250" t="inlineStr">
+        <is>
+          <t>物語コーポレーション／「丸源ラーメン イオンモール甲府昭和店」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2250" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100273.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2251">
+      <c r="A2251" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2251" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2251" t="inlineStr">
+        <is>
+          <t>JR東日本／商業・ホテル複合「武蔵境駅東側駅ビル」28年度冬オープン</t>
+        </is>
+      </c>
+      <c r="D2251" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100175.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2252">
+      <c r="A2252" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2252" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2252" t="inlineStr">
+        <is>
+          <t>オーケーほか／東京都北区に「（仮称）北区豊島四丁目SC計画（店舗面積2670m2）」27年3月23日新設</t>
+        </is>
+      </c>
+      <c r="D2252" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1001011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2253">
+      <c r="A2253" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2253" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2253" t="inlineStr">
+        <is>
+          <t>しまむら／東京都練馬区に「（仮称）ファッションセンターしまむら中村南店」27年3月29日新設</t>
+        </is>
+      </c>
+      <c r="D2253" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1001012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2254">
+      <c r="A2254" t="inlineStr">
+        <is>
+          <t>2026年10月04日</t>
+        </is>
+      </c>
+      <c r="B2254" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2254" t="inlineStr">
+        <is>
+          <t>東京ソラマチ／10月以降「Eggs ’n Things」など新規6店舗オープン</t>
+        </is>
+      </c>
+      <c r="D2254" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100176.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-05
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2254"/>
+  <dimension ref="A1:D2323"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50004,6 +50004,1524 @@
         </is>
       </c>
     </row>
+    <row r="2255">
+      <c r="A2255" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2255" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2255" t="inlineStr">
+        <is>
+          <t>・12/1炭焼きレストランさわやか御殿場ぐみ沢店</t>
+        </is>
+      </c>
+      <c r="D2255" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gwe</t>
+        </is>
+      </c>
+    </row>
+    <row r="2256">
+      <c r="A2256" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2256" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2256" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D2256" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="2257">
+      <c r="A2257" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2257" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2257" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D2257" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="2258">
+      <c r="A2258" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2258" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2258" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D2258" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2259">
+      <c r="A2259" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2259" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2259" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D2259" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="2260">
+      <c r="A2260" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2260" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2260" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D2260" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2261">
+      <c r="A2261" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2261" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2261" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D2261" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="2262">
+      <c r="A2262" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2262" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2262" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D2262" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2263">
+      <c r="A2263" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2263" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2263" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D2263" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="2264">
+      <c r="A2264" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2264" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2264" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2264" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2265">
+      <c r="A2265" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2265" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2265" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2265" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2266">
+      <c r="A2266" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2266" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2266" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2266" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2267">
+      <c r="A2267" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2267" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2267" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2267" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2268">
+      <c r="A2268" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2268" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2268" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2268" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2269">
+      <c r="A2269" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2269" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2269" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2269" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2270">
+      <c r="A2270" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2270" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2270" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2270" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2271">
+      <c r="A2271" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2271" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2271" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2271" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2272">
+      <c r="A2272" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2272" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2272" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2272" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2273">
+      <c r="A2273" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2273" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2273" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2273" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2274">
+      <c r="A2274" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2274" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2274" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2274" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2275">
+      <c r="A2275" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2275" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2275" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2275" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2276">
+      <c r="A2276" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2276" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2276" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2276" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2277">
+      <c r="A2277" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2277" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2277" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2277" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2278">
+      <c r="A2278" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2278" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2278" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2278" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2279">
+      <c r="A2279" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2279" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2279" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2279" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2280">
+      <c r="A2280" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2280" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2280" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2280" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2281">
+      <c r="A2281" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2281" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2281" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2281" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2282">
+      <c r="A2282" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2282" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2282" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2282" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2283">
+      <c r="A2283" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2283" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2283" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2283" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2284">
+      <c r="A2284" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2284" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2284" t="inlineStr">
+        <is>
+          <t>関東地方イオン藤沢店 2026年1月末で一旦閉店し建て替えへ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2284" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/46012</t>
+        </is>
+      </c>
+    </row>
+    <row r="2285">
+      <c r="A2285" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2285" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2285" t="inlineStr">
+        <is>
+          <t>関東地方品川駅西口地区 B-1地区再開発 2035年度開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2285" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49707</t>
+        </is>
+      </c>
+    </row>
+    <row r="2286">
+      <c r="A2286" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2286" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2286" t="inlineStr">
+        <is>
+          <t>関東地方アトレ中野 2026年12月9日(水)開業！全73テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2286" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/27599</t>
+        </is>
+      </c>
+    </row>
+    <row r="2287">
+      <c r="A2287" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2287" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2287" t="inlineStr">
+        <is>
+          <t>東北地方いろは蔵パーク 2025年3月27日(木)開業！無印良品が出店へ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2287" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/38677</t>
+        </is>
+      </c>
+    </row>
+    <row r="2288">
+      <c r="A2288" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2288" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2288" t="inlineStr">
+        <is>
+          <t>関西地方OttoTerrace南芦屋浜店 2026年4月30日(木)開業！全13テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2288" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/30566</t>
+        </is>
+      </c>
+    </row>
+    <row r="2289">
+      <c r="A2289" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2289" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2289" t="inlineStr">
+        <is>
+          <t>北海道地方札幌駅・パセオ跡地 高架下商業施設 2028年冬開業！200店舗が出店へ！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2289" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/43941</t>
+        </is>
+      </c>
+    </row>
+    <row r="2290">
+      <c r="A2290" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2290" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2290" t="inlineStr">
+        <is>
+          <t>関東地方ハーモニーヒルズパーク入間 ベルクと屋上公園 2028年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2290" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/45967</t>
+        </is>
+      </c>
+    </row>
+    <row r="2291">
+      <c r="A2291" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2291" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2291" t="inlineStr">
+        <is>
+          <t>関東地方スーパーセンタートライアル秦野店 2026年10月開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2291" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48975</t>
+        </is>
+      </c>
+    </row>
+    <row r="2292">
+      <c r="A2292" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2292" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2292" t="inlineStr">
+        <is>
+          <t>関東地方みと好文テラス 2026年4月23日(木)開業！全11テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2292" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48066</t>
+        </is>
+      </c>
+    </row>
+    <row r="2293">
+      <c r="A2293" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2293" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2293" t="inlineStr">
+        <is>
+          <t>関東地方鷺沼駅前地区市街地再開発事業 2031年度竣工予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2293" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/24281</t>
+        </is>
+      </c>
+    </row>
+    <row r="2294">
+      <c r="A2294" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2294" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2294" t="inlineStr">
+        <is>
+          <t>中部地方カインズ笛吹石和店 2026年7月17日(金)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2294" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/43688</t>
+        </is>
+      </c>
+    </row>
+    <row r="2295">
+      <c r="A2295" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2295" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2295" t="inlineStr">
+        <is>
+          <t>中部地方三井アウトレットパーク岡崎 2025年11月4日(火)開業！テナント情報180店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2295" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/32467</t>
+        </is>
+      </c>
+    </row>
+    <row r="2296">
+      <c r="A2296" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2296" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2296" t="inlineStr">
+        <is>
+          <t>関東地方渋谷二丁目西地区市街地再開発事業 2029年度竣工予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2296" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/24394</t>
+        </is>
+      </c>
+    </row>
+    <row r="2297">
+      <c r="A2297" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2297" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2297" t="inlineStr">
+        <is>
+          <t>関西地方そよら小野 2027年秋開業！イオン小野店跡地 21店舗が出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2297" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/43512</t>
+        </is>
+      </c>
+    </row>
+    <row r="2298">
+      <c r="A2298" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2298" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2298" t="inlineStr">
+        <is>
+          <t>関東地方マチノマ小手指 トライアル西友小手指 2026年冬開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2298" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/39507</t>
+        </is>
+      </c>
+    </row>
+    <row r="2299">
+      <c r="A2299" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2299" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2299" t="inlineStr">
+        <is>
+          <t>関東地方本八幡駅北口駅前地区市街地再開発事業 2032年11月竣工！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2299" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49749</t>
+        </is>
+      </c>
+    </row>
+    <row r="2300">
+      <c r="A2300" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2300" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2300" t="inlineStr">
+        <is>
+          <t>関東地方ヨークタウン小山羽川 2026年8月28日(金)開業！全4テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2300" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48080</t>
+        </is>
+      </c>
+    </row>
+    <row r="2301">
+      <c r="A2301" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2301" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2301" t="inlineStr">
+        <is>
+          <t>関東地方リコパ東大和 2026年春全館開業！テラス棟含む 全46テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2301" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/32977</t>
+        </is>
+      </c>
+    </row>
+    <row r="2302">
+      <c r="A2302" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2302" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2302" t="inlineStr">
+        <is>
+          <t>四国地方フジ三町店 イヨテツスポーツセンター跡地 2028年開業！テナントは？最新情報も！愛媛県松山市三町の「イヨテツスポーツセンター」跡地に、株式会社フジによる新たな商業施設「フジ三町店（仮称）」が2028年ごろ開業予定！県内唯一のアイススケート場や屋外プールとして約60年にわたり親しまれた「イヨテツスポーツセンター」跡地を中...2026.10.04四国地方</t>
+        </is>
+      </c>
+      <c r="D2302" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/shikoku/49886</t>
+        </is>
+      </c>
+    </row>
+    <row r="2303">
+      <c r="A2303" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2303" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2303" t="inlineStr">
+        <is>
+          <t>関東地方湯島三丁目地区市街地再開発事業 2035年度完成予定！どのような施設に？最新情報も！東京都文京区湯島に、地上40階建ての超高層ランドマーク複合ビル「湯島三丁目地区市街地再開発事業」が2035年度に完成予定！東京メトロ千代田線「湯島駅」直結！高さ約170m・延床面積約11万㎡の超高層タワーが誕生！低層階の商業ゾーンをはじめ、...2026.10.04関東地方</t>
+        </is>
+      </c>
+      <c r="D2303" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49878</t>
+        </is>
+      </c>
+    </row>
+    <row r="2304">
+      <c r="A2304" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2304" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2304" t="inlineStr">
+        <is>
+          <t>ヤオコー／埼玉県入間市「まるひろ入間SC店」10月9日オープン、年商予定は22億円</t>
+        </is>
+      </c>
+      <c r="D2304" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100541.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2305">
+      <c r="A2305" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2305" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2305" t="inlineStr">
+        <is>
+          <t>川崎とどろきパーク／等々力緑地の正面広場にマクドナルド・スタバなど4店舗オープン</t>
+        </is>
+      </c>
+      <c r="D2305" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100545.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2306">
+      <c r="A2306" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2306" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2306" t="inlineStr">
+        <is>
+          <t>有隣堂／大船ルミネウィングに文具・雑貨の新ブランド「ペンノ ペンナ」11月5日オープン</t>
+        </is>
+      </c>
+      <c r="D2306" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2307">
+      <c r="A2307" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2307" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2307" t="inlineStr">
+        <is>
+          <t>ウオロク／新潟県加茂市に「加茂店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D2307" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100544.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2308">
+      <c r="A2308" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2308" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2308" t="inlineStr">
+        <is>
+          <t>まいばすけっと／埼玉県さいたま市に「北浦和駅西店」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2308" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100516.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2309">
+      <c r="A2309" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2309" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2309" t="inlineStr">
+        <is>
+          <t>エディオン／佐賀県唐津市「イオン唐津店」10月23日移転オープン</t>
+        </is>
+      </c>
+      <c r="D2309" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100542.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2310">
+      <c r="A2310" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2310" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2310" t="inlineStr">
+        <is>
+          <t>コメリ／富山県に「コメリPRO小矢部」10月17日オープン、ハード＆グリーンに併設</t>
+        </is>
+      </c>
+      <c r="D2310" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100574.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2311">
+      <c r="A2311" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2311" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2311" t="inlineStr">
+        <is>
+          <t>神奈川県「ミウィ橋本」／開業25周年、抽選会やポイント5倍キャンペーン実施</t>
+        </is>
+      </c>
+      <c r="D2311" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100511.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2312">
+      <c r="A2312" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2312" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2312" t="inlineStr">
+        <is>
+          <t>レインズ／京都府3店舗目「牛角焼肉食堂 イオン京都洛南店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D2312" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100572.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2313">
+      <c r="A2313" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2313" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2313" t="inlineStr">
+        <is>
+          <t>平和堂／平松社長「富山県でドミナント強化、富山掛尾店の滑り出し好調」注目</t>
+        </is>
+      </c>
+      <c r="D2313" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100214.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2314">
+      <c r="A2314" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2314" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2314" t="inlineStr">
+        <is>
+          <t>イオンリテール／イオン諏訪店跡地に「イオンスタイル」10月21日オープン</t>
+        </is>
+      </c>
+      <c r="D2314" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100278.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2315">
+      <c r="A2315" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2315" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2315" t="inlineStr">
+        <is>
+          <t>ユニクロ京都／西日本初登場の「UNIQLO COFFEE」導入、地元コラボTシャツも登場</t>
+        </is>
+      </c>
+      <c r="D2315" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100275.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2316">
+      <c r="A2316" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2316" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2316" t="inlineStr">
+        <is>
+          <t>大阪屋ショップ／愛知県2店舗目「日進店」オープン、鮮魚・魚総菜に注力</t>
+        </is>
+      </c>
+      <c r="D2316" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100271.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2317">
+      <c r="A2317" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2317" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2317" t="inlineStr">
+        <is>
+          <t>ジーユー／熊本県「ゆめタウン光の森」に10月9日移転・増床オープン</t>
+        </is>
+      </c>
+      <c r="D2317" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100211.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2318">
+      <c r="A2318" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2318" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2318" t="inlineStr">
+        <is>
+          <t>ヨークベニマル／福島県南相馬市に「ヨークベニマル原町西店衣料館」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2318" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100219.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2319">
+      <c r="A2319" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2319" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2319" t="inlineStr">
+        <is>
+          <t>ロイヤルホームセンター／京都府城陽市に「ロイヤルプロ城陽インター（店舗面積2400m2）」27年5月21日新設</t>
+        </is>
+      </c>
+      <c r="D2319" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1002011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2320">
+      <c r="A2320" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2320" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2320" t="inlineStr">
+        <is>
+          <t>コスモス薬品／群馬県渋川市に「ドラッグコスモス阿久津店」27年9月30日新設</t>
+        </is>
+      </c>
+      <c r="D2320" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1002012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2321">
+      <c r="A2321" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2321" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2321" t="inlineStr">
+        <is>
+          <t>ビームス／新宿区に初のスポーツコンセプトストア10月12日オープン</t>
+        </is>
+      </c>
+      <c r="D2321" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100276.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2322">
+      <c r="A2322" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2322" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2322" t="inlineStr">
+        <is>
+          <t>西鉄ストア／福岡市城南区「レガネット七隈」リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D2322" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100272.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2323">
+      <c r="A2323" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2323" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2323" t="inlineStr">
+        <is>
+          <t>キルフェボン／東京・新宿「明治安田新宿ビル」に新店舗11月28日オープン</t>
+        </is>
+      </c>
+      <c r="D2323" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100274.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-06
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2323"/>
+  <dimension ref="A1:D2392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51522,6 +51522,1524 @@
         </is>
       </c>
     </row>
+    <row r="2324">
+      <c r="A2324" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2324" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2324" t="inlineStr">
+        <is>
+          <t>・12/1炭焼きレストランさわやか御殿場ぐみ沢店</t>
+        </is>
+      </c>
+      <c r="D2324" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gwe</t>
+        </is>
+      </c>
+    </row>
+    <row r="2325">
+      <c r="A2325" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2325" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2325" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D2325" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="2326">
+      <c r="A2326" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2326" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2326" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D2326" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="2327">
+      <c r="A2327" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2327" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2327" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D2327" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2328">
+      <c r="A2328" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2328" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2328" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D2328" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="2329">
+      <c r="A2329" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2329" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2329" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D2329" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2330">
+      <c r="A2330" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2330" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2330" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D2330" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="2331">
+      <c r="A2331" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2331" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2331" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D2331" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2332">
+      <c r="A2332" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2332" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2332" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D2332" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="2333">
+      <c r="A2333" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2333" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2333" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2333" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2334">
+      <c r="A2334" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2334" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2334" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2334" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2335">
+      <c r="A2335" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2335" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2335" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2335" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2336">
+      <c r="A2336" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2336" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2336" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2336" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2337">
+      <c r="A2337" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2337" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2337" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2337" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2338">
+      <c r="A2338" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2338" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2338" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2338" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2339">
+      <c r="A2339" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2339" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2339" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2339" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2340">
+      <c r="A2340" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2340" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2340" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2340" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2341">
+      <c r="A2341" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2341" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2341" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2341" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2342">
+      <c r="A2342" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2342" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2342" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2342" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2343">
+      <c r="A2343" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2343" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2343" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2343" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2344">
+      <c r="A2344" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2344" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2344" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2344" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2345">
+      <c r="A2345" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2345" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2345" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2345" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2346">
+      <c r="A2346" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2346" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2346" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2346" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2347">
+      <c r="A2347" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2347" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2347" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2347" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2348">
+      <c r="A2348" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2348" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2348" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2348" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2349">
+      <c r="A2349" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2349" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2349" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2349" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2350">
+      <c r="A2350" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2350" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2350" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2350" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2351">
+      <c r="A2351" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2351" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2351" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2351" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2352">
+      <c r="A2352" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2352" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2352" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2352" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2353">
+      <c r="A2353" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2353" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2353" t="inlineStr">
+        <is>
+          <t>中部地方ミュープラット豊田市 2026年8月26日(水)開業！全7店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2353" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48621</t>
+        </is>
+      </c>
+    </row>
+    <row r="2354">
+      <c r="A2354" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2354" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2354" t="inlineStr">
+        <is>
+          <t>関東地方神田小川町三丁目西部南地区市街地再開発事業 進捗状況は？テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2354" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/31895</t>
+        </is>
+      </c>
+    </row>
+    <row r="2355">
+      <c r="A2355" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2355" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2355" t="inlineStr">
+        <is>
+          <t>中部地方そよら三条須頃 2025年11月7日(金)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2355" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/36987</t>
+        </is>
+      </c>
+    </row>
+    <row r="2356">
+      <c r="A2356" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2356" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2356" t="inlineStr">
+        <is>
+          <t>関東地方北小金駅南口東地区市街地再開発事業 2028年度完成 テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2356" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49735</t>
+        </is>
+      </c>
+    </row>
+    <row r="2357">
+      <c r="A2357" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2357" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2357" t="inlineStr">
+        <is>
+          <t>北海道地方SAPPORO ONE サッポロワン 大通西4南地区市街地再開発事業 2029年8月完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2357" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/26256</t>
+        </is>
+      </c>
+    </row>
+    <row r="2358">
+      <c r="A2358" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2358" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2358" t="inlineStr">
+        <is>
+          <t>東北地方ニトリ福島御山店 2027年3月開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2358" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/49620</t>
+        </is>
+      </c>
+    </row>
+    <row r="2359">
+      <c r="A2359" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2359" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2359" t="inlineStr">
+        <is>
+          <t>関西地方アイユータウン マルアイ長田店 2025年9月17日(水)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2359" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/42358</t>
+        </is>
+      </c>
+    </row>
+    <row r="2360">
+      <c r="A2360" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2360" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2360" t="inlineStr">
+        <is>
+          <t>北海道地方札幌4丁目プレイス 4PLA 2025年4月25日(金)から順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2360" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/32449</t>
+        </is>
+      </c>
+    </row>
+    <row r="2361">
+      <c r="A2361" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2361" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2361" t="inlineStr">
+        <is>
+          <t>関西地方ミラモール東岸和田駅前 住友商事が2025年9月25日(木)~順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2361" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39056</t>
+        </is>
+      </c>
+    </row>
+    <row r="2362">
+      <c r="A2362" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2362" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2362" t="inlineStr">
+        <is>
+          <t>中国地方カインズ日吉津店 2025年3月12日(水)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2362" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/34869</t>
+        </is>
+      </c>
+    </row>
+    <row r="2363">
+      <c r="A2363" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2363" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2363" t="inlineStr">
+        <is>
+          <t>関東地方太田駅南口再開発 ベルクの複合商業施設 2026年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2363" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47305</t>
+        </is>
+      </c>
+    </row>
+    <row r="2364">
+      <c r="A2364" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2364" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2364" t="inlineStr">
+        <is>
+          <t>中国地方ハローズ西岐波店 2026年8月6日(木)開業！全4テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2364" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/48261</t>
+        </is>
+      </c>
+    </row>
+    <row r="2365">
+      <c r="A2365" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2365" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2365" t="inlineStr">
+        <is>
+          <t>関東地方福生駅西口地区市街地再開発事業 2027年春完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2365" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36735</t>
+        </is>
+      </c>
+    </row>
+    <row r="2366">
+      <c r="A2366" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2366" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2366" t="inlineStr">
+        <is>
+          <t>関東地方KAMISEYA PARK 三菱地所がテーマパーク 2031年頃開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2366" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/34224</t>
+        </is>
+      </c>
+    </row>
+    <row r="2367">
+      <c r="A2367" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2367" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2367" t="inlineStr">
+        <is>
+          <t>中国地方そよら鳥取駅南 2026年10月上旬開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2367" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/49474</t>
+        </is>
+      </c>
+    </row>
+    <row r="2368">
+      <c r="A2368" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2368" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2368" t="inlineStr">
+        <is>
+          <t>関東地方渋谷アッパー・ウエスト・プロジェクト(東急百貨店本店跡地) 2029年夏竣工！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2368" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26447</t>
+        </is>
+      </c>
+    </row>
+    <row r="2369">
+      <c r="A2369" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2369" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2369" t="inlineStr">
+        <is>
+          <t>九州地方クロスモール花ヶ島 2026年1月29日(木)開業！全5店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2369" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/34622</t>
+        </is>
+      </c>
+    </row>
+    <row r="2370">
+      <c r="A2370" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2370" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2370" t="inlineStr">
+        <is>
+          <t>関西地方J.GRAN TOWER 京都向日町 2028年夏開業！駅ビルのテナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2370" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39560</t>
+        </is>
+      </c>
+    </row>
+    <row r="2371">
+      <c r="A2371" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2371" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2371" t="inlineStr">
+        <is>
+          <t>中国地方ケーズデンキ山口店 2026年秋開業予定！最新情報も！山口県山口市にビッグ・エスの店舗「ケーズデンキ山口店」が2026年秋に開業予定！ケーズデンキの中では中～大型店舗となります。隣接地には「ウォンツ山口黒川店」も新設！そんな、ケーズデンキ山口店について、テナントや開業日などを見ていきましょう！...2026.10.06中国地方</t>
+        </is>
+      </c>
+      <c r="D2371" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/44477</t>
+        </is>
+      </c>
+    </row>
+    <row r="2372">
+      <c r="A2372" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2372" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2372" t="inlineStr">
+        <is>
+          <t>関西地方スーパーセンタートライアル愛知川店 2026年10月下旬に開業予定！最新情報も！滋賀県愛知郡にトライアルカンパニーの店舗「スーパーセンタートライアル愛知川店」が2026年10月下旬に開業予定！スーパーセンタートライアルが愛荘町に初出店！そんな、スーパーセンタートライアル愛知川店について、テナントや開業日などを見ていきま...2026.10.06関西地方</t>
+        </is>
+      </c>
+      <c r="D2372" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/47736</t>
+        </is>
+      </c>
+    </row>
+    <row r="2373">
+      <c r="A2373" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2373" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2373" t="inlineStr">
+        <is>
+          <t>自由が丘駅南口／新たな文化発信拠点「ミミミ自由が丘」10月9日オープン、新業態充実注目</t>
+        </is>
+      </c>
+      <c r="D2373" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s100673.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2374">
+      <c r="A2374" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2374" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2374" t="inlineStr">
+        <is>
+          <t>サンエー 決算／3～8月増収増益、季節商材・食品・土産が好調</t>
+        </is>
+      </c>
+      <c r="D2374" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100616.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2375">
+      <c r="A2375" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2375" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2375" t="inlineStr">
+        <is>
+          <t>ラスカ平塚／「リンツ ショコラ ブティック」など4店舗が11月にオープン</t>
+        </is>
+      </c>
+      <c r="D2375" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100672.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2376">
+      <c r="A2376" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2376" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2376" t="inlineStr">
+        <is>
+          <t>ニトリ／横浜市鶴見区にアパレルブランド「N+島忠ホームズ新川崎店」オープン</t>
+        </is>
+      </c>
+      <c r="D2376" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100644.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2377">
+      <c r="A2377" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2377" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2377" t="inlineStr">
+        <is>
+          <t>オリジン東秀／東京・五反田に「れんげ食堂Toshu 五反田TOC店」オープン</t>
+        </is>
+      </c>
+      <c r="D2377" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100645.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2378">
+      <c r="A2378" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2378" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2378" t="inlineStr">
+        <is>
+          <t>キーコーヒー／岩手県盛岡市に「KEY’S CAFE 盛岡フェザン店」オープン</t>
+        </is>
+      </c>
+      <c r="D2378" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100647.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2379">
+      <c r="A2379" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2379" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2379" t="inlineStr">
+        <is>
+          <t>相鉄ライフさがみ野／2027年1月下旬に閉館、46年の歴史に幕</t>
+        </is>
+      </c>
+      <c r="D2379" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100651.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2380">
+      <c r="A2380" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2380" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2380" t="inlineStr">
+        <is>
+          <t>大創産業／DAISO公式キャラ「だいぞう」初のコラボカフェ、東京・大阪で開催</t>
+        </is>
+      </c>
+      <c r="D2380" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100612.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2381">
+      <c r="A2381" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2381" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2381" t="inlineStr">
+        <is>
+          <t>ヤオコー／埼玉県入間市「まるひろ入間SC店」10月9日オープン、年商予定は22億円</t>
+        </is>
+      </c>
+      <c r="D2381" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100541.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2382">
+      <c r="A2382" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2382" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2382" t="inlineStr">
+        <is>
+          <t>川崎とどろきパーク／等々力緑地の正面広場にマクドナルド・スタバなど4店舗オープン</t>
+        </is>
+      </c>
+      <c r="D2382" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100545.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2383">
+      <c r="A2383" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2383" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2383" t="inlineStr">
+        <is>
+          <t>有隣堂／大船ルミネウィングに文具・雑貨の新ブランド「ペンノ ペンナ」11月5日オープン</t>
+        </is>
+      </c>
+      <c r="D2383" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2384">
+      <c r="A2384" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2384" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2384" t="inlineStr">
+        <is>
+          <t>ウオロク／新潟県加茂市に「加茂店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D2384" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100544.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2385">
+      <c r="A2385" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2385" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2385" t="inlineStr">
+        <is>
+          <t>まいばすけっと／埼玉県さいたま市に「北浦和駅西店」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2385" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100516.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2386">
+      <c r="A2386" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2386" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2386" t="inlineStr">
+        <is>
+          <t>エディオン／佐賀県唐津市「イオン唐津店」10月23日移転オープン</t>
+        </is>
+      </c>
+      <c r="D2386" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100542.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2387">
+      <c r="A2387" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2387" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2387" t="inlineStr">
+        <is>
+          <t>コメリ／富山県に「コメリPRO小矢部」10月17日オープン、ハード＆グリーンに併設</t>
+        </is>
+      </c>
+      <c r="D2387" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100574.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2388">
+      <c r="A2388" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2388" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2388" t="inlineStr">
+        <is>
+          <t>神奈川県「ミウィ橋本」／開業25周年、抽選会やポイント5倍キャンペーン実施</t>
+        </is>
+      </c>
+      <c r="D2388" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100511.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2389">
+      <c r="A2389" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2389" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2389" t="inlineStr">
+        <is>
+          <t>レインズ／京都府3店舗目「牛角焼肉食堂 イオン京都洛南店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D2389" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100572.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2390">
+      <c r="A2390" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2390" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2390" t="inlineStr">
+        <is>
+          <t>平和堂／平松社長「富山県でドミナント強化、富山掛尾店の滑り出し好調」注目</t>
+        </is>
+      </c>
+      <c r="D2390" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100214.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2391">
+      <c r="A2391" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2391" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2391" t="inlineStr">
+        <is>
+          <t>イオンリテール／イオン諏訪店跡地に「イオンスタイル」10月21日オープン</t>
+        </is>
+      </c>
+      <c r="D2391" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100278.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2392">
+      <c r="A2392" t="inlineStr">
+        <is>
+          <t>2026年10月06日</t>
+        </is>
+      </c>
+      <c r="B2392" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2392" t="inlineStr">
+        <is>
+          <t>ユニクロ京都／西日本初登場の「UNIQLO COFFEE」導入、地元コラボTシャツも登場</t>
+        </is>
+      </c>
+      <c r="D2392" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100275.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-07
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2392"/>
+  <dimension ref="A1:D2452"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53040,6 +53040,1326 @@
         </is>
       </c>
     </row>
+    <row r="2393">
+      <c r="A2393" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2393" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2393" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2393" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2394">
+      <c r="A2394" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2394" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2394" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2394" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2395">
+      <c r="A2395" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2395" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2395" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2395" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2396">
+      <c r="A2396" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2396" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2396" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2396" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2397">
+      <c r="A2397" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2397" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2397" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2397" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2398">
+      <c r="A2398" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2398" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2398" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2398" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2399">
+      <c r="A2399" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2399" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2399" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2399" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2400">
+      <c r="A2400" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2400" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2400" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2400" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2401">
+      <c r="A2401" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2401" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2401" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2401" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2402">
+      <c r="A2402" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2402" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2402" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2402" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2403">
+      <c r="A2403" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2403" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2403" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2403" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2404">
+      <c r="A2404" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2404" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2404" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2404" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2405">
+      <c r="A2405" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2405" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2405" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2405" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2406">
+      <c r="A2406" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2406" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2406" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2406" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2407">
+      <c r="A2407" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2407" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2407" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2407" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2408">
+      <c r="A2408" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2408" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2408" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2408" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2409">
+      <c r="A2409" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2409" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2409" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2409" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2410">
+      <c r="A2410" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2410" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2410" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2410" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2411">
+      <c r="A2411" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2411" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2411" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2411" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2412">
+      <c r="A2412" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2412" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2412" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2412" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2413">
+      <c r="A2413" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2413" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2413" t="inlineStr">
+        <is>
+          <t>東北地方旧青森国際ホテル跡地地区市街地再開発事業 完成はいつ？どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2413" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/39897</t>
+        </is>
+      </c>
+    </row>
+    <row r="2414">
+      <c r="A2414" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2414" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2414" t="inlineStr">
+        <is>
+          <t>関東地方ヨークベニマル古河店 カインズ古河店 2025年2月14日(金)開業！無印良品とスタバが出店！全6テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2414" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/37708</t>
+        </is>
+      </c>
+    </row>
+    <row r="2415">
+      <c r="A2415" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2415" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2415" t="inlineStr">
+        <is>
+          <t>九州地方スプリングガーデン御代志2025年3月24日(月)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2415" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/36931</t>
+        </is>
+      </c>
+    </row>
+    <row r="2416">
+      <c r="A2416" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2416" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2416" t="inlineStr">
+        <is>
+          <t>関東地方原宿クエスト 建て替え 2025年11月18日(火)から順次開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2416" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/28345</t>
+        </is>
+      </c>
+    </row>
+    <row r="2417">
+      <c r="A2417" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2417" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2417" t="inlineStr">
+        <is>
+          <t>関西地方【計画白紙】コストコ たつの市 2029年度開業計画！場所は？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2417" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39958</t>
+        </is>
+      </c>
+    </row>
+    <row r="2418">
+      <c r="A2418" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2418" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2418" t="inlineStr">
+        <is>
+          <t>関東地方鎌倉梶原商業施設 2026年8月28日(金)より順次開業！ライフやカインズが出店！全4店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2418" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/43953</t>
+        </is>
+      </c>
+    </row>
+    <row r="2419">
+      <c r="A2419" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2419" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2419" t="inlineStr">
+        <is>
+          <t>関東地方大宮駅東口大門町３丁目中地区再開発事業 が計画中！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2419" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/34117</t>
+        </is>
+      </c>
+    </row>
+    <row r="2420">
+      <c r="A2420" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2420" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2420" t="inlineStr">
+        <is>
+          <t>関西地方アクロスプラザ和泉観音寺 2026年11月開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2420" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/47867</t>
+        </is>
+      </c>
+    </row>
+    <row r="2421">
+      <c r="A2421" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2421" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2421" t="inlineStr">
+        <is>
+          <t>関東地方武蔵小金井駅北口駅前東地区市街地再開発事業 2030年1月完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2421" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48940</t>
+        </is>
+      </c>
+    </row>
+    <row r="2422">
+      <c r="A2422" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2422" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2422" t="inlineStr">
+        <is>
+          <t>関東地方渋谷スクランブルスクエア第Ⅱ期（中央棟・西棟）2031年度開業！大規模商業施設誕生！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2422" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47883</t>
+        </is>
+      </c>
+    </row>
+    <row r="2423">
+      <c r="A2423" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2423" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2423" t="inlineStr">
+        <is>
+          <t>東北地方スーパーセンタートライアル金ケ崎店 2026年9月16日(水)開業！15日(火)プレオープン！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2423" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/47232</t>
+        </is>
+      </c>
+    </row>
+    <row r="2424">
+      <c r="A2424" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2424" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2424" t="inlineStr">
+        <is>
+          <t>東北地方アスマチ多賀城 2025年10月着工！商業施設も！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2424" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/35915</t>
+        </is>
+      </c>
+    </row>
+    <row r="2425">
+      <c r="A2425" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2425" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2425" t="inlineStr">
+        <is>
+          <t>関東地方逗子駅ビル 2028年春開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2425" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49835</t>
+        </is>
+      </c>
+    </row>
+    <row r="2426">
+      <c r="A2426" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2426" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2426" t="inlineStr">
+        <is>
+          <t>東北地方マイヤ宮古磯鶏 2025年3月27日(木)開業！最新情報は？求人情報も！</t>
+        </is>
+      </c>
+      <c r="D2426" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/43583</t>
+        </is>
+      </c>
+    </row>
+    <row r="2427">
+      <c r="A2427" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2427" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2427" t="inlineStr">
+        <is>
+          <t>関東地方コープ幕張駅北口店 2025年2月25日(火)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2427" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/39459</t>
+        </is>
+      </c>
+    </row>
+    <row r="2428">
+      <c r="A2428" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2428" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2428" t="inlineStr">
+        <is>
+          <t>北海道地方スーパーセンタートライアル砂川店 2025年6月4日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2428" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/41719</t>
+        </is>
+      </c>
+    </row>
+    <row r="2429">
+      <c r="A2429" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2429" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2429" t="inlineStr">
+        <is>
+          <t>九州地方九州大学箱崎キャンパス跡地地区 2028年度より街びらき！商業施設も誕生！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2429" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/46612</t>
+        </is>
+      </c>
+    </row>
+    <row r="2430">
+      <c r="A2430" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2430" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2430" t="inlineStr">
+        <is>
+          <t>中国地方ハローズ西古松モール 2025年6月20日(金)開業！全8テナント一覧 最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2430" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/42181</t>
+        </is>
+      </c>
+    </row>
+    <row r="2431">
+      <c r="A2431" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2431" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2431" t="inlineStr">
+        <is>
+          <t>中国地方ケーズデンキ山口店 2026年秋開業予定！最新情報も！山口県山口市にビッグ・エスの店舗「ケーズデンキ山口店」が2026年秋に開業予定！ケーズデンキの中では中～大型店舗となります。隣接地には「ウォンツ山口黒川店」も新設！そんな、ケーズデンキ山口店について、テナントや開業日などを見ていきましょう！...2026.10.06中国地方</t>
+        </is>
+      </c>
+      <c r="D2431" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/44477</t>
+        </is>
+      </c>
+    </row>
+    <row r="2432">
+      <c r="A2432" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2432" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2432" t="inlineStr">
+        <is>
+          <t>関西地方スーパーセンタートライアル愛知川店 2026年10月下旬に開業予定！最新情報も！滋賀県愛知郡にトライアルカンパニーの店舗「スーパーセンタートライアル愛知川店」が2026年10月下旬に開業予定！スーパーセンタートライアルが愛荘町に初出店！そんな、スーパーセンタートライアル愛知川店について、テナントや開業日などを見ていきま...2026.10.06関西地方</t>
+        </is>
+      </c>
+      <c r="D2432" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/47736</t>
+        </is>
+      </c>
+    </row>
+    <row r="2433">
+      <c r="A2433" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2433" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2433" t="inlineStr">
+        <is>
+          <t>あべのハルカス近鉄本店／洋菓子フロアの大規模リニューアル10月21日開始</t>
+        </is>
+      </c>
+      <c r="D2433" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100778.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2434">
+      <c r="A2434" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2434" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2434" t="inlineStr">
+        <is>
+          <t>ベイシア高萩モール店／「Beisia Foods Park」に10月9日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D2434" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100715.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2435">
+      <c r="A2435" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2435" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2435" t="inlineStr">
+        <is>
+          <t>大創産業／「Standard Products」福井県初出店、DAISOとの複合店をフェアモール福井にオープン</t>
+        </is>
+      </c>
+      <c r="D2435" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100716.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2436">
+      <c r="A2436" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2436" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2436" t="inlineStr">
+        <is>
+          <t>資さんうどん／神奈川県「横浜霧ケ丘店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D2436" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100779.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2437">
+      <c r="A2437" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2437" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2437" t="inlineStr">
+        <is>
+          <t>渋谷スクランブルスクエア／NY発チョコブランド「マリベル」10月28日オープン</t>
+        </is>
+      </c>
+      <c r="D2437" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100720.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2438">
+      <c r="A2438" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2438" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2438" t="inlineStr">
+        <is>
+          <t>ジェラート ピケ／「ららぽーと豊洲」「シャミネ松江」に新店舗10月オープン</t>
+        </is>
+      </c>
+      <c r="D2438" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100772.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2439">
+      <c r="A2439" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2439" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2439" t="inlineStr">
+        <is>
+          <t>中部薬品／愛知県一宮市に「V・drug一宮三条薬局」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D2439" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100717.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2440">
+      <c r="A2440" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2440" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2440" t="inlineStr">
+        <is>
+          <t>サブウェイ／大阪府守口市「イオンモール大日店」10月14日オープン</t>
+        </is>
+      </c>
+      <c r="D2440" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100777.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2441">
+      <c r="A2441" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2441" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2441" t="inlineStr">
+        <is>
+          <t>自由が丘駅南口／新たな文化発信拠点「ミミミ自由が丘」10月9日オープン、新業態充実注目</t>
+        </is>
+      </c>
+      <c r="D2441" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s100673.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2442">
+      <c r="A2442" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2442" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2442" t="inlineStr">
+        <is>
+          <t>サンエー 決算／3～8月増収増益、季節商材・食品・土産が好調</t>
+        </is>
+      </c>
+      <c r="D2442" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100616.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2443">
+      <c r="A2443" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2443" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2443" t="inlineStr">
+        <is>
+          <t>ラスカ平塚／「リンツ ショコラ ブティック」など4店舗が11月にオープン</t>
+        </is>
+      </c>
+      <c r="D2443" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100672.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2444">
+      <c r="A2444" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2444" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2444" t="inlineStr">
+        <is>
+          <t>ニトリ／横浜市鶴見区にアパレルブランド「N+島忠ホームズ新川崎店」オープン</t>
+        </is>
+      </c>
+      <c r="D2444" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100644.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2445">
+      <c r="A2445" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2445" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2445" t="inlineStr">
+        <is>
+          <t>オリジン東秀／東京・五反田に「れんげ食堂Toshu 五反田TOC店」オープン</t>
+        </is>
+      </c>
+      <c r="D2445" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100645.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2446">
+      <c r="A2446" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2446" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2446" t="inlineStr">
+        <is>
+          <t>キーコーヒー／岩手県盛岡市に「KEY’S CAFE 盛岡フェザン店」オープン</t>
+        </is>
+      </c>
+      <c r="D2446" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100647.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2447">
+      <c r="A2447" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2447" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2447" t="inlineStr">
+        <is>
+          <t>相鉄ライフさがみ野／2027年1月下旬に閉館、46年の歴史に幕</t>
+        </is>
+      </c>
+      <c r="D2447" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100651.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2448">
+      <c r="A2448" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2448" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2448" t="inlineStr">
+        <is>
+          <t>大創産業／DAISO公式キャラ「だいぞう」初のコラボカフェ、東京・大阪で開催</t>
+        </is>
+      </c>
+      <c r="D2448" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100612.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2449">
+      <c r="A2449" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2449" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2449" t="inlineStr">
+        <is>
+          <t>ヤオコー／埼玉県入間市「まるひろ入間SC店」10月9日オープン、年商予定は22億円</t>
+        </is>
+      </c>
+      <c r="D2449" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100541.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2450">
+      <c r="A2450" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2450" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2450" t="inlineStr">
+        <is>
+          <t>川崎とどろきパーク／等々力緑地の正面広場にマクドナルド・スタバなど4店舗オープン</t>
+        </is>
+      </c>
+      <c r="D2450" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100545.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2451">
+      <c r="A2451" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2451" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2451" t="inlineStr">
+        <is>
+          <t>マミーマート／「生鮮市場TOP！川口柳崎店」オープン、足元商圏のファミリー層狙う</t>
+        </is>
+      </c>
+      <c r="D2451" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091771.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2452">
+      <c r="A2452" t="inlineStr">
+        <is>
+          <t>2026年10月08日</t>
+        </is>
+      </c>
+      <c r="B2452" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2452" t="inlineStr">
+        <is>
+          <t>東京建物／川口市にNSC「ミナノバ」2号店オープン、2km商圏11万人の住宅地に出店</t>
+        </is>
+      </c>
+      <c r="D2452" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091672.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-08
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2452"/>
+  <dimension ref="A1:D2512"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54360,6 +54360,1326 @@
         </is>
       </c>
     </row>
+    <row r="2453">
+      <c r="A2453" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2453" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2453" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2453" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2454">
+      <c r="A2454" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2454" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2454" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2454" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2455">
+      <c r="A2455" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2455" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2455" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2455" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2456">
+      <c r="A2456" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2456" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2456" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2456" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2457">
+      <c r="A2457" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2457" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2457" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2457" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2458">
+      <c r="A2458" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2458" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2458" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2458" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2459">
+      <c r="A2459" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2459" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2459" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2459" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2460">
+      <c r="A2460" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2460" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2460" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2460" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2461">
+      <c r="A2461" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2461" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2461" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2461" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2462">
+      <c r="A2462" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2462" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2462" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2462" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2463">
+      <c r="A2463" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2463" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2463" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2463" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2464">
+      <c r="A2464" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2464" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2464" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2464" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2465">
+      <c r="A2465" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2465" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2465" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2465" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2466">
+      <c r="A2466" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2466" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2466" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2466" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2467">
+      <c r="A2467" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2467" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2467" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2467" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2468">
+      <c r="A2468" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2468" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2468" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2468" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2469">
+      <c r="A2469" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2469" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2469" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2469" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2470">
+      <c r="A2470" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2470" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2470" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2470" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2471">
+      <c r="A2471" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2471" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2471" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2471" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2472">
+      <c r="A2472" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2472" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2472" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2472" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2473">
+      <c r="A2473" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2473" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2473" t="inlineStr">
+        <is>
+          <t>東北地方アスマチ多賀城 2025年10月着工！商業施設も！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2473" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/35915</t>
+        </is>
+      </c>
+    </row>
+    <row r="2474">
+      <c r="A2474" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2474" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2474" t="inlineStr">
+        <is>
+          <t>関西地方高島屋堺店跡地にHiViE堺東が2027年春全体開業！ライフが出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2474" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/41410</t>
+        </is>
+      </c>
+    </row>
+    <row r="2475">
+      <c r="A2475" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2475" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2475" t="inlineStr">
+        <is>
+          <t>関東地方HIBIYA CROSSPARK（日比谷クロスパーク）2029年春街びらき！2037年全体開業！どのような街に？</t>
+        </is>
+      </c>
+      <c r="D2475" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/24411</t>
+        </is>
+      </c>
+    </row>
+    <row r="2476">
+      <c r="A2476" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2476" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2476" t="inlineStr">
+        <is>
+          <t>関東地方上板橋駅南口駅前東地区市街地再開発事業 2028年完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2476" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48931</t>
+        </is>
+      </c>
+    </row>
+    <row r="2477">
+      <c r="A2477" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2477" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2477" t="inlineStr">
+        <is>
+          <t>北海道地方札幌ダイビル PIVOT(ピヴォ) 建て替え 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2477" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/32542</t>
+        </is>
+      </c>
+    </row>
+    <row r="2478">
+      <c r="A2478" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2478" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2478" t="inlineStr">
+        <is>
+          <t>九州地方新一日橋ショッピングセンター 2026年冬開業！30店舗が出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2478" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/45078</t>
+        </is>
+      </c>
+    </row>
+    <row r="2479">
+      <c r="A2479" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2479" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2479" t="inlineStr">
+        <is>
+          <t>関東地方六町駅前に東神開発の商業施設 2026年6月開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2479" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/31860</t>
+        </is>
+      </c>
+    </row>
+    <row r="2480">
+      <c r="A2480" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2480" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2480" t="inlineStr">
+        <is>
+          <t>関東地方新綱島MICCA 2026年10月28日(水)開業！全21テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2480" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49470</t>
+        </is>
+      </c>
+    </row>
+    <row r="2481">
+      <c r="A2481" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2481" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2481" t="inlineStr">
+        <is>
+          <t>関東地方川崎アリーナシティプロジェクト 2030年10月開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2481" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/33041</t>
+        </is>
+      </c>
+    </row>
+    <row r="2482">
+      <c r="A2482" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2482" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2482" t="inlineStr">
+        <is>
+          <t>関西地方イオンタウン堺水賀池 2027年冬開業！30店舗が出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2482" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/45734</t>
+        </is>
+      </c>
+    </row>
+    <row r="2483">
+      <c r="A2483" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2483" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2483" t="inlineStr">
+        <is>
+          <t>中部地方ウオロク加茂店 2026年秋(11月頃)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2483" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48531</t>
+        </is>
+      </c>
+    </row>
+    <row r="2484">
+      <c r="A2484" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2484" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2484" t="inlineStr">
+        <is>
+          <t>関東地方みなとみらい21中央地区60・61街区開発事業 2029年春開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2484" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36914</t>
+        </is>
+      </c>
+    </row>
+    <row r="2485">
+      <c r="A2485" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2485" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2485" t="inlineStr">
+        <is>
+          <t>中部地方【ツインタワー】岐阜駅北中央東・中央西地区市街地再開発事業 2029年度竣工予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2485" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/24349</t>
+        </is>
+      </c>
+    </row>
+    <row r="2486">
+      <c r="A2486" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2486" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2486" t="inlineStr">
+        <is>
+          <t>関西地方高槻グリーンプレイス 2025年5月1日(木)開業！12店舗が出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2486" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/38803</t>
+        </is>
+      </c>
+    </row>
+    <row r="2487">
+      <c r="A2487" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2487" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2487" t="inlineStr">
+        <is>
+          <t>北海道地方コープさっぽろ すながわ店 2026年9月10日(木)開業！無印良品も出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2487" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/48252</t>
+        </is>
+      </c>
+    </row>
+    <row r="2488">
+      <c r="A2488" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2488" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2488" t="inlineStr">
+        <is>
+          <t>四国地方スーパーセンタートライアル阿波土成店 2026年6月10日(水)グランドオープン！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2488" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/shikoku/46692</t>
+        </is>
+      </c>
+    </row>
+    <row r="2489">
+      <c r="A2489" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2489" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2489" t="inlineStr">
+        <is>
+          <t>中部地方アスナル金山 2036年3月閉店！当初計画の再開発の内容は？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2489" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/45176</t>
+        </is>
+      </c>
+    </row>
+    <row r="2490">
+      <c r="A2490" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2490" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2490" t="inlineStr">
+        <is>
+          <t>東北地方ドン・キホーテ東根店 蟹沢複合商業施設 2026年11月開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2490" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/47620</t>
+        </is>
+      </c>
+    </row>
+    <row r="2491">
+      <c r="A2491" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2491" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2491" t="inlineStr">
+        <is>
+          <t>中国地方ケーズデンキ山口店 2026年秋開業予定！最新情報も！山口県山口市にビッグ・エスの店舗「ケーズデンキ山口店」が2026年秋に開業予定！ケーズデンキの中では中～大型店舗となります。隣接地には「ウォンツ山口黒川店」も新設！そんな、ケーズデンキ山口店について、テナントや開業日などを見ていきましょう！...2026.10.06中国地方</t>
+        </is>
+      </c>
+      <c r="D2491" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/44477</t>
+        </is>
+      </c>
+    </row>
+    <row r="2492">
+      <c r="A2492" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2492" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2492" t="inlineStr">
+        <is>
+          <t>関西地方スーパーセンタートライアル愛知川店 2026年10月下旬に開業予定！最新情報も！滋賀県愛知郡にトライアルカンパニーの店舗「スーパーセンタートライアル愛知川店」が2026年10月下旬に開業予定！スーパーセンタートライアルが愛荘町に初出店！そんな、スーパーセンタートライアル愛知川店について、テナントや開業日などを見ていきま...2026.10.06関西地方</t>
+        </is>
+      </c>
+      <c r="D2492" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/47736</t>
+        </is>
+      </c>
+    </row>
+    <row r="2493">
+      <c r="A2493" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2493" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2493" t="inlineStr">
+        <is>
+          <t>ロピア／神戸市垂水区に「ブルメール舞多聞店」10月15日オープン</t>
+        </is>
+      </c>
+      <c r="D2493" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100813.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2494">
+      <c r="A2494" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2494" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2494" t="inlineStr">
+        <is>
+          <t>ふかや花園プレミアム・アウトレット／第2期増設で30店舗オープン、28年夏開業へ</t>
+        </is>
+      </c>
+      <c r="D2494" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100812.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2495">
+      <c r="A2495" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2495" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2495" t="inlineStr">
+        <is>
+          <t>三井不動産、野村不動産／「東京ミッドタウン日本橋」竣工、商業ゾーンは100区画2万m2</t>
+        </is>
+      </c>
+      <c r="D2495" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100872.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2496">
+      <c r="A2496" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2496" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2496" t="inlineStr">
+        <is>
+          <t>秋葉原UDX／商業ゾーン12月10日リニューアル、新規含む飲食27店舗オープン</t>
+        </is>
+      </c>
+      <c r="D2496" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100875.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2497">
+      <c r="A2497" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2497" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2497" t="inlineStr">
+        <is>
+          <t>AOKI／駅前型の新フォーマット店舗「川崎駅東口店」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2497" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100871.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2498">
+      <c r="A2498" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2498" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2498" t="inlineStr">
+        <is>
+          <t>グラニフ／京都に新旗艦店11月19日オープン、カフェ・アミューズメントエリア併設</t>
+        </is>
+      </c>
+      <c r="D2498" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100876.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2499">
+      <c r="A2499" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2499" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2499" t="inlineStr">
+        <is>
+          <t>マキヤ／静岡県裾野市に「（仮称）裾野複合店舗A棟・B棟」27年2月25日新設</t>
+        </is>
+      </c>
+      <c r="D2499" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1008012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2500">
+      <c r="A2500" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2500" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2500" t="inlineStr">
+        <is>
+          <t>コスモス薬品／岐阜県安八郡安八町に「ドラッグコスモス東結店」27年2月5日新設</t>
+        </is>
+      </c>
+      <c r="D2500" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1008011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2501">
+      <c r="A2501" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2501" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2501" t="inlineStr">
+        <is>
+          <t>あべのハルカス近鉄本店／洋菓子フロアの大規模リニューアル10月21日開始</t>
+        </is>
+      </c>
+      <c r="D2501" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100778.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2502">
+      <c r="A2502" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2502" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2502" t="inlineStr">
+        <is>
+          <t>ベイシア高萩モール店／「Beisia Foods Park」に10月9日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D2502" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100715.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2503">
+      <c r="A2503" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2503" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2503" t="inlineStr">
+        <is>
+          <t>大創産業／「Standard Products」福井県初出店、DAISOとの複合店をフェアモール福井にオープン</t>
+        </is>
+      </c>
+      <c r="D2503" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100716.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2504">
+      <c r="A2504" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2504" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2504" t="inlineStr">
+        <is>
+          <t>資さんうどん／神奈川県「横浜霧ケ丘店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D2504" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100779.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2505">
+      <c r="A2505" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2505" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2505" t="inlineStr">
+        <is>
+          <t>渋谷スクランブルスクエア／NY発チョコブランド「マリベル」10月28日オープン</t>
+        </is>
+      </c>
+      <c r="D2505" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100720.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2506">
+      <c r="A2506" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2506" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2506" t="inlineStr">
+        <is>
+          <t>ジェラート ピケ／「ららぽーと豊洲」「シャミネ松江」に新店舗10月オープン</t>
+        </is>
+      </c>
+      <c r="D2506" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100772.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2507">
+      <c r="A2507" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2507" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2507" t="inlineStr">
+        <is>
+          <t>中部薬品／愛知県一宮市に「V・drug一宮三条薬局」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D2507" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100717.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2508">
+      <c r="A2508" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2508" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2508" t="inlineStr">
+        <is>
+          <t>サブウェイ／大阪府守口市「イオンモール大日店」10月14日オープン</t>
+        </is>
+      </c>
+      <c r="D2508" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100777.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2509">
+      <c r="A2509" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2509" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2509" t="inlineStr">
+        <is>
+          <t>自由が丘駅南口／新たな文化発信拠点「ミミミ自由が丘」10月9日オープン、新業態充実注目</t>
+        </is>
+      </c>
+      <c r="D2509" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s100673.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2510">
+      <c r="A2510" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2510" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2510" t="inlineStr">
+        <is>
+          <t>サンエー 決算／3～8月増収増益、季節商材・食品・土産が好調</t>
+        </is>
+      </c>
+      <c r="D2510" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100616.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2511">
+      <c r="A2511" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2511" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2511" t="inlineStr">
+        <is>
+          <t>マミーマート／「生鮮市場TOP！川口柳崎店」オープン、足元商圏のファミリー層狙う</t>
+        </is>
+      </c>
+      <c r="D2511" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091771.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2512">
+      <c r="A2512" t="inlineStr">
+        <is>
+          <t>2026年10月09日</t>
+        </is>
+      </c>
+      <c r="B2512" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2512" t="inlineStr">
+        <is>
+          <t>東京建物／川口市にNSC「ミナノバ」2号店オープン、2km商圏11万人の住宅地に出店</t>
+        </is>
+      </c>
+      <c r="D2512" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091672.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-09
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2512"/>
+  <dimension ref="A1:D2572"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55680,6 +55680,1326 @@
         </is>
       </c>
     </row>
+    <row r="2513">
+      <c r="A2513" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2513" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2513" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2513" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2514">
+      <c r="A2514" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2514" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2514" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2514" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2515">
+      <c r="A2515" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2515" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2515" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2515" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2516">
+      <c r="A2516" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2516" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2516" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2516" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2517">
+      <c r="A2517" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2517" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2517" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2517" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2518">
+      <c r="A2518" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2518" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2518" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2518" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2519">
+      <c r="A2519" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2519" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2519" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2519" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2520">
+      <c r="A2520" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2520" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2520" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2520" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2521">
+      <c r="A2521" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2521" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2521" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2521" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2522">
+      <c r="A2522" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2522" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2522" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2522" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2523">
+      <c r="A2523" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2523" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2523" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2523" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2524">
+      <c r="A2524" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2524" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2524" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2524" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2525">
+      <c r="A2525" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2525" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2525" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2525" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2526">
+      <c r="A2526" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2526" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2526" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2526" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2527">
+      <c r="A2527" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2527" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2527" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2527" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2528">
+      <c r="A2528" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2528" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2528" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2528" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2529">
+      <c r="A2529" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2529" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2529" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2529" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2530">
+      <c r="A2530" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2530" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2530" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2530" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2531">
+      <c r="A2531" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2531" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2531" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2531" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2532">
+      <c r="A2532" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2532" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2532" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2532" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2533">
+      <c r="A2533" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2533" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2533" t="inlineStr">
+        <is>
+          <t>関東地方イオンスタイル竹ノ塚 ヤマダデンキ竹ノ塚店 2025年6月26日(木)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2533" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36038</t>
+        </is>
+      </c>
+    </row>
+    <row r="2534">
+      <c r="A2534" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2534" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2534" t="inlineStr">
+        <is>
+          <t>九州地方西日本シティビル 2026年7月21日(火)開業！全5テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2534" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/20689</t>
+        </is>
+      </c>
+    </row>
+    <row r="2535">
+      <c r="A2535" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2535" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2535" t="inlineStr">
+        <is>
+          <t>中国地方広島駅ビル「minamoa（ミナモア）」2025年3月24日(月)開業！全220テナント公開！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2535" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/7700</t>
+        </is>
+      </c>
+    </row>
+    <row r="2536">
+      <c r="A2536" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2536" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2536" t="inlineStr">
+        <is>
+          <t>関西地方ヒラカタウーヴン（枚方woven）・OPH枚方駅前 2025年早春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2536" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/25362</t>
+        </is>
+      </c>
+    </row>
+    <row r="2537">
+      <c r="A2537" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2537" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2537" t="inlineStr">
+        <is>
+          <t>関東地方新横浜プリンスペペ 2027年3月閉店の理由は？跡地はマクニカ新社屋に！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2537" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47961</t>
+        </is>
+      </c>
+    </row>
+    <row r="2538">
+      <c r="A2538" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2538" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2538" t="inlineStr">
+        <is>
+          <t>関東地方イオン八王子滝山 2026年6月26日(金)10:00~開業！次世代型商業施設が誕生！全21店舗一覧！</t>
+        </is>
+      </c>
+      <c r="D2538" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/17987</t>
+        </is>
+      </c>
+    </row>
+    <row r="2539">
+      <c r="A2539" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2539" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2539" t="inlineStr">
+        <is>
+          <t>関東地方藍テラス（あおてらす）青梅駅前に2026年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2539" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26304</t>
+        </is>
+      </c>
+    </row>
+    <row r="2540">
+      <c r="A2540" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2540" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2540" t="inlineStr">
+        <is>
+          <t>関東地方池袋マルイ跡「IT TOWER TOKYO」2026年3月14日(土)開業！全14店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2540" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/40793</t>
+        </is>
+      </c>
+    </row>
+    <row r="2541">
+      <c r="A2541" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2541" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2541" t="inlineStr">
+        <is>
+          <t>関東地方ニトリふじみ野店 2026年10月開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2541" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48589</t>
+        </is>
+      </c>
+    </row>
+    <row r="2542">
+      <c r="A2542" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2542" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2542" t="inlineStr">
+        <is>
+          <t>関東地方伊勢崎境ショッピングパーク 2027年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2542" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47294</t>
+        </is>
+      </c>
+    </row>
+    <row r="2543">
+      <c r="A2543" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2543" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2543" t="inlineStr">
+        <is>
+          <t>北海道地方ケーズデンキ帯広店 2025年3月20日(木・祝)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2543" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/40212</t>
+        </is>
+      </c>
+    </row>
+    <row r="2544">
+      <c r="A2544" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2544" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2544" t="inlineStr">
+        <is>
+          <t>関東地方平井テラス(プラウドタワー平井) 2025年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2544" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/19549</t>
+        </is>
+      </c>
+    </row>
+    <row r="2545">
+      <c r="A2545" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2545" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2545" t="inlineStr">
+        <is>
+          <t>九州地方スーパーセンタートライアル加納店 2025年4月29日(火・祝)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2545" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/40580</t>
+        </is>
+      </c>
+    </row>
+    <row r="2546">
+      <c r="A2546" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2546" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2546" t="inlineStr">
+        <is>
+          <t>関西地方ハローズ本多聞店 2026年6月24日(水)から順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2546" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/46204</t>
+        </is>
+      </c>
+    </row>
+    <row r="2547">
+      <c r="A2547" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2547" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2547" t="inlineStr">
+        <is>
+          <t>中部地方マックスバリュ豊橋西幸町店 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2547" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48626</t>
+        </is>
+      </c>
+    </row>
+    <row r="2548">
+      <c r="A2548" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2548" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2548" t="inlineStr">
+        <is>
+          <t>関西地方平和堂大久保店 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2548" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49605</t>
+        </is>
+      </c>
+    </row>
+    <row r="2549">
+      <c r="A2549" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2549" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2549" t="inlineStr">
+        <is>
+          <t>関東地方カスミ赤羽神谷店 2026年1月23日(金)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2549" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42132</t>
+        </is>
+      </c>
+    </row>
+    <row r="2550">
+      <c r="A2550" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2550" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2550" t="inlineStr">
+        <is>
+          <t>関東地方横須賀・若松町1丁目地区市街地再開発事業 2030年春開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2550" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47566</t>
+        </is>
+      </c>
+    </row>
+    <row r="2551">
+      <c r="A2551" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2551" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2551" t="inlineStr">
+        <is>
+          <t>中国地方ケーズデンキ山口店 2026年秋開業予定！最新情報も！山口県山口市にビッグ・エスの店舗「ケーズデンキ山口店」が2026年秋に開業予定！ケーズデンキの中では中～大型店舗となります。隣接地には「ウォンツ山口黒川店」も新設！そんな、ケーズデンキ山口店について、テナントや開業日などを見ていきましょう！...2026.10.06中国地方</t>
+        </is>
+      </c>
+      <c r="D2551" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/44477</t>
+        </is>
+      </c>
+    </row>
+    <row r="2552">
+      <c r="A2552" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2552" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2552" t="inlineStr">
+        <is>
+          <t>関西地方スーパーセンタートライアル愛知川店 2026年10月下旬に開業予定！最新情報も！滋賀県愛知郡にトライアルカンパニーの店舗「スーパーセンタートライアル愛知川店」が2026年10月下旬に開業予定！スーパーセンタートライアルが愛荘町に初出店！そんな、スーパーセンタートライアル愛知川店について、テナントや開業日などを見ていきま...2026.10.06関西地方</t>
+        </is>
+      </c>
+      <c r="D2552" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/47736</t>
+        </is>
+      </c>
+    </row>
+    <row r="2553">
+      <c r="A2553" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2553" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2553" t="inlineStr">
+        <is>
+          <t>イオンリテール／「そよら鳥取駅南」10月9日オープン、イオン鳥取店を全館リニューアル</t>
+        </is>
+      </c>
+      <c r="D2553" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100911.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2554">
+      <c r="A2554" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2554" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2554" t="inlineStr">
+        <is>
+          <t>イオンリテールほか／兵庫県三田市に「（仮称）そよら三田・サンフラワー（店舗面積7481m2）」27年4月27日新設</t>
+        </is>
+      </c>
+      <c r="D2554" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1009012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2555">
+      <c r="A2555" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2555" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2555" t="inlineStr">
+        <is>
+          <t>ユニクロ／東京都「世田谷千歳台店」10月23日リニューアル、新サービス充実</t>
+        </is>
+      </c>
+      <c r="D2555" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100980.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2556">
+      <c r="A2556" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2556" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2556" t="inlineStr">
+        <is>
+          <t>近鉄不動産／大阪上本町に商業・オフィス複合施設「上本町ネクサス」27年2月オープン</t>
+        </is>
+      </c>
+      <c r="D2556" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100976.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2557">
+      <c r="A2557" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2557" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2557" t="inlineStr">
+        <is>
+          <t>たかき、ウェディングエルティ／山形県東根市に「（仮称）東根一本木商業施設」27年3月31日新設</t>
+        </is>
+      </c>
+      <c r="D2557" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1009011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2558">
+      <c r="A2558" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2558" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2558" t="inlineStr">
+        <is>
+          <t>資さんうどん／群馬県に「倉賀野店」10月15日オープン、ガストを業態転換</t>
+        </is>
+      </c>
+      <c r="D2558" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100973.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2559">
+      <c r="A2559" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2559" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2559" t="inlineStr">
+        <is>
+          <t>ロイヤルHD／池袋のスパにハワイアン・アジアンレストラン10月16日オープン</t>
+        </is>
+      </c>
+      <c r="D2559" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100913.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2560">
+      <c r="A2560" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2560" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2560" t="inlineStr">
+        <is>
+          <t>ランディーズドーナツ／東京ソラマチにテイクアウト専門店10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D2560" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100975.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2561">
+      <c r="A2561" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2561" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2561" t="inlineStr">
+        <is>
+          <t>レインズ／さいたま市浦和区「しゃぶしゃぶ温野菜 浦和店」オープン</t>
+        </is>
+      </c>
+      <c r="D2561" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100978.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2562">
+      <c r="A2562" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2562" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2562" t="inlineStr">
+        <is>
+          <t>ヒマラヤ／愛知県「ヒマラヤスポーツ＆ゴルフ アピタ稲沢店」リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D2562" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100974.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2563">
+      <c r="A2563" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2563" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2563" t="inlineStr">
+        <is>
+          <t>ロピア／神戸市垂水区に「ブルメール舞多聞店」10月15日オープン</t>
+        </is>
+      </c>
+      <c r="D2563" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100813.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2564">
+      <c r="A2564" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2564" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2564" t="inlineStr">
+        <is>
+          <t>ふかや花園プレミアム・アウトレット／第2期増設で30店舗オープン、28年夏開業へ</t>
+        </is>
+      </c>
+      <c r="D2564" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100812.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2565">
+      <c r="A2565" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2565" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2565" t="inlineStr">
+        <is>
+          <t>三井不動産、野村不動産／「東京ミッドタウン日本橋」竣工、商業ゾーンは100区画2万m2</t>
+        </is>
+      </c>
+      <c r="D2565" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100872.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2566">
+      <c r="A2566" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2566" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2566" t="inlineStr">
+        <is>
+          <t>秋葉原UDX／商業ゾーン12月10日リニューアル、新規含む飲食27店舗オープン</t>
+        </is>
+      </c>
+      <c r="D2566" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100875.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2567">
+      <c r="A2567" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2567" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2567" t="inlineStr">
+        <is>
+          <t>AOKI／駅前型の新フォーマット店舗「川崎駅東口店」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2567" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100871.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2568">
+      <c r="A2568" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2568" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2568" t="inlineStr">
+        <is>
+          <t>グラニフ／京都に新旗艦店11月19日オープン、カフェ・アミューズメントエリア併設</t>
+        </is>
+      </c>
+      <c r="D2568" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100876.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2569">
+      <c r="A2569" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2569" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2569" t="inlineStr">
+        <is>
+          <t>マキヤ／静岡県裾野市に「（仮称）裾野複合店舗A棟・B棟」27年2月25日新設</t>
+        </is>
+      </c>
+      <c r="D2569" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1008012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2570">
+      <c r="A2570" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2570" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2570" t="inlineStr">
+        <is>
+          <t>コスモス薬品／岐阜県安八郡安八町に「ドラッグコスモス東結店」27年2月5日新設</t>
+        </is>
+      </c>
+      <c r="D2570" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1008011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2571">
+      <c r="A2571" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2571" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2571" t="inlineStr">
+        <is>
+          <t>あべのハルカス近鉄本店／洋菓子フロアの大規模リニューアル10月21日開始</t>
+        </is>
+      </c>
+      <c r="D2571" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100778.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2572">
+      <c r="A2572" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2572" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2572" t="inlineStr">
+        <is>
+          <t>ベイシア高萩モール店／「Beisia Foods Park」に10月9日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D2572" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100715.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-10
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2572"/>
+  <dimension ref="A1:D2644"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57000,6 +57000,1590 @@
         </is>
       </c>
     </row>
+    <row r="2573">
+      <c r="A2573" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2573" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2573" t="inlineStr">
+        <is>
+          <t>11/6移転 デリシアまめじま店</t>
+        </is>
+      </c>
+      <c r="D2573" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2574">
+      <c r="A2574" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2574" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2574" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D2574" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="2575">
+      <c r="A2575" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2575" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2575" t="inlineStr">
+        <is>
+          <t>10/8建替 ツルヤなぎさ店(長野県松本市)</t>
+        </is>
+      </c>
+      <c r="D2575" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="2576">
+      <c r="A2576" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2576" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2576" t="inlineStr">
+        <is>
+          <t>10/9そよら鳥取駅南</t>
+        </is>
+      </c>
+      <c r="D2576" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gyC</t>
+        </is>
+      </c>
+    </row>
+    <row r="2577">
+      <c r="A2577" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2577" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2577" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D2577" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="2578">
+      <c r="A2578" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2578" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2578" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D2578" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2579">
+      <c r="A2579" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2579" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2579" t="inlineStr">
+        <is>
+          <t>10/27やまのぶ赤池店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D2579" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1dGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2580">
+      <c r="A2580" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2580" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2580" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D2580" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="2581">
+      <c r="A2581" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2581" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2581" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D2581" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2582">
+      <c r="A2582" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2582" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2582" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D2582" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="2583">
+      <c r="A2583" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2583" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2583" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D2583" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2584">
+      <c r="A2584" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2584" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2584" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D2584" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="2585">
+      <c r="A2585" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2585" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2585" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2585" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2586">
+      <c r="A2586" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2586" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2586" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2586" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2587">
+      <c r="A2587" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2587" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2587" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2587" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2588">
+      <c r="A2588" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2588" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2588" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2588" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2589">
+      <c r="A2589" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2589" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2589" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2589" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2590">
+      <c r="A2590" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2590" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2590" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2590" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2591">
+      <c r="A2591" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2591" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2591" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2591" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2592">
+      <c r="A2592" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2592" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2592" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2592" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2593">
+      <c r="A2593" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2593" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2593" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2593" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2594">
+      <c r="A2594" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2594" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2594" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2594" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2595">
+      <c r="A2595" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2595" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2595" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2595" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2596">
+      <c r="A2596" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2596" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2596" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2596" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2597">
+      <c r="A2597" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2597" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2597" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2597" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2598">
+      <c r="A2598" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2598" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2598" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2598" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2599">
+      <c r="A2599" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2599" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2599" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2599" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2600">
+      <c r="A2600" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2600" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2600" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2600" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2601">
+      <c r="A2601" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2601" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2601" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2601" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2602">
+      <c r="A2602" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2602" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2602" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2602" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2603">
+      <c r="A2603" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2603" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2603" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2603" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2604">
+      <c r="A2604" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2604" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2604" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2604" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2605">
+      <c r="A2605" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2605" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2605" t="inlineStr">
+        <is>
+          <t>東北地方寒河江市にヨークベニマルの大型商業施設 2026年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2605" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/42945</t>
+        </is>
+      </c>
+    </row>
+    <row r="2606">
+      <c r="A2606" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2606" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2606" t="inlineStr">
+        <is>
+          <t>関東地方品川駅街区地区開発計画 2030年度より順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2606" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/33795</t>
+        </is>
+      </c>
+    </row>
+    <row r="2607">
+      <c r="A2607" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2607" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2607" t="inlineStr">
+        <is>
+          <t>九州地方九州大学箱崎キャンパス跡地地区 2028年度より街びらき！商業施設も誕生！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2607" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/46612</t>
+        </is>
+      </c>
+    </row>
+    <row r="2608">
+      <c r="A2608" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2608" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2608" t="inlineStr">
+        <is>
+          <t>関東地方平井テラス(プラウドタワー平井) 2025年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2608" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/19549</t>
+        </is>
+      </c>
+    </row>
+    <row r="2609">
+      <c r="A2609" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2609" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2609" t="inlineStr">
+        <is>
+          <t>中部地方ウオロク加茂店 2026年秋(11月頃)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2609" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48531</t>
+        </is>
+      </c>
+    </row>
+    <row r="2610">
+      <c r="A2610" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2610" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2610" t="inlineStr">
+        <is>
+          <t>中部地方イオンモール須坂 2025年10月3日(金)開業！全テナント166店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2610" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/11811</t>
+        </is>
+      </c>
+    </row>
+    <row r="2611">
+      <c r="A2611" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2611" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2611" t="inlineStr">
+        <is>
+          <t>関東地方追浜駅前第2街区市街地再開発事業 2029年11月完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2611" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/32533</t>
+        </is>
+      </c>
+    </row>
+    <row r="2612">
+      <c r="A2612" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2612" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2612" t="inlineStr">
+        <is>
+          <t>関東地方ブルーフロント芝浦 商業施設 2025年9月1日(月)11:00~開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2612" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/21848</t>
+        </is>
+      </c>
+    </row>
+    <row r="2613">
+      <c r="A2613" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2613" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2613" t="inlineStr">
+        <is>
+          <t>関西地方淀屋橋ゲートタワー 2026年7月9日(木)開業！どのような建物に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2613" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/26392</t>
+        </is>
+      </c>
+    </row>
+    <row r="2614">
+      <c r="A2614" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2614" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2614" t="inlineStr">
+        <is>
+          <t>関東地方品川駅西口地区 B-1地区再開発 2035年度開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2614" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49707</t>
+        </is>
+      </c>
+    </row>
+    <row r="2615">
+      <c r="A2615" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2615" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2615" t="inlineStr">
+        <is>
+          <t>関東地方コーナン江戸川船堀店 2025年12月10日(水)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2615" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42263</t>
+        </is>
+      </c>
+    </row>
+    <row r="2616">
+      <c r="A2616" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2616" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2616" t="inlineStr">
+        <is>
+          <t>東北地方スーパーセンタートライアル錦ケ丘店 2025年5月21日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2616" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/40364</t>
+        </is>
+      </c>
+    </row>
+    <row r="2617">
+      <c r="A2617" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2617" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2617" t="inlineStr">
+        <is>
+          <t>東北地方江釣子ショッピングセンター・パル 増床 2026年4月17日(金)開業！新規7テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2617" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/47925</t>
+        </is>
+      </c>
+    </row>
+    <row r="2618">
+      <c r="A2618" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2618" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2618" t="inlineStr">
+        <is>
+          <t>関東地方大宮駅西口第3-A･D地区市街地再開発事業 2031年以降開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2618" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/16908</t>
+        </is>
+      </c>
+    </row>
+    <row r="2619">
+      <c r="A2619" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2619" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2619" t="inlineStr">
+        <is>
+          <t>関西地方Kubota field(クボタフィールド) 2032年以降開業予定！クボタららアリーナや商業施設が誕生！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2619" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49228</t>
+        </is>
+      </c>
+    </row>
+    <row r="2620">
+      <c r="A2620" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2620" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2620" t="inlineStr">
+        <is>
+          <t>北海道地方札幌4丁目プレイス 4PLA 2025年4月25日(金)から順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2620" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/32449</t>
+        </is>
+      </c>
+    </row>
+    <row r="2621">
+      <c r="A2621" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2621" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2621" t="inlineStr">
+        <is>
+          <t>中国地方ケーズデンキ山口店 2026年秋開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2621" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/44477</t>
+        </is>
+      </c>
+    </row>
+    <row r="2622">
+      <c r="A2622" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2622" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2622" t="inlineStr">
+        <is>
+          <t>東北地方イオンモール郡山 フェスタ跡地 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2622" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/28173</t>
+        </is>
+      </c>
+    </row>
+    <row r="2623">
+      <c r="A2623" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2623" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2623" t="inlineStr">
+        <is>
+          <t>中部地方スーパーセンタートライアル名古屋みなと店 2027年2月上旬に開業予定！最新情報も！愛知県名古屋市港区にトライアルカンパニーの店舗「スーパーセンタートライアル名古屋みなと店」が2027年2月上旬に開業予定！スーパーセンタートライアルが名古屋市港区に2店舗目の出店！そんな、スーパーセンタートライアル名古屋みなと店について、テ...2026.10.10中部地方</t>
+        </is>
+      </c>
+      <c r="D2623" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48009</t>
+        </is>
+      </c>
+    </row>
+    <row r="2624">
+      <c r="A2624" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2624" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2624" t="inlineStr">
+        <is>
+          <t>関西地方スーパーセンタートライアル愛知川店 2026年10月下旬に開業予定！最新情報も！滋賀県愛知郡にトライアルカンパニーの店舗「スーパーセンタートライアル愛知川店」が2026年10月下旬に開業予定！スーパーセンタートライアルが愛荘町に初出店！そんな、スーパーセンタートライアル愛知川店について、テナントや開業日などを見ていきま...2026.10.06関西地方</t>
+        </is>
+      </c>
+      <c r="D2624" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/47736</t>
+        </is>
+      </c>
+    </row>
+    <row r="2625">
+      <c r="A2625" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2625" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2625" t="inlineStr">
+        <is>
+          <t>イオンリテール／「そよら鳥取駅南」10月9日オープン、イオン鳥取店を全館リニューアル</t>
+        </is>
+      </c>
+      <c r="D2625" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100911.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2626">
+      <c r="A2626" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2626" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2626" t="inlineStr">
+        <is>
+          <t>イオンリテールほか／兵庫県三田市に「（仮称）そよら三田・サンフラワー（店舗面積7481m2）」27年4月27日新設</t>
+        </is>
+      </c>
+      <c r="D2626" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1009012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2627">
+      <c r="A2627" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2627" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2627" t="inlineStr">
+        <is>
+          <t>ユニクロ／東京都「世田谷千歳台店」10月23日リニューアル、新サービス充実</t>
+        </is>
+      </c>
+      <c r="D2627" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100980.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2628">
+      <c r="A2628" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2628" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2628" t="inlineStr">
+        <is>
+          <t>近鉄不動産／大阪上本町に商業・オフィス複合施設「上本町ネクサス」27年2月オープン</t>
+        </is>
+      </c>
+      <c r="D2628" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100976.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2629">
+      <c r="A2629" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2629" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2629" t="inlineStr">
+        <is>
+          <t>たかき、ウェディングエルティ／山形県東根市に「（仮称）東根一本木商業施設」27年3月31日新設</t>
+        </is>
+      </c>
+      <c r="D2629" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1009011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2630">
+      <c r="A2630" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2630" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2630" t="inlineStr">
+        <is>
+          <t>資さんうどん／群馬県に「倉賀野店」10月15日オープン、ガストを業態転換</t>
+        </is>
+      </c>
+      <c r="D2630" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100973.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2631">
+      <c r="A2631" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2631" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2631" t="inlineStr">
+        <is>
+          <t>ロイヤルHD／池袋のスパにハワイアン・アジアンレストラン10月16日オープン</t>
+        </is>
+      </c>
+      <c r="D2631" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100913.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2632">
+      <c r="A2632" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2632" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2632" t="inlineStr">
+        <is>
+          <t>ランディーズドーナツ／東京ソラマチにテイクアウト専門店10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D2632" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100975.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2633">
+      <c r="A2633" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2633" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2633" t="inlineStr">
+        <is>
+          <t>レインズ／さいたま市浦和区「しゃぶしゃぶ温野菜 浦和店」オープン</t>
+        </is>
+      </c>
+      <c r="D2633" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100978.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2634">
+      <c r="A2634" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2634" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2634" t="inlineStr">
+        <is>
+          <t>ヒマラヤ／愛知県「ヒマラヤスポーツ＆ゴルフ アピタ稲沢店」リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D2634" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100974.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2635">
+      <c r="A2635" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2635" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2635" t="inlineStr">
+        <is>
+          <t>ロピア／神戸市垂水区に「ブルメール舞多聞店」10月15日オープン</t>
+        </is>
+      </c>
+      <c r="D2635" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100813.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2636">
+      <c r="A2636" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2636" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2636" t="inlineStr">
+        <is>
+          <t>ふかや花園プレミアム・アウトレット／第2期増設で30店舗オープン、28年夏開業へ</t>
+        </is>
+      </c>
+      <c r="D2636" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100812.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2637">
+      <c r="A2637" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2637" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2637" t="inlineStr">
+        <is>
+          <t>三井不動産、野村不動産／「東京ミッドタウン日本橋」竣工、商業ゾーンは100区画2万m2</t>
+        </is>
+      </c>
+      <c r="D2637" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100872.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2638">
+      <c r="A2638" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2638" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2638" t="inlineStr">
+        <is>
+          <t>秋葉原UDX／商業ゾーン12月10日リニューアル、新規含む飲食27店舗オープン</t>
+        </is>
+      </c>
+      <c r="D2638" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100875.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2639">
+      <c r="A2639" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2639" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2639" t="inlineStr">
+        <is>
+          <t>AOKI／駅前型の新フォーマット店舗「川崎駅東口店」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2639" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100871.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2640">
+      <c r="A2640" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2640" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2640" t="inlineStr">
+        <is>
+          <t>グラニフ／京都に新旗艦店11月19日オープン、カフェ・アミューズメントエリア併設</t>
+        </is>
+      </c>
+      <c r="D2640" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100876.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2641">
+      <c r="A2641" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2641" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2641" t="inlineStr">
+        <is>
+          <t>マキヤ／静岡県裾野市に「（仮称）裾野複合店舗A棟・B棟」27年2月25日新設</t>
+        </is>
+      </c>
+      <c r="D2641" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1008012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2642">
+      <c r="A2642" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2642" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2642" t="inlineStr">
+        <is>
+          <t>コスモス薬品／岐阜県安八郡安八町に「ドラッグコスモス東結店」27年2月5日新設</t>
+        </is>
+      </c>
+      <c r="D2642" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1008011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2643">
+      <c r="A2643" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2643" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2643" t="inlineStr">
+        <is>
+          <t>あべのハルカス近鉄本店／洋菓子フロアの大規模リニューアル10月21日開始</t>
+        </is>
+      </c>
+      <c r="D2643" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100778.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2644">
+      <c r="A2644" t="inlineStr">
+        <is>
+          <t>2026年10月10日</t>
+        </is>
+      </c>
+      <c r="B2644" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2644" t="inlineStr">
+        <is>
+          <t>ベイシア高萩モール店／「Beisia Foods Park」に10月9日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D2644" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100715.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-11
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2644"/>
+  <dimension ref="A1:D2720"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -58584,6 +58584,1678 @@
         </is>
       </c>
     </row>
+    <row r="2645">
+      <c r="A2645" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2645" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2645" t="inlineStr">
+        <is>
+          <t>10/15ロピア ブルメール舞多聞店</t>
+        </is>
+      </c>
+      <c r="D2645" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gBq</t>
+        </is>
+      </c>
+    </row>
+    <row r="2646">
+      <c r="A2646" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2646" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2646" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D2646" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="2647">
+      <c r="A2647" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2647" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2647" t="inlineStr">
+        <is>
+          <t>10/8建替 ツルヤなぎさ店(長野県松本市)</t>
+        </is>
+      </c>
+      <c r="D2647" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="2648">
+      <c r="A2648" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2648" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2648" t="inlineStr">
+        <is>
+          <t>10/9そよら鳥取駅南</t>
+        </is>
+      </c>
+      <c r="D2648" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gyC</t>
+        </is>
+      </c>
+    </row>
+    <row r="2649">
+      <c r="A2649" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2649" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2649" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D2649" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="2650">
+      <c r="A2650" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2650" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2650" t="inlineStr">
+        <is>
+          <t>10/22移転 業務スーパー天理店</t>
+        </is>
+      </c>
+      <c r="D2650" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gzx</t>
+        </is>
+      </c>
+    </row>
+    <row r="2651">
+      <c r="A2651" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2651" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2651" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D2651" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2652">
+      <c r="A2652" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2652" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2652" t="inlineStr">
+        <is>
+          <t>10/27やまのぶ赤池店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D2652" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1dGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2653">
+      <c r="A2653" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2653" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2653" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D2653" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="2654">
+      <c r="A2654" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2654" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2654" t="inlineStr">
+        <is>
+          <t>11/6移転 デリシアまめじま店</t>
+        </is>
+      </c>
+      <c r="D2654" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2655">
+      <c r="A2655" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2655" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2655" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D2655" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2656">
+      <c r="A2656" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2656" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2656" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D2656" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="2657">
+      <c r="A2657" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2657" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2657" t="inlineStr">
+        <is>
+          <t>12/3フェルナ武豊店(愛知県知多郡)</t>
+        </is>
+      </c>
+      <c r="D2657" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gBM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2658">
+      <c r="A2658" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2658" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2658" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D2658" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2659">
+      <c r="A2659" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2659" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2659" t="inlineStr">
+        <is>
+          <t>&lt;4/1予定&gt;(仮称)マックスバリュ豊橋西幸町店</t>
+        </is>
+      </c>
+      <c r="D2659" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gBH</t>
+        </is>
+      </c>
+    </row>
+    <row r="2660">
+      <c r="A2660" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2660" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2660" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D2660" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="2661">
+      <c r="A2661" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2661" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2661" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2661" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2662">
+      <c r="A2662" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2662" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2662" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2662" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2663">
+      <c r="A2663" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2663" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2663" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2663" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2664">
+      <c r="A2664" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2664" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2664" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2664" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2665">
+      <c r="A2665" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2665" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2665" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2665" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2666">
+      <c r="A2666" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2666" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2666" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2666" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2667">
+      <c r="A2667" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2667" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2667" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2667" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2668">
+      <c r="A2668" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2668" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2668" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2668" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2669">
+      <c r="A2669" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2669" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2669" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2669" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2670">
+      <c r="A2670" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2670" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2670" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2670" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2671">
+      <c r="A2671" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2671" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2671" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2671" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2672">
+      <c r="A2672" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2672" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2672" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2672" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2673">
+      <c r="A2673" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2673" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2673" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2673" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2674">
+      <c r="A2674" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2674" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2674" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2674" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2675">
+      <c r="A2675" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2675" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2675" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2675" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2676">
+      <c r="A2676" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2676" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2676" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2676" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2677">
+      <c r="A2677" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2677" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2677" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2677" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2678">
+      <c r="A2678" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2678" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2678" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2678" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2679">
+      <c r="A2679" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2679" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2679" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2679" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2680">
+      <c r="A2680" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2680" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2680" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2680" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2681">
+      <c r="A2681" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2681" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2681" t="inlineStr">
+        <is>
+          <t>関東地方赤羽一丁目第一地区市街地再開発事業 2029年度竣工！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2681" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36586</t>
+        </is>
+      </c>
+    </row>
+    <row r="2682">
+      <c r="A2682" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2682" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2682" t="inlineStr">
+        <is>
+          <t>関西地方京都城陽プレミアム・アウトレット 2028年以降開業！150店舗が出店予定！どのような商業施設に？</t>
+        </is>
+      </c>
+      <c r="D2682" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/10189</t>
+        </is>
+      </c>
+    </row>
+    <row r="2683">
+      <c r="A2683" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2683" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2683" t="inlineStr">
+        <is>
+          <t>中国地方ケーズデンキ山口店 2026年秋開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2683" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/44477</t>
+        </is>
+      </c>
+    </row>
+    <row r="2684">
+      <c r="A2684" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2684" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2684" t="inlineStr">
+        <is>
+          <t>東北地方イオンモール伊達 2026年11月27日(金)9：00~開業！どのような施設に？テナント情報随時更新中！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2684" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/17982</t>
+        </is>
+      </c>
+    </row>
+    <row r="2685">
+      <c r="A2685" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2685" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2685" t="inlineStr">
+        <is>
+          <t>中部地方デンソー池田工場跡地 日本エスコンが商業施設を計画！2027年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2685" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/39672</t>
+        </is>
+      </c>
+    </row>
+    <row r="2686">
+      <c r="A2686" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2686" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2686" t="inlineStr">
+        <is>
+          <t>関西地方(仮称)三条駅周辺プロジェクト 商業施設計画が2029年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2686" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/41582</t>
+        </is>
+      </c>
+    </row>
+    <row r="2687">
+      <c r="A2687" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2687" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2687" t="inlineStr">
+        <is>
+          <t>関東地方板橋駅西口地区市街地再開発事業 2029年10月完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2687" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26695</t>
+        </is>
+      </c>
+    </row>
+    <row r="2688">
+      <c r="A2688" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2688" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2688" t="inlineStr">
+        <is>
+          <t>関東地方イオン藤沢店 2026年1月末で一旦閉店し建て替えへ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2688" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/46012</t>
+        </is>
+      </c>
+    </row>
+    <row r="2689">
+      <c r="A2689" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2689" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2689" t="inlineStr">
+        <is>
+          <t>九州地方ケーズデンキ小倉東インター店 2026年7月2日(木)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2689" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/46276</t>
+        </is>
+      </c>
+    </row>
+    <row r="2690">
+      <c r="A2690" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2690" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2690" t="inlineStr">
+        <is>
+          <t>関東地方桜川ショッピングセンター(仮称) 2027年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2690" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/34191</t>
+        </is>
+      </c>
+    </row>
+    <row r="2691">
+      <c r="A2691" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2691" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2691" t="inlineStr">
+        <is>
+          <t>関東地方ヴィータモールせいせき 2025年10月31日(金)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2691" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/45333</t>
+        </is>
+      </c>
+    </row>
+    <row r="2692">
+      <c r="A2692" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2692" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2692" t="inlineStr">
+        <is>
+          <t>関東地方minanoba相模原（ミナノバ相模原） 2025年3月5日(水)開業！全11テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2692" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/35264</t>
+        </is>
+      </c>
+    </row>
+    <row r="2693">
+      <c r="A2693" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2693" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2693" t="inlineStr">
+        <is>
+          <t>関東地方まえばし赤城モール 2026年秋開業！カインズや劇安ワンダーランド ココトク！出店 テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2693" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/38254</t>
+        </is>
+      </c>
+    </row>
+    <row r="2694">
+      <c r="A2694" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2694" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2694" t="inlineStr">
+        <is>
+          <t>関西地方ライフ大仙店・ケーズデンキ堺大仙店 2026年11月開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2694" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/48721</t>
+        </is>
+      </c>
+    </row>
+    <row r="2695">
+      <c r="A2695" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2695" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2695" t="inlineStr">
+        <is>
+          <t>関東地方京王プラザホテル多摩 跡地 分譲マンションと商業施設 2028年度開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2695" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/35148</t>
+        </is>
+      </c>
+    </row>
+    <row r="2696">
+      <c r="A2696" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2696" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2696" t="inlineStr">
+        <is>
+          <t>九州地方西日本シティビル 2026年7月21日(火)開業！全5テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2696" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/20689</t>
+        </is>
+      </c>
+    </row>
+    <row r="2697">
+      <c r="A2697" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2697" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2697" t="inlineStr">
+        <is>
+          <t>関東地方生鮮市場TOP栃木合戦場店 2026年8月1日(土)8時~開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2697" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47134</t>
+        </is>
+      </c>
+    </row>
+    <row r="2698">
+      <c r="A2698" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2698" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2698" t="inlineStr">
+        <is>
+          <t>関東地方新綱島MICCA 2026年10月28日(水)開業！全21テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2698" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49470</t>
+        </is>
+      </c>
+    </row>
+    <row r="2699">
+      <c r="A2699" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2699" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2699" t="inlineStr">
+        <is>
+          <t>中部地方スーパーセンタートライアル名古屋みなと店 2027年2月上旬に開業予定！最新情報も！愛知県名古屋市港区にトライアルカンパニーの店舗「スーパーセンタートライアル名古屋みなと店」が2027年2月上旬に開業予定！スーパーセンタートライアルが名古屋市港区に2店舗目の出店！そんな、スーパーセンタートライアル名古屋みなと店について、テ...2026.10.10中部地方</t>
+        </is>
+      </c>
+      <c r="D2699" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48009</t>
+        </is>
+      </c>
+    </row>
+    <row r="2700">
+      <c r="A2700" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2700" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2700" t="inlineStr">
+        <is>
+          <t>関西地方スーパーセンタートライアル愛知川店 2026年10月下旬に開業予定！最新情報も！滋賀県愛知郡にトライアルカンパニーの店舗「スーパーセンタートライアル愛知川店」が2026年10月下旬に開業予定！スーパーセンタートライアルが愛荘町に初出店！そんな、スーパーセンタートライアル愛知川店について、テナントや開業日などを見ていきま...2026.10.06関西地方</t>
+        </is>
+      </c>
+      <c r="D2700" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/47736</t>
+        </is>
+      </c>
+    </row>
+    <row r="2701">
+      <c r="A2701" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2701" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2701" t="inlineStr">
+        <is>
+          <t>イオンリテール／「そよら鳥取駅南」10月9日オープン、イオン鳥取店を全館リニューアル</t>
+        </is>
+      </c>
+      <c r="D2701" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100911.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2702">
+      <c r="A2702" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2702" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2702" t="inlineStr">
+        <is>
+          <t>イオンリテールほか／兵庫県三田市に「（仮称）そよら三田・サンフラワー（店舗面積7481m2）」27年4月27日新設</t>
+        </is>
+      </c>
+      <c r="D2702" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1009012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2703">
+      <c r="A2703" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2703" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2703" t="inlineStr">
+        <is>
+          <t>ユニクロ／東京都「世田谷千歳台店」10月23日リニューアル、新サービス充実</t>
+        </is>
+      </c>
+      <c r="D2703" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100980.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2704">
+      <c r="A2704" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2704" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2704" t="inlineStr">
+        <is>
+          <t>近鉄不動産／大阪上本町に商業・オフィス複合施設「上本町ネクサス」27年2月オープン</t>
+        </is>
+      </c>
+      <c r="D2704" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100976.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2705">
+      <c r="A2705" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2705" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2705" t="inlineStr">
+        <is>
+          <t>たかき、ウェディングエルティ／山形県東根市に「（仮称）東根一本木商業施設」27年3月31日新設</t>
+        </is>
+      </c>
+      <c r="D2705" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1009011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2706">
+      <c r="A2706" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2706" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2706" t="inlineStr">
+        <is>
+          <t>資さんうどん／群馬県に「倉賀野店」10月15日オープン、ガストを業態転換</t>
+        </is>
+      </c>
+      <c r="D2706" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100973.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2707">
+      <c r="A2707" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2707" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2707" t="inlineStr">
+        <is>
+          <t>ロイヤルHD／池袋のスパにハワイアン・アジアンレストラン10月16日オープン</t>
+        </is>
+      </c>
+      <c r="D2707" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100913.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2708">
+      <c r="A2708" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2708" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2708" t="inlineStr">
+        <is>
+          <t>ランディーズドーナツ／東京ソラマチにテイクアウト専門店10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D2708" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100975.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2709">
+      <c r="A2709" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2709" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2709" t="inlineStr">
+        <is>
+          <t>レインズ／さいたま市浦和区「しゃぶしゃぶ温野菜 浦和店」オープン</t>
+        </is>
+      </c>
+      <c r="D2709" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100978.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2710">
+      <c r="A2710" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2710" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2710" t="inlineStr">
+        <is>
+          <t>ヒマラヤ／愛知県「ヒマラヤスポーツ＆ゴルフ アピタ稲沢店」リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D2710" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100974.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2711">
+      <c r="A2711" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2711" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2711" t="inlineStr">
+        <is>
+          <t>ロピア／神戸市垂水区に「ブルメール舞多聞店」10月15日オープン</t>
+        </is>
+      </c>
+      <c r="D2711" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100813.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2712">
+      <c r="A2712" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2712" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2712" t="inlineStr">
+        <is>
+          <t>ふかや花園プレミアム・アウトレット／第2期増設で30店舗オープン、28年夏開業へ</t>
+        </is>
+      </c>
+      <c r="D2712" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100812.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2713">
+      <c r="A2713" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2713" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2713" t="inlineStr">
+        <is>
+          <t>三井不動産、野村不動産／「東京ミッドタウン日本橋」竣工、商業ゾーンは100区画2万m2</t>
+        </is>
+      </c>
+      <c r="D2713" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100872.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2714">
+      <c r="A2714" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2714" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2714" t="inlineStr">
+        <is>
+          <t>秋葉原UDX／商業ゾーン12月10日リニューアル、新規含む飲食27店舗オープン</t>
+        </is>
+      </c>
+      <c r="D2714" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100875.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2715">
+      <c r="A2715" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2715" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2715" t="inlineStr">
+        <is>
+          <t>AOKI／駅前型の新フォーマット店舗「川崎駅東口店」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2715" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100871.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2716">
+      <c r="A2716" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2716" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2716" t="inlineStr">
+        <is>
+          <t>グラニフ／京都に新旗艦店11月19日オープン、カフェ・アミューズメントエリア併設</t>
+        </is>
+      </c>
+      <c r="D2716" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100876.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2717">
+      <c r="A2717" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2717" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2717" t="inlineStr">
+        <is>
+          <t>マキヤ／静岡県裾野市に「（仮称）裾野複合店舗A棟・B棟」27年2月25日新設</t>
+        </is>
+      </c>
+      <c r="D2717" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1008012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2718">
+      <c r="A2718" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2718" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2718" t="inlineStr">
+        <is>
+          <t>コスモス薬品／岐阜県安八郡安八町に「ドラッグコスモス東結店」27年2月5日新設</t>
+        </is>
+      </c>
+      <c r="D2718" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1008011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2719">
+      <c r="A2719" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2719" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2719" t="inlineStr">
+        <is>
+          <t>あべのハルカス近鉄本店／洋菓子フロアの大規模リニューアル10月21日開始</t>
+        </is>
+      </c>
+      <c r="D2719" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100778.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2720">
+      <c r="A2720" t="inlineStr">
+        <is>
+          <t>2026年10月11日</t>
+        </is>
+      </c>
+      <c r="B2720" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2720" t="inlineStr">
+        <is>
+          <t>ベイシア高萩モール店／「Beisia Foods Park」に10月9日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D2720" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100715.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-12
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2720"/>
+  <dimension ref="A1:D2797"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -60256,6 +60256,1700 @@
         </is>
       </c>
     </row>
+    <row r="2721">
+      <c r="A2721" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2721" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2721" t="inlineStr">
+        <is>
+          <t>12/3フェルナ武豊店 (カネスエ,愛知県知多郡)</t>
+        </is>
+      </c>
+      <c r="D2721" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gBM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2722">
+      <c r="A2722" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2722" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2722" t="inlineStr">
+        <is>
+          <t>2027/6/1炭焼きレストランさわやか イオンセントラルスクエア静岡店</t>
+        </is>
+      </c>
+      <c r="D2722" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gCI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2723">
+      <c r="A2723" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2723" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2723" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D2723" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="2724">
+      <c r="A2724" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2724" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2724" t="inlineStr">
+        <is>
+          <t>10/8建替 ツルヤなぎさ店(長野県松本市)</t>
+        </is>
+      </c>
+      <c r="D2724" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="2725">
+      <c r="A2725" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2725" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2725" t="inlineStr">
+        <is>
+          <t>10/9そよら鳥取駅南</t>
+        </is>
+      </c>
+      <c r="D2725" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gyC</t>
+        </is>
+      </c>
+    </row>
+    <row r="2726">
+      <c r="A2726" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2726" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2726" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D2726" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="2727">
+      <c r="A2727" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2727" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2727" t="inlineStr">
+        <is>
+          <t>10/15ロピア ブルメール舞多聞店</t>
+        </is>
+      </c>
+      <c r="D2727" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gBq</t>
+        </is>
+      </c>
+    </row>
+    <row r="2728">
+      <c r="A2728" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2728" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2728" t="inlineStr">
+        <is>
+          <t>10/22移転 業務スーパー天理店</t>
+        </is>
+      </c>
+      <c r="D2728" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gzx</t>
+        </is>
+      </c>
+    </row>
+    <row r="2729">
+      <c r="A2729" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2729" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2729" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D2729" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2730">
+      <c r="A2730" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2730" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2730" t="inlineStr">
+        <is>
+          <t>10/27やまのぶ赤池店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D2730" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1dGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2731">
+      <c r="A2731" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2731" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2731" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D2731" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="2732">
+      <c r="A2732" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2732" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2732" t="inlineStr">
+        <is>
+          <t>11/6移転 デリシアまめじま店</t>
+        </is>
+      </c>
+      <c r="D2732" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2733">
+      <c r="A2733" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2733" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2733" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D2733" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2734">
+      <c r="A2734" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2734" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2734" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D2734" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="2735">
+      <c r="A2735" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2735" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2735" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D2735" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2736">
+      <c r="A2736" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2736" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2736" t="inlineStr">
+        <is>
+          <t>&lt;4/1予定&gt;(仮称)マックスバリュ豊橋西幸町店</t>
+        </is>
+      </c>
+      <c r="D2736" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gBH</t>
+        </is>
+      </c>
+    </row>
+    <row r="2737">
+      <c r="A2737" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2737" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2737" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D2737" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="2738">
+      <c r="A2738" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2738" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2738" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2738" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2739">
+      <c r="A2739" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2739" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2739" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2739" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2740">
+      <c r="A2740" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2740" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2740" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2740" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2741">
+      <c r="A2741" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2741" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2741" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2741" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2742">
+      <c r="A2742" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2742" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2742" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2742" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2743">
+      <c r="A2743" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2743" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2743" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2743" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2744">
+      <c r="A2744" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2744" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2744" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2744" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2745">
+      <c r="A2745" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2745" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2745" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2745" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2746">
+      <c r="A2746" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2746" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2746" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2746" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2747">
+      <c r="A2747" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2747" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2747" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2747" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2748">
+      <c r="A2748" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2748" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2748" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2748" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2749">
+      <c r="A2749" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2749" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2749" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2749" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2750">
+      <c r="A2750" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2750" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2750" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2750" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2751">
+      <c r="A2751" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2751" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2751" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2751" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2752">
+      <c r="A2752" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2752" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2752" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2752" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2753">
+      <c r="A2753" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2753" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2753" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2753" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2754">
+      <c r="A2754" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2754" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2754" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2754" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2755">
+      <c r="A2755" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2755" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2755" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2755" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2756">
+      <c r="A2756" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2756" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2756" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2756" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2757">
+      <c r="A2757" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2757" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2757" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2757" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2758">
+      <c r="A2758" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2758" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2758" t="inlineStr">
+        <is>
+          <t>関西地方グラングリーン大阪 2025年3月21日(金)南館開業！テナントは？どのような街に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2758" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/4448</t>
+        </is>
+      </c>
+    </row>
+    <row r="2759">
+      <c r="A2759" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2759" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2759" t="inlineStr">
+        <is>
+          <t>関東地方武蔵村山商業施設計画 2026年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2759" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/39426</t>
+        </is>
+      </c>
+    </row>
+    <row r="2760">
+      <c r="A2760" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2760" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2760" t="inlineStr">
+        <is>
+          <t>関東地方JR小岩駅北口地区再開発事業 2027年春完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2760" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/20970</t>
+        </is>
+      </c>
+    </row>
+    <row r="2761">
+      <c r="A2761" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2761" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2761" t="inlineStr">
+        <is>
+          <t>関東地方伊勢崎境ショッピングパーク 2027年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2761" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47294</t>
+        </is>
+      </c>
+    </row>
+    <row r="2762">
+      <c r="A2762" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2762" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2762" t="inlineStr">
+        <is>
+          <t>関東地方ビバタウン沼田再開発 ベルクが出店 2025年7月23日(水)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2762" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/40309</t>
+        </is>
+      </c>
+    </row>
+    <row r="2763">
+      <c r="A2763" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2763" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2763" t="inlineStr">
+        <is>
+          <t>関東地方品川駅西口地区 B-1地区再開発 2035年度開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2763" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49707</t>
+        </is>
+      </c>
+    </row>
+    <row r="2764">
+      <c r="A2764" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2764" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2764" t="inlineStr">
+        <is>
+          <t>関東地方新綱島MICCA 2026年10月28日(水)開業！全21テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2764" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49470</t>
+        </is>
+      </c>
+    </row>
+    <row r="2765">
+      <c r="A2765" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2765" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2765" t="inlineStr">
+        <is>
+          <t>中国地方マルアイ川西店 複合商業施設が開業！2027年冬開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2765" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/44825</t>
+        </is>
+      </c>
+    </row>
+    <row r="2766">
+      <c r="A2766" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2766" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2766" t="inlineStr">
+        <is>
+          <t>九州地方アクロスプラザ篠栗 2025年春グランドオープン！全10テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2766" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/38349</t>
+        </is>
+      </c>
+    </row>
+    <row r="2767">
+      <c r="A2767" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2767" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2767" t="inlineStr">
+        <is>
+          <t>東北地方イオンタウン 福島市南矢野目に進出！2028年10月開業！ テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2767" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/38134</t>
+        </is>
+      </c>
+    </row>
+    <row r="2768">
+      <c r="A2768" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2768" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2768" t="inlineStr">
+        <is>
+          <t>北海道地方フレスポ旭川龍谷 2025年10月30日(木)~順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2768" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/32723</t>
+        </is>
+      </c>
+    </row>
+    <row r="2769">
+      <c r="A2769" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2769" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2769" t="inlineStr">
+        <is>
+          <t>関東地方竹ノ塚駅東口地区市街地再開発事業 2035年以降開業！どのような施設になる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2769" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48886</t>
+        </is>
+      </c>
+    </row>
+    <row r="2770">
+      <c r="A2770" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2770" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2770" t="inlineStr">
+        <is>
+          <t>中国地方ニトリ岡山南店 2026年1月23日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2770" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/44181</t>
+        </is>
+      </c>
+    </row>
+    <row r="2771">
+      <c r="A2771" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2771" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2771" t="inlineStr">
+        <is>
+          <t>関西地方アイユータウン マルアイ長田店 2025年9月17日(水)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2771" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/42358</t>
+        </is>
+      </c>
+    </row>
+    <row r="2772">
+      <c r="A2772" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2772" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2772" t="inlineStr">
+        <is>
+          <t>関東地方門前仲町駅前地区市街地再開発事業 2031年度完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2772" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49704</t>
+        </is>
+      </c>
+    </row>
+    <row r="2773">
+      <c r="A2773" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2773" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2773" t="inlineStr">
+        <is>
+          <t>関東地方松戸駅 新駅ビルに商業施設 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2773" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/29225</t>
+        </is>
+      </c>
+    </row>
+    <row r="2774">
+      <c r="A2774" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2774" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2774" t="inlineStr">
+        <is>
+          <t>関東地方鎌倉梶原商業施設 2026年8月28日(金)より順次開業！ライフやカインズが出店！全4店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2774" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/43953</t>
+        </is>
+      </c>
+    </row>
+    <row r="2775">
+      <c r="A2775" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2775" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2775" t="inlineStr">
+        <is>
+          <t>関東地方西新宿三丁目西地区市街地再開発事業 2035年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2775" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26862</t>
+        </is>
+      </c>
+    </row>
+    <row r="2776">
+      <c r="A2776" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2776" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2776" t="inlineStr">
+        <is>
+          <t>中部地方スーパーセンタートライアル名古屋みなと店 2027年2月上旬に開業予定！最新情報も！愛知県名古屋市港区にトライアルカンパニーの店舗「スーパーセンタートライアル名古屋みなと店」が2027年2月上旬に開業予定！スーパーセンタートライアルが名古屋市港区に2店舗目の出店！そんな、スーパーセンタートライアル名古屋みなと店について、テ...2026.10.10中部地方</t>
+        </is>
+      </c>
+      <c r="D2776" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48009</t>
+        </is>
+      </c>
+    </row>
+    <row r="2777">
+      <c r="A2777" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2777" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2777" t="inlineStr">
+        <is>
+          <t>中国地方ケーズデンキ山口店 2026年秋開業予定！最新情報も！山口県山口市にビッグ・エスの店舗「ケーズデンキ山口店」が2026年秋に開業予定！ケーズデンキの中では中～大型店舗となります。隣接地には「ウォンツ山口黒川店」も新設！そんな、ケーズデンキ山口店について、テナントや開業日などを見ていきましょう！...2026.10.06中国地方</t>
+        </is>
+      </c>
+      <c r="D2777" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/44477</t>
+        </is>
+      </c>
+    </row>
+    <row r="2778">
+      <c r="A2778" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2778" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2778" t="inlineStr">
+        <is>
+          <t>イオンリテール／「そよら鳥取駅南」10月9日オープン、イオン鳥取店を全館リニューアル</t>
+        </is>
+      </c>
+      <c r="D2778" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100911.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2779">
+      <c r="A2779" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2779" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2779" t="inlineStr">
+        <is>
+          <t>イオンリテールほか／兵庫県三田市に「（仮称）そよら三田・サンフラワー（店舗面積7481m2）」27年4月27日新設</t>
+        </is>
+      </c>
+      <c r="D2779" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1009012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2780">
+      <c r="A2780" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2780" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2780" t="inlineStr">
+        <is>
+          <t>ユニクロ／東京都「世田谷千歳台店」10月23日リニューアル、新サービス充実</t>
+        </is>
+      </c>
+      <c r="D2780" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100980.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2781">
+      <c r="A2781" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2781" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2781" t="inlineStr">
+        <is>
+          <t>近鉄不動産／大阪上本町に商業・オフィス複合施設「上本町ネクサス」27年2月オープン</t>
+        </is>
+      </c>
+      <c r="D2781" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100976.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2782">
+      <c r="A2782" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2782" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2782" t="inlineStr">
+        <is>
+          <t>たかき、ウェディングエルティ／山形県東根市に「（仮称）東根一本木商業施設」27年3月31日新設</t>
+        </is>
+      </c>
+      <c r="D2782" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1009011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2783">
+      <c r="A2783" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2783" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2783" t="inlineStr">
+        <is>
+          <t>資さんうどん／群馬県に「倉賀野店」10月15日オープン、ガストを業態転換</t>
+        </is>
+      </c>
+      <c r="D2783" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100973.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2784">
+      <c r="A2784" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2784" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2784" t="inlineStr">
+        <is>
+          <t>ロイヤルHD／池袋のスパにハワイアン・アジアンレストラン10月16日オープン</t>
+        </is>
+      </c>
+      <c r="D2784" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100913.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2785">
+      <c r="A2785" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2785" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2785" t="inlineStr">
+        <is>
+          <t>ランディーズドーナツ／東京ソラマチにテイクアウト専門店10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D2785" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100975.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2786">
+      <c r="A2786" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2786" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2786" t="inlineStr">
+        <is>
+          <t>レインズ／さいたま市浦和区「しゃぶしゃぶ温野菜 浦和店」オープン</t>
+        </is>
+      </c>
+      <c r="D2786" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100978.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2787">
+      <c r="A2787" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2787" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2787" t="inlineStr">
+        <is>
+          <t>ヒマラヤ／愛知県「ヒマラヤスポーツ＆ゴルフ アピタ稲沢店」リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D2787" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100974.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2788">
+      <c r="A2788" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2788" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2788" t="inlineStr">
+        <is>
+          <t>ロピア／神戸市垂水区に「ブルメール舞多聞店」10月15日オープン</t>
+        </is>
+      </c>
+      <c r="D2788" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100813.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2789">
+      <c r="A2789" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2789" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2789" t="inlineStr">
+        <is>
+          <t>ふかや花園プレミアム・アウトレット／第2期増設で30店舗オープン、28年夏開業へ</t>
+        </is>
+      </c>
+      <c r="D2789" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100812.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2790">
+      <c r="A2790" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2790" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2790" t="inlineStr">
+        <is>
+          <t>三井不動産、野村不動産／「東京ミッドタウン日本橋」竣工、商業ゾーンは100区画2万m2</t>
+        </is>
+      </c>
+      <c r="D2790" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100872.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2791">
+      <c r="A2791" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2791" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2791" t="inlineStr">
+        <is>
+          <t>秋葉原UDX／商業ゾーン12月10日リニューアル、新規含む飲食27店舗オープン</t>
+        </is>
+      </c>
+      <c r="D2791" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100875.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2792">
+      <c r="A2792" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2792" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2792" t="inlineStr">
+        <is>
+          <t>AOKI／駅前型の新フォーマット店舗「川崎駅東口店」10月9日オープン</t>
+        </is>
+      </c>
+      <c r="D2792" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100871.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2793">
+      <c r="A2793" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2793" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2793" t="inlineStr">
+        <is>
+          <t>グラニフ／京都に新旗艦店11月19日オープン、カフェ・アミューズメントエリア併設</t>
+        </is>
+      </c>
+      <c r="D2793" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100876.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2794">
+      <c r="A2794" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2794" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2794" t="inlineStr">
+        <is>
+          <t>マキヤ／静岡県裾野市に「（仮称）裾野複合店舗A棟・B棟」27年2月25日新設</t>
+        </is>
+      </c>
+      <c r="D2794" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1008012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2795">
+      <c r="A2795" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2795" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2795" t="inlineStr">
+        <is>
+          <t>コスモス薬品／岐阜県安八郡安八町に「ドラッグコスモス東結店」27年2月5日新設</t>
+        </is>
+      </c>
+      <c r="D2795" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1008011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2796">
+      <c r="A2796" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2796" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2796" t="inlineStr">
+        <is>
+          <t>あべのハルカス近鉄本店／洋菓子フロアの大規模リニューアル10月21日開始</t>
+        </is>
+      </c>
+      <c r="D2796" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100778.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2797">
+      <c r="A2797" t="inlineStr">
+        <is>
+          <t>2026年10月13日</t>
+        </is>
+      </c>
+      <c r="B2797" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2797" t="inlineStr">
+        <is>
+          <t>ベイシア高萩モール店／「Beisia Foods Park」に10月9日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D2797" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100715.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-13
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2797"/>
+  <dimension ref="A1:D2857"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61950,6 +61950,1326 @@
         </is>
       </c>
     </row>
+    <row r="2798">
+      <c r="A2798" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2798" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2798" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2798" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2799">
+      <c r="A2799" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2799" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2799" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2799" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2800">
+      <c r="A2800" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2800" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2800" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2800" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2801">
+      <c r="A2801" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2801" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2801" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2801" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2802">
+      <c r="A2802" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2802" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2802" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2802" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2803">
+      <c r="A2803" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2803" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2803" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2803" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2804">
+      <c r="A2804" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2804" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2804" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2804" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2805">
+      <c r="A2805" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2805" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2805" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2805" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2806">
+      <c r="A2806" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2806" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2806" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2806" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2807">
+      <c r="A2807" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2807" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2807" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2807" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2808">
+      <c r="A2808" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2808" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2808" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2808" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2809">
+      <c r="A2809" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2809" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2809" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2809" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2810">
+      <c r="A2810" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2810" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2810" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2810" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2811">
+      <c r="A2811" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2811" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2811" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2811" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2812">
+      <c r="A2812" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2812" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2812" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2812" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2813">
+      <c r="A2813" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2813" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2813" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2813" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2814">
+      <c r="A2814" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2814" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2814" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2814" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2815">
+      <c r="A2815" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2815" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2815" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2815" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2816">
+      <c r="A2816" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2816" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2816" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2816" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2817">
+      <c r="A2817" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2817" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2817" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2817" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2818">
+      <c r="A2818" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2818" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2818" t="inlineStr">
+        <is>
+          <t>関東地方W シティタワーズ 蕨駅西口地区市街地再開発事業 2027年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2818" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/16952</t>
+        </is>
+      </c>
+    </row>
+    <row r="2819">
+      <c r="A2819" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2819" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2819" t="inlineStr">
+        <is>
+          <t>九州地方天神ビジネスセンターII 2026年8月4日(火)開業！全16テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2819" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/41150</t>
+        </is>
+      </c>
+    </row>
+    <row r="2820">
+      <c r="A2820" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2820" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2820" t="inlineStr">
+        <is>
+          <t>関東地方イオン石岡店が建て替えへ！2028年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2820" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/45661</t>
+        </is>
+      </c>
+    </row>
+    <row r="2821">
+      <c r="A2821" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2821" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2821" t="inlineStr">
+        <is>
+          <t>中国地方ケーズデンキ山口店 2026年秋開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2821" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/44477</t>
+        </is>
+      </c>
+    </row>
+    <row r="2822">
+      <c r="A2822" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2822" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2822" t="inlineStr">
+        <is>
+          <t>中部地方ベルク町田相原店 2026年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2822" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/47130</t>
+        </is>
+      </c>
+    </row>
+    <row r="2823">
+      <c r="A2823" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2823" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2823" t="inlineStr">
+        <is>
+          <t>関東地方セントラルガーデン月島 ザ タワー 2028年春完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2823" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26835</t>
+        </is>
+      </c>
+    </row>
+    <row r="2824">
+      <c r="A2824" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2824" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2824" t="inlineStr">
+        <is>
+          <t>関東地方グランドシティタワー月島 2026年6月より順次開業！月島WESTのテナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2824" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/23131</t>
+        </is>
+      </c>
+    </row>
+    <row r="2825">
+      <c r="A2825" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2825" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2825" t="inlineStr">
+        <is>
+          <t>中部地方イオンタウン岐阜北方 2026年3月27日(金)開業！全24テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2825" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/16776</t>
+        </is>
+      </c>
+    </row>
+    <row r="2826">
+      <c r="A2826" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2826" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2826" t="inlineStr">
+        <is>
+          <t>関東地方つくば学園南プロジェクト 2029年春完成！商業施設誕生！カスミが進出 最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2826" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36105</t>
+        </is>
+      </c>
+    </row>
+    <row r="2827">
+      <c r="A2827" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2827" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2827" t="inlineStr">
+        <is>
+          <t>関東地方豊洲セイルパーク 2025年7月24日~順次開業！全21テナント一覧 最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2827" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/18680</t>
+        </is>
+      </c>
+    </row>
+    <row r="2828">
+      <c r="A2828" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2828" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2828" t="inlineStr">
+        <is>
+          <t>関東地方習志野市旧庁舎跡地にベルク・フォルテが出店！2028年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2828" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/43905</t>
+        </is>
+      </c>
+    </row>
+    <row r="2829">
+      <c r="A2829" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2829" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2829" t="inlineStr">
+        <is>
+          <t>関東地方京王プラザホテル多摩 跡地 分譲マンションと商業施設 2028年度開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2829" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/35148</t>
+        </is>
+      </c>
+    </row>
+    <row r="2830">
+      <c r="A2830" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2830" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2830" t="inlineStr">
+        <is>
+          <t>中部地方アークスクエア須坂 ホームセンタームサシ・ヤマダデンキ 2025年8月6日(水)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2830" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/21807</t>
+        </is>
+      </c>
+    </row>
+    <row r="2831">
+      <c r="A2831" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2831" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2831" t="inlineStr">
+        <is>
+          <t>中部地方ロピアモール滝ノ水 2026年5月21日(木)開業！全7テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2831" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48558</t>
+        </is>
+      </c>
+    </row>
+    <row r="2832">
+      <c r="A2832" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2832" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2832" t="inlineStr">
+        <is>
+          <t>関東地方ヤオコー岩槻本丸店 2025年10月29日(水)9時~開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2832" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/39888</t>
+        </is>
+      </c>
+    </row>
+    <row r="2833">
+      <c r="A2833" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2833" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2833" t="inlineStr">
+        <is>
+          <t>関東地方スーパーセンタートライアル山武成東店 2026年5月20日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2833" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/46150</t>
+        </is>
+      </c>
+    </row>
+    <row r="2834">
+      <c r="A2834" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2834" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2834" t="inlineStr">
+        <is>
+          <t>関東地方コトエ橋本 2026年5月29日(金)開業！全21テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2834" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/41085</t>
+        </is>
+      </c>
+    </row>
+    <row r="2835">
+      <c r="A2835" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2835" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2835" t="inlineStr">
+        <is>
+          <t>関東地方王子駅前地区市街地再開発事業 2034年度開業予定！商業施設も誕生！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2835" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47579</t>
+        </is>
+      </c>
+    </row>
+    <row r="2836">
+      <c r="A2836" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2836" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2836" t="inlineStr">
+        <is>
+          <t>中部地方スーパーセンタートライアル名古屋みなと店 2027年2月上旬に開業予定！最新情報も！愛知県名古屋市港区にトライアルカンパニーの店舗「スーパーセンタートライアル名古屋みなと店」が2027年2月上旬に開業予定！スーパーセンタートライアルが名古屋市港区に2店舗目の出店！そんな、スーパーセンタートライアル名古屋みなと店について、テ...2026.10.10中部地方</t>
+        </is>
+      </c>
+      <c r="D2836" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48009</t>
+        </is>
+      </c>
+    </row>
+    <row r="2837">
+      <c r="A2837" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2837" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2837" t="inlineStr">
+        <is>
+          <t>関西地方スーパーセンタートライアル愛知川店 2026年10月下旬に開業予定！最新情報も！滋賀県愛知郡にトライアルカンパニーの店舗「スーパーセンタートライアル愛知川店」が2026年10月下旬に開業予定！スーパーセンタートライアルが愛荘町に初出店！そんな、スーパーセンタートライアル愛知川店について、テナントや開業日などを見ていきま...2026.10.06関西地方</t>
+        </is>
+      </c>
+      <c r="D2837" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/47736</t>
+        </is>
+      </c>
+    </row>
+    <row r="2838">
+      <c r="A2838" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2838" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2838" t="inlineStr">
+        <is>
+          <t>三井不動産ほか／東京都足立区の大規模複合開発「アクアゲート千住大川端」30年1期竣工</t>
+        </is>
+      </c>
+      <c r="D2838" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101376.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2839">
+      <c r="A2839" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2839" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2839" t="inlineStr">
+        <is>
+          <t>三菱商事都市開発×奥村組／大阪に商業施設、ライフ・ヤマダデンキが27年春オープン</t>
+        </is>
+      </c>
+      <c r="D2839" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101315.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2840">
+      <c r="A2840" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2840" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2840" t="inlineStr">
+        <is>
+          <t>イオンリテール／兵庫県小野市に「（仮称）そよら小野（店舗面積1万360m2）」27年4月1日新設</t>
+        </is>
+      </c>
+      <c r="D2840" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1013011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2841">
+      <c r="A2841" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2841" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2841" t="inlineStr">
+        <is>
+          <t>大丸梅田店／「ヤマダストアー大阪 梅田店」12月12日オープン、大阪初出店</t>
+        </is>
+      </c>
+      <c r="D2841" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101373.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2842">
+      <c r="A2842" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2842" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2842" t="inlineStr">
+        <is>
+          <t>ライフ／さいたま市「指扇店」リニューアル、ビオラルコーナー新設</t>
+        </is>
+      </c>
+      <c r="D2842" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101311.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2843">
+      <c r="A2843" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2843" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2843" t="inlineStr">
+        <is>
+          <t>モラージュ菖蒲／今秋新規含む5店舗オープン、無印良品が移転・増床リニューアル</t>
+        </is>
+      </c>
+      <c r="D2843" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101375.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2844">
+      <c r="A2844" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2844" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2844" t="inlineStr">
+        <is>
+          <t>イズミ／「ゆめタウン防府」10月15日リニューアル、食品売場にベーカリー・寿司コーナー導入</t>
+        </is>
+      </c>
+      <c r="D2844" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101374.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2845">
+      <c r="A2845" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2845" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2845" t="inlineStr">
+        <is>
+          <t>資さんうどん／東海地域1号店「熱田一番店」名古屋市に27年1月下旬オープン</t>
+        </is>
+      </c>
+      <c r="D2845" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101379.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2846">
+      <c r="A2846" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2846" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2846" t="inlineStr">
+        <is>
+          <t>まいばすけっと／東京・横浜・川崎に新店舗10月16日オープン</t>
+        </is>
+      </c>
+      <c r="D2846" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101313.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2847">
+      <c r="A2847" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2847" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2847" t="inlineStr">
+        <is>
+          <t>エブリイ／広島県に「リベモール深川（店舗面積4785m2）」27年4月27日新設</t>
+        </is>
+      </c>
+      <c r="D2847" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1013012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2848">
+      <c r="A2848" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2848" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2848" t="inlineStr">
+        <is>
+          <t>ピソラ／群馬県初出店「PISOLA前橋三俣店」10月15日オープン</t>
+        </is>
+      </c>
+      <c r="D2848" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101371.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2849">
+      <c r="A2849" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2849" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2849" t="inlineStr">
+        <is>
+          <t>銀座ルノアール／「喫茶室ルノアール 新宿3丁目T＆Tビル店」10月18日オープン</t>
+        </is>
+      </c>
+      <c r="D2849" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101372.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2850">
+      <c r="A2850" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2850" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2850" t="inlineStr">
+        <is>
+          <t>イオンリテール／「そよら鳥取駅南」10月9日オープン、イオン鳥取店を全館リニューアル</t>
+        </is>
+      </c>
+      <c r="D2850" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100911.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2851">
+      <c r="A2851" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2851" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2851" t="inlineStr">
+        <is>
+          <t>イオンリテールほか／兵庫県三田市に「（仮称）そよら三田・サンフラワー（店舗面積7481m2）」27年4月27日新設</t>
+        </is>
+      </c>
+      <c r="D2851" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1009012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2852">
+      <c r="A2852" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2852" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2852" t="inlineStr">
+        <is>
+          <t>ユニクロ／東京都「世田谷千歳台店」10月23日リニューアル、新サービス充実</t>
+        </is>
+      </c>
+      <c r="D2852" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100980.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2853">
+      <c r="A2853" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2853" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2853" t="inlineStr">
+        <is>
+          <t>近鉄不動産／大阪上本町に商業・オフィス複合施設「上本町ネクサス」27年2月オープン</t>
+        </is>
+      </c>
+      <c r="D2853" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100976.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2854">
+      <c r="A2854" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2854" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2854" t="inlineStr">
+        <is>
+          <t>たかき、ウェディングエルティ／山形県東根市に「（仮称）東根一本木商業施設」27年3月31日新設</t>
+        </is>
+      </c>
+      <c r="D2854" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1009011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2855">
+      <c r="A2855" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2855" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2855" t="inlineStr">
+        <is>
+          <t>資さんうどん／群馬県に「倉賀野店」10月15日オープン、ガストを業態転換</t>
+        </is>
+      </c>
+      <c r="D2855" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100973.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2856">
+      <c r="A2856" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2856" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2856" t="inlineStr">
+        <is>
+          <t>ロイヤルHD／池袋のスパにハワイアン・アジアンレストラン10月16日オープン</t>
+        </is>
+      </c>
+      <c r="D2856" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100913.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2857">
+      <c r="A2857" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2857" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2857" t="inlineStr">
+        <is>
+          <t>ランディーズドーナツ／東京ソラマチにテイクアウト専門店10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D2857" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s100975.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-14
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2857"/>
+  <dimension ref="A1:D2937"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63270,6 +63270,1766 @@
         </is>
       </c>
     </row>
+    <row r="2858">
+      <c r="A2858" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2858" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2858" t="inlineStr">
+        <is>
+          <t>10/16改装 平和堂大野店（食品売場）</t>
+        </is>
+      </c>
+      <c r="D2858" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gDK</t>
+        </is>
+      </c>
+    </row>
+    <row r="2859">
+      <c r="A2859" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2859" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2859" t="inlineStr">
+        <is>
+          <t>10/22移転 業務スーパー天理店</t>
+        </is>
+      </c>
+      <c r="D2859" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gCg</t>
+        </is>
+      </c>
+    </row>
+    <row r="2860">
+      <c r="A2860" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2860" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2860" t="inlineStr">
+        <is>
+          <t>「おじさんブランド」はなぜ生まれるのか。合理性を追求した男たちの行き着く先。モンベル、ロレックス、TUMI、ニューバランス(2026/10/12記事)</t>
+        </is>
+      </c>
+      <c r="D2860" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg1kmQ-1cH3</t>
+        </is>
+      </c>
+    </row>
+    <row r="2861">
+      <c r="A2861" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2861" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2861" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D2861" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="2862">
+      <c r="A2862" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2862" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2862" t="inlineStr">
+        <is>
+          <t>10/8建替 ツルヤなぎさ店(長野県松本市)</t>
+        </is>
+      </c>
+      <c r="D2862" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="2863">
+      <c r="A2863" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2863" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2863" t="inlineStr">
+        <is>
+          <t>10/9そよら鳥取駅南</t>
+        </is>
+      </c>
+      <c r="D2863" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gyC</t>
+        </is>
+      </c>
+    </row>
+    <row r="2864">
+      <c r="A2864" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2864" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2864" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D2864" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="2865">
+      <c r="A2865" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2865" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2865" t="inlineStr">
+        <is>
+          <t>10/15ロピア ブルメール舞多聞店</t>
+        </is>
+      </c>
+      <c r="D2865" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gBq</t>
+        </is>
+      </c>
+    </row>
+    <row r="2866">
+      <c r="A2866" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2866" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2866" t="inlineStr">
+        <is>
+          <t>10/22移転 業務スーパー天理店</t>
+        </is>
+      </c>
+      <c r="D2866" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gzx</t>
+        </is>
+      </c>
+    </row>
+    <row r="2867">
+      <c r="A2867" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2867" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2867" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D2867" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2868">
+      <c r="A2868" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2868" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2868" t="inlineStr">
+        <is>
+          <t>10/27やまのぶ赤池店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D2868" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1dGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2869">
+      <c r="A2869" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2869" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2869" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D2869" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="2870">
+      <c r="A2870" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2870" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2870" t="inlineStr">
+        <is>
+          <t>11/6移転 デリシアまめじま店</t>
+        </is>
+      </c>
+      <c r="D2870" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2871">
+      <c r="A2871" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2871" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2871" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D2871" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2872">
+      <c r="A2872" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2872" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2872" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D2872" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="2873">
+      <c r="A2873" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2873" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2873" t="inlineStr">
+        <is>
+          <t>12/3フェルナ武豊店(愛知県知多郡)</t>
+        </is>
+      </c>
+      <c r="D2873" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gBM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2874">
+      <c r="A2874" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2874" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2874" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D2874" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2875">
+      <c r="A2875" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2875" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2875" t="inlineStr">
+        <is>
+          <t>&lt;4/1予定&gt;(仮称)マックスバリュ豊橋西幸町店</t>
+        </is>
+      </c>
+      <c r="D2875" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gBH</t>
+        </is>
+      </c>
+    </row>
+    <row r="2876">
+      <c r="A2876" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2876" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2876" t="inlineStr">
+        <is>
+          <t>2027/6/1炭焼きレストランさわやか イオンセントラルスクエア静岡店</t>
+        </is>
+      </c>
+      <c r="D2876" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gCI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2877">
+      <c r="A2877" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2877" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2877" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D2877" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="2878">
+      <c r="A2878" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2878" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2878" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2878" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2879">
+      <c r="A2879" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2879" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2879" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2879" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2880">
+      <c r="A2880" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2880" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2880" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2880" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2881">
+      <c r="A2881" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2881" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2881" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2881" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2882">
+      <c r="A2882" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2882" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2882" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2882" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2883">
+      <c r="A2883" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2883" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2883" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2883" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2884">
+      <c r="A2884" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2884" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2884" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2884" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2885">
+      <c r="A2885" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2885" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2885" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2885" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2886">
+      <c r="A2886" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2886" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2886" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2886" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2887">
+      <c r="A2887" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2887" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2887" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2887" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2888">
+      <c r="A2888" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2888" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2888" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2888" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2889">
+      <c r="A2889" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2889" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2889" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2889" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2890">
+      <c r="A2890" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2890" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2890" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2890" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2891">
+      <c r="A2891" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2891" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2891" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2891" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2892">
+      <c r="A2892" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2892" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2892" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2892" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2893">
+      <c r="A2893" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2893" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2893" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2893" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2894">
+      <c r="A2894" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2894" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2894" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2894" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2895">
+      <c r="A2895" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2895" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2895" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2895" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2896">
+      <c r="A2896" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2896" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2896" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2896" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2897">
+      <c r="A2897" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2897" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2897" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D2897" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2898">
+      <c r="A2898" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2898" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2898" t="inlineStr">
+        <is>
+          <t>関東地方中野三丁目拠点施設 2029年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2898" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49231</t>
+        </is>
+      </c>
+    </row>
+    <row r="2899">
+      <c r="A2899" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2899" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2899" t="inlineStr">
+        <is>
+          <t>関東地方川崎市千年商業施設計画 ノジマが出店へ 2029年初頭開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2899" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42082</t>
+        </is>
+      </c>
+    </row>
+    <row r="2900">
+      <c r="A2900" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2900" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2900" t="inlineStr">
+        <is>
+          <t>九州地方ゆめモール那珂川 2026年2月20日(金)~順次開業！全20店舗一覧！</t>
+        </is>
+      </c>
+      <c r="D2900" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/31176</t>
+        </is>
+      </c>
+    </row>
+    <row r="2901">
+      <c r="A2901" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2901" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2901" t="inlineStr">
+        <is>
+          <t>関東地方コープ幕張駅北口店 2025年2月25日(火)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2901" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/39459</t>
+        </is>
+      </c>
+    </row>
+    <row r="2902">
+      <c r="A2902" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2902" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2902" t="inlineStr">
+        <is>
+          <t>関東地方福生駅西口地区市街地再開発事業 2027年春完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2902" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36735</t>
+        </is>
+      </c>
+    </row>
+    <row r="2903">
+      <c r="A2903" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2903" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2903" t="inlineStr">
+        <is>
+          <t>関東地方JR目黒ビル 2029年初頭開業！アトレ目黒が増床へ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2903" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47870</t>
+        </is>
+      </c>
+    </row>
+    <row r="2904">
+      <c r="A2904" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2904" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2904" t="inlineStr">
+        <is>
+          <t>関西地方GLION ARENA KOBE・TOTTEI PARKが 2025年4月4日(金)開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2904" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/33025</t>
+        </is>
+      </c>
+    </row>
+    <row r="2905">
+      <c r="A2905" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2905" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2905" t="inlineStr">
+        <is>
+          <t>中部地方スーパーセンタートライアル・コメリパワー垂井店 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2905" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48537</t>
+        </is>
+      </c>
+    </row>
+    <row r="2906">
+      <c r="A2906" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2906" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2906" t="inlineStr">
+        <is>
+          <t>九州地方ニトリ熊本はません店 2026年7月31日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2906" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/48407</t>
+        </is>
+      </c>
+    </row>
+    <row r="2907">
+      <c r="A2907" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2907" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2907" t="inlineStr">
+        <is>
+          <t>関東地方碓氷川右岸拠点商業地 フレッセイが出店へ 2029年以降開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2907" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/44330</t>
+        </is>
+      </c>
+    </row>
+    <row r="2908">
+      <c r="A2908" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2908" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2908" t="inlineStr">
+        <is>
+          <t>関東地方新所沢パルコ 跡地はヤオコーの商業施設に！2030年ごろ開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2908" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36676</t>
+        </is>
+      </c>
+    </row>
+    <row r="2909">
+      <c r="A2909" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2909" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2909" t="inlineStr">
+        <is>
+          <t>九州地方スーパーセンタートライアル加納店 2025年4月29日(火・祝)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2909" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/40580</t>
+        </is>
+      </c>
+    </row>
+    <row r="2910">
+      <c r="A2910" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2910" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2910" t="inlineStr">
+        <is>
+          <t>中部地方アルビス太閤山店 太閤山ショッピングセンター「パスコ」 建て替えて2025年10月24日(金)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2910" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/34574</t>
+        </is>
+      </c>
+    </row>
+    <row r="2911">
+      <c r="A2911" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2911" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2911" t="inlineStr">
+        <is>
+          <t>関西地方ヤマイチGARDEN桜井 マツゲンが出店！2025年11月21日(金)~順次開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2911" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39875</t>
+        </is>
+      </c>
+    </row>
+    <row r="2912">
+      <c r="A2912" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2912" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2912" t="inlineStr">
+        <is>
+          <t>関東地方ららテラス北綾瀬 北綾瀬駅前に2025年6月24日(火)開業！全テナント51店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2912" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26173</t>
+        </is>
+      </c>
+    </row>
+    <row r="2913">
+      <c r="A2913" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2913" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2913" t="inlineStr">
+        <is>
+          <t>四国地方ゆめタウン四国中央(仮称) フジグラン川之江 2027年春開業！ 最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2913" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/shikoku/47945</t>
+        </is>
+      </c>
+    </row>
+    <row r="2914">
+      <c r="A2914" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2914" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2914" t="inlineStr">
+        <is>
+          <t>関西地方淀屋橋ゲートタワー 2026年7月9日(木)開業！どのような建物に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2914" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/26392</t>
+        </is>
+      </c>
+    </row>
+    <row r="2915">
+      <c r="A2915" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2915" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2915" t="inlineStr">
+        <is>
+          <t>関西地方バルチカM 2027年3月開業！大阪駅高架下 全14テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2915" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49863</t>
+        </is>
+      </c>
+    </row>
+    <row r="2916">
+      <c r="A2916" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2916" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2916" t="inlineStr">
+        <is>
+          <t>関西地方スーパーセンタートライアル愛知川店 2026年10月21日(水)グランドオープン！最新情報も！滋賀県愛知郡にトライアルカンパニーの店舗「スーパーセンタートライアル愛知川店」が2026年10月21日(水)AM8: 30グランドオープン！10月20日(火)10:00〜19:00 プレオープン！スーパーセンタートライアルが愛荘町に初出店！...2026.10.14関西地方</t>
+        </is>
+      </c>
+      <c r="D2916" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/47736</t>
+        </is>
+      </c>
+    </row>
+    <row r="2917">
+      <c r="A2917" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2917" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2917" t="inlineStr">
+        <is>
+          <t>九州地方トライアルスマート小倉熊谷店 2026年12月初旬に開業予定！最新情報も！福岡県北九州市にトライアルカンパニーの店舗「トライアルスマート小倉熊谷店」が2026年12月初旬に開業予定！トライアルスマートが小倉北区熊谷に出店！そんな、トライアルスマート小倉熊谷店について、テナントや開業日などを見ていきましょう！202...2026.10.14九州地方</t>
+        </is>
+      </c>
+      <c r="D2917" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/48785</t>
+        </is>
+      </c>
+    </row>
+    <row r="2918">
+      <c r="A2918" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2918" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2918" t="inlineStr">
+        <is>
+          <t>ロピア／埼玉県「加須ビバモール店」10月21日オープン、肉総菜・アジア食品訴求</t>
+        </is>
+      </c>
+      <c r="D2918" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101475.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2919">
+      <c r="A2919" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2919" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2919" t="inlineStr">
+        <is>
+          <t>大黒天物産／愛知県知多郡東浦町に「（仮称）ラ・ムー東浦店」27年3月28日新設</t>
+        </is>
+      </c>
+      <c r="D2919" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1014011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2920">
+      <c r="A2920" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2920" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2920" t="inlineStr">
+        <is>
+          <t>コスモス薬品／愛知県・富山県に「ドラッグコスモス」計3店舗、27年4月新設</t>
+        </is>
+      </c>
+      <c r="D2920" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1014012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2921">
+      <c r="A2921" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2921" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2921" t="inlineStr">
+        <is>
+          <t>レデイ薬局／愛媛県四国中央市に「くすりのレデイ イオンタウン川之江店」オープン</t>
+        </is>
+      </c>
+      <c r="D2921" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101442.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2922">
+      <c r="A2922" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2922" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2922" t="inlineStr">
+        <is>
+          <t>タリーズコーヒー／北海道に「小樽ポートスクエア店」オープン、小樽エリアに初出店</t>
+        </is>
+      </c>
+      <c r="D2922" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101443.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2923">
+      <c r="A2923" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2923" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2923" t="inlineStr">
+        <is>
+          <t>松屋フーズ／熊本県八代市に松屋・松のや複合店「八代店」10月15日オープン</t>
+        </is>
+      </c>
+      <c r="D2923" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101473.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2924">
+      <c r="A2924" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2924" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2924" t="inlineStr">
+        <is>
+          <t>三井不動産ほか／東京都足立区の大規模複合開発「アクアゲート千住大川端」30年1期竣工</t>
+        </is>
+      </c>
+      <c r="D2924" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101376.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2925">
+      <c r="A2925" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2925" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2925" t="inlineStr">
+        <is>
+          <t>三菱商事都市開発×奥村組／大阪に商業施設、ライフ・ヤマダデンキが27年春オープン</t>
+        </is>
+      </c>
+      <c r="D2925" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101315.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2926">
+      <c r="A2926" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2926" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2926" t="inlineStr">
+        <is>
+          <t>イオンリテール／兵庫県小野市に「（仮称）そよら小野（店舗面積1万360m2）」27年4月1日新設</t>
+        </is>
+      </c>
+      <c r="D2926" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1013011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2927">
+      <c r="A2927" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2927" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2927" t="inlineStr">
+        <is>
+          <t>大丸梅田店／「ヤマダストアー大阪 梅田店」12月12日オープン、大阪初出店</t>
+        </is>
+      </c>
+      <c r="D2927" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101373.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2928">
+      <c r="A2928" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2928" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2928" t="inlineStr">
+        <is>
+          <t>ライフ／さいたま市「指扇店」リニューアル、ビオラルコーナー新設</t>
+        </is>
+      </c>
+      <c r="D2928" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101311.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2929">
+      <c r="A2929" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2929" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2929" t="inlineStr">
+        <is>
+          <t>モラージュ菖蒲／今秋新規含む5店舗オープン、無印良品が移転・増床リニューアル</t>
+        </is>
+      </c>
+      <c r="D2929" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101375.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2930">
+      <c r="A2930" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2930" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2930" t="inlineStr">
+        <is>
+          <t>イズミ／「ゆめタウン防府」10月15日リニューアル、食品売場にベーカリー・寿司コーナー導入</t>
+        </is>
+      </c>
+      <c r="D2930" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101374.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2931">
+      <c r="A2931" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2931" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2931" t="inlineStr">
+        <is>
+          <t>資さんうどん／東海地域1号店「熱田一番店」名古屋市に27年1月下旬オープン</t>
+        </is>
+      </c>
+      <c r="D2931" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101379.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2932">
+      <c r="A2932" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2932" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2932" t="inlineStr">
+        <is>
+          <t>まいばすけっと／東京・横浜・川崎に新店舗10月16日オープン</t>
+        </is>
+      </c>
+      <c r="D2932" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101313.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2933">
+      <c r="A2933" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2933" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2933" t="inlineStr">
+        <is>
+          <t>エブリイ／広島県に「リベモール深川（店舗面積4785m2）」27年4月27日新設</t>
+        </is>
+      </c>
+      <c r="D2933" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1013012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2934">
+      <c r="A2934" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2934" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2934" t="inlineStr">
+        <is>
+          <t>ピソラ／群馬県初出店「PISOLA前橋三俣店」10月15日オープン</t>
+        </is>
+      </c>
+      <c r="D2934" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101371.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2935">
+      <c r="A2935" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2935" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2935" t="inlineStr">
+        <is>
+          <t>銀座ルノアール／「喫茶室ルノアール 新宿3丁目T＆Tビル店」10月18日オープン</t>
+        </is>
+      </c>
+      <c r="D2935" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101372.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2936">
+      <c r="A2936" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2936" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2936" t="inlineStr">
+        <is>
+          <t>自由が丘駅南口／新たな文化発信拠点「ミミミ自由が丘」10月9日オープン、新業態充実</t>
+        </is>
+      </c>
+      <c r="D2936" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s100673.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2937">
+      <c r="A2937" t="inlineStr">
+        <is>
+          <t>2026年10月14日</t>
+        </is>
+      </c>
+      <c r="B2937" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2937" t="inlineStr">
+        <is>
+          <t>マミーマート／「生鮮市場TOP！川口柳崎店」オープン、足元商圏のファミリー層狙う</t>
+        </is>
+      </c>
+      <c r="D2937" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s091771.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-15
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2937"/>
+  <dimension ref="A1:D3012"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -65030,6 +65030,1656 @@
         </is>
       </c>
     </row>
+    <row r="2938">
+      <c r="A2938" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2938" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2938" t="inlineStr">
+        <is>
+          <t>10/21ロピア加須ビバモール店(埼玉県加須市)</t>
+        </is>
+      </c>
+      <c r="D2938" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gE6</t>
+        </is>
+      </c>
+    </row>
+    <row r="2939">
+      <c r="A2939" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2939" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2939" t="inlineStr">
+        <is>
+          <t>10/30松屋可児店（松のや併設）</t>
+        </is>
+      </c>
+      <c r="D2939" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gEg</t>
+        </is>
+      </c>
+    </row>
+    <row r="2940">
+      <c r="A2940" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2940" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2940" t="inlineStr">
+        <is>
+          <t>10/15ロピアブルメール舞多聞店</t>
+        </is>
+      </c>
+      <c r="D2940" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gBq</t>
+        </is>
+      </c>
+    </row>
+    <row r="2941">
+      <c r="A2941" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2941" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2941" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D2941" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="2942">
+      <c r="A2942" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2942" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2942" t="inlineStr">
+        <is>
+          <t>10/8建替 ツルヤなぎさ店(長野県松本市)</t>
+        </is>
+      </c>
+      <c r="D2942" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="2943">
+      <c r="A2943" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2943" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2943" t="inlineStr">
+        <is>
+          <t>10/9そよら鳥取駅南</t>
+        </is>
+      </c>
+      <c r="D2943" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gyC</t>
+        </is>
+      </c>
+    </row>
+    <row r="2944">
+      <c r="A2944" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2944" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2944" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D2944" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="2945">
+      <c r="A2945" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2945" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2945" t="inlineStr">
+        <is>
+          <t>10/16改装 平和堂大野店（食品売場）</t>
+        </is>
+      </c>
+      <c r="D2945" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gDK</t>
+        </is>
+      </c>
+    </row>
+    <row r="2946">
+      <c r="A2946" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2946" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2946" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D2946" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2947">
+      <c r="A2947" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2947" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2947" t="inlineStr">
+        <is>
+          <t>10/27やまのぶ赤池店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D2947" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1dGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2948">
+      <c r="A2948" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2948" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2948" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D2948" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="2949">
+      <c r="A2949" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2949" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2949" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D2949" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2950">
+      <c r="A2950" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2950" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2950" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D2950" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="2951">
+      <c r="A2951" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2951" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2951" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D2951" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2952">
+      <c r="A2952" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2952" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C2952" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D2952" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="2953">
+      <c r="A2953" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2953" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2953" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2953" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2954">
+      <c r="A2954" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2954" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2954" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2954" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2955">
+      <c r="A2955" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2955" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2955" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2955" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2956">
+      <c r="A2956" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2956" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2956" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2956" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2957">
+      <c r="A2957" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2957" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2957" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2957" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2958">
+      <c r="A2958" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2958" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2958" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2958" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2959">
+      <c r="A2959" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2959" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2959" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2959" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2960">
+      <c r="A2960" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2960" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2960" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2960" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2961">
+      <c r="A2961" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2961" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2961" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2961" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2962">
+      <c r="A2962" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2962" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2962" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2962" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2963">
+      <c r="A2963" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2963" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2963" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2963" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2964">
+      <c r="A2964" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2964" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2964" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D2964" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2965">
+      <c r="A2965" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2965" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2965" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D2965" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2966">
+      <c r="A2966" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2966" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2966" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D2966" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2967">
+      <c r="A2967" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2967" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2967" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D2967" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2968">
+      <c r="A2968" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2968" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2968" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D2968" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2969">
+      <c r="A2969" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2969" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2969" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2969" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2970">
+      <c r="A2970" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2970" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2970" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D2970" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2971">
+      <c r="A2971" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2971" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2971" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D2971" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2972">
+      <c r="A2972" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2972" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C2972" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D2972" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2973">
+      <c r="A2973" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2973" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2973" t="inlineStr">
+        <is>
+          <t>関東地方武蔵小金井駅北口駅前東地区市街地再開発事業 2030年1月完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2973" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48940</t>
+        </is>
+      </c>
+    </row>
+    <row r="2974">
+      <c r="A2974" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2974" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2974" t="inlineStr">
+        <is>
+          <t>中国地方カミハチクロス 2027年度開業！アンダーズ広島が進出！商業施設も！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2974" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/27582</t>
+        </is>
+      </c>
+    </row>
+    <row r="2975">
+      <c r="A2975" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2975" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2975" t="inlineStr">
+        <is>
+          <t>東北地方スーパーセンタートライアル亘理店 2025年7月16日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2975" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/41583</t>
+        </is>
+      </c>
+    </row>
+    <row r="2976">
+      <c r="A2976" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2976" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2976" t="inlineStr">
+        <is>
+          <t>中部地方アークガレリア長岡 再開発 2026年春リニューアル完了！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2976" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/37232</t>
+        </is>
+      </c>
+    </row>
+    <row r="2977">
+      <c r="A2977" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2977" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2977" t="inlineStr">
+        <is>
+          <t>関東地方イオン藤沢店 2026年1月末で一旦閉店し建て替えへ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2977" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/46012</t>
+        </is>
+      </c>
+    </row>
+    <row r="2978">
+      <c r="A2978" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2978" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2978" t="inlineStr">
+        <is>
+          <t>中国地方ハローズ呉広モール 2025年12月17日(水)開業！全7店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2978" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/42161</t>
+        </is>
+      </c>
+    </row>
+    <row r="2979">
+      <c r="A2979" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2979" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2979" t="inlineStr">
+        <is>
+          <t>関東地方南小岩七丁目地区市街地再開発事業 2030年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2979" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/19966</t>
+        </is>
+      </c>
+    </row>
+    <row r="2980">
+      <c r="A2980" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2980" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2980" t="inlineStr">
+        <is>
+          <t>関東地方綱島駅東口駅前地区市街地再開発事業 完成はいつ？テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2980" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26111</t>
+        </is>
+      </c>
+    </row>
+    <row r="2981">
+      <c r="A2981" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2981" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2981" t="inlineStr">
+        <is>
+          <t>関東地方スーパーセンタートライアル深谷川本店 2026年4月29日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2981" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/44915</t>
+        </is>
+      </c>
+    </row>
+    <row r="2982">
+      <c r="A2982" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2982" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2982" t="inlineStr">
+        <is>
+          <t>四国地方スーパーセンタートライアル三木店 2025年7月16日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2982" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/shikoku/41508</t>
+        </is>
+      </c>
+    </row>
+    <row r="2983">
+      <c r="A2983" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2983" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2983" t="inlineStr">
+        <is>
+          <t>関東地方ヨークベニマル古河店 カインズ古河店 2025年2月14日(金)開業！無印良品とスタバが出店！全6テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2983" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/37708</t>
+        </is>
+      </c>
+    </row>
+    <row r="2984">
+      <c r="A2984" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2984" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2984" t="inlineStr">
+        <is>
+          <t>九州地方スーパーセンタートライアル阿蘇店 2026年11月中旬に開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2984" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/48550</t>
+        </is>
+      </c>
+    </row>
+    <row r="2985">
+      <c r="A2985" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2985" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2985" t="inlineStr">
+        <is>
+          <t>関西地方アイユータウン マルアイ長田店 2025年9月17日(水)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2985" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/42358</t>
+        </is>
+      </c>
+    </row>
+    <row r="2986">
+      <c r="A2986" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2986" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2986" t="inlineStr">
+        <is>
+          <t>中部地方M20 cosa（コーサ）静岡駅北口 2024年10月28日(月)開業！全13テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2986" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/26298</t>
+        </is>
+      </c>
+    </row>
+    <row r="2987">
+      <c r="A2987" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2987" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2987" t="inlineStr">
+        <is>
+          <t>中部地方アークスクエア須坂 ホームセンタームサシ・ヤマダデンキ 2025年8月6日(水)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2987" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/21807</t>
+        </is>
+      </c>
+    </row>
+    <row r="2988">
+      <c r="A2988" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2988" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2988" t="inlineStr">
+        <is>
+          <t>関東地方カインズ伊勢崎境保泉店 2028年春開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2988" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47795</t>
+        </is>
+      </c>
+    </row>
+    <row r="2989">
+      <c r="A2989" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2989" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2989" t="inlineStr">
+        <is>
+          <t>関東地方そよら入曽駅前 2025年3月21日(金)開業！全テナント10店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D2989" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/22304</t>
+        </is>
+      </c>
+    </row>
+    <row r="2990">
+      <c r="A2990" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2990" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2990" t="inlineStr">
+        <is>
+          <t>中部地方HAERA(ハエラ） ザ・ランドマーク名古屋栄 2026年6月11日(木)開業！コンラッド名古屋や高級商業施設！全65店舗一覧！</t>
+        </is>
+      </c>
+      <c r="D2990" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/23200</t>
+        </is>
+      </c>
+    </row>
+    <row r="2991">
+      <c r="A2991" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2991" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2991" t="inlineStr">
+        <is>
+          <t>関西地方スーパーセンタートライアル愛知川店 2026年10月21日(水)グランドオープン！最新情報も！滋賀県愛知郡にトライアルカンパニーの店舗「スーパーセンタートライアル愛知川店」が2026年10月21日(水)AM8: 30グランドオープン！10月20日(火)10:00〜19:00 プレオープン！スーパーセンタートライアルが愛荘町に初出店！...2026.10.14関西地方</t>
+        </is>
+      </c>
+      <c r="D2991" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/47736</t>
+        </is>
+      </c>
+    </row>
+    <row r="2992">
+      <c r="A2992" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2992" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C2992" t="inlineStr">
+        <is>
+          <t>九州地方トライアルスマート小倉熊谷店 2026年12月初旬に開業予定！最新情報も！福岡県北九州市にトライアルカンパニーの店舗「トライアルスマート小倉熊谷店」が2026年12月初旬に開業予定！トライアルスマートが小倉北区熊谷に出店！そんな、トライアルスマート小倉熊谷店について、テナントや開業日などを見ていきましょう！202...2026.10.14九州地方</t>
+        </is>
+      </c>
+      <c r="D2992" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/48785</t>
+        </is>
+      </c>
+    </row>
+    <row r="2993">
+      <c r="A2993" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2993" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2993" t="inlineStr">
+        <is>
+          <t>西武池袋本店／11～12月の7・8階リニューアルで新百貨店モデルが完成</t>
+        </is>
+      </c>
+      <c r="D2993" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101515.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2994">
+      <c r="A2994" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2994" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2994" t="inlineStr">
+        <is>
+          <t>大丸梅田店／新ストアコンセプト発表、27年春3フロアを先行リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D2994" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101577.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2995">
+      <c r="A2995" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2995" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2995" t="inlineStr">
+        <is>
+          <t>エキュート大宮／今秋「銀座おのでら」の新業態含む9店舗が順次オープン</t>
+        </is>
+      </c>
+      <c r="D2995" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101579.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2996">
+      <c r="A2996" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2996" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2996" t="inlineStr">
+        <is>
+          <t>コスモス薬品／京都府・静岡県に「ドラッグコスモス」計2店舗、27年4月新設</t>
+        </is>
+      </c>
+      <c r="D2996" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1015012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2997">
+      <c r="A2997" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2997" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2997" t="inlineStr">
+        <is>
+          <t>クリエイトSD／神奈川県綾瀬市に「綾瀬北上土棚店」27年4月4日新設</t>
+        </is>
+      </c>
+      <c r="D2997" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1015011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2998">
+      <c r="A2998" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2998" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2998" t="inlineStr">
+        <is>
+          <t>カインズ／ユアエルム青戸にリフォーム専門の小型店舗オープン</t>
+        </is>
+      </c>
+      <c r="D2998" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101514.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2999">
+      <c r="A2999" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B2999" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C2999" t="inlineStr">
+        <is>
+          <t>アミュプラザくまもと／家具・インテリアブランド「LOWYA」の新店27年春オープン</t>
+        </is>
+      </c>
+      <c r="D2999" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101571.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3000">
+      <c r="A3000" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B3000" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3000" t="inlineStr">
+        <is>
+          <t>京都ヨドバシ／「nana’s green tea」のテイクアウト新業態12月初旬オープン</t>
+        </is>
+      </c>
+      <c r="D3000" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101574.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3001">
+      <c r="A3001" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B3001" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3001" t="inlineStr">
+        <is>
+          <t>エノテカ／東京・丸の内に新店舗10月28日オープン、贈答用ワイン約600種そろう</t>
+        </is>
+      </c>
+      <c r="D3001" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101576.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3002">
+      <c r="A3002" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B3002" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3002" t="inlineStr">
+        <is>
+          <t>ジョイフル／「JOYFULL EXPRESS イオンモール高岡店」10月27日オープン</t>
+        </is>
+      </c>
+      <c r="D3002" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101575.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3003">
+      <c r="A3003" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B3003" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3003" t="inlineStr">
+        <is>
+          <t>すたみな太郎／青森県八戸市に「PREMIUM BUFFET八戸店」10月17日オープン</t>
+        </is>
+      </c>
+      <c r="D3003" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101573.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3004">
+      <c r="A3004" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B3004" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3004" t="inlineStr">
+        <is>
+          <t>ロピア／埼玉県「加須ビバモール店」10月21日オープン、肉総菜・アジア食品訴求</t>
+        </is>
+      </c>
+      <c r="D3004" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101475.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3005">
+      <c r="A3005" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B3005" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3005" t="inlineStr">
+        <is>
+          <t>大黒天物産／愛知県知多郡東浦町に「（仮称）ラ・ムー東浦店」27年3月28日新設</t>
+        </is>
+      </c>
+      <c r="D3005" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1014011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3006">
+      <c r="A3006" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B3006" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3006" t="inlineStr">
+        <is>
+          <t>コスモス薬品／愛知県・富山県に「ドラッグコスモス」計3店舗、27年4月新設</t>
+        </is>
+      </c>
+      <c r="D3006" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1014012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3007">
+      <c r="A3007" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B3007" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3007" t="inlineStr">
+        <is>
+          <t>レデイ薬局／愛媛県四国中央市に「くすりのレデイ イオンタウン川之江店」オープン</t>
+        </is>
+      </c>
+      <c r="D3007" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101442.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3008">
+      <c r="A3008" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B3008" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3008" t="inlineStr">
+        <is>
+          <t>タリーズコーヒー／北海道に「小樽ポートスクエア店」オープン、小樽エリアに初出店</t>
+        </is>
+      </c>
+      <c r="D3008" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101443.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3009">
+      <c r="A3009" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B3009" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3009" t="inlineStr">
+        <is>
+          <t>松屋フーズ／熊本県八代市に松屋・松のや複合店「八代店」10月15日オープン</t>
+        </is>
+      </c>
+      <c r="D3009" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101473.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3010">
+      <c r="A3010" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B3010" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3010" t="inlineStr">
+        <is>
+          <t>三井不動産ほか／東京都足立区の大規模複合開発「アクアゲート千住大川端」30年1期竣工</t>
+        </is>
+      </c>
+      <c r="D3010" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101376.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3011">
+      <c r="A3011" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B3011" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3011" t="inlineStr">
+        <is>
+          <t>三菱商事都市開発×奥村組／大阪に商業施設、ライフ・ヤマダデンキが27年春オープン</t>
+        </is>
+      </c>
+      <c r="D3011" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101315.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3012">
+      <c r="A3012" t="inlineStr">
+        <is>
+          <t>2026年10月15日</t>
+        </is>
+      </c>
+      <c r="B3012" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3012" t="inlineStr">
+        <is>
+          <t>イオンリテール／兵庫県小野市に「（仮称）そよら小野（店舗面積1万360m2）」27年4月1日新設</t>
+        </is>
+      </c>
+      <c r="D3012" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1013011.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-16
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3012"/>
+  <dimension ref="A1:D3087"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -66680,6 +66680,1656 @@
         </is>
       </c>
     </row>
+    <row r="3013">
+      <c r="A3013" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3013" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3013" t="inlineStr">
+        <is>
+          <t>10/16改装 平和堂大野店（食品売場)</t>
+        </is>
+      </c>
+      <c r="D3013" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gDK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3014">
+      <c r="A3014" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3014" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3014" t="inlineStr">
+        <is>
+          <t>10/16KOmart fine長泉店</t>
+        </is>
+      </c>
+      <c r="D3014" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gFD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3015">
+      <c r="A3015" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3015" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3015" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3015" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="3016">
+      <c r="A3016" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3016" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3016" t="inlineStr">
+        <is>
+          <t>10/8建替 ツルヤなぎさ店(長野県松本市)</t>
+        </is>
+      </c>
+      <c r="D3016" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="3017">
+      <c r="A3017" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3017" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3017" t="inlineStr">
+        <is>
+          <t>10/9そよら鳥取駅南</t>
+        </is>
+      </c>
+      <c r="D3017" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gyC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3018">
+      <c r="A3018" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3018" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3018" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D3018" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="3019">
+      <c r="A3019" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3019" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3019" t="inlineStr">
+        <is>
+          <t>10/21ロピア加須ビバモール店(埼玉県加須市)</t>
+        </is>
+      </c>
+      <c r="D3019" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gE6</t>
+        </is>
+      </c>
+    </row>
+    <row r="3020">
+      <c r="A3020" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3020" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3020" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D3020" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="3021">
+      <c r="A3021" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3021" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3021" t="inlineStr">
+        <is>
+          <t>10/27やまのぶ赤池店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3021" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1dGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3022">
+      <c r="A3022" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3022" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3022" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D3022" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3023">
+      <c r="A3023" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3023" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3023" t="inlineStr">
+        <is>
+          <t>10/30松屋可児店（松のや併設）</t>
+        </is>
+      </c>
+      <c r="D3023" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gEg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3024">
+      <c r="A3024" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3024" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3024" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D3024" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3025">
+      <c r="A3025" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3025" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3025" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D3025" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="3026">
+      <c r="A3026" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3026" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3026" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D3026" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="3027">
+      <c r="A3027" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3027" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3027" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D3027" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="3028">
+      <c r="A3028" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3028" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3028" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3028" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3029">
+      <c r="A3029" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3029" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3029" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3029" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3030">
+      <c r="A3030" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3030" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3030" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3030" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3031">
+      <c r="A3031" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3031" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3031" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3031" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3032">
+      <c r="A3032" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3032" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3032" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3032" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3033">
+      <c r="A3033" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3033" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3033" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3033" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3034">
+      <c r="A3034" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3034" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3034" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3034" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3035">
+      <c r="A3035" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3035" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3035" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3035" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3036">
+      <c r="A3036" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3036" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3036" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3036" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3037">
+      <c r="A3037" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3037" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3037" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3037" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3038">
+      <c r="A3038" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3038" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3038" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3038" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3039">
+      <c r="A3039" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3039" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3039" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3039" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3040">
+      <c r="A3040" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3040" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3040" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3040" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3041">
+      <c r="A3041" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3041" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3041" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3041" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3042">
+      <c r="A3042" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3042" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3042" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3042" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3043">
+      <c r="A3043" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3043" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3043" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3043" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3044">
+      <c r="A3044" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3044" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3044" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3044" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3045">
+      <c r="A3045" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3045" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3045" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3045" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3046">
+      <c r="A3046" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3046" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3046" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3046" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3047">
+      <c r="A3047" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3047" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3047" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3047" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3048">
+      <c r="A3048" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3048" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3048" t="inlineStr">
+        <is>
+          <t>九州地方旦過市場いちばん館 2026年11月24日~順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3048" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/47032</t>
+        </is>
+      </c>
+    </row>
+    <row r="3049">
+      <c r="A3049" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3049" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3049" t="inlineStr">
+        <is>
+          <t>関東地方ミナモニ有明 江東区有明1丁目計画 大和ハウスのマンションと商業施設に！2026年5月13日(水)9時~開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3049" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/35626</t>
+        </is>
+      </c>
+    </row>
+    <row r="3050">
+      <c r="A3050" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3050" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3050" t="inlineStr">
+        <is>
+          <t>関東地方かすかべテラス 2025年6月10日(火)開業！コープみらいが出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3050" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/29383</t>
+        </is>
+      </c>
+    </row>
+    <row r="3051">
+      <c r="A3051" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3051" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3051" t="inlineStr">
+        <is>
+          <t>中部地方三島駅南口東街区Ａ地区市街地再開発事業 2027年竣工予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3051" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/25890</t>
+        </is>
+      </c>
+    </row>
+    <row r="3052">
+      <c r="A3052" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3052" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3052" t="inlineStr">
+        <is>
+          <t>中国地方リベモール深川 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3052" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/48520</t>
+        </is>
+      </c>
+    </row>
+    <row r="3053">
+      <c r="A3053" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3053" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3053" t="inlineStr">
+        <is>
+          <t>九州地方福岡空港国内線ターミナル 大型商業施設が誕生！2027年夏開業！180店舗が出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3053" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/43493</t>
+        </is>
+      </c>
+    </row>
+    <row r="3054">
+      <c r="A3054" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3054" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3054" t="inlineStr">
+        <is>
+          <t>関東地方神田小川町三丁目西部南地区市街地再開発事業 進捗状況は？テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3054" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/31895</t>
+        </is>
+      </c>
+    </row>
+    <row r="3055">
+      <c r="A3055" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3055" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3055" t="inlineStr">
+        <is>
+          <t>九州地方アクロスプラザ飯塚太郎丸 2026年5月28日(木)開業！全8テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3055" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/44863</t>
+        </is>
+      </c>
+    </row>
+    <row r="3056">
+      <c r="A3056" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3056" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3056" t="inlineStr">
+        <is>
+          <t>関東地方相模原駅北口地区土地利用計画 商業施設も開業へ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3056" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/44641</t>
+        </is>
+      </c>
+    </row>
+    <row r="3057">
+      <c r="A3057" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3057" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3057" t="inlineStr">
+        <is>
+          <t>関西地方ニトリ平野店 2026年4月24日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3057" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/46499</t>
+        </is>
+      </c>
+    </row>
+    <row r="3058">
+      <c r="A3058" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3058" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3058" t="inlineStr">
+        <is>
+          <t>関西地方平和堂岸辺店 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3058" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49465</t>
+        </is>
+      </c>
+    </row>
+    <row r="3059">
+      <c r="A3059" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3059" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3059" t="inlineStr">
+        <is>
+          <t>東北地方オルフィーカ美田園 2025年5月23日(金)より順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3059" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/39130</t>
+        </is>
+      </c>
+    </row>
+    <row r="3060">
+      <c r="A3060" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3060" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3060" t="inlineStr">
+        <is>
+          <t>関西地方難波宮跡公園 なノにわ 2025年3月28日(金)12時に開業！全13テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3060" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/41360</t>
+        </is>
+      </c>
+    </row>
+    <row r="3061">
+      <c r="A3061" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3061" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3061" t="inlineStr">
+        <is>
+          <t>関西地方北千里駅前地区市街地再開発事業 2037年までに段階整備！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3061" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39517</t>
+        </is>
+      </c>
+    </row>
+    <row r="3062">
+      <c r="A3062" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3062" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3062" t="inlineStr">
+        <is>
+          <t>関東地方碓氷川右岸拠点商業地 フレッセイが出店へ 2029年以降開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3062" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/44330</t>
+        </is>
+      </c>
+    </row>
+    <row r="3063">
+      <c r="A3063" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3063" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3063" t="inlineStr">
+        <is>
+          <t>関東地方ロヂャース熊谷新島店 2027年春開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3063" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49874</t>
+        </is>
+      </c>
+    </row>
+    <row r="3064">
+      <c r="A3064" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3064" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3064" t="inlineStr">
+        <is>
+          <t>関東地方ブルーフロント芝浦 商業施設 2025年9月1日(月)11:00~開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3064" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/21848</t>
+        </is>
+      </c>
+    </row>
+    <row r="3065">
+      <c r="A3065" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3065" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3065" t="inlineStr">
+        <is>
+          <t>関東地方Beisia Foods Park 伊勢崎境保泉店 2028年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3065" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47770</t>
+        </is>
+      </c>
+    </row>
+    <row r="3066">
+      <c r="A3066" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3066" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3066" t="inlineStr">
+        <is>
+          <t>関西地方スーパーセンタートライアル愛知川店 2026年10月21日(水)グランドオープン！最新情報も！滋賀県愛知郡にトライアルカンパニーの店舗「スーパーセンタートライアル愛知川店」が2026年10月21日(水)AM8: 30グランドオープン！10月20日(火)10:00〜19:00 プレオープン！スーパーセンタートライアルが愛荘町に初出店！...2026.10.14関西地方</t>
+        </is>
+      </c>
+      <c r="D3066" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/47736</t>
+        </is>
+      </c>
+    </row>
+    <row r="3067">
+      <c r="A3067" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3067" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3067" t="inlineStr">
+        <is>
+          <t>九州地方トライアルスマート小倉熊谷店 2026年12月初旬に開業予定！最新情報も！福岡県北九州市にトライアルカンパニーの店舗「トライアルスマート小倉熊谷店」が2026年12月初旬に開業予定！トライアルスマートが小倉北区熊谷に出店！そんな、トライアルスマート小倉熊谷店について、テナントや開業日などを見ていきましょう！202...2026.10.14九州地方</t>
+        </is>
+      </c>
+      <c r="D3067" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/48785</t>
+        </is>
+      </c>
+    </row>
+    <row r="3068">
+      <c r="A3068" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3068" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3068" t="inlineStr">
+        <is>
+          <t>玉川高島屋S.C.／27年3月本館食品フロア刷新、南館にサウナほか新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3068" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101673.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3069">
+      <c r="A3069" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3069" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3069" t="inlineStr">
+        <is>
+          <t>バロー／大府市に「大府北山店」10月23日オープン、愛知県70店舗目</t>
+        </is>
+      </c>
+      <c r="D3069" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101612.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3070">
+      <c r="A3070" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3070" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3070" t="inlineStr">
+        <is>
+          <t>野村不動産／東京・門前仲町で住宅・商業複合施設を開発</t>
+        </is>
+      </c>
+      <c r="D3070" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101613.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3071">
+      <c r="A3071" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3071" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3071" t="inlineStr">
+        <is>
+          <t>イオン北海道／「ザ・ビッグ千歳武道館前店」10月23日オープン</t>
+        </is>
+      </c>
+      <c r="D3071" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101615.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3072">
+      <c r="A3072" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3072" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3072" t="inlineStr">
+        <is>
+          <t>京阪HD／京都府に「三条PJ本館新築工事（店舗面積6895m2）」27年5月1日新設</t>
+        </is>
+      </c>
+      <c r="D3072" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1016011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3073">
+      <c r="A3073" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3073" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3073" t="inlineStr">
+        <is>
+          <t>コスモス薬品／栃木県・新潟県に「ドラッグコスモス」計2店舗、27年5月新設</t>
+        </is>
+      </c>
+      <c r="D3073" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1016012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3074">
+      <c r="A3074" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3074" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3074" t="inlineStr">
+        <is>
+          <t>串カツ田中／全国制覇達成「串カツ田中 和歌山駅前店」10月23日オープン</t>
+        </is>
+      </c>
+      <c r="D3074" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101681.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3075">
+      <c r="A3075" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3075" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3075" t="inlineStr">
+        <is>
+          <t>コメダ／愛知県安城市に「おかげ庵」12月オープン</t>
+        </is>
+      </c>
+      <c r="D3075" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101616.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3076">
+      <c r="A3076" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3076" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3076" t="inlineStr">
+        <is>
+          <t>ミズノ／「ミズノ大阪心斎橋」10月23日オープン、若年層・インバウンドに照準</t>
+        </is>
+      </c>
+      <c r="D3076" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101672.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3077">
+      <c r="A3077" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3077" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3077" t="inlineStr">
+        <is>
+          <t>東急百貨店たまプラーザ店／「メンズビギ」の新店舗オープン、限定アイテムも販売</t>
+        </is>
+      </c>
+      <c r="D3077" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101680.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3078">
+      <c r="A3078" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3078" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3078" t="inlineStr">
+        <is>
+          <t>ゴンチャ／銀座・有楽町エリア初出店「ルミネ有楽町店」10月23日オープン</t>
+        </is>
+      </c>
+      <c r="D3078" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101674.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3079">
+      <c r="A3079" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3079" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3079" t="inlineStr">
+        <is>
+          <t>サンマルクカフェ＆茶／東京都墨田区に「両国東口店」10月21日オープン</t>
+        </is>
+      </c>
+      <c r="D3079" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101675.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3080">
+      <c r="A3080" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3080" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3080" t="inlineStr">
+        <is>
+          <t>西武池袋本店／11～12月の7・8階リニューアルで新百貨店モデルが完成</t>
+        </is>
+      </c>
+      <c r="D3080" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101515.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3081">
+      <c r="A3081" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3081" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3081" t="inlineStr">
+        <is>
+          <t>大丸梅田店／新ストアコンセプト発表、27年春3フロアを先行リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D3081" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101577.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3082">
+      <c r="A3082" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3082" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3082" t="inlineStr">
+        <is>
+          <t>エキュート大宮／今秋「銀座おのでら」の新業態含む9店舗が順次オープン</t>
+        </is>
+      </c>
+      <c r="D3082" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101579.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3083">
+      <c r="A3083" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3083" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3083" t="inlineStr">
+        <is>
+          <t>コスモス薬品／京都府・静岡県に「ドラッグコスモス」計2店舗、27年4月新設</t>
+        </is>
+      </c>
+      <c r="D3083" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1015012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3084">
+      <c r="A3084" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3084" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3084" t="inlineStr">
+        <is>
+          <t>クリエイトSD／神奈川県綾瀬市に「綾瀬北上土棚店」27年4月4日新設</t>
+        </is>
+      </c>
+      <c r="D3084" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1015011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3085">
+      <c r="A3085" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3085" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3085" t="inlineStr">
+        <is>
+          <t>カインズ／ユアエルム青戸にリフォーム専門の小型店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3085" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101514.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3086">
+      <c r="A3086" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3086" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3086" t="inlineStr">
+        <is>
+          <t>アミュプラザくまもと／家具・インテリアブランド「LOWYA」の新店27年春オープン</t>
+        </is>
+      </c>
+      <c r="D3086" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101571.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3087">
+      <c r="A3087" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="B3087" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3087" t="inlineStr">
+        <is>
+          <t>京都ヨドバシ／「nana’s green tea」のテイクアウト新業態12月初旬オープン</t>
+        </is>
+      </c>
+      <c r="D3087" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101574.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-17
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3087"/>
+  <dimension ref="A1:D3145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -68330,6 +68330,1282 @@
         </is>
       </c>
     </row>
+    <row r="3088">
+      <c r="A3088" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3088" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3088" t="inlineStr">
+        <is>
+          <t>10/22業務スーパー西帯広店</t>
+        </is>
+      </c>
+      <c r="D3088" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gG7</t>
+        </is>
+      </c>
+    </row>
+    <row r="3089">
+      <c r="A3089" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3089" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3089" t="inlineStr">
+        <is>
+          <t>10/23スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D3089" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="3090">
+      <c r="A3090" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3090" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3090" t="inlineStr">
+        <is>
+          <t>ラ・ムー草津店</t>
+        </is>
+      </c>
+      <c r="D3090" t="inlineStr">
+        <is>
+          <t>https://www.dkt-s.com/map.html?id=341</t>
+        </is>
+      </c>
+    </row>
+    <row r="3091">
+      <c r="A3091" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3091" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3091" t="inlineStr">
+        <is>
+          <t>(10/19プレ)10/21コノミヤJR鴫野店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D3091" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1aBE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3092">
+      <c r="A3092" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3092" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3092" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3092" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="3093">
+      <c r="A3093" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3093" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3093" t="inlineStr">
+        <is>
+          <t>10/8建替 ツルヤなぎさ店(長野県松本市)</t>
+        </is>
+      </c>
+      <c r="D3093" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="3094">
+      <c r="A3094" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3094" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3094" t="inlineStr">
+        <is>
+          <t>10/9そよら鳥取駅南</t>
+        </is>
+      </c>
+      <c r="D3094" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gyC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3095">
+      <c r="A3095" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3095" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3095" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D3095" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="3096">
+      <c r="A3096" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3096" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3096" t="inlineStr">
+        <is>
+          <t>10/16改装 平和堂大野店（食品売場）</t>
+        </is>
+      </c>
+      <c r="D3096" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gDK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3097">
+      <c r="A3097" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3097" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3097" t="inlineStr">
+        <is>
+          <t>10/16KOmart fine長泉店</t>
+        </is>
+      </c>
+      <c r="D3097" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gFD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3098">
+      <c r="A3098" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3098" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3098" t="inlineStr">
+        <is>
+          <t>10/21ロピア加須ビバモール店(埼玉県加須市)</t>
+        </is>
+      </c>
+      <c r="D3098" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gE6</t>
+        </is>
+      </c>
+    </row>
+    <row r="3099">
+      <c r="A3099" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3099" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3099" t="inlineStr">
+        <is>
+          <t>10/27やまのぶ赤池店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3099" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1dGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3100">
+      <c r="A3100" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3100" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3100" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D3100" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3101">
+      <c r="A3101" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3101" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3101" t="inlineStr">
+        <is>
+          <t>10/30松屋可児店（松のや併設）</t>
+        </is>
+      </c>
+      <c r="D3101" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gEg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3102">
+      <c r="A3102" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3102" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3102" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D3102" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3103">
+      <c r="A3103" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3103" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3103" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D3103" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="3104">
+      <c r="A3104" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3104" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3104" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D3104" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="3105">
+      <c r="A3105" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3105" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3105" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D3105" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="3106">
+      <c r="A3106" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3106" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3106" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3106" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3107">
+      <c r="A3107" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3107" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3107" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3107" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3108">
+      <c r="A3108" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3108" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3108" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3108" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3109">
+      <c r="A3109" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3109" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3109" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3109" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3110">
+      <c r="A3110" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3110" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3110" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3110" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3111">
+      <c r="A3111" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3111" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3111" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3111" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3112">
+      <c r="A3112" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3112" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3112" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3112" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3113">
+      <c r="A3113" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3113" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3113" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3113" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3114">
+      <c r="A3114" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3114" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3114" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3114" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3115">
+      <c r="A3115" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3115" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3115" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3115" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3116">
+      <c r="A3116" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3116" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3116" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3116" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3117">
+      <c r="A3117" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3117" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3117" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3117" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3118">
+      <c r="A3118" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3118" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3118" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3118" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3119">
+      <c r="A3119" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3119" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3119" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3119" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3120">
+      <c r="A3120" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3120" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3120" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3120" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3121">
+      <c r="A3121" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3121" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3121" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3121" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3122">
+      <c r="A3122" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3122" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3122" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3122" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3123">
+      <c r="A3123" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3123" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3123" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3123" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3124">
+      <c r="A3124" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3124" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3124" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3124" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3125">
+      <c r="A3125" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3125" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3125" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3125" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3126">
+      <c r="A3126" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3126" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3126" t="inlineStr">
+        <is>
+          <t>玉川高島屋S.C.／27年3月本館食品フロア刷新、南館にサウナほか新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3126" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101673.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3127">
+      <c r="A3127" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3127" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3127" t="inlineStr">
+        <is>
+          <t>バロー／大府市に「大府北山店」10月23日オープン、愛知県70店舗目</t>
+        </is>
+      </c>
+      <c r="D3127" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101612.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3128">
+      <c r="A3128" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3128" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3128" t="inlineStr">
+        <is>
+          <t>野村不動産／東京・門前仲町で住宅・商業複合施設を開発</t>
+        </is>
+      </c>
+      <c r="D3128" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101613.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3129">
+      <c r="A3129" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3129" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3129" t="inlineStr">
+        <is>
+          <t>イオン北海道／「ザ・ビッグ千歳武道館前店」10月23日オープン</t>
+        </is>
+      </c>
+      <c r="D3129" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101615.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3130">
+      <c r="A3130" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3130" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3130" t="inlineStr">
+        <is>
+          <t>京阪HD／京都府に「三条PJ本館新築工事（店舗面積6895m2）」27年5月1日新設</t>
+        </is>
+      </c>
+      <c r="D3130" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1016011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3131">
+      <c r="A3131" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3131" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3131" t="inlineStr">
+        <is>
+          <t>コスモス薬品／栃木県・新潟県に「ドラッグコスモス」計2店舗、27年5月新設</t>
+        </is>
+      </c>
+      <c r="D3131" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1016012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3132">
+      <c r="A3132" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3132" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3132" t="inlineStr">
+        <is>
+          <t>串カツ田中／全国制覇達成「串カツ田中 和歌山駅前店」10月23日オープン</t>
+        </is>
+      </c>
+      <c r="D3132" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101681.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3133">
+      <c r="A3133" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3133" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3133" t="inlineStr">
+        <is>
+          <t>コメダ／愛知県安城市に「おかげ庵」12月オープン</t>
+        </is>
+      </c>
+      <c r="D3133" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101616.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3134">
+      <c r="A3134" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3134" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3134" t="inlineStr">
+        <is>
+          <t>ミズノ／「ミズノ大阪心斎橋」10月23日オープン、若年層・インバウンドに照準</t>
+        </is>
+      </c>
+      <c r="D3134" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101672.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3135">
+      <c r="A3135" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3135" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3135" t="inlineStr">
+        <is>
+          <t>東急百貨店たまプラーザ店／「メンズビギ」の新店舗オープン、限定アイテムも販売</t>
+        </is>
+      </c>
+      <c r="D3135" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101680.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3136">
+      <c r="A3136" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3136" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3136" t="inlineStr">
+        <is>
+          <t>ゴンチャ／銀座・有楽町エリア初出店「ルミネ有楽町店」10月23日オープン</t>
+        </is>
+      </c>
+      <c r="D3136" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101674.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3137">
+      <c r="A3137" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3137" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3137" t="inlineStr">
+        <is>
+          <t>サンマルクカフェ＆茶／東京都墨田区に「両国東口店」10月21日オープン</t>
+        </is>
+      </c>
+      <c r="D3137" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101675.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3138">
+      <c r="A3138" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3138" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3138" t="inlineStr">
+        <is>
+          <t>西武池袋本店／11～12月の7・8階リニューアルで新百貨店モデルが完成</t>
+        </is>
+      </c>
+      <c r="D3138" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101515.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3139">
+      <c r="A3139" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3139" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3139" t="inlineStr">
+        <is>
+          <t>大丸梅田店／新ストアコンセプト発表、27年春3フロアを先行リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D3139" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101577.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3140">
+      <c r="A3140" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3140" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3140" t="inlineStr">
+        <is>
+          <t>エキュート大宮／今秋「銀座おのでら」の新業態含む9店舗が順次オープン</t>
+        </is>
+      </c>
+      <c r="D3140" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101579.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3141">
+      <c r="A3141" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3141" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3141" t="inlineStr">
+        <is>
+          <t>コスモス薬品／京都府・静岡県に「ドラッグコスモス」計2店舗、27年4月新設</t>
+        </is>
+      </c>
+      <c r="D3141" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1015012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3142">
+      <c r="A3142" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3142" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3142" t="inlineStr">
+        <is>
+          <t>クリエイトSD／神奈川県綾瀬市に「綾瀬北上土棚店」27年4月4日新設</t>
+        </is>
+      </c>
+      <c r="D3142" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1015011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3143">
+      <c r="A3143" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3143" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3143" t="inlineStr">
+        <is>
+          <t>カインズ／ユアエルム青戸にリフォーム専門の小型店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3143" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101514.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3144">
+      <c r="A3144" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3144" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3144" t="inlineStr">
+        <is>
+          <t>アミュプラザくまもと／家具・インテリアブランド「LOWYA」の新店27年春オープン</t>
+        </is>
+      </c>
+      <c r="D3144" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101571.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3145">
+      <c r="A3145" t="inlineStr">
+        <is>
+          <t>2026年10月17日</t>
+        </is>
+      </c>
+      <c r="B3145" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3145" t="inlineStr">
+        <is>
+          <t>京都ヨドバシ／「nana’s green tea」のテイクアウト新業態12月初旬オープン</t>
+        </is>
+      </c>
+      <c r="D3145" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101574.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-18
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3145"/>
+  <dimension ref="A1:D3223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -69606,6 +69606,1722 @@
         </is>
       </c>
     </row>
+    <row r="3146">
+      <c r="A3146" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3146" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3146" t="inlineStr">
+        <is>
+          <t>10/21魚市場食堂平の屋(愛知県岡崎市)</t>
+        </is>
+      </c>
+      <c r="D3146" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gGK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3147">
+      <c r="A3147" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3147" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3147" t="inlineStr">
+        <is>
+          <t>(10/20プレ)10/21スーパーセンタートライアル愛知川店</t>
+        </is>
+      </c>
+      <c r="D3147" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gHm</t>
+        </is>
+      </c>
+    </row>
+    <row r="3148">
+      <c r="A3148" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3148" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3148" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3148" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="3149">
+      <c r="A3149" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3149" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3149" t="inlineStr">
+        <is>
+          <t>10/8建替 ツルヤなぎさ店(長野県松本市)</t>
+        </is>
+      </c>
+      <c r="D3149" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="3150">
+      <c r="A3150" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3150" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3150" t="inlineStr">
+        <is>
+          <t>10/9そよら鳥取駅南</t>
+        </is>
+      </c>
+      <c r="D3150" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gyC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3151">
+      <c r="A3151" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3151" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3151" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D3151" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="3152">
+      <c r="A3152" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3152" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3152" t="inlineStr">
+        <is>
+          <t>10/16KOmart fine長泉店</t>
+        </is>
+      </c>
+      <c r="D3152" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gFD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3153">
+      <c r="A3153" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3153" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3153" t="inlineStr">
+        <is>
+          <t>10/16改装 平和堂大野店（食品売場）</t>
+        </is>
+      </c>
+      <c r="D3153" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gDK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3154">
+      <c r="A3154" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3154" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3154" t="inlineStr">
+        <is>
+          <t>10/21ロピア加須ビバモール店(埼玉県加須市)</t>
+        </is>
+      </c>
+      <c r="D3154" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gE6</t>
+        </is>
+      </c>
+    </row>
+    <row r="3155">
+      <c r="A3155" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3155" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3155" t="inlineStr">
+        <is>
+          <t>10/22業務スーパー西帯広店</t>
+        </is>
+      </c>
+      <c r="D3155" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gG7</t>
+        </is>
+      </c>
+    </row>
+    <row r="3156">
+      <c r="A3156" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3156" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3156" t="inlineStr">
+        <is>
+          <t>10/23スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D3156" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="3157">
+      <c r="A3157" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3157" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3157" t="inlineStr">
+        <is>
+          <t>10/27やまのぶ赤池店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3157" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1dGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3158">
+      <c r="A3158" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3158" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3158" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D3158" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3159">
+      <c r="A3159" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3159" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3159" t="inlineStr">
+        <is>
+          <t>10/30松屋可児店（松のや併設）</t>
+        </is>
+      </c>
+      <c r="D3159" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gEg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3160">
+      <c r="A3160" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3160" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3160" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D3160" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3161">
+      <c r="A3161" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3161" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3161" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D3161" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="3162">
+      <c r="A3162" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3162" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3162" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D3162" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="3163">
+      <c r="A3163" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3163" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3163" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D3163" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="3164">
+      <c r="A3164" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3164" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3164" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3164" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3165">
+      <c r="A3165" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3165" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3165" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3165" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3166">
+      <c r="A3166" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3166" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3166" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3166" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3167">
+      <c r="A3167" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3167" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3167" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3167" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3168">
+      <c r="A3168" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3168" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3168" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3168" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3169">
+      <c r="A3169" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3169" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3169" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3169" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3170">
+      <c r="A3170" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3170" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3170" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3170" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3171">
+      <c r="A3171" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3171" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3171" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3171" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3172">
+      <c r="A3172" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3172" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3172" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3172" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3173">
+      <c r="A3173" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3173" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3173" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3173" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3174">
+      <c r="A3174" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3174" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3174" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3174" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3175">
+      <c r="A3175" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3175" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3175" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3175" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3176">
+      <c r="A3176" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3176" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3176" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3176" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3177">
+      <c r="A3177" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3177" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3177" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3177" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3178">
+      <c r="A3178" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3178" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3178" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3178" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3179">
+      <c r="A3179" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3179" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3179" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3179" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3180">
+      <c r="A3180" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3180" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3180" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3180" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3181">
+      <c r="A3181" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3181" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3181" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3181" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3182">
+      <c r="A3182" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3182" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3182" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3182" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3183">
+      <c r="A3183" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3183" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3183" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3183" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3184">
+      <c r="A3184" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3184" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3184" t="inlineStr">
+        <is>
+          <t>関西地方コメリパワー平群店 2025年7月16日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3184" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39836</t>
+        </is>
+      </c>
+    </row>
+    <row r="3185">
+      <c r="A3185" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3185" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3185" t="inlineStr">
+        <is>
+          <t>中部地方ベルク町田相原店 2026年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3185" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/47130</t>
+        </is>
+      </c>
+    </row>
+    <row r="3186">
+      <c r="A3186" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3186" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3186" t="inlineStr">
+        <is>
+          <t>中国地方ゆめモール山陽 2025年6月12日(木)開業！全14テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3186" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/35608</t>
+        </is>
+      </c>
+    </row>
+    <row r="3187">
+      <c r="A3187" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3187" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3187" t="inlineStr">
+        <is>
+          <t>関西地方ハローズ伊川谷店 2026年2月7日(土)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3187" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39546</t>
+        </is>
+      </c>
+    </row>
+    <row r="3188">
+      <c r="A3188" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3188" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3188" t="inlineStr">
+        <is>
+          <t>関東地方WORLD TOWER RESIDENCE 2026年12月完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3188" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/19463</t>
+        </is>
+      </c>
+    </row>
+    <row r="3189">
+      <c r="A3189" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3189" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3189" t="inlineStr">
+        <is>
+          <t>関東地方ヤオコー岩槻本丸店 2025年10月29日(水)9時~開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3189" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/39888</t>
+        </is>
+      </c>
+    </row>
+    <row r="3190">
+      <c r="A3190" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3190" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3190" t="inlineStr">
+        <is>
+          <t>中部地方そよら飯田アップルロード 2025年7月18日(金)開業！全30店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3190" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/40463</t>
+        </is>
+      </c>
+    </row>
+    <row r="3191">
+      <c r="A3191" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3191" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3191" t="inlineStr">
+        <is>
+          <t>関西地方そよら長原駅前 2025年4月28日(月)開業！全15店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3191" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/31820</t>
+        </is>
+      </c>
+    </row>
+    <row r="3192">
+      <c r="A3192" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3192" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3192" t="inlineStr">
+        <is>
+          <t>関西地方イオン姫路店 2026年8月末で一旦閉店し建て替えへ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3192" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49763</t>
+        </is>
+      </c>
+    </row>
+    <row r="3193">
+      <c r="A3193" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3193" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3193" t="inlineStr">
+        <is>
+          <t>関東地方ケーズデンキ厚木妻田東店 2027年春に開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3193" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47111</t>
+        </is>
+      </c>
+    </row>
+    <row r="3194">
+      <c r="A3194" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3194" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3194" t="inlineStr">
+        <is>
+          <t>関西地方ケーズデンキ桜井店 2026年9月17日(木)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3194" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49275</t>
+        </is>
+      </c>
+    </row>
+    <row r="3195">
+      <c r="A3195" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3195" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3195" t="inlineStr">
+        <is>
+          <t>中部地方スーパーセンタートライアル名古屋みなと店 2027年2月上旬に開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3195" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48009</t>
+        </is>
+      </c>
+    </row>
+    <row r="3196">
+      <c r="A3196" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3196" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3196" t="inlineStr">
+        <is>
+          <t>関東地方ベルク古河中田店 2026年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3196" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47848</t>
+        </is>
+      </c>
+    </row>
+    <row r="3197">
+      <c r="A3197" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3197" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3197" t="inlineStr">
+        <is>
+          <t>東北地方ヨークタウン富久山 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3197" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/49459</t>
+        </is>
+      </c>
+    </row>
+    <row r="3198">
+      <c r="A3198" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3198" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3198" t="inlineStr">
+        <is>
+          <t>中部地方三郷駅前地区市街地再開発事業 2029年春完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3198" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/24605</t>
+        </is>
+      </c>
+    </row>
+    <row r="3199">
+      <c r="A3199" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3199" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3199" t="inlineStr">
+        <is>
+          <t>中部地方フォレストモール東海太田川 2026年4月16日(木)開業！全13テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3199" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/39446</t>
+        </is>
+      </c>
+    </row>
+    <row r="3200">
+      <c r="A3200" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3200" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3200" t="inlineStr">
+        <is>
+          <t>関東地方ニトリふじみ野店 2026年10月開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3200" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48589</t>
+        </is>
+      </c>
+    </row>
+    <row r="3201">
+      <c r="A3201" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3201" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3201" t="inlineStr">
+        <is>
+          <t>中部地方カインズ岡崎美合店 2025年10月23日(木)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3201" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/39138</t>
+        </is>
+      </c>
+    </row>
+    <row r="3202">
+      <c r="A3202" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3202" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3202" t="inlineStr">
+        <is>
+          <t>中部地方イオンスタイル諏訪 2026年10月21日(水)開業！全5テナント一覧！最新情報も！長野県諏訪郡下諏訪町の「イオン諏訪店」跡地に、イオンリテールの新商業施設「イオンスタイル諏訪」が2026年10月21日(水)グランドオープン！旧イオン諏訪店の閉店から約8年、待望の新店舗が2026年10月21日（水）に開業決定！平屋建ての「...2026.10.18中部地方</t>
+        </is>
+      </c>
+      <c r="D3202" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/36918</t>
+        </is>
+      </c>
+    </row>
+    <row r="3203">
+      <c r="A3203" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3203" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3203" t="inlineStr">
+        <is>
+          <t>九州地方旦過市場いちばん館 2026年11月24日~順次開業！テナントは？最新情報も！福岡県北九州市小倉北区の市場「旦過市場」が再開発・再整備され、新たな市場（商業棟）「旦過市場いちばん館」として2026年11月24日以降順次開業予定です！旦過市場の再開発により、1階には市場店舗が入り、2階には北九州の食文化を体験できる約2...2026.10.18九州地方</t>
+        </is>
+      </c>
+      <c r="D3203" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/47032</t>
+        </is>
+      </c>
+    </row>
+    <row r="3204">
+      <c r="A3204" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3204" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3204" t="inlineStr">
+        <is>
+          <t>玉川高島屋S.C.／27年3月本館食品フロア刷新、南館にサウナほか新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3204" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101673.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3205">
+      <c r="A3205" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3205" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3205" t="inlineStr">
+        <is>
+          <t>バロー／大府市に「大府北山店」10月23日オープン、愛知県70店舗目</t>
+        </is>
+      </c>
+      <c r="D3205" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101612.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3206">
+      <c r="A3206" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3206" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3206" t="inlineStr">
+        <is>
+          <t>野村不動産／東京・門前仲町で住宅・商業複合施設を開発</t>
+        </is>
+      </c>
+      <c r="D3206" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101613.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3207">
+      <c r="A3207" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3207" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3207" t="inlineStr">
+        <is>
+          <t>イオン北海道／「ザ・ビッグ千歳武道館前店」10月23日オープン</t>
+        </is>
+      </c>
+      <c r="D3207" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101615.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3208">
+      <c r="A3208" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3208" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3208" t="inlineStr">
+        <is>
+          <t>京阪HD／京都府に「三条PJ本館新築工事（店舗面積6895m2）」27年5月1日新設</t>
+        </is>
+      </c>
+      <c r="D3208" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1016011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3209">
+      <c r="A3209" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3209" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3209" t="inlineStr">
+        <is>
+          <t>コスモス薬品／栃木県・新潟県に「ドラッグコスモス」計2店舗、27年5月新設</t>
+        </is>
+      </c>
+      <c r="D3209" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1016012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3210">
+      <c r="A3210" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3210" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3210" t="inlineStr">
+        <is>
+          <t>串カツ田中／全国制覇達成「串カツ田中 和歌山駅前店」10月23日オープン</t>
+        </is>
+      </c>
+      <c r="D3210" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101681.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3211">
+      <c r="A3211" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3211" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3211" t="inlineStr">
+        <is>
+          <t>コメダ／愛知県安城市に「おかげ庵」12月オープン</t>
+        </is>
+      </c>
+      <c r="D3211" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101616.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3212">
+      <c r="A3212" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3212" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3212" t="inlineStr">
+        <is>
+          <t>ミズノ／「ミズノ大阪心斎橋」10月23日オープン、若年層・インバウンドに照準</t>
+        </is>
+      </c>
+      <c r="D3212" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101672.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3213">
+      <c r="A3213" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3213" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3213" t="inlineStr">
+        <is>
+          <t>東急百貨店たまプラーザ店／「メンズビギ」の新店舗オープン、限定アイテムも販売</t>
+        </is>
+      </c>
+      <c r="D3213" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101680.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3214">
+      <c r="A3214" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3214" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3214" t="inlineStr">
+        <is>
+          <t>ゴンチャ／銀座・有楽町エリア初出店「ルミネ有楽町店」10月23日オープン</t>
+        </is>
+      </c>
+      <c r="D3214" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101674.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3215">
+      <c r="A3215" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3215" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3215" t="inlineStr">
+        <is>
+          <t>サンマルクカフェ＆茶／東京都墨田区に「両国東口店」10月21日オープン</t>
+        </is>
+      </c>
+      <c r="D3215" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101675.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3216">
+      <c r="A3216" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3216" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3216" t="inlineStr">
+        <is>
+          <t>西武池袋本店／11～12月の7・8階リニューアルで新百貨店モデルが完成</t>
+        </is>
+      </c>
+      <c r="D3216" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101515.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3217">
+      <c r="A3217" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3217" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3217" t="inlineStr">
+        <is>
+          <t>大丸梅田店／新ストアコンセプト発表、27年春3フロアを先行リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D3217" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101577.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3218">
+      <c r="A3218" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3218" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3218" t="inlineStr">
+        <is>
+          <t>エキュート大宮／今秋「銀座おのでら」の新業態含む9店舗が順次オープン</t>
+        </is>
+      </c>
+      <c r="D3218" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101579.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3219">
+      <c r="A3219" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3219" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3219" t="inlineStr">
+        <is>
+          <t>コスモス薬品／京都府・静岡県に「ドラッグコスモス」計2店舗、27年4月新設</t>
+        </is>
+      </c>
+      <c r="D3219" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1015012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3220">
+      <c r="A3220" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3220" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3220" t="inlineStr">
+        <is>
+          <t>クリエイトSD／神奈川県綾瀬市に「綾瀬北上土棚店」27年4月4日新設</t>
+        </is>
+      </c>
+      <c r="D3220" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1015011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3221">
+      <c r="A3221" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3221" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3221" t="inlineStr">
+        <is>
+          <t>カインズ／ユアエルム青戸にリフォーム専門の小型店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3221" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101514.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3222">
+      <c r="A3222" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3222" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3222" t="inlineStr">
+        <is>
+          <t>アミュプラザくまもと／家具・インテリアブランド「LOWYA」の新店27年春オープン</t>
+        </is>
+      </c>
+      <c r="D3222" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101571.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3223">
+      <c r="A3223" t="inlineStr">
+        <is>
+          <t>2026年10月18日</t>
+        </is>
+      </c>
+      <c r="B3223" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3223" t="inlineStr">
+        <is>
+          <t>京都ヨドバシ／「nana’s green tea」のテイクアウト新業態12月初旬オープン</t>
+        </is>
+      </c>
+      <c r="D3223" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101574.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-19
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3223"/>
+  <dimension ref="A1:D3283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -71322,6 +71322,1326 @@
         </is>
       </c>
     </row>
+    <row r="3224">
+      <c r="A3224" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3224" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3224" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3224" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3225">
+      <c r="A3225" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3225" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3225" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3225" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3226">
+      <c r="A3226" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3226" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3226" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3226" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3227">
+      <c r="A3227" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3227" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3227" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3227" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3228">
+      <c r="A3228" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3228" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3228" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3228" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3229">
+      <c r="A3229" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3229" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3229" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3229" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3230">
+      <c r="A3230" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3230" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3230" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3230" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3231">
+      <c r="A3231" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3231" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3231" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3231" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3232">
+      <c r="A3232" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3232" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3232" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3232" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3233">
+      <c r="A3233" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3233" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3233" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3233" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3234">
+      <c r="A3234" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3234" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3234" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3234" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3235">
+      <c r="A3235" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3235" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3235" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3235" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3236">
+      <c r="A3236" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3236" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3236" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3236" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3237">
+      <c r="A3237" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3237" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3237" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3237" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3238">
+      <c r="A3238" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3238" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3238" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3238" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3239">
+      <c r="A3239" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3239" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3239" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3239" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3240">
+      <c r="A3240" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3240" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3240" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3240" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3241">
+      <c r="A3241" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3241" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3241" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3241" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3242">
+      <c r="A3242" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3242" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3242" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3242" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3243">
+      <c r="A3243" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3243" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3243" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3243" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3244">
+      <c r="A3244" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3244" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3244" t="inlineStr">
+        <is>
+          <t>関東地方フォレストスクエア仙川 2025年12月9日(火)開業！全16テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3244" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42193</t>
+        </is>
+      </c>
+    </row>
+    <row r="3245">
+      <c r="A3245" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3245" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3245" t="inlineStr">
+        <is>
+          <t>関東地方宇都宮Yo-To BASE 2028年春開業！ベルクが出店へ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3245" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48277</t>
+        </is>
+      </c>
+    </row>
+    <row r="3246">
+      <c r="A3246" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3246" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3246" t="inlineStr">
+        <is>
+          <t>関西地方高槻グリーンプレイス 2025年5月1日(木)開業！12店舗が出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3246" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/38803</t>
+        </is>
+      </c>
+    </row>
+    <row r="3247">
+      <c r="A3247" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3247" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3247" t="inlineStr">
+        <is>
+          <t>関西地方Kubota field(クボタフィールド) 2032年以降開業予定！クボタららアリーナや商業施設が誕生！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3247" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49228</t>
+        </is>
+      </c>
+    </row>
+    <row r="3248">
+      <c r="A3248" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3248" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3248" t="inlineStr">
+        <is>
+          <t>中部地方イオンタウン松阪船江 2025年4月25日(金)開業！全31テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3248" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/28643</t>
+        </is>
+      </c>
+    </row>
+    <row r="3249">
+      <c r="A3249" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3249" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3249" t="inlineStr">
+        <is>
+          <t>関東地方アクロスプラザ宇都宮インターパーク 2025年10月3日(木)10時~順次開業！全5テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3249" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/39701</t>
+        </is>
+      </c>
+    </row>
+    <row r="3250">
+      <c r="A3250" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3250" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3250" t="inlineStr">
+        <is>
+          <t>中部地方牧之原ヒルズプロジェクト 商業施設も誕生！2028年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3250" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/47123</t>
+        </is>
+      </c>
+    </row>
+    <row r="3251">
+      <c r="A3251" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3251" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3251" t="inlineStr">
+        <is>
+          <t>関東地方取手駅西口A街区市街地再開発事業 2031年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3251" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/22823</t>
+        </is>
+      </c>
+    </row>
+    <row r="3252">
+      <c r="A3252" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3252" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3252" t="inlineStr">
+        <is>
+          <t>関東地方コープ幕張駅北口店 2025年2月25日(火)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3252" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/39459</t>
+        </is>
+      </c>
+    </row>
+    <row r="3253">
+      <c r="A3253" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3253" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3253" t="inlineStr">
+        <is>
+          <t>関東地方(仮称)小杉町一丁目計画 武蔵小杉駅北口 タワマンと商業施設に！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3253" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/35200</t>
+        </is>
+      </c>
+    </row>
+    <row r="3254">
+      <c r="A3254" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3254" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3254" t="inlineStr">
+        <is>
+          <t>関東地方ニュウマン高輪 2025年9月12日(金)開業！テナント164店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3254" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/40621</t>
+        </is>
+      </c>
+    </row>
+    <row r="3255">
+      <c r="A3255" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3255" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3255" t="inlineStr">
+        <is>
+          <t>関東地方ハーモニーヒルズパーク入間 ベルクと屋上公園 2028年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3255" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/45967</t>
+        </is>
+      </c>
+    </row>
+    <row r="3256">
+      <c r="A3256" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3256" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3256" t="inlineStr">
+        <is>
+          <t>関東地方ミライト一条 2025年5月30日(金)9時~開業！一条中学校跡地 テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3256" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/29186</t>
+        </is>
+      </c>
+    </row>
+    <row r="3257">
+      <c r="A3257" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3257" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3257" t="inlineStr">
+        <is>
+          <t>関東地方TAIRAYA与野店 与野フード建て替え 2025年4月24日(木)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3257" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/37854</t>
+        </is>
+      </c>
+    </row>
+    <row r="3258">
+      <c r="A3258" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3258" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3258" t="inlineStr">
+        <is>
+          <t>関東地方藤沢駅南口391地区市街地再開発事業 2035年完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3258" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/32666</t>
+        </is>
+      </c>
+    </row>
+    <row r="3259">
+      <c r="A3259" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3259" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3259" t="inlineStr">
+        <is>
+          <t>関東地方ヤオコーまるひろ上尾SC 2025年9月12日(金)開業！全テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3259" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42379</t>
+        </is>
+      </c>
+    </row>
+    <row r="3260">
+      <c r="A3260" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3260" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3260" t="inlineStr">
+        <is>
+          <t>九州地方スーパーセンタートライアル阿蘇店 2026年11月中旬に開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3260" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/48550</t>
+        </is>
+      </c>
+    </row>
+    <row r="3261">
+      <c r="A3261" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3261" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3261" t="inlineStr">
+        <is>
+          <t>九州地方OHASHI HILL ゆめアール大橋跡地に2025年4月18日(金)先行開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3261" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/27364</t>
+        </is>
+      </c>
+    </row>
+    <row r="3262">
+      <c r="A3262" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3262" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3262" t="inlineStr">
+        <is>
+          <t>中部地方イオンスタイル諏訪 2026年10月21日(水)開業！全5テナント一覧！最新情報も！長野県諏訪郡下諏訪町の「イオン諏訪店」跡地に、イオンリテールの新商業施設「イオンスタイル諏訪」が2026年10月21日(水)グランドオープン！旧イオン諏訪店の閉店から約8年、待望の新店舗が2026年10月21日（水）に開業決定！平屋建ての「...2026.10.18中部地方</t>
+        </is>
+      </c>
+      <c r="D3262" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/36918</t>
+        </is>
+      </c>
+    </row>
+    <row r="3263">
+      <c r="A3263" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3263" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3263" t="inlineStr">
+        <is>
+          <t>九州地方旦過市場いちばん館 2026年11月24日~順次開業！テナントは？最新情報も！福岡県北九州市小倉北区の市場「旦過市場」が再開発・再整備され、新たな市場（商業棟）「旦過市場いちばん館」として2026年11月24日以降順次開業予定です！旦過市場の再開発により、1階には市場店舗が入り、2階には北九州の食文化を体験できる約2...2026.10.18九州地方</t>
+        </is>
+      </c>
+      <c r="D3263" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/47032</t>
+        </is>
+      </c>
+    </row>
+    <row r="3264">
+      <c r="A3264" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3264" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3264" t="inlineStr">
+        <is>
+          <t>明治屋／東京・広尾の旗艦店「明治屋広尾ストアー」10月30日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D3264" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101945.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3265">
+      <c r="A3265" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3265" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3265" t="inlineStr">
+        <is>
+          <t>コメダ／DXモデル店舗「コメダ珈琲店 板橋仲宿店」オープン、レジで注文式に</t>
+        </is>
+      </c>
+      <c r="D3265" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101912.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3266">
+      <c r="A3266" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3266" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3266" t="inlineStr">
+        <is>
+          <t>マミーマート／群馬県「生鮮市場TOPガーデン前橋店」リニューアルオープン、日用品を新規導入</t>
+        </is>
+      </c>
+      <c r="D3266" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101916.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3267">
+      <c r="A3267" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3267" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3267" t="inlineStr">
+        <is>
+          <t>JR東海／「アスティ静岡」11月18日リニューアル、治一郎など4店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3267" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101978.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3268">
+      <c r="A3268" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3268" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3268" t="inlineStr">
+        <is>
+          <t>マミーマートほか／埼玉県川口市に「（仮称）川口市上青木プロジェクト（店舗面積3054m2）」27年5月4日新設</t>
+        </is>
+      </c>
+      <c r="D3268" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1019011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3269">
+      <c r="A3269" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3269" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3269" t="inlineStr">
+        <is>
+          <t>コスモス薬品／岡山県・宮崎県に「ドラッグコスモス」計2店舗、27年5月新設</t>
+        </is>
+      </c>
+      <c r="D3269" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1019012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3270">
+      <c r="A3270" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3270" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3270" t="inlineStr">
+        <is>
+          <t>エディオン／兵庫県尼崎市「エディオン塚口店」11月13日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D3270" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101944.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3271">
+      <c r="A3271" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3271" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3271" t="inlineStr">
+        <is>
+          <t>相鉄／シャトレーゼのフランチャイズ事業に参入「横浜片倉町店」10月26日オープン</t>
+        </is>
+      </c>
+      <c r="D3271" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101972.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3272">
+      <c r="A3272" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3272" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3272" t="inlineStr">
+        <is>
+          <t>ローソン／九州で車中泊サービス「RVパーク」開始</t>
+        </is>
+      </c>
+      <c r="D3272" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101913.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3273">
+      <c r="A3273" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3273" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3273" t="inlineStr">
+        <is>
+          <t>シェイク シャック／東京・新宿「明治安田新宿ビル」に新店舗11月28日オープン</t>
+        </is>
+      </c>
+      <c r="D3273" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101974.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3274">
+      <c r="A3274" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3274" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3274" t="inlineStr">
+        <is>
+          <t>ニラックス／「イタリアン リゾート ペルティカ 多摩境店」10月30日オープン</t>
+        </is>
+      </c>
+      <c r="D3274" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101976.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3275">
+      <c r="A3275" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3275" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3275" t="inlineStr">
+        <is>
+          <t>金沢フォーラス／開業20周年キャンペーン実施、NiziU・MAYAさんとのコラボも</t>
+        </is>
+      </c>
+      <c r="D3275" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101914.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3276">
+      <c r="A3276" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3276" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3276" t="inlineStr">
+        <is>
+          <t>スープストックトーキョー／東京都「アトレ中野店」12月9日オープン</t>
+        </is>
+      </c>
+      <c r="D3276" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101977.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3277">
+      <c r="A3277" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3277" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3277" t="inlineStr">
+        <is>
+          <t>コープながの／「コープ安曇野豊科店」10月23日リニューアル、地元の食を強化</t>
+        </is>
+      </c>
+      <c r="D3277" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101973.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3278">
+      <c r="A3278" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3278" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3278" t="inlineStr">
+        <is>
+          <t>玉川高島屋S.C.／27年3月本館食品フロア刷新、南館にサウナほか新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3278" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101673.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3279">
+      <c r="A3279" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3279" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3279" t="inlineStr">
+        <is>
+          <t>バロー／大府市に「大府北山店」10月23日オープン、愛知県70店舗目</t>
+        </is>
+      </c>
+      <c r="D3279" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101612.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3280">
+      <c r="A3280" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3280" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3280" t="inlineStr">
+        <is>
+          <t>野村不動産／東京・門前仲町で住宅・商業複合施設を開発</t>
+        </is>
+      </c>
+      <c r="D3280" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101613.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3281">
+      <c r="A3281" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3281" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3281" t="inlineStr">
+        <is>
+          <t>イオン北海道／「ザ・ビッグ千歳武道館前店」10月23日オープン</t>
+        </is>
+      </c>
+      <c r="D3281" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101615.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3282">
+      <c r="A3282" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3282" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3282" t="inlineStr">
+        <is>
+          <t>京阪HD／京都府に「三条PJ本館新築工事（店舗面積6895m2）」27年5月1日新設</t>
+        </is>
+      </c>
+      <c r="D3282" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1016011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3283">
+      <c r="A3283" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3283" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3283" t="inlineStr">
+        <is>
+          <t>コスモス薬品／栃木県・新潟県に「ドラッグコスモス」計2店舗、27年5月新設</t>
+        </is>
+      </c>
+      <c r="D3283" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1016012.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-20
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3283"/>
+  <dimension ref="A1:D3362"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -72642,6 +72642,1744 @@
         </is>
       </c>
     </row>
+    <row r="3284">
+      <c r="A3284" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3284" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3284" t="inlineStr">
+        <is>
+          <t>10/21ベルク太田駅前店(群馬県太田市)</t>
+        </is>
+      </c>
+      <c r="D3284" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gJJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3285">
+      <c r="A3285" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3285" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3285" t="inlineStr">
+        <is>
+          <t>(10/20プレ)10/21スーパーセンタートライアル愛知川店</t>
+        </is>
+      </c>
+      <c r="D3285" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gHm</t>
+        </is>
+      </c>
+    </row>
+    <row r="3286">
+      <c r="A3286" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3286" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3286" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3286" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="3287">
+      <c r="A3287" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3287" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3287" t="inlineStr">
+        <is>
+          <t>10/8建替 ツルヤなぎさ店(長野県松本市)</t>
+        </is>
+      </c>
+      <c r="D3287" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="3288">
+      <c r="A3288" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3288" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3288" t="inlineStr">
+        <is>
+          <t>10/9そよら鳥取駅南</t>
+        </is>
+      </c>
+      <c r="D3288" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gyC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3289">
+      <c r="A3289" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3289" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3289" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D3289" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="3290">
+      <c r="A3290" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3290" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3290" t="inlineStr">
+        <is>
+          <t>10/16KOmart fine長泉店</t>
+        </is>
+      </c>
+      <c r="D3290" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gFD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3291">
+      <c r="A3291" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3291" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3291" t="inlineStr">
+        <is>
+          <t>10/16改装 平和堂大野店（食品売場）</t>
+        </is>
+      </c>
+      <c r="D3291" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gDK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3292">
+      <c r="A3292" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3292" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3292" t="inlineStr">
+        <is>
+          <t>10/21魚市場食堂平の屋(愛知県岡崎市)</t>
+        </is>
+      </c>
+      <c r="D3292" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gGK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3293">
+      <c r="A3293" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3293" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3293" t="inlineStr">
+        <is>
+          <t>10/21ロピア加須ビバモール店(埼玉県加須市)</t>
+        </is>
+      </c>
+      <c r="D3293" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gE6</t>
+        </is>
+      </c>
+    </row>
+    <row r="3294">
+      <c r="A3294" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3294" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3294" t="inlineStr">
+        <is>
+          <t>10/22業務スーパー西帯広店</t>
+        </is>
+      </c>
+      <c r="D3294" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gG7</t>
+        </is>
+      </c>
+    </row>
+    <row r="3295">
+      <c r="A3295" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3295" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3295" t="inlineStr">
+        <is>
+          <t>10/23スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D3295" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="3296">
+      <c r="A3296" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3296" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3296" t="inlineStr">
+        <is>
+          <t>10/27やまのぶ赤池店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3296" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1dGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3297">
+      <c r="A3297" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3297" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3297" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D3297" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3298">
+      <c r="A3298" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3298" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3298" t="inlineStr">
+        <is>
+          <t>10/30松屋可児店（松のや併設）</t>
+        </is>
+      </c>
+      <c r="D3298" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gEg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3299">
+      <c r="A3299" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3299" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3299" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D3299" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3300">
+      <c r="A3300" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3300" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3300" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D3300" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="3301">
+      <c r="A3301" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3301" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3301" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D3301" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="3302">
+      <c r="A3302" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3302" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3302" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D3302" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="3303">
+      <c r="A3303" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3303" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3303" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3303" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3304">
+      <c r="A3304" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3304" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3304" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3304" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3305">
+      <c r="A3305" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3305" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3305" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3305" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3306">
+      <c r="A3306" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3306" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3306" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3306" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3307">
+      <c r="A3307" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3307" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3307" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3307" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3308">
+      <c r="A3308" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3308" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3308" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3308" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3309">
+      <c r="A3309" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3309" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3309" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3309" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3310">
+      <c r="A3310" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3310" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3310" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3310" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3311">
+      <c r="A3311" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3311" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3311" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3311" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3312">
+      <c r="A3312" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3312" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3312" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3312" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3313">
+      <c r="A3313" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3313" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3313" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3313" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3314">
+      <c r="A3314" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3314" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3314" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3314" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3315">
+      <c r="A3315" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3315" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3315" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3315" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3316">
+      <c r="A3316" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3316" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3316" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3316" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3317">
+      <c r="A3317" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3317" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3317" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3317" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3318">
+      <c r="A3318" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3318" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3318" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3318" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3319">
+      <c r="A3319" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3319" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3319" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3319" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3320">
+      <c r="A3320" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3320" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3320" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3320" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3321">
+      <c r="A3321" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3321" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3321" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3321" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3322">
+      <c r="A3322" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3322" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3322" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3322" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3323">
+      <c r="A3323" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3323" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3323" t="inlineStr">
+        <is>
+          <t>関東地方逗子駅ビル 2028年春開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3323" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49835</t>
+        </is>
+      </c>
+    </row>
+    <row r="3324">
+      <c r="A3324" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3324" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3324" t="inlineStr">
+        <is>
+          <t>東北地方イオンモール仙台上杉 2025年10月8日(水)開業！全テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3324" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/2380</t>
+        </is>
+      </c>
+    </row>
+    <row r="3325">
+      <c r="A3325" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3325" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3325" t="inlineStr">
+        <is>
+          <t>中部地方知立西新地地区市街地再開発事業 2029年度完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3325" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/37537</t>
+        </is>
+      </c>
+    </row>
+    <row r="3326">
+      <c r="A3326" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3326" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3326" t="inlineStr">
+        <is>
+          <t>東北地方ヨークタウン富久山 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3326" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/49459</t>
+        </is>
+      </c>
+    </row>
+    <row r="3327">
+      <c r="A3327" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3327" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3327" t="inlineStr">
+        <is>
+          <t>関東地方マミーマート 見沼区東新井 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3327" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47301</t>
+        </is>
+      </c>
+    </row>
+    <row r="3328">
+      <c r="A3328" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3328" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3328" t="inlineStr">
+        <is>
+          <t>九州地方ワンフクオカビルディング 2025年4月24日(木)開業！全126テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3328" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/13237</t>
+        </is>
+      </c>
+    </row>
+    <row r="3329">
+      <c r="A3329" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3329" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3329" t="inlineStr">
+        <is>
+          <t>九州地方スーパーセンタートライアル上毛店 2025年7月23日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3329" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/40427</t>
+        </is>
+      </c>
+    </row>
+    <row r="3330">
+      <c r="A3330" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3330" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3330" t="inlineStr">
+        <is>
+          <t>関東地方登戸駅前地区市街地再開発事業 2029年竣工！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3330" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/24273</t>
+        </is>
+      </c>
+    </row>
+    <row r="3331">
+      <c r="A3331" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3331" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3331" t="inlineStr">
+        <is>
+          <t>関東地方新松田駅北口地区市街地再開発事業 2030年初頭開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3331" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48018</t>
+        </is>
+      </c>
+    </row>
+    <row r="3332">
+      <c r="A3332" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3332" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3332" t="inlineStr">
+        <is>
+          <t>関東地方ヴィータモールせいせき 2025年10月31日(金)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3332" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/45333</t>
+        </is>
+      </c>
+    </row>
+    <row r="3333">
+      <c r="A3333" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3333" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3333" t="inlineStr">
+        <is>
+          <t>関西地方高島屋堺店跡地にHiViE堺東が2027年春全体開業！ライフが出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3333" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/41410</t>
+        </is>
+      </c>
+    </row>
+    <row r="3334">
+      <c r="A3334" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3334" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3334" t="inlineStr">
+        <is>
+          <t>関西地方イオンタウン堺水賀池 2027年冬開業！30店舗が出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3334" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/45734</t>
+        </is>
+      </c>
+    </row>
+    <row r="3335">
+      <c r="A3335" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3335" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3335" t="inlineStr">
+        <is>
+          <t>中部地方富士駅北口第一地区市街地再開発事業 2030年初頭開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3335" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/26250</t>
+        </is>
+      </c>
+    </row>
+    <row r="3336">
+      <c r="A3336" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3336" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3336" t="inlineStr">
+        <is>
+          <t>関西地方神戸三宮TWINGATE（ツインゲート） 2028年春開業予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3336" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/25375</t>
+        </is>
+      </c>
+    </row>
+    <row r="3337">
+      <c r="A3337" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3337" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3337" t="inlineStr">
+        <is>
+          <t>中部地方スーパーセンタートライアル本巣店 2026年7月22日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3337" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/45851</t>
+        </is>
+      </c>
+    </row>
+    <row r="3338">
+      <c r="A3338" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3338" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3338" t="inlineStr">
+        <is>
+          <t>関東地方板橋駅西口地区市街地再開発事業 2029年10月完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3338" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26695</t>
+        </is>
+      </c>
+    </row>
+    <row r="3339">
+      <c r="A3339" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3339" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3339" t="inlineStr">
+        <is>
+          <t>九州地方LAプラザ ランドアーク島瀬 マックスバリュ佐世保島瀬店 2026年5月14日(木)9:00~開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3339" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/39475</t>
+        </is>
+      </c>
+    </row>
+    <row r="3340">
+      <c r="A3340" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3340" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3340" t="inlineStr">
+        <is>
+          <t>関東地方ケーズデンキ厚木妻田東店 2027年春に開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3340" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47111</t>
+        </is>
+      </c>
+    </row>
+    <row r="3341">
+      <c r="A3341" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3341" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3341" t="inlineStr">
+        <is>
+          <t>中国地方ケーズデンキ山口店 2026年10月29日(木)開業！最新情報も！山口県山口市にビッグ・エスの店舗「ケーズデンキ山口店」が2026年10月29日(木)開業予定！ケーズデンキの中では中～大型店舗となります。隣接地には「ウォンツ山口黒川店」も新設！そんな、ケーズデンキ山口店について、テナントや開業日などを見て...2026.10.20中国地方</t>
+        </is>
+      </c>
+      <c r="D3341" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/44477</t>
+        </is>
+      </c>
+    </row>
+    <row r="3342">
+      <c r="A3342" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3342" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3342" t="inlineStr">
+        <is>
+          <t>関西地方スーパーセンタートライアル愛知川店 2026年10月21日(水)グランドオープン！最新情報も！滋賀県愛知郡にトライアルカンパニーの店舗「スーパーセンタートライアル愛知川店」が2026年10月21日(水)AM8: 30グランドオープン！10月20日(火)10:00〜19:00 プレオープン！スーパーセンタートライアルが愛荘町に初出店！...2026.10.20関西地方</t>
+        </is>
+      </c>
+      <c r="D3342" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/47736</t>
+        </is>
+      </c>
+    </row>
+    <row r="3343">
+      <c r="A3343" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3343" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3343" t="inlineStr">
+        <is>
+          <t>御殿場プレミアム・アウトレット／常設・ポップアップ計9ブランドが今秋オープン</t>
+        </is>
+      </c>
+      <c r="D3343" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102073.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3344">
+      <c r="A3344" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3344" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3344" t="inlineStr">
+        <is>
+          <t>イオンリテール／衣料品レンタル「ルルティ」旗艦店、サンシャインシティに11月20日オープン</t>
+        </is>
+      </c>
+      <c r="D3344" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102074.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3345">
+      <c r="A3345" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3345" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3345" t="inlineStr">
+        <is>
+          <t>平和堂／「丸善守山店」10月23日リニューアルオープン、個店仕入れで生鮮を強化</t>
+        </is>
+      </c>
+      <c r="D3345" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3346">
+      <c r="A3346" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3346" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3346" t="inlineStr">
+        <is>
+          <t>クスリのアオキ／静岡県・愛媛県・愛知県に計3店舗、27年5～6月新設</t>
+        </is>
+      </c>
+      <c r="D3346" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1020011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3347">
+      <c r="A3347" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3347" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3347" t="inlineStr">
+        <is>
+          <t>コスモス薬品／香川県・愛媛県に「ドラッグコスモス」計2店舗、27年5月新設</t>
+        </is>
+      </c>
+      <c r="D3347" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1020012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3348">
+      <c r="A3348" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3348" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3348" t="inlineStr">
+        <is>
+          <t>タリーズ／神奈川県に「タリーズコーヒー＆TEA 武蔵小杉東急スクエア店」オープン</t>
+        </is>
+      </c>
+      <c r="D3348" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102044.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3349">
+      <c r="A3349" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3349" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3349" t="inlineStr">
+        <is>
+          <t>三越伊勢丹HD／横浜駅の「FOOD＆TIME ISETAN」2027年3月28日閉店</t>
+        </is>
+      </c>
+      <c r="D3349" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102016.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3350">
+      <c r="A3350" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3350" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3350" t="inlineStr">
+        <is>
+          <t>アイスタイル／「＠cosme STORE 函館 蔦屋書店」11月13日増床リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D3350" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102075.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3351">
+      <c r="A3351" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3351" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3351" t="inlineStr">
+        <is>
+          <t>サンリオハウス／渋谷パルコに11月13日新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3351" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102013.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3352">
+      <c r="A3352" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3352" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3352" t="inlineStr">
+        <is>
+          <t>やよい軒／長野県下諏訪町「イオンスタイル諏訪店」新規オープン</t>
+        </is>
+      </c>
+      <c r="D3352" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102045.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3353">
+      <c r="A3353" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3353" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3353" t="inlineStr">
+        <is>
+          <t>明治屋／東京・広尾の旗艦店「明治屋広尾ストアー」10月30日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D3353" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101945.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3354">
+      <c r="A3354" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3354" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3354" t="inlineStr">
+        <is>
+          <t>コメダ／DXモデル店舗「コメダ珈琲店 板橋仲宿店」オープン、レジで注文式に</t>
+        </is>
+      </c>
+      <c r="D3354" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101912.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3355">
+      <c r="A3355" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3355" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3355" t="inlineStr">
+        <is>
+          <t>マミーマート／群馬県「生鮮市場TOPガーデン前橋店」リニューアルオープン、日用品を新規導入</t>
+        </is>
+      </c>
+      <c r="D3355" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101916.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3356">
+      <c r="A3356" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3356" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3356" t="inlineStr">
+        <is>
+          <t>JR東海／「アスティ静岡」11月18日リニューアル、治一郎など4店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3356" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101978.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3357">
+      <c r="A3357" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3357" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3357" t="inlineStr">
+        <is>
+          <t>マミーマートほか／埼玉県川口市に「（仮称）川口市上青木プロジェクト（店舗面積3054m2）」27年5月4日新設</t>
+        </is>
+      </c>
+      <c r="D3357" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1019011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3358">
+      <c r="A3358" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3358" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3358" t="inlineStr">
+        <is>
+          <t>コスモス薬品／岡山県・宮崎県に「ドラッグコスモス」計2店舗、27年5月新設</t>
+        </is>
+      </c>
+      <c r="D3358" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1019012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3359">
+      <c r="A3359" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3359" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3359" t="inlineStr">
+        <is>
+          <t>エディオン／兵庫県尼崎市「エディオン塚口店」11月13日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D3359" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101944.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3360">
+      <c r="A3360" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3360" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3360" t="inlineStr">
+        <is>
+          <t>相鉄／シャトレーゼのフランチャイズ事業に参入「横浜片倉町店」10月26日オープン</t>
+        </is>
+      </c>
+      <c r="D3360" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101972.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3361">
+      <c r="A3361" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3361" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3361" t="inlineStr">
+        <is>
+          <t>ローソン／九州で車中泊サービス「RVパーク」開始</t>
+        </is>
+      </c>
+      <c r="D3361" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101913.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3362">
+      <c r="A3362" t="inlineStr">
+        <is>
+          <t>2026年10月20日</t>
+        </is>
+      </c>
+      <c r="B3362" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3362" t="inlineStr">
+        <is>
+          <t>シェイク シャック／東京・新宿「明治安田新宿ビル」に新店舗11月28日オープン</t>
+        </is>
+      </c>
+      <c r="D3362" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101974.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-21
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3362"/>
+  <dimension ref="A1:D3444"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74380,6 +74380,1810 @@
         </is>
       </c>
     </row>
+    <row r="3363">
+      <c r="A3363" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3363" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3363" t="inlineStr">
+        <is>
+          <t>10/21ベルク太田駅前店(群馬県太田市)</t>
+        </is>
+      </c>
+      <c r="D3363" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gJJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3364">
+      <c r="A3364" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3364" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3364" t="inlineStr">
+        <is>
+          <t>10/21ロピア加須ビバモール店(埼玉県加須市)</t>
+        </is>
+      </c>
+      <c r="D3364" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gE6</t>
+        </is>
+      </c>
+    </row>
+    <row r="3365">
+      <c r="A3365" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3365" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3365" t="inlineStr">
+        <is>
+          <t>マクドナルド丸岡高柳店</t>
+        </is>
+      </c>
+      <c r="D3365" t="inlineStr">
+        <is>
+          <t>https://www.mcdonalds.co.jp</t>
+        </is>
+      </c>
+    </row>
+    <row r="3366">
+      <c r="A3366" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3366" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3366" t="inlineStr">
+        <is>
+          <t>10/21イオンスタイル諏訪(長野県諏訪市)</t>
+        </is>
+      </c>
+      <c r="D3366" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1abH</t>
+        </is>
+      </c>
+    </row>
+    <row r="3367">
+      <c r="A3367" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3367" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3367" t="inlineStr">
+        <is>
+          <t>10/21魚市場食堂平の屋(愛知県岡崎市)</t>
+        </is>
+      </c>
+      <c r="D3367" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gGK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3368">
+      <c r="A3368" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3368" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3368" t="inlineStr">
+        <is>
+          <t>12/14マクドナルド池田本郷店(岐阜県)</t>
+        </is>
+      </c>
+      <c r="D3368" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3369">
+      <c r="A3369" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3369" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3369" t="inlineStr">
+        <is>
+          <t>10/21 (10/20プレ)  スーパーセンタートライアル愛知川店</t>
+        </is>
+      </c>
+      <c r="D3369" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gHm</t>
+        </is>
+      </c>
+    </row>
+    <row r="3370">
+      <c r="A3370" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3370" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3370" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3370" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="3371">
+      <c r="A3371" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3371" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3371" t="inlineStr">
+        <is>
+          <t>10/8建替 ツルヤなぎさ店(長野県松本市)</t>
+        </is>
+      </c>
+      <c r="D3371" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="3372">
+      <c r="A3372" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3372" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3372" t="inlineStr">
+        <is>
+          <t>10/9そよら鳥取駅南</t>
+        </is>
+      </c>
+      <c r="D3372" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gyC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3373">
+      <c r="A3373" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3373" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3373" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D3373" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="3374">
+      <c r="A3374" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3374" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3374" t="inlineStr">
+        <is>
+          <t>10/16KOmart fine長泉店</t>
+        </is>
+      </c>
+      <c r="D3374" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gFD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3375">
+      <c r="A3375" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3375" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3375" t="inlineStr">
+        <is>
+          <t>10/16改装 平和堂大野店（食品売場）</t>
+        </is>
+      </c>
+      <c r="D3375" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gDK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3376">
+      <c r="A3376" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3376" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3376" t="inlineStr">
+        <is>
+          <t>10/22業務スーパー西帯広店</t>
+        </is>
+      </c>
+      <c r="D3376" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gG7</t>
+        </is>
+      </c>
+    </row>
+    <row r="3377">
+      <c r="A3377" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3377" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3377" t="inlineStr">
+        <is>
+          <t>10/23スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D3377" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="3378">
+      <c r="A3378" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3378" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3378" t="inlineStr">
+        <is>
+          <t>10/27やまのぶ赤池店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3378" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1dGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3379">
+      <c r="A3379" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3379" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3379" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D3379" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3380">
+      <c r="A3380" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3380" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3380" t="inlineStr">
+        <is>
+          <t>10/30松屋可児店（松のや併設）</t>
+        </is>
+      </c>
+      <c r="D3380" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gEg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3381">
+      <c r="A3381" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3381" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3381" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D3381" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3382">
+      <c r="A3382" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3382" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3382" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D3382" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="3383">
+      <c r="A3383" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3383" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3383" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D3383" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="3384">
+      <c r="A3384" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3384" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3384" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D3384" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="3385">
+      <c r="A3385" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3385" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3385" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3385" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3386">
+      <c r="A3386" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3386" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3386" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3386" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3387">
+      <c r="A3387" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3387" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3387" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3387" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3388">
+      <c r="A3388" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3388" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3388" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3388" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3389">
+      <c r="A3389" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3389" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3389" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3389" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3390">
+      <c r="A3390" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3390" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3390" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3390" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3391">
+      <c r="A3391" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3391" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3391" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3391" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3392">
+      <c r="A3392" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3392" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3392" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3392" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3393">
+      <c r="A3393" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3393" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3393" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3393" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3394">
+      <c r="A3394" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3394" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3394" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3394" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3395">
+      <c r="A3395" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3395" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3395" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3395" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3396">
+      <c r="A3396" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3396" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3396" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3396" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3397">
+      <c r="A3397" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3397" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3397" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3397" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3398">
+      <c r="A3398" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3398" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3398" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3398" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3399">
+      <c r="A3399" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3399" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3399" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3399" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3400">
+      <c r="A3400" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3400" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3400" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3400" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3401">
+      <c r="A3401" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3401" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3401" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3401" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3402">
+      <c r="A3402" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3402" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3402" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3402" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3403">
+      <c r="A3403" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3403" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3403" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3403" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3404">
+      <c r="A3404" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3404" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3404" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3404" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3405">
+      <c r="A3405" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3405" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3405" t="inlineStr">
+        <is>
+          <t>中部地方鳥屋野潟南部地区 商業施設計画 2028年4月開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3405" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/43227</t>
+        </is>
+      </c>
+    </row>
+    <row r="3406">
+      <c r="A3406" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3406" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3406" t="inlineStr">
+        <is>
+          <t>関西地方イオンスタイル大津京 一旦閉店し建て替えて2028年開業！分譲マンションとの一体開発！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3406" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/35154</t>
+        </is>
+      </c>
+    </row>
+    <row r="3407">
+      <c r="A3407" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3407" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3407" t="inlineStr">
+        <is>
+          <t>中部地方中央通りＤ北地区市街地再開発事業 2027年春開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3407" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/25993</t>
+        </is>
+      </c>
+    </row>
+    <row r="3408">
+      <c r="A3408" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3408" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3408" t="inlineStr">
+        <is>
+          <t>関東地方中山駅南口地区市街地再開発事業 2029年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3408" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26880</t>
+        </is>
+      </c>
+    </row>
+    <row r="3409">
+      <c r="A3409" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3409" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3409" t="inlineStr">
+        <is>
+          <t>関東地方武蔵小金井駅北口駅前東地区市街地再開発事業 2030年1月完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3409" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48940</t>
+        </is>
+      </c>
+    </row>
+    <row r="3410">
+      <c r="A3410" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3410" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3410" t="inlineStr">
+        <is>
+          <t>関西地方神戸市役所本庁舎2号館再整備事業 2030年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3410" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/27303</t>
+        </is>
+      </c>
+    </row>
+    <row r="3411">
+      <c r="A3411" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3411" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3411" t="inlineStr">
+        <is>
+          <t>関東地方ヨークベニマル古河店 カインズ古河店 2025年2月14日(金)開業！無印良品とスタバが出店！全6テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3411" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/37708</t>
+        </is>
+      </c>
+    </row>
+    <row r="3412">
+      <c r="A3412" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3412" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3412" t="inlineStr">
+        <is>
+          <t>関西地方ブランズタワー西宮 2027年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3412" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/23230</t>
+        </is>
+      </c>
+    </row>
+    <row r="3413">
+      <c r="A3413" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3413" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3413" t="inlineStr">
+        <is>
+          <t>関東地方カインズ八潮店 2026年冬開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3413" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48076</t>
+        </is>
+      </c>
+    </row>
+    <row r="3414">
+      <c r="A3414" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3414" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3414" t="inlineStr">
+        <is>
+          <t>関東地方みなとみらい21中央地区60・61街区開発事業 2029年春開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3414" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36914</t>
+        </is>
+      </c>
+    </row>
+    <row r="3415">
+      <c r="A3415" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3415" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3415" t="inlineStr">
+        <is>
+          <t>北海道地方Fビレッジ複合施設 2028年春開業！駅前に商業施設併設 テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3415" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/47835</t>
+        </is>
+      </c>
+    </row>
+    <row r="3416">
+      <c r="A3416" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3416" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3416" t="inlineStr">
+        <is>
+          <t>四国地方コストコ東温倉庫店 2027年末開業！愛媛県初出店！場所は？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3416" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/shikoku/45913</t>
+        </is>
+      </c>
+    </row>
+    <row r="3417">
+      <c r="A3417" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3417" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3417" t="inlineStr">
+        <is>
+          <t>東北地方イオンスタイル山王 2025年3月20日(木)開業！無印良品も出店へ！全8テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3417" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/37974</t>
+        </is>
+      </c>
+    </row>
+    <row r="3418">
+      <c r="A3418" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3418" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3418" t="inlineStr">
+        <is>
+          <t>関東地方コトエ橋本 2026年5月29日(金)開業！全21テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3418" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/41085</t>
+        </is>
+      </c>
+    </row>
+    <row r="3419">
+      <c r="A3419" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3419" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3419" t="inlineStr">
+        <is>
+          <t>東北地方【電力ビル】一番町三丁目七番地区市街地再開発事業 2029年開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3419" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/31239</t>
+        </is>
+      </c>
+    </row>
+    <row r="3420">
+      <c r="A3420" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3420" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3420" t="inlineStr">
+        <is>
+          <t>関東地方三河島駅前北地区市街地再開発事業 2031年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3420" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26830</t>
+        </is>
+      </c>
+    </row>
+    <row r="3421">
+      <c r="A3421" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3421" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3421" t="inlineStr">
+        <is>
+          <t>関東地方ららぽーとTOKYO-BAY 北館 建て替えへ！2025年10月31日(金)開業！Ⅰ期では96店舗が出店！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3421" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/29408</t>
+        </is>
+      </c>
+    </row>
+    <row r="3422">
+      <c r="A3422" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3422" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3422" t="inlineStr">
+        <is>
+          <t>九州地方ゆめモール那珂川 2026年2月20日(金)~順次開業！全20店舗一覧！</t>
+        </is>
+      </c>
+      <c r="D3422" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/31176</t>
+        </is>
+      </c>
+    </row>
+    <row r="3423">
+      <c r="A3423" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3423" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3423" t="inlineStr">
+        <is>
+          <t>九州地方イオン鹿児島鴨池店 2024年8月31日(土)に閉店し建て替えへ！イオンモールが取得！最新情報も！鹿児島県鹿児島市の商業施設「イオン鹿児島鴨池店」が2024年8月31日(土)をもって閉店し、現在跡地の再開発計画が大きく動き出しています！旧店舗の解体工事が完了し、約3.6万㎡（約1.1万坪）におよぶ広大な敷地を「イオンモール」が取得！既存...2026.10.21九州地方</t>
+        </is>
+      </c>
+      <c r="D3423" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/36900</t>
+        </is>
+      </c>
+    </row>
+    <row r="3424">
+      <c r="A3424" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3424" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3424" t="inlineStr">
+        <is>
+          <t>関東地方ベルク平塚田村店 2027年春開業！テナントは？最新情報も！神奈川県平塚市の相模小学校跡地に、ベルクの大型ショッピングセンター「ベルク平塚田村店（仮称）」が2027年春開業予定！平塚市に埼玉発の人気食品スーパー「ベルク」が初出店！国道129号沿いの広大な小学校跡地に、スーパーマーケット棟と物販店舗2...2026.10.21関東地方</t>
+        </is>
+      </c>
+      <c r="D3424" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47482</t>
+        </is>
+      </c>
+    </row>
+    <row r="3425">
+      <c r="A3425" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3425" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3425" t="inlineStr">
+        <is>
+          <t>ユニクロ／都内の超大型店「世田谷千歳台店」リニューアル、地域密着で多彩な協業注目</t>
+        </is>
+      </c>
+      <c r="D3425" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s102144.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3426">
+      <c r="A3426" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3426" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3426" t="inlineStr">
+        <is>
+          <t>トライアル／徳島県阿波市に「スーパーセンタートライアル阿波岩津店（店舗面積3292m2）」27年5月12日新設</t>
+        </is>
+      </c>
+      <c r="D3426" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1021012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3427">
+      <c r="A3427" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3427" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3427" t="inlineStr">
+        <is>
+          <t>築地食堂 源ちゃん／埼玉・新座にロードサイド2号店「新座RS店」今冬オープン</t>
+        </is>
+      </c>
+      <c r="D3427" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102177.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3428">
+      <c r="A3428" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3428" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3428" t="inlineStr">
+        <is>
+          <t>ノジマ／埼玉県「ラ・ヴィーニュ 新座」に新店舗10月22日オープン</t>
+        </is>
+      </c>
+      <c r="D3428" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102176.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3429">
+      <c r="A3429" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3429" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3429" t="inlineStr">
+        <is>
+          <t>河淳／埼玉県新座市に「ケユカ エキア志木店」新規オープン</t>
+        </is>
+      </c>
+      <c r="D3429" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102175.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3430">
+      <c r="A3430" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3430" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3430" t="inlineStr">
+        <is>
+          <t>ドラッグストアモリ／徳島県・長崎県に計2店舗、27年4月新設</t>
+        </is>
+      </c>
+      <c r="D3430" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1021011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3431">
+      <c r="A3431" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3431" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3431" t="inlineStr">
+        <is>
+          <t>サイプレス／福島県「イオンモール伊達」に新業態の天丼専門店11月27日オープン</t>
+        </is>
+      </c>
+      <c r="D3431" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102178.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3432">
+      <c r="A3432" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3432" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3432" t="inlineStr">
+        <is>
+          <t>南魚沼市／新潟・南魚沼市図書館内に「ドトールコーヒーショップ」11月4日オープン</t>
+        </is>
+      </c>
+      <c r="D3432" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102143.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3433">
+      <c r="A3433" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3433" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3433" t="inlineStr">
+        <is>
+          <t>戸塚モディ／「40周年感謝祭」を11月1～30日開催</t>
+        </is>
+      </c>
+      <c r="D3433" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102112.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3434">
+      <c r="A3434" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3434" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3434" t="inlineStr">
+        <is>
+          <t>御殿場プレミアム・アウトレット／常設・ポップアップ計9ブランドが今秋オープン</t>
+        </is>
+      </c>
+      <c r="D3434" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102073.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3435">
+      <c r="A3435" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3435" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3435" t="inlineStr">
+        <is>
+          <t>イオンリテール／衣料品レンタル「ルルティ」旗艦店、サンシャインシティに11月20日オープン</t>
+        </is>
+      </c>
+      <c r="D3435" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102074.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3436">
+      <c r="A3436" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3436" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3436" t="inlineStr">
+        <is>
+          <t>平和堂／「丸善守山店」10月23日リニューアルオープン、個店仕入れで生鮮を強化</t>
+        </is>
+      </c>
+      <c r="D3436" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3437">
+      <c r="A3437" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3437" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3437" t="inlineStr">
+        <is>
+          <t>クスリのアオキ／静岡県・愛媛県・愛知県に計3店舗、27年5～6月新設</t>
+        </is>
+      </c>
+      <c r="D3437" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1020011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3438">
+      <c r="A3438" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3438" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3438" t="inlineStr">
+        <is>
+          <t>コスモス薬品／香川県・愛媛県に「ドラッグコスモス」計2店舗、27年5月新設</t>
+        </is>
+      </c>
+      <c r="D3438" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1020012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3439">
+      <c r="A3439" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3439" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3439" t="inlineStr">
+        <is>
+          <t>タリーズ／神奈川県に「タリーズコーヒー＆TEA 武蔵小杉東急スクエア店」オープン</t>
+        </is>
+      </c>
+      <c r="D3439" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102044.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3440">
+      <c r="A3440" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3440" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3440" t="inlineStr">
+        <is>
+          <t>三越伊勢丹HD／横浜駅の「FOOD＆TIME ISETAN」2027年3月28日閉店</t>
+        </is>
+      </c>
+      <c r="D3440" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102016.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3441">
+      <c r="A3441" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3441" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3441" t="inlineStr">
+        <is>
+          <t>アイスタイル／「＠cosme STORE 函館 蔦屋書店」11月13日増床リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D3441" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102075.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3442">
+      <c r="A3442" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3442" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3442" t="inlineStr">
+        <is>
+          <t>サンリオハウス／渋谷パルコに11月13日新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3442" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102013.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3443">
+      <c r="A3443" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3443" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3443" t="inlineStr">
+        <is>
+          <t>やよい軒／長野県下諏訪町「イオンスタイル諏訪店」新規オープン</t>
+        </is>
+      </c>
+      <c r="D3443" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102045.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3444">
+      <c r="A3444" t="inlineStr">
+        <is>
+          <t>2026年10月21日</t>
+        </is>
+      </c>
+      <c r="B3444" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3444" t="inlineStr">
+        <is>
+          <t>明治屋／東京・広尾の旗艦店「明治屋広尾ストアー」10月30日リニューアルオープン</t>
+        </is>
+      </c>
+      <c r="D3444" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s101945.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-22
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3444"/>
+  <dimension ref="A1:D3529"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -76184,6 +76184,1876 @@
         </is>
       </c>
     </row>
+    <row r="3445">
+      <c r="A3445" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3445" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3445" t="inlineStr">
+        <is>
+          <t>10/22業務スーパー西帯広店</t>
+        </is>
+      </c>
+      <c r="D3445" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gG7</t>
+        </is>
+      </c>
+    </row>
+    <row r="3446">
+      <c r="A3446" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3446" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3446" t="inlineStr">
+        <is>
+          <t>10/22マックスバリュエクスプレス栄5丁目店(名古屋市中区)</t>
+        </is>
+      </c>
+      <c r="D3446" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eRp</t>
+        </is>
+      </c>
+    </row>
+    <row r="3447">
+      <c r="A3447" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3447" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3447" t="inlineStr">
+        <is>
+          <t>12/30マクドナルド各務原いちょう通り店</t>
+        </is>
+      </c>
+      <c r="D3447" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gMH</t>
+        </is>
+      </c>
+    </row>
+    <row r="3448">
+      <c r="A3448" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3448" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3448" t="inlineStr">
+        <is>
+          <t>10/22移転 業務スーパー天理店</t>
+        </is>
+      </c>
+      <c r="D3448" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gCg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3449">
+      <c r="A3449" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3449" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3449" t="inlineStr">
+        <is>
+          <t>10/22サンディ千船店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D3449" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3450">
+      <c r="A3450" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3450" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3450" t="inlineStr">
+        <is>
+          <t>https://www.ksdenki.co.jp/store/open/2026/10/17/post-497.html</t>
+        </is>
+      </c>
+      <c r="D3450" t="inlineStr">
+        <is>
+          <t>https://www.ksdenki.co.jp/store/open/2026/10/17/post-497.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3451">
+      <c r="A3451" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3451" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3451" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3451" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="3452">
+      <c r="A3452" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3452" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3452" t="inlineStr">
+        <is>
+          <t>10/8建替 ツルヤなぎさ店(長野県松本市)</t>
+        </is>
+      </c>
+      <c r="D3452" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="3453">
+      <c r="A3453" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3453" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3453" t="inlineStr">
+        <is>
+          <t>10/9そよら鳥取駅南</t>
+        </is>
+      </c>
+      <c r="D3453" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gyC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3454">
+      <c r="A3454" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3454" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3454" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D3454" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="3455">
+      <c r="A3455" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3455" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3455" t="inlineStr">
+        <is>
+          <t>10/16KOmart fine長泉店</t>
+        </is>
+      </c>
+      <c r="D3455" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gFD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3456">
+      <c r="A3456" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3456" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3456" t="inlineStr">
+        <is>
+          <t>10/16改装 平和堂大野店（食品売場）</t>
+        </is>
+      </c>
+      <c r="D3456" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gDK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3457">
+      <c r="A3457" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3457" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3457" t="inlineStr">
+        <is>
+          <t>(10/20プレ)10/21スーパーセンタートライアル愛知川店</t>
+        </is>
+      </c>
+      <c r="D3457" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gHm</t>
+        </is>
+      </c>
+    </row>
+    <row r="3458">
+      <c r="A3458" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3458" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3458" t="inlineStr">
+        <is>
+          <t>10/21魚市場食堂平の屋(愛知県岡崎市)</t>
+        </is>
+      </c>
+      <c r="D3458" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gGK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3459">
+      <c r="A3459" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3459" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3459" t="inlineStr">
+        <is>
+          <t>10/21ロピア加須ビバモール店(埼玉県加須市)</t>
+        </is>
+      </c>
+      <c r="D3459" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gE6</t>
+        </is>
+      </c>
+    </row>
+    <row r="3460">
+      <c r="A3460" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3460" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3460" t="inlineStr">
+        <is>
+          <t>10/21ベルク太田駅前店(群馬県太田市)</t>
+        </is>
+      </c>
+      <c r="D3460" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gJJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3461">
+      <c r="A3461" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3461" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3461" t="inlineStr">
+        <is>
+          <t>10/23スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D3461" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="3462">
+      <c r="A3462" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3462" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3462" t="inlineStr">
+        <is>
+          <t>10/27やまのぶ赤池店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3462" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1dGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3463">
+      <c r="A3463" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3463" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3463" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D3463" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3464">
+      <c r="A3464" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3464" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3464" t="inlineStr">
+        <is>
+          <t>10/30松屋可児店（松のや併設）</t>
+        </is>
+      </c>
+      <c r="D3464" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gEg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3465">
+      <c r="A3465" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3465" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3465" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D3465" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3466">
+      <c r="A3466" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3466" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3466" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D3466" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="3467">
+      <c r="A3467" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3467" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3467" t="inlineStr">
+        <is>
+          <t>12/14マクドナルド池田本郷店(岐阜県)</t>
+        </is>
+      </c>
+      <c r="D3467" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3468">
+      <c r="A3468" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3468" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3468" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D3468" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="3469">
+      <c r="A3469" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3469" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3469" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D3469" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="3470">
+      <c r="A3470" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3470" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3470" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3470" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3471">
+      <c r="A3471" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3471" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3471" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3471" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3472">
+      <c r="A3472" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3472" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3472" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3472" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3473">
+      <c r="A3473" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3473" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3473" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3473" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3474">
+      <c r="A3474" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3474" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3474" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3474" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3475">
+      <c r="A3475" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3475" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3475" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3475" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3476">
+      <c r="A3476" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3476" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3476" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3476" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3477">
+      <c r="A3477" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3477" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3477" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3477" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3478">
+      <c r="A3478" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3478" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3478" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3478" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3479">
+      <c r="A3479" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3479" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3479" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3479" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3480">
+      <c r="A3480" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3480" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3480" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3480" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3481">
+      <c r="A3481" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3481" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3481" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3481" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3482">
+      <c r="A3482" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3482" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3482" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3482" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3483">
+      <c r="A3483" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3483" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3483" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3483" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3484">
+      <c r="A3484" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3484" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3484" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3484" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3485">
+      <c r="A3485" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3485" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3485" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3485" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3486">
+      <c r="A3486" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3486" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3486" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3486" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3487">
+      <c r="A3487" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3487" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3487" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3487" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3488">
+      <c r="A3488" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3488" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3488" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3488" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3489">
+      <c r="A3489" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3489" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3489" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3489" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3490">
+      <c r="A3490" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3490" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3490" t="inlineStr">
+        <is>
+          <t>関東地方BLiX茅ヶ崎(ブリックス茅ヶ崎) 2025年11月27日(木)開業！テナント随時更新中！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3490" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/38752</t>
+        </is>
+      </c>
+    </row>
+    <row r="3491">
+      <c r="A3491" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3491" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3491" t="inlineStr">
+        <is>
+          <t>関東地方品川駅街区地区開発計画 2030年度より順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3491" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/33795</t>
+        </is>
+      </c>
+    </row>
+    <row r="3492">
+      <c r="A3492" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3492" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3492" t="inlineStr">
+        <is>
+          <t>関西地方クオーツ心斎橋 2026年4月25日(土)開業！全52店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3492" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/25158</t>
+        </is>
+      </c>
+    </row>
+    <row r="3493">
+      <c r="A3493" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3493" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3493" t="inlineStr">
+        <is>
+          <t>中部地方武蔵ヶ辻A地区市街地再開発事業 エムザ再開発！どのような施設になる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3493" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/49728</t>
+        </is>
+      </c>
+    </row>
+    <row r="3494">
+      <c r="A3494" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3494" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3494" t="inlineStr">
+        <is>
+          <t>関東地方小川パレット 小川駅西口複合施設 2026年11月1日(日)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3494" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26411</t>
+        </is>
+      </c>
+    </row>
+    <row r="3495">
+      <c r="A3495" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3495" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3495" t="inlineStr">
+        <is>
+          <t>北海道地方コメリパワー恵庭店 2025年3月21日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3495" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/40058</t>
+        </is>
+      </c>
+    </row>
+    <row r="3496">
+      <c r="A3496" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3496" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3496" t="inlineStr">
+        <is>
+          <t>関西地方淀屋橋ステーションワン 2025年6月23日(月)に開業！テナント13店舗一覧！どのような建物に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3496" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/26225</t>
+        </is>
+      </c>
+    </row>
+    <row r="3497">
+      <c r="A3497" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3497" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3497" t="inlineStr">
+        <is>
+          <t>東北地方福島ピボット 2026年3月28日(土)開業！ロピアも出店！11店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3497" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/47552</t>
+        </is>
+      </c>
+    </row>
+    <row r="3498">
+      <c r="A3498" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3498" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3498" t="inlineStr">
+        <is>
+          <t>関東地方ジョイホン小山駅前店 2026年7月3日(金)リニューアル開業！全22テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3498" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48918</t>
+        </is>
+      </c>
+    </row>
+    <row r="3499">
+      <c r="A3499" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3499" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3499" t="inlineStr">
+        <is>
+          <t>中部地方中央通りＤ北地区市街地再開発事業 2027年春開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3499" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/25993</t>
+        </is>
+      </c>
+    </row>
+    <row r="3500">
+      <c r="A3500" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3500" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3500" t="inlineStr">
+        <is>
+          <t>九州地方中井口・高見台商業施設 2026年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3500" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/44099</t>
+        </is>
+      </c>
+    </row>
+    <row r="3501">
+      <c r="A3501" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3501" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3501" t="inlineStr">
+        <is>
+          <t>中部地方アークスクエア須坂 ホームセンタームサシ・ヤマダデンキ 2025年8月6日(水)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3501" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/21807</t>
+        </is>
+      </c>
+    </row>
+    <row r="3502">
+      <c r="A3502" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3502" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3502" t="inlineStr">
+        <is>
+          <t>関東地方ザ・パークハウス 赤羽台タワー＆レジデンス 2028年10月完成予定！商業施設も誕生 最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3502" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/39853</t>
+        </is>
+      </c>
+    </row>
+    <row r="3503">
+      <c r="A3503" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3503" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3503" t="inlineStr">
+        <is>
+          <t>関西地方豊中市立庄内さくら学園中学校跡地 複合商業施設 2028年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3503" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/46363</t>
+        </is>
+      </c>
+    </row>
+    <row r="3504">
+      <c r="A3504" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3504" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3504" t="inlineStr">
+        <is>
+          <t>関東地方ヤオコー福生牛浜店 2026年1月20日(火)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3504" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42926</t>
+        </is>
+      </c>
+    </row>
+    <row r="3505">
+      <c r="A3505" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3505" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3505" t="inlineStr">
+        <is>
+          <t>関東地方プレミストタワー船橋 2028年秋開業！西武船橋店跡地 最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3505" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/30141</t>
+        </is>
+      </c>
+    </row>
+    <row r="3506">
+      <c r="A3506" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3506" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3506" t="inlineStr">
+        <is>
+          <t>関東地方大宮駅西口第3-A･D地区市街地再開発事業 2031年以降開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3506" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/16908</t>
+        </is>
+      </c>
+    </row>
+    <row r="3507">
+      <c r="A3507" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3507" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3507" t="inlineStr">
+        <is>
+          <t>中国地方コストコ赤磐計画は白紙に！計画地は商業施設計画始動！2027年以降開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3507" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/39978</t>
+        </is>
+      </c>
+    </row>
+    <row r="3508">
+      <c r="A3508" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3508" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3508" t="inlineStr">
+        <is>
+          <t>中部地方ヤマダデンキ Tecc LIFE SELECT 豊田広路店(仮称) 2027年冬オープン予定！最新情報も！愛知県豊田市にヤマダデンキの大型店舗「ヤマダデンキ Tecc LIFE SELECT 豊田広路店(仮称)」が2027年冬に開業予定！ヤマダデンキの中では大型店舗となります！そんな、ヤマダデンキ Tecc LIFE SELECT 豊田広路店(...2026.10.22中部地方</t>
+        </is>
+      </c>
+      <c r="D3508" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/49945</t>
+        </is>
+      </c>
+    </row>
+    <row r="3509">
+      <c r="A3509" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3509" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3509" t="inlineStr">
+        <is>
+          <t>関西地方そよら小野 2027年秋開業！イオン小野店跡地 21店舗が出店！テナントは？最新情報も！兵庫県小野市のイオンリテールの商業施設「イオン小野店」が2025年1月15日(水)に閉店し、都市型オープンモール「そよら小野（仮称）」として2027年秋（8月〜9月頃）に生まれ変わります！敷地面積約4.5万㎡に広がる地上1〜2階建てのオープ...2026.10.22関西地方</t>
+        </is>
+      </c>
+      <c r="D3509" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/43512</t>
+        </is>
+      </c>
+    </row>
+    <row r="3510">
+      <c r="A3510" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3510" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3510" t="inlineStr">
+        <is>
+          <t>三菱地所プロパティマネジメント／丸の内エリア、今秋20店舗が新規・改装オープン</t>
+        </is>
+      </c>
+      <c r="D3510" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102212.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3511">
+      <c r="A3511" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3511" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3511" t="inlineStr">
+        <is>
+          <t>イオンフードスタイル／「フードスタイル東五反田店」10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D3511" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102214.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3512">
+      <c r="A3512" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3512" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3512" t="inlineStr">
+        <is>
+          <t>イオンウエルシア九州／熊本市東区に「ウエルシアプラス長嶺南店」10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D3512" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102279.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3513">
+      <c r="A3513" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3513" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3513" t="inlineStr">
+        <is>
+          <t>ロピア／鹿児島県に初出店「鹿児島宇宿店」来夏オープン</t>
+        </is>
+      </c>
+      <c r="D3513" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102275.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3514">
+      <c r="A3514" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3514" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3514" t="inlineStr">
+        <is>
+          <t>ジェイアール名古屋タカシマヤ／和洋菓子売場に新業態含む4店舗10月30日オープン</t>
+        </is>
+      </c>
+      <c r="D3514" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102278.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3515">
+      <c r="A3515" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3515" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3515" t="inlineStr">
+        <is>
+          <t>神戸港／スーパーヨットの受入・滞在拠点を整備、28年飲食などの複合施設オープン</t>
+        </is>
+      </c>
+      <c r="D3515" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102274.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3516">
+      <c r="A3516" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3516" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3516" t="inlineStr">
+        <is>
+          <t>ベルクほか／埼玉県入間市に「（仮称）フレスポ入間（店舗面積3210m2）」28年3月31日新設</t>
+        </is>
+      </c>
+      <c r="D3516" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1022012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3517">
+      <c r="A3517" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3517" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3517" t="inlineStr">
+        <is>
+          <t>ベイシア／長野県千曲市「更埴店」10月23日リニューアル、総菜強化・レイアウト刷新</t>
+        </is>
+      </c>
+      <c r="D3517" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102272.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3518">
+      <c r="A3518" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3518" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3518" t="inlineStr">
+        <is>
+          <t>カインズ／東京・赤羽ビビオにリフォーム専門の小型店オープン</t>
+        </is>
+      </c>
+      <c r="D3518" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102215.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3519">
+      <c r="A3519" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3519" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3519" t="inlineStr">
+        <is>
+          <t>サブウェイ／東京都千代田区「住友不動産秋葉原ファーストビル店」10月28日オープン</t>
+        </is>
+      </c>
+      <c r="D3519" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102271.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3520">
+      <c r="A3520" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3520" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3520" t="inlineStr">
+        <is>
+          <t>ロック・フィールド／JR川口駅構内に「神戸コロッケ 川口駅店」オープン</t>
+        </is>
+      </c>
+      <c r="D3520" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102276.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3521">
+      <c r="A3521" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3521" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3521" t="inlineStr">
+        <is>
+          <t>リカーマウンテン／埼玉県行田市に「行田店」11月5日オープン</t>
+        </is>
+      </c>
+      <c r="D3521" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102277.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3522">
+      <c r="A3522" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3522" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3522" t="inlineStr">
+        <is>
+          <t>ドラッグストアモリ／熊本県・福岡県に計2店舗、27年5月新設</t>
+        </is>
+      </c>
+      <c r="D3522" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1022011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3523">
+      <c r="A3523" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3523" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3523" t="inlineStr">
+        <is>
+          <t>ユニクロ／都内の超大型店「世田谷千歳台店」リニューアル、地域密着で多彩な協業注目</t>
+        </is>
+      </c>
+      <c r="D3523" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s102144.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3524">
+      <c r="A3524" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3524" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3524" t="inlineStr">
+        <is>
+          <t>トライアル／徳島県阿波市に「スーパーセンタートライアル阿波岩津店（店舗面積3292m2）」27年5月12日新設</t>
+        </is>
+      </c>
+      <c r="D3524" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1021012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3525">
+      <c r="A3525" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3525" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3525" t="inlineStr">
+        <is>
+          <t>築地食堂 源ちゃん／埼玉・新座にロードサイド2号店「新座RS店」今冬オープン</t>
+        </is>
+      </c>
+      <c r="D3525" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102177.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3526">
+      <c r="A3526" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3526" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3526" t="inlineStr">
+        <is>
+          <t>ノジマ／埼玉県「ラ・ヴィーニュ 新座」に新店舗10月22日オープン</t>
+        </is>
+      </c>
+      <c r="D3526" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102176.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3527">
+      <c r="A3527" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3527" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3527" t="inlineStr">
+        <is>
+          <t>河淳／埼玉県新座市に「ケユカ エキア志木店」新規オープン</t>
+        </is>
+      </c>
+      <c r="D3527" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102175.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3528">
+      <c r="A3528" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3528" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3528" t="inlineStr">
+        <is>
+          <t>ドラッグストアモリ／徳島県・長崎県に計2店舗、27年4月新設</t>
+        </is>
+      </c>
+      <c r="D3528" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1021011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3529">
+      <c r="A3529" t="inlineStr">
+        <is>
+          <t>2026年10月22日</t>
+        </is>
+      </c>
+      <c r="B3529" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3529" t="inlineStr">
+        <is>
+          <t>サイプレス／福島県「イオンモール伊達」に新業態の天丼専門店11月27日オープン</t>
+        </is>
+      </c>
+      <c r="D3529" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102178.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-23
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3529"/>
+  <dimension ref="A1:D3616"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -78054,6 +78054,1920 @@
         </is>
       </c>
     </row>
+    <row r="3530">
+      <c r="A3530" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3530" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3530" t="inlineStr">
+        <is>
+          <t>10/23ザ・ビッグ千歳武道館前店</t>
+        </is>
+      </c>
+      <c r="D3530" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3531">
+      <c r="A3531" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3531" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3531" t="inlineStr">
+        <is>
+          <t>10/23廻転鮨 銀座おのでらハレザ池袋店</t>
+        </is>
+      </c>
+      <c r="D3531" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gOs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3532">
+      <c r="A3532" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3532" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3532" t="inlineStr">
+        <is>
+          <t>10/23トライアル西友町田店</t>
+        </is>
+      </c>
+      <c r="D3532" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gOi</t>
+        </is>
+      </c>
+    </row>
+    <row r="3533">
+      <c r="A3533" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3533" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3533" t="inlineStr">
+        <is>
+          <t>10/23スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D3533" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="3534">
+      <c r="A3534" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3534" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3534" t="inlineStr">
+        <is>
+          <t>10/23タチヤ豊田小坂店(愛知県豊田市)</t>
+        </is>
+      </c>
+      <c r="D3534" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1goQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3535">
+      <c r="A3535" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3535" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3535" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3535" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="3536">
+      <c r="A3536" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3536" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3536" t="inlineStr">
+        <is>
+          <t>10/8建替 ツルヤなぎさ店(長野県松本市)</t>
+        </is>
+      </c>
+      <c r="D3536" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="3537">
+      <c r="A3537" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3537" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3537" t="inlineStr">
+        <is>
+          <t>10/9そよら鳥取駅南</t>
+        </is>
+      </c>
+      <c r="D3537" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gyC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3538">
+      <c r="A3538" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3538" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3538" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D3538" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="3539">
+      <c r="A3539" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3539" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3539" t="inlineStr">
+        <is>
+          <t>10/16KOmart fine長泉店</t>
+        </is>
+      </c>
+      <c r="D3539" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gFD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3540">
+      <c r="A3540" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3540" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3540" t="inlineStr">
+        <is>
+          <t>10/16改装 平和堂大野店（食品売場）</t>
+        </is>
+      </c>
+      <c r="D3540" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gDK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3541">
+      <c r="A3541" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3541" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3541" t="inlineStr">
+        <is>
+          <t>(10/20プレ)10/21スーパーセンタートライアル愛知川店</t>
+        </is>
+      </c>
+      <c r="D3541" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gHm</t>
+        </is>
+      </c>
+    </row>
+    <row r="3542">
+      <c r="A3542" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3542" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3542" t="inlineStr">
+        <is>
+          <t>10/21魚市場食堂平の屋(愛知県岡崎市)</t>
+        </is>
+      </c>
+      <c r="D3542" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gGK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3543">
+      <c r="A3543" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3543" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3543" t="inlineStr">
+        <is>
+          <t>10/21ロピア加須ビバモール店(埼玉県加須市)</t>
+        </is>
+      </c>
+      <c r="D3543" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gE6</t>
+        </is>
+      </c>
+    </row>
+    <row r="3544">
+      <c r="A3544" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3544" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3544" t="inlineStr">
+        <is>
+          <t>10/21ベルク太田駅前店(群馬県太田市)</t>
+        </is>
+      </c>
+      <c r="D3544" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gJJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3545">
+      <c r="A3545" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3545" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3545" t="inlineStr">
+        <is>
+          <t>10/22業務スーパー西帯広店</t>
+        </is>
+      </c>
+      <c r="D3545" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gG7</t>
+        </is>
+      </c>
+    </row>
+    <row r="3546">
+      <c r="A3546" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3546" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3546" t="inlineStr">
+        <is>
+          <t>10/22サンディ千船店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D3546" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3547">
+      <c r="A3547" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3547" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3547" t="inlineStr">
+        <is>
+          <t>10/22マックスバリュエクスプレス栄5丁目店(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D3547" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eRp</t>
+        </is>
+      </c>
+    </row>
+    <row r="3548">
+      <c r="A3548" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3548" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3548" t="inlineStr">
+        <is>
+          <t>10/27やまのぶ赤池店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3548" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1dGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3549">
+      <c r="A3549" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3549" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3549" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D3549" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3550">
+      <c r="A3550" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3550" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3550" t="inlineStr">
+        <is>
+          <t>10/30松屋可児店（松のや併設）</t>
+        </is>
+      </c>
+      <c r="D3550" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gEg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3551">
+      <c r="A3551" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3551" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3551" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D3551" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3552">
+      <c r="A3552" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3552" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3552" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D3552" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="3553">
+      <c r="A3553" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3553" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3553" t="inlineStr">
+        <is>
+          <t>12/14マクドナルド池田本郷店(岐阜県)</t>
+        </is>
+      </c>
+      <c r="D3553" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3554">
+      <c r="A3554" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3554" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3554" t="inlineStr">
+        <is>
+          <t>12/30マクドナルド各務原いちょう通り店</t>
+        </is>
+      </c>
+      <c r="D3554" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gMH</t>
+        </is>
+      </c>
+    </row>
+    <row r="3555">
+      <c r="A3555" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3555" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3555" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D3555" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="3556">
+      <c r="A3556" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3556" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3556" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D3556" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="3557">
+      <c r="A3557" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3557" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3557" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3557" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3558">
+      <c r="A3558" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3558" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3558" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3558" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3559">
+      <c r="A3559" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3559" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3559" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3559" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3560">
+      <c r="A3560" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3560" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3560" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3560" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3561">
+      <c r="A3561" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3561" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3561" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3561" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3562">
+      <c r="A3562" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3562" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3562" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3562" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3563">
+      <c r="A3563" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3563" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3563" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3563" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3564">
+      <c r="A3564" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3564" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3564" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3564" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3565">
+      <c r="A3565" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3565" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3565" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3565" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3566">
+      <c r="A3566" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3566" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3566" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3566" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3567">
+      <c r="A3567" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3567" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3567" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3567" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3568">
+      <c r="A3568" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3568" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3568" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3568" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3569">
+      <c r="A3569" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3569" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3569" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3569" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3570">
+      <c r="A3570" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3570" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3570" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3570" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3571">
+      <c r="A3571" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3571" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3571" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3571" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3572">
+      <c r="A3572" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3572" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3572" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3572" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3573">
+      <c r="A3573" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3573" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3573" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3573" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3574">
+      <c r="A3574" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3574" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3574" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3574" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3575">
+      <c r="A3575" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3575" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3575" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3575" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3576">
+      <c r="A3576" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3576" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3576" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3576" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3577">
+      <c r="A3577" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3577" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3577" t="inlineStr">
+        <is>
+          <t>中部地方スーパーセンタートライアル石和店 2026年3月18日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3577" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/41684</t>
+        </is>
+      </c>
+    </row>
+    <row r="3578">
+      <c r="A3578" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3578" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3578" t="inlineStr">
+        <is>
+          <t>関東地方藍テラス（あおてらす）青梅駅前に2026年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3578" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26304</t>
+        </is>
+      </c>
+    </row>
+    <row r="3579">
+      <c r="A3579" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3579" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3579" t="inlineStr">
+        <is>
+          <t>関西地方プリコ西明石 南館 2026年6月26日(金)開業！全6テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3579" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/42350</t>
+        </is>
+      </c>
+    </row>
+    <row r="3580">
+      <c r="A3580" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3580" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3580" t="inlineStr">
+        <is>
+          <t>九州地方NTT西日本宮崎支店商業施設「HAROW」2025年4月18日(金)全面開業！ 全テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3580" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/39808</t>
+        </is>
+      </c>
+    </row>
+    <row r="3581">
+      <c r="A3581" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3581" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3581" t="inlineStr">
+        <is>
+          <t>九州地方福岡空港国内線ターミナル 大型商業施設が誕生！2027年夏開業！180店舗が出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3581" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/43493</t>
+        </is>
+      </c>
+    </row>
+    <row r="3582">
+      <c r="A3582" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3582" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3582" t="inlineStr">
+        <is>
+          <t>関東地方アクロスプラザ昭島 2025年3月27日(木)より順次開業！全7テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3582" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/43645</t>
+        </is>
+      </c>
+    </row>
+    <row r="3583">
+      <c r="A3583" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3583" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3583" t="inlineStr">
+        <is>
+          <t>関西地方ハローズ洲本モール 2026年冬開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3583" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/42115</t>
+        </is>
+      </c>
+    </row>
+    <row r="3584">
+      <c r="A3584" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3584" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3584" t="inlineStr">
+        <is>
+          <t>関西地方ニトリ江坂店が2027年早春に開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3584" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/43247</t>
+        </is>
+      </c>
+    </row>
+    <row r="3585">
+      <c r="A3585" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3585" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3585" t="inlineStr">
+        <is>
+          <t>関東地方上板橋駅南口駅前東地区市街地再開発事業 2028年完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3585" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48931</t>
+        </is>
+      </c>
+    </row>
+    <row r="3586">
+      <c r="A3586" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3586" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3586" t="inlineStr">
+        <is>
+          <t>東北地方イオン相馬店 建て替え 2027年夏開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3586" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/49770</t>
+        </is>
+      </c>
+    </row>
+    <row r="3587">
+      <c r="A3587" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3587" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3587" t="inlineStr">
+        <is>
+          <t>中国地方マルアイ川西店 複合商業施設が開業！2027年冬開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3587" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/44825</t>
+        </is>
+      </c>
+    </row>
+    <row r="3588">
+      <c r="A3588" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3588" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3588" t="inlineStr">
+        <is>
+          <t>中国地方スーパーセンタートライアル大田店 2025年6月18日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3588" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/40704</t>
+        </is>
+      </c>
+    </row>
+    <row r="3589">
+      <c r="A3589" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3589" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3589" t="inlineStr">
+        <is>
+          <t>東北地方イオンモール伊達 2026年11月27日(金)9：00~開業！どのような施設に？テナント情報随時更新中！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3589" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/17982</t>
+        </is>
+      </c>
+    </row>
+    <row r="3590">
+      <c r="A3590" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3590" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3590" t="inlineStr">
+        <is>
+          <t>東北地方仙台工業団地跡地 大型商業施設 2027年以降開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3590" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/23173</t>
+        </is>
+      </c>
+    </row>
+    <row r="3591">
+      <c r="A3591" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3591" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3591" t="inlineStr">
+        <is>
+          <t>中部地方そよら三条須頃 2025年11月7日(金)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3591" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/36987</t>
+        </is>
+      </c>
+    </row>
+    <row r="3592">
+      <c r="A3592" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3592" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3592" t="inlineStr">
+        <is>
+          <t>関東地方マルイシティ横浜 2026年2月28日(土)閉店！ 跡地はどうなる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3592" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/46498</t>
+        </is>
+      </c>
+    </row>
+    <row r="3593">
+      <c r="A3593" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3593" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3593" t="inlineStr">
+        <is>
+          <t>九州地方トライアルスマート小倉熊谷店 2026年12月初旬に開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3593" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/48785</t>
+        </is>
+      </c>
+    </row>
+    <row r="3594">
+      <c r="A3594" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3594" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3594" t="inlineStr">
+        <is>
+          <t>中部地方三郷駅前地区市街地再開発事業 2029年春完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3594" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/24605</t>
+        </is>
+      </c>
+    </row>
+    <row r="3595">
+      <c r="A3595" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3595" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3595" t="inlineStr">
+        <is>
+          <t>九州地方HAKOZAKI BLOCK（ハコザキブロック） 2028年度より街びらき！商業施設も誕生！最新情報も！福岡市東区の九州大学箱崎キャンパス跡地で、日本最大級の次世代スマートシティプロジェクト「HAKOZAKI BLOCK（ハコザキブロック）」が本格始動し、2028年度より順次まちびらき！プロジェクト名称が「HAKOZAKI BLOCK（ハコザ...2026.10.23九州地方</t>
+        </is>
+      </c>
+      <c r="D3595" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/46612</t>
+        </is>
+      </c>
+    </row>
+    <row r="3596">
+      <c r="A3596" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3596" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3596" t="inlineStr">
+        <is>
+          <t>関東地方太田駅南口再開発 ベルク太田駅前店 2026年10月21日(水)開業！全3テナント一覧！最新情報も！群馬県太田市の太田駅南口、旧ドン・キホーテ太田店跡地の大規模再開発施設「ベルク太田駅前店」が2026年10月21日(水)にグランドオープンしました！太田駅前に待望の大型生活拠点SCが誕生！食品スーパーマーケット「ベルク太田駅前店」を核店舗に...2026.10.23関東地方</t>
+        </is>
+      </c>
+      <c r="D3596" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47305</t>
+        </is>
+      </c>
+    </row>
+    <row r="3597">
+      <c r="A3597" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3597" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3597" t="inlineStr">
+        <is>
+          <t>イオンリテール／茨城県牛久市に「そよらひたち野うしく」11月18日オープン</t>
+        </is>
+      </c>
+      <c r="D3597" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102342.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3598">
+      <c r="A3598" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3598" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3598" t="inlineStr">
+        <is>
+          <t>ニトリ／世界最大の旗艦店「梅田茶屋町店」10月30日オープン、梅田ロフト跡地に出店</t>
+        </is>
+      </c>
+      <c r="D3598" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102379.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3599">
+      <c r="A3599" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3599" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3599" t="inlineStr">
+        <is>
+          <t>マルエツ／東京都大田区「新糀谷店」10月30日リニューアルオープン、鮮魚を対面販売</t>
+        </is>
+      </c>
+      <c r="D3599" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102343.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3600">
+      <c r="A3600" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3600" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3600" t="inlineStr">
+        <is>
+          <t>大和ハウス／福岡市に「ボートレース福岡 天神ストリートパーク」10月30日オープン</t>
+        </is>
+      </c>
+      <c r="D3600" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102381.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3601">
+      <c r="A3601" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3601" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3601" t="inlineStr">
+        <is>
+          <t>NTT都市開発／広島市「パセーラ」11月6日リニューアル、来春までに5店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3601" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102378.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3602">
+      <c r="A3602" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3602" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3602" t="inlineStr">
+        <is>
+          <t>ヤマダデンキ／「広島本店」11月6日オープン、体験型の展示充実・トレンド商品そろう</t>
+        </is>
+      </c>
+      <c r="D3602" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102377.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3603">
+      <c r="A3603" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3603" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3603" t="inlineStr">
+        <is>
+          <t>バローグループ／大阪府高槻市に「たこ一高槻駅前店」10月30日オープン</t>
+        </is>
+      </c>
+      <c r="D3603" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102311.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3604">
+      <c r="A3604" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3604" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3604" t="inlineStr">
+        <is>
+          <t>阪急オアシスマルシェ武庫之荘店／10月30日オープン、価値訴求型店舗に転換</t>
+        </is>
+      </c>
+      <c r="D3604" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102314.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3605">
+      <c r="A3605" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3605" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3605" t="inlineStr">
+        <is>
+          <t>メガネトップ／東京都国分寺市に「眼鏡市場 セレオ国分寺店」オープン</t>
+        </is>
+      </c>
+      <c r="D3605" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102371.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3606">
+      <c r="A3606" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3606" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3606" t="inlineStr">
+        <is>
+          <t>バーガーキング／「そよらつくば学園の森店」「下丸子駅前店」10月下旬オープン</t>
+        </is>
+      </c>
+      <c r="D3606" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102376.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3607">
+      <c r="A3607" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3607" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3607" t="inlineStr">
+        <is>
+          <t>ゴンチャ／東京都墨田区「東京ソラマチ店」10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D3607" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102373.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3608">
+      <c r="A3608" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3608" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3608" t="inlineStr">
+        <is>
+          <t>ホットランド／「厚切りとんかつ よし平 各務原店」10月28日オープン、岐阜県初出店</t>
+        </is>
+      </c>
+      <c r="D3608" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102380.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3609">
+      <c r="A3609" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3609" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3609" t="inlineStr">
+        <is>
+          <t>コロワイド／「チーズガーデン 遠鉄百貨店」11月20日オープン、静岡県初出店</t>
+        </is>
+      </c>
+      <c r="D3609" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102374.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3610">
+      <c r="A3610" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3610" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3610" t="inlineStr">
+        <is>
+          <t>やまや／宮城県仙台市「泉パークタウンタピオ店」オープン、世界各国の酒・食品充実</t>
+        </is>
+      </c>
+      <c r="D3610" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102372.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3611">
+      <c r="A3611" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3611" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3611" t="inlineStr">
+        <is>
+          <t>オンデーズ／「鹿児島天文館店」「ヴェルサウォーク西尾店」同日オープン</t>
+        </is>
+      </c>
+      <c r="D3611" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102375.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3612">
+      <c r="A3612" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3612" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3612" t="inlineStr">
+        <is>
+          <t>チヨダ／1号店「高円寺店」をリニューアル、ハンズフリーシューズを拡充</t>
+        </is>
+      </c>
+      <c r="D3612" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102344.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3613">
+      <c r="A3613" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3613" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3613" t="inlineStr">
+        <is>
+          <t>三菱地所プロパティマネジメント／丸の内エリア、今秋20店舗が新規・改装オープン</t>
+        </is>
+      </c>
+      <c r="D3613" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102212.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3614">
+      <c r="A3614" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3614" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3614" t="inlineStr">
+        <is>
+          <t>イオンフードスタイル／「フードスタイル東五反田店」10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D3614" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102214.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3615">
+      <c r="A3615" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3615" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3615" t="inlineStr">
+        <is>
+          <t>イオンウエルシア九州／熊本市東区に「ウエルシアプラス長嶺南店」10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D3615" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102279.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3616">
+      <c r="A3616" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="B3616" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3616" t="inlineStr">
+        <is>
+          <t>ロピア／鹿児島県に初出店「鹿児島宇宿店」来夏オープン</t>
+        </is>
+      </c>
+      <c r="D3616" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102275.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-24
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3616"/>
+  <dimension ref="A1:D3700"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -79968,6 +79968,1854 @@
         </is>
       </c>
     </row>
+    <row r="3617">
+      <c r="A3617" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3617" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3617" t="inlineStr">
+        <is>
+          <t>10/28厚切りとんかつ よし平 各務原店</t>
+        </is>
+      </c>
+      <c r="D3617" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3618">
+      <c r="A3618" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3618" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3618" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3618" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="3619">
+      <c r="A3619" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3619" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3619" t="inlineStr">
+        <is>
+          <t>10/8建替 ツルヤなぎさ店(長野県松本市)</t>
+        </is>
+      </c>
+      <c r="D3619" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="3620">
+      <c r="A3620" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3620" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3620" t="inlineStr">
+        <is>
+          <t>10/9そよら鳥取駅南</t>
+        </is>
+      </c>
+      <c r="D3620" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gyC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3621">
+      <c r="A3621" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3621" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3621" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D3621" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="3622">
+      <c r="A3622" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3622" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3622" t="inlineStr">
+        <is>
+          <t>10/16KOmart fine長泉店</t>
+        </is>
+      </c>
+      <c r="D3622" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gFD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3623">
+      <c r="A3623" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3623" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3623" t="inlineStr">
+        <is>
+          <t>10/16改装 平和堂大野店（食品売場）</t>
+        </is>
+      </c>
+      <c r="D3623" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gDK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3624">
+      <c r="A3624" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3624" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3624" t="inlineStr">
+        <is>
+          <t>(10/20プレ)10/21スーパーセンタートライアル愛知川店</t>
+        </is>
+      </c>
+      <c r="D3624" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gHm</t>
+        </is>
+      </c>
+    </row>
+    <row r="3625">
+      <c r="A3625" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3625" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3625" t="inlineStr">
+        <is>
+          <t>10/21魚市場食堂平の屋(愛知県岡崎市)</t>
+        </is>
+      </c>
+      <c r="D3625" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gGK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3626">
+      <c r="A3626" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3626" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3626" t="inlineStr">
+        <is>
+          <t>10/21ロピア加須ビバモール店(埼玉県加須市)</t>
+        </is>
+      </c>
+      <c r="D3626" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gE6</t>
+        </is>
+      </c>
+    </row>
+    <row r="3627">
+      <c r="A3627" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3627" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3627" t="inlineStr">
+        <is>
+          <t>10/21ベルク太田駅前店(群馬県太田市)</t>
+        </is>
+      </c>
+      <c r="D3627" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gJJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3628">
+      <c r="A3628" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3628" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3628" t="inlineStr">
+        <is>
+          <t>10/22業務スーパー西帯広店</t>
+        </is>
+      </c>
+      <c r="D3628" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gG7</t>
+        </is>
+      </c>
+    </row>
+    <row r="3629">
+      <c r="A3629" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3629" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3629" t="inlineStr">
+        <is>
+          <t>10/22サンディ千船店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D3629" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3630">
+      <c r="A3630" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3630" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3630" t="inlineStr">
+        <is>
+          <t>10/22マックスバリュエクスプレス栄5丁目店(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D3630" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eRp</t>
+        </is>
+      </c>
+    </row>
+    <row r="3631">
+      <c r="A3631" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3631" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3631" t="inlineStr">
+        <is>
+          <t>10/23スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D3631" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="3632">
+      <c r="A3632" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3632" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3632" t="inlineStr">
+        <is>
+          <t>10/27やまのぶ赤池店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3632" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1dGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3633">
+      <c r="A3633" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3633" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3633" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D3633" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3634">
+      <c r="A3634" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3634" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3634" t="inlineStr">
+        <is>
+          <t>10/30松屋可児店（松のや併設）</t>
+        </is>
+      </c>
+      <c r="D3634" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gEg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3635">
+      <c r="A3635" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3635" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3635" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D3635" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3636">
+      <c r="A3636" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3636" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3636" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D3636" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="3637">
+      <c r="A3637" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3637" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3637" t="inlineStr">
+        <is>
+          <t>12/14マクドナルド池田本郷店(岐阜県)</t>
+        </is>
+      </c>
+      <c r="D3637" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3638">
+      <c r="A3638" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3638" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3638" t="inlineStr">
+        <is>
+          <t>12/30マクドナルド各務原いちょう通り店</t>
+        </is>
+      </c>
+      <c r="D3638" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gMH</t>
+        </is>
+      </c>
+    </row>
+    <row r="3639">
+      <c r="A3639" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3639" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3639" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D3639" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="3640">
+      <c r="A3640" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3640" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3640" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D3640" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="3641">
+      <c r="A3641" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3641" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3641" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3641" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3642">
+      <c r="A3642" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3642" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3642" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3642" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3643">
+      <c r="A3643" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3643" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3643" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3643" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3644">
+      <c r="A3644" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3644" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3644" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3644" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3645">
+      <c r="A3645" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3645" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3645" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3645" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3646">
+      <c r="A3646" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3646" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3646" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3646" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3647">
+      <c r="A3647" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3647" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3647" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3647" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3648">
+      <c r="A3648" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3648" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3648" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3648" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3649">
+      <c r="A3649" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3649" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3649" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3649" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3650">
+      <c r="A3650" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3650" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3650" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3650" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3651">
+      <c r="A3651" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3651" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3651" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3651" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3652">
+      <c r="A3652" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3652" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3652" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3652" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3653">
+      <c r="A3653" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3653" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3653" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3653" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3654">
+      <c r="A3654" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3654" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3654" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3654" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3655">
+      <c r="A3655" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3655" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3655" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3655" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3656">
+      <c r="A3656" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3656" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3656" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3656" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3657">
+      <c r="A3657" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3657" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3657" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3657" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3658">
+      <c r="A3658" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3658" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3658" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3658" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3659">
+      <c r="A3659" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3659" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3659" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3659" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3660">
+      <c r="A3660" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3660" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3660" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3660" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3661">
+      <c r="A3661" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3661" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3661" t="inlineStr">
+        <is>
+          <t>九州地方諫早プロジェクト(ゆめタウン諫早) 2028年春開業！どのような商業施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3661" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/14603</t>
+        </is>
+      </c>
+    </row>
+    <row r="3662">
+      <c r="A3662" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3662" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3662" t="inlineStr">
+        <is>
+          <t>関東地方日本橋一丁目東地区市街地再開発事業 2032年開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3662" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36113</t>
+        </is>
+      </c>
+    </row>
+    <row r="3663">
+      <c r="A3663" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3663" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3663" t="inlineStr">
+        <is>
+          <t>関西地方神戸市役所本庁舎2号館再整備事業 2030年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3663" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/27303</t>
+        </is>
+      </c>
+    </row>
+    <row r="3664">
+      <c r="A3664" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3664" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3664" t="inlineStr">
+        <is>
+          <t>東北地方ニトリ福島御山店 2027年3月開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3664" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/49620</t>
+        </is>
+      </c>
+    </row>
+    <row r="3665">
+      <c r="A3665" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3665" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3665" t="inlineStr">
+        <is>
+          <t>関東地方太田駅南口再開発 ベルク太田駅前店 2026年10月21日(水)開業！全3テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3665" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47305</t>
+        </is>
+      </c>
+    </row>
+    <row r="3666">
+      <c r="A3666" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3666" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3666" t="inlineStr">
+        <is>
+          <t>関東地方TOCビル 建て替えて2027年竣工！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3666" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/23255</t>
+        </is>
+      </c>
+    </row>
+    <row r="3667">
+      <c r="A3667" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3667" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3667" t="inlineStr">
+        <is>
+          <t>関西地方アクロスプラザ和泉観音寺 2026年11月開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3667" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/47867</t>
+        </is>
+      </c>
+    </row>
+    <row r="3668">
+      <c r="A3668" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3668" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3668" t="inlineStr">
+        <is>
+          <t>関東地方西武渋谷店 2026年9月30日(水)閉店 跡地はどうなる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3668" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47951</t>
+        </is>
+      </c>
+    </row>
+    <row r="3669">
+      <c r="A3669" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3669" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3669" t="inlineStr">
+        <is>
+          <t>関西地方ミラモール東岸和田駅前 住友商事が2025年9月25日(木)~順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3669" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39056</t>
+        </is>
+      </c>
+    </row>
+    <row r="3670">
+      <c r="A3670" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3670" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3670" t="inlineStr">
+        <is>
+          <t>関東地方ミラゾ池袋 グランドシティタワー池袋 2026年夏より順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3670" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26771</t>
+        </is>
+      </c>
+    </row>
+    <row r="3671">
+      <c r="A3671" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3671" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3671" t="inlineStr">
+        <is>
+          <t>関東地方スーパーセンタートライアル深谷川本店 2026年4月29日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3671" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/44915</t>
+        </is>
+      </c>
+    </row>
+    <row r="3672">
+      <c r="A3672" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3672" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3672" t="inlineStr">
+        <is>
+          <t>関西地方クオーツ心斎橋 2026年4月25日(土)開業！全52店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3672" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/25158</t>
+        </is>
+      </c>
+    </row>
+    <row r="3673">
+      <c r="A3673" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3673" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3673" t="inlineStr">
+        <is>
+          <t>中部地方武蔵ヶ辻A地区市街地再開発事業 エムザ再開発！どのような施設になる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3673" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/49728</t>
+        </is>
+      </c>
+    </row>
+    <row r="3674">
+      <c r="A3674" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3674" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3674" t="inlineStr">
+        <is>
+          <t>中部地方コメリパワー亀山店 2027年3月開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3674" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48442</t>
+        </is>
+      </c>
+    </row>
+    <row r="3675">
+      <c r="A3675" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3675" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3675" t="inlineStr">
+        <is>
+          <t>東北地方イオンモール伊達 2026年11月27日(金)9：00~開業！どのような施設に？テナント情報随時更新中！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3675" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/17982</t>
+        </is>
+      </c>
+    </row>
+    <row r="3676">
+      <c r="A3676" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3676" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3676" t="inlineStr">
+        <is>
+          <t>関東地方明治安田新宿ビル 2026年11月下旬以降開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3676" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26240</t>
+        </is>
+      </c>
+    </row>
+    <row r="3677">
+      <c r="A3677" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3677" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3677" t="inlineStr">
+        <is>
+          <t>関東地方SHIKANISHI Terrace 鹿西テラス(ベルクス足立鹿浜店) 2026年3月19日(木)~順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3677" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/31997</t>
+        </is>
+      </c>
+    </row>
+    <row r="3678">
+      <c r="A3678" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3678" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3678" t="inlineStr">
+        <is>
+          <t>中部地方新潟駅万代口東地区開発計画 2028年夏開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3678" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48895</t>
+        </is>
+      </c>
+    </row>
+    <row r="3679">
+      <c r="A3679" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3679" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3679" t="inlineStr">
+        <is>
+          <t>関東地方境北商業集積計画 2027年春開業！テナントは？最新情報も！群馬県伊勢崎市の国道354号線沿い、東武伊勢崎線「境町」駅近くにフレッセイの商業施設「境北商業集積計画」が2027年春開業！境北商業集積計画は、食品スーパーマーケットのフレッセイを中心に、コメリの大型店舗など複数店舗が出店！境北商業集積計画...2026.10.24関東地方</t>
+        </is>
+      </c>
+      <c r="D3679" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42268</t>
+        </is>
+      </c>
+    </row>
+    <row r="3680">
+      <c r="A3680" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3680" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3680" t="inlineStr">
+        <is>
+          <t>九州地方イオン鹿児島鴨池店 2024年8月31日(土)に閉店し建て替えへ！イオンモールが取得！最新情報も！鹿児島県鹿児島市の商業施設「イオン鹿児島鴨池店」が2024年8月31日(土)をもって閉店し、現在跡地の再開発計画が大きく動き出しています！旧店舗の解体工事が完了し、約3.6万㎡（約1.1万坪）におよぶ広大な敷地を「イオンモール」が取得！既存...2026.10.24九州地方</t>
+        </is>
+      </c>
+      <c r="D3680" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/36900</t>
+        </is>
+      </c>
+    </row>
+    <row r="3681">
+      <c r="A3681" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3681" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3681" t="inlineStr">
+        <is>
+          <t>イオンリテール／茨城県牛久市に「そよらひたち野うしく」11月18日オープン</t>
+        </is>
+      </c>
+      <c r="D3681" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102342.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3682">
+      <c r="A3682" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3682" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3682" t="inlineStr">
+        <is>
+          <t>ニトリ／世界最大の旗艦店「梅田茶屋町店」10月30日オープン、梅田ロフト跡地に出店</t>
+        </is>
+      </c>
+      <c r="D3682" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102379.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3683">
+      <c r="A3683" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3683" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3683" t="inlineStr">
+        <is>
+          <t>マルエツ／東京都大田区「新糀谷店」10月30日リニューアルオープン、鮮魚を対面販売</t>
+        </is>
+      </c>
+      <c r="D3683" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102343.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3684">
+      <c r="A3684" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3684" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3684" t="inlineStr">
+        <is>
+          <t>大和ハウス／福岡市に「ボートレース福岡 天神ストリートパーク」10月30日オープン</t>
+        </is>
+      </c>
+      <c r="D3684" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102381.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3685">
+      <c r="A3685" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3685" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3685" t="inlineStr">
+        <is>
+          <t>NTT都市開発／広島市「パセーラ」11月6日リニューアル、来春までに5店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3685" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102378.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3686">
+      <c r="A3686" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3686" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3686" t="inlineStr">
+        <is>
+          <t>ヤマダデンキ／「広島本店」11月6日オープン、体験型の展示充実・トレンド商品そろう</t>
+        </is>
+      </c>
+      <c r="D3686" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102377.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3687">
+      <c r="A3687" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3687" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3687" t="inlineStr">
+        <is>
+          <t>バローグループ／大阪府高槻市に「たこ一高槻駅前店」10月30日オープン</t>
+        </is>
+      </c>
+      <c r="D3687" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102311.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3688">
+      <c r="A3688" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3688" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3688" t="inlineStr">
+        <is>
+          <t>阪急オアシスマルシェ武庫之荘店／10月30日オープン、価値訴求型店舗に転換</t>
+        </is>
+      </c>
+      <c r="D3688" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102314.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3689">
+      <c r="A3689" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3689" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3689" t="inlineStr">
+        <is>
+          <t>メガネトップ／東京都国分寺市に「眼鏡市場 セレオ国分寺店」オープン</t>
+        </is>
+      </c>
+      <c r="D3689" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102371.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3690">
+      <c r="A3690" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3690" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3690" t="inlineStr">
+        <is>
+          <t>バーガーキング／「そよらつくば学園の森店」「下丸子駅前店」10月下旬オープン</t>
+        </is>
+      </c>
+      <c r="D3690" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102376.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3691">
+      <c r="A3691" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3691" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3691" t="inlineStr">
+        <is>
+          <t>ゴンチャ／東京都墨田区「東京ソラマチ店」10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D3691" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102373.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3692">
+      <c r="A3692" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3692" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3692" t="inlineStr">
+        <is>
+          <t>ホットランド／「厚切りとんかつ よし平 各務原店」10月28日オープン、岐阜県初出店</t>
+        </is>
+      </c>
+      <c r="D3692" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102380.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3693">
+      <c r="A3693" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3693" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3693" t="inlineStr">
+        <is>
+          <t>コロワイド／「チーズガーデン 遠鉄百貨店」11月20日オープン、静岡県初出店</t>
+        </is>
+      </c>
+      <c r="D3693" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102374.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3694">
+      <c r="A3694" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3694" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3694" t="inlineStr">
+        <is>
+          <t>やまや／宮城県仙台市「泉パークタウンタピオ店」オープン、世界各国の酒・食品充実</t>
+        </is>
+      </c>
+      <c r="D3694" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102372.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3695">
+      <c r="A3695" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3695" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3695" t="inlineStr">
+        <is>
+          <t>オンデーズ／「鹿児島天文館店」「ヴェルサウォーク西尾店」同日オープン</t>
+        </is>
+      </c>
+      <c r="D3695" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102375.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3696">
+      <c r="A3696" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3696" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3696" t="inlineStr">
+        <is>
+          <t>チヨダ／1号店「高円寺店」をリニューアル、ハンズフリーシューズを拡充</t>
+        </is>
+      </c>
+      <c r="D3696" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102344.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3697">
+      <c r="A3697" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3697" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3697" t="inlineStr">
+        <is>
+          <t>三菱地所プロパティマネジメント／丸の内エリア、今秋20店舗が新規・改装オープン</t>
+        </is>
+      </c>
+      <c r="D3697" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102212.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3698">
+      <c r="A3698" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3698" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3698" t="inlineStr">
+        <is>
+          <t>イオンフードスタイル／「フードスタイル東五反田店」10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D3698" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102214.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3699">
+      <c r="A3699" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3699" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3699" t="inlineStr">
+        <is>
+          <t>イオンウエルシア九州／熊本市東区に「ウエルシアプラス長嶺南店」10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D3699" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102279.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3700">
+      <c r="A3700" t="inlineStr">
+        <is>
+          <t>2026年10月24日</t>
+        </is>
+      </c>
+      <c r="B3700" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3700" t="inlineStr">
+        <is>
+          <t>ロピア／鹿児島県に初出店「鹿児島宇宿店」来夏オープン</t>
+        </is>
+      </c>
+      <c r="D3700" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102275.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-25
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3700"/>
+  <dimension ref="A1:D3788"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81816,6 +81816,1942 @@
         </is>
       </c>
     </row>
+    <row r="3701">
+      <c r="A3701" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3701" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3701" t="inlineStr">
+        <is>
+          <t>10/25そよらつくば学園の森(茨城県つくば市)</t>
+        </is>
+      </c>
+      <c r="D3701" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gvs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3702">
+      <c r="A3702" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3702" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3702" t="inlineStr">
+        <is>
+          <t>タウンプラザかねひで南風原市場</t>
+        </is>
+      </c>
+      <c r="D3702" t="inlineStr">
+        <is>
+          <t>https://www.kanehideshj.com/store/%E3%82%BF%E3%82%A6%E3%83%B3%E3%83%97%E3%83%A9%E3%82%B6-%E6%9C%AC%E5%B3%B6%E5%8D%97%E9%83%A8%E5%9C%B0%E5%8C%BA%E3%80%90%E9%82%A3%E8%A6%87%E5%B8%82%E3%80%91%EF%BC%9A%E3%82%BF%E3%82%A6%E3%83%B3-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3703">
+      <c r="A3703" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3703" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3703" t="inlineStr">
+        <is>
+          <t>10/2大阪屋ショップ日進店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3703" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-18La</t>
+        </is>
+      </c>
+    </row>
+    <row r="3704">
+      <c r="A3704" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3704" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3704" t="inlineStr">
+        <is>
+          <t>10/8建替 ツルヤなぎさ店(長野県松本市)</t>
+        </is>
+      </c>
+      <c r="D3704" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="3705">
+      <c r="A3705" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3705" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3705" t="inlineStr">
+        <is>
+          <t>10/9そよら鳥取駅南</t>
+        </is>
+      </c>
+      <c r="D3705" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gyC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3706">
+      <c r="A3706" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3706" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3706" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D3706" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="3707">
+      <c r="A3707" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3707" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3707" t="inlineStr">
+        <is>
+          <t>10/16KOmart fine長泉店</t>
+        </is>
+      </c>
+      <c r="D3707" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gFD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3708">
+      <c r="A3708" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3708" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3708" t="inlineStr">
+        <is>
+          <t>10/16改装 平和堂大野店（食品売場）</t>
+        </is>
+      </c>
+      <c r="D3708" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gDK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3709">
+      <c r="A3709" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3709" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3709" t="inlineStr">
+        <is>
+          <t>(10/20プレ)10/21スーパーセンタートライアル愛知川店</t>
+        </is>
+      </c>
+      <c r="D3709" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gHm</t>
+        </is>
+      </c>
+    </row>
+    <row r="3710">
+      <c r="A3710" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3710" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3710" t="inlineStr">
+        <is>
+          <t>10/21魚市場食堂平の屋(愛知県岡崎市)</t>
+        </is>
+      </c>
+      <c r="D3710" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gGK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3711">
+      <c r="A3711" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3711" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3711" t="inlineStr">
+        <is>
+          <t>10/21ロピア加須ビバモール店(埼玉県加須市)</t>
+        </is>
+      </c>
+      <c r="D3711" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gE6</t>
+        </is>
+      </c>
+    </row>
+    <row r="3712">
+      <c r="A3712" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3712" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3712" t="inlineStr">
+        <is>
+          <t>10/21ベルク太田駅前店(群馬県太田市)</t>
+        </is>
+      </c>
+      <c r="D3712" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gJJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3713">
+      <c r="A3713" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3713" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3713" t="inlineStr">
+        <is>
+          <t>10/22業務スーパー西帯広店</t>
+        </is>
+      </c>
+      <c r="D3713" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gG7</t>
+        </is>
+      </c>
+    </row>
+    <row r="3714">
+      <c r="A3714" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3714" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3714" t="inlineStr">
+        <is>
+          <t>10/22サンディ千船店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D3714" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3715">
+      <c r="A3715" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3715" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3715" t="inlineStr">
+        <is>
+          <t>10/22マックスバリュエクスプレス栄5丁目店(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D3715" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eRp</t>
+        </is>
+      </c>
+    </row>
+    <row r="3716">
+      <c r="A3716" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3716" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3716" t="inlineStr">
+        <is>
+          <t>10/23スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D3716" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="3717">
+      <c r="A3717" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3717" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3717" t="inlineStr">
+        <is>
+          <t>10/23トライアル西友町田店</t>
+        </is>
+      </c>
+      <c r="D3717" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gOi</t>
+        </is>
+      </c>
+    </row>
+    <row r="3718">
+      <c r="A3718" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3718" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3718" t="inlineStr">
+        <is>
+          <t>10/23ザ・ビッグ千歳武道館前店</t>
+        </is>
+      </c>
+      <c r="D3718" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3719">
+      <c r="A3719" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3719" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3719" t="inlineStr">
+        <is>
+          <t>10/23廻転鮨 銀座おのでらハレザ池袋店</t>
+        </is>
+      </c>
+      <c r="D3719" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gOs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3720">
+      <c r="A3720" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3720" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3720" t="inlineStr">
+        <is>
+          <t>10/27やまのぶ赤池店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3720" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1dGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3721">
+      <c r="A3721" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3721" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3721" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D3721" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3722">
+      <c r="A3722" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3722" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3722" t="inlineStr">
+        <is>
+          <t>10/30松屋可児店（松のや併設）</t>
+        </is>
+      </c>
+      <c r="D3722" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gEg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3723">
+      <c r="A3723" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3723" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3723" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D3723" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3724">
+      <c r="A3724" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3724" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3724" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D3724" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="3725">
+      <c r="A3725" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3725" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3725" t="inlineStr">
+        <is>
+          <t>12/14マクドナルド池田本郷店(岐阜県)</t>
+        </is>
+      </c>
+      <c r="D3725" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3726">
+      <c r="A3726" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3726" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3726" t="inlineStr">
+        <is>
+          <t>12/30マクドナルド各務原いちょう通り店</t>
+        </is>
+      </c>
+      <c r="D3726" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gMH</t>
+        </is>
+      </c>
+    </row>
+    <row r="3727">
+      <c r="A3727" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3727" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3727" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D3727" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="3728">
+      <c r="A3728" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3728" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3728" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D3728" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="3729">
+      <c r="A3729" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3729" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3729" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3729" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3730">
+      <c r="A3730" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3730" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3730" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3730" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3731">
+      <c r="A3731" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3731" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3731" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3731" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3732">
+      <c r="A3732" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3732" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3732" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3732" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3733">
+      <c r="A3733" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3733" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3733" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3733" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3734">
+      <c r="A3734" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3734" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3734" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3734" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3735">
+      <c r="A3735" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3735" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3735" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3735" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3736">
+      <c r="A3736" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3736" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3736" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3736" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3737">
+      <c r="A3737" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3737" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3737" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3737" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3738">
+      <c r="A3738" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3738" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3738" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3738" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3739">
+      <c r="A3739" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3739" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3739" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3739" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3740">
+      <c r="A3740" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3740" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3740" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3740" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3741">
+      <c r="A3741" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3741" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3741" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3741" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3742">
+      <c r="A3742" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3742" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3742" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3742" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3743">
+      <c r="A3743" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3743" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3743" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3743" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3744">
+      <c r="A3744" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3744" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3744" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3744" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3745">
+      <c r="A3745" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3745" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3745" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3745" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3746">
+      <c r="A3746" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3746" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3746" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3746" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3747">
+      <c r="A3747" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3747" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3747" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3747" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3748">
+      <c r="A3748" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3748" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3748" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3748" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3749">
+      <c r="A3749" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3749" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3749" t="inlineStr">
+        <is>
+          <t>関西地方【計画延期】大阪ガスビルディング（ガスビル） 再開発 2027年以降開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3749" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/30050</t>
+        </is>
+      </c>
+    </row>
+    <row r="3750">
+      <c r="A3750" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3750" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3750" t="inlineStr">
+        <is>
+          <t>関東地方星天qlay 2025年3月27日(木)全エリア グランドオープン！全28テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3750" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/24855</t>
+        </is>
+      </c>
+    </row>
+    <row r="3751">
+      <c r="A3751" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3751" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3751" t="inlineStr">
+        <is>
+          <t>中部地方カインズ東海店 2026年3月25日(水)開業！全6テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3751" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/44325</t>
+        </is>
+      </c>
+    </row>
+    <row r="3752">
+      <c r="A3752" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3752" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3752" t="inlineStr">
+        <is>
+          <t>関東地方そよらひたち野うしく 西友跡地 2026年11月18日(水)開業！全29テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3752" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/44853</t>
+        </is>
+      </c>
+    </row>
+    <row r="3753">
+      <c r="A3753" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3753" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3753" t="inlineStr">
+        <is>
+          <t>中国地方ハローズ呉広モール 2025年12月17日(水)開業！全7店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3753" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/42161</t>
+        </is>
+      </c>
+    </row>
+    <row r="3754">
+      <c r="A3754" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3754" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3754" t="inlineStr">
+        <is>
+          <t>関西地方iyouTown（アイユータウン）須磨 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3754" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/43508</t>
+        </is>
+      </c>
+    </row>
+    <row r="3755">
+      <c r="A3755" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3755" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3755" t="inlineStr">
+        <is>
+          <t>関西地方アークスクエア茨木 2025年5月21日(水)より順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3755" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/21729</t>
+        </is>
+      </c>
+    </row>
+    <row r="3756">
+      <c r="A3756" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3756" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3756" t="inlineStr">
+        <is>
+          <t>関東地方マミーマート 見沼区東新井 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3756" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47301</t>
+        </is>
+      </c>
+    </row>
+    <row r="3757">
+      <c r="A3757" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3757" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3757" t="inlineStr">
+        <is>
+          <t>関西地方泉ケ丘駅前活性化計画 計画再始動！商業施設は2028年度開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3757" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/23983</t>
+        </is>
+      </c>
+    </row>
+    <row r="3758">
+      <c r="A3758" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3758" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3758" t="inlineStr">
+        <is>
+          <t>中国地方広島駅ビル「minamoa（ミナモア）」2025年3月24日(月)開業！全220テナント公開！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3758" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/7700</t>
+        </is>
+      </c>
+    </row>
+    <row r="3759">
+      <c r="A3759" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3759" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3759" t="inlineStr">
+        <is>
+          <t>関東地方ミラゾ池袋 グランドシティタワー池袋 2026年夏より順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3759" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26771</t>
+        </is>
+      </c>
+    </row>
+    <row r="3760">
+      <c r="A3760" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3760" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3760" t="inlineStr">
+        <is>
+          <t>東北地方イオン土崎港店跡地 2026年2月28日閉店 跡地はどうなる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3760" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/45956</t>
+        </is>
+      </c>
+    </row>
+    <row r="3761">
+      <c r="A3761" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3761" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3761" t="inlineStr">
+        <is>
+          <t>関東地方ヨークタウン小山羽川 2026年8月28日(金)開業！全4テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3761" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48080</t>
+        </is>
+      </c>
+    </row>
+    <row r="3762">
+      <c r="A3762" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3762" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3762" t="inlineStr">
+        <is>
+          <t>関西地方レイクウェル堅田 2025年10月31日(金)より順次開業！全4テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3762" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/42148</t>
+        </is>
+      </c>
+    </row>
+    <row r="3763">
+      <c r="A3763" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3763" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3763" t="inlineStr">
+        <is>
+          <t>中部地方イオン今池店 ブランズタワー名古屋今池 2024年2月29日(木)に閉店し建て替え！2028年以降開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3763" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/33420</t>
+        </is>
+      </c>
+    </row>
+    <row r="3764">
+      <c r="A3764" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3764" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3764" t="inlineStr">
+        <is>
+          <t>九州地方ミーナ天神が建て替え検討！2030年代開業！どのような施設になる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3764" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/49546</t>
+        </is>
+      </c>
+    </row>
+    <row r="3765">
+      <c r="A3765" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3765" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3765" t="inlineStr">
+        <is>
+          <t>関東地方TAIRAYA与野店 与野フード建て替え 2025年4月24日(木)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3765" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/37854</t>
+        </is>
+      </c>
+    </row>
+    <row r="3766">
+      <c r="A3766" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3766" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3766" t="inlineStr">
+        <is>
+          <t>関東地方イオンシネマ土岐 2025年4月18日(金)開業！どのような映画館に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3766" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/38692</t>
+        </is>
+      </c>
+    </row>
+    <row r="3767">
+      <c r="A3767" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3767" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3767" t="inlineStr">
+        <is>
+          <t>関東地方境北商業集積計画 2027年春開業！テナントは？最新情報も！群馬県伊勢崎市の国道354号線沿い、東武伊勢崎線「境町」駅近くにフレッセイの商業施設「境北商業集積計画」が2027年春開業！境北商業集積計画は、食品スーパーマーケットのフレッセイを中心に、コメリの大型店舗など複数店舗が出店！境北商業集積計画...2026.10.24関東地方</t>
+        </is>
+      </c>
+      <c r="D3767" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42268</t>
+        </is>
+      </c>
+    </row>
+    <row r="3768">
+      <c r="A3768" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3768" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3768" t="inlineStr">
+        <is>
+          <t>九州地方イオン鹿児島鴨池店 2024年8月31日(土)に閉店し建て替えへ！イオンモールが取得！最新情報も！鹿児島県鹿児島市の商業施設「イオン鹿児島鴨池店」が2024年8月31日(土)をもって閉店し、現在跡地の再開発計画が大きく動き出しています！旧店舗の解体工事が完了し、約3.6万㎡（約1.1万坪）におよぶ広大な敷地を「イオンモール」が取得！既存...2026.10.24九州地方</t>
+        </is>
+      </c>
+      <c r="D3768" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/36900</t>
+        </is>
+      </c>
+    </row>
+    <row r="3769">
+      <c r="A3769" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3769" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3769" t="inlineStr">
+        <is>
+          <t>イオンリテール／茨城県牛久市に「そよらひたち野うしく」11月18日オープン</t>
+        </is>
+      </c>
+      <c r="D3769" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102342.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3770">
+      <c r="A3770" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3770" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3770" t="inlineStr">
+        <is>
+          <t>ニトリ／世界最大の旗艦店「梅田茶屋町店」10月30日オープン、梅田ロフト跡地に出店</t>
+        </is>
+      </c>
+      <c r="D3770" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102379.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3771">
+      <c r="A3771" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3771" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3771" t="inlineStr">
+        <is>
+          <t>マルエツ／東京都大田区「新糀谷店」10月30日リニューアルオープン、鮮魚を対面販売</t>
+        </is>
+      </c>
+      <c r="D3771" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102343.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3772">
+      <c r="A3772" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3772" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3772" t="inlineStr">
+        <is>
+          <t>大和ハウス／福岡市に「ボートレース福岡 天神ストリートパーク」10月30日オープン</t>
+        </is>
+      </c>
+      <c r="D3772" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102381.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3773">
+      <c r="A3773" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3773" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3773" t="inlineStr">
+        <is>
+          <t>NTT都市開発／広島市「パセーラ」11月6日リニューアル、来春までに5店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3773" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102378.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3774">
+      <c r="A3774" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3774" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3774" t="inlineStr">
+        <is>
+          <t>ヤマダデンキ／「広島本店」11月6日オープン、体験型の展示充実・トレンド商品そろう</t>
+        </is>
+      </c>
+      <c r="D3774" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102377.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3775">
+      <c r="A3775" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3775" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3775" t="inlineStr">
+        <is>
+          <t>バローグループ／大阪府高槻市に「たこ一高槻駅前店」10月30日オープン</t>
+        </is>
+      </c>
+      <c r="D3775" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102311.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3776">
+      <c r="A3776" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3776" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3776" t="inlineStr">
+        <is>
+          <t>阪急オアシスマルシェ武庫之荘店／10月30日オープン、価値訴求型店舗に転換</t>
+        </is>
+      </c>
+      <c r="D3776" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102314.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3777">
+      <c r="A3777" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3777" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3777" t="inlineStr">
+        <is>
+          <t>メガネトップ／東京都国分寺市に「眼鏡市場 セレオ国分寺店」オープン</t>
+        </is>
+      </c>
+      <c r="D3777" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102371.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3778">
+      <c r="A3778" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3778" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3778" t="inlineStr">
+        <is>
+          <t>バーガーキング／「そよらつくば学園の森店」「下丸子駅前店」10月下旬オープン</t>
+        </is>
+      </c>
+      <c r="D3778" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102376.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3779">
+      <c r="A3779" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3779" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3779" t="inlineStr">
+        <is>
+          <t>ゴンチャ／東京都墨田区「東京ソラマチ店」10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D3779" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102373.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3780">
+      <c r="A3780" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3780" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3780" t="inlineStr">
+        <is>
+          <t>ホットランド／「厚切りとんかつ よし平 各務原店」10月28日オープン、岐阜県初出店</t>
+        </is>
+      </c>
+      <c r="D3780" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102380.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3781">
+      <c r="A3781" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3781" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3781" t="inlineStr">
+        <is>
+          <t>コロワイド／「チーズガーデン 遠鉄百貨店」11月20日オープン、静岡県初出店</t>
+        </is>
+      </c>
+      <c r="D3781" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102374.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3782">
+      <c r="A3782" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3782" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3782" t="inlineStr">
+        <is>
+          <t>やまや／宮城県仙台市「泉パークタウンタピオ店」オープン、世界各国の酒・食品充実</t>
+        </is>
+      </c>
+      <c r="D3782" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102372.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3783">
+      <c r="A3783" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3783" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3783" t="inlineStr">
+        <is>
+          <t>オンデーズ／「鹿児島天文館店」「ヴェルサウォーク西尾店」同日オープン</t>
+        </is>
+      </c>
+      <c r="D3783" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102375.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3784">
+      <c r="A3784" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3784" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3784" t="inlineStr">
+        <is>
+          <t>チヨダ／1号店「高円寺店」をリニューアル、ハンズフリーシューズを拡充</t>
+        </is>
+      </c>
+      <c r="D3784" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102344.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3785">
+      <c r="A3785" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3785" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3785" t="inlineStr">
+        <is>
+          <t>三菱地所プロパティマネジメント／丸の内エリア、今秋20店舗が新規・改装オープン</t>
+        </is>
+      </c>
+      <c r="D3785" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102212.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3786">
+      <c r="A3786" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3786" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3786" t="inlineStr">
+        <is>
+          <t>イオンフードスタイル／「フードスタイル東五反田店」10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D3786" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102214.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3787">
+      <c r="A3787" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3787" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3787" t="inlineStr">
+        <is>
+          <t>イオンウエルシア九州／熊本市東区に「ウエルシアプラス長嶺南店」10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D3787" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102279.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3788">
+      <c r="A3788" t="inlineStr">
+        <is>
+          <t>2026年10月25日</t>
+        </is>
+      </c>
+      <c r="B3788" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3788" t="inlineStr">
+        <is>
+          <t>ロピア／鹿児島県に初出店「鹿児島宇宿店」来夏オープン</t>
+        </is>
+      </c>
+      <c r="D3788" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102275.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-26
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3788"/>
+  <dimension ref="A1:D3848"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -83752,6 +83752,1326 @@
         </is>
       </c>
     </row>
+    <row r="3789">
+      <c r="A3789" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3789" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3789" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3789" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3790">
+      <c r="A3790" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3790" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3790" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3790" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3791">
+      <c r="A3791" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3791" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3791" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3791" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3792">
+      <c r="A3792" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3792" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3792" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3792" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3793">
+      <c r="A3793" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3793" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3793" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3793" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3794">
+      <c r="A3794" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3794" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3794" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3794" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3795">
+      <c r="A3795" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3795" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3795" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3795" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3796">
+      <c r="A3796" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3796" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3796" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3796" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3797">
+      <c r="A3797" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3797" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3797" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3797" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3798">
+      <c r="A3798" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3798" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3798" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3798" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3799">
+      <c r="A3799" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3799" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3799" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3799" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3800">
+      <c r="A3800" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3800" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3800" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3800" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3801">
+      <c r="A3801" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3801" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3801" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3801" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3802">
+      <c r="A3802" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3802" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3802" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3802" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3803">
+      <c r="A3803" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3803" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3803" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3803" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3804">
+      <c r="A3804" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3804" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3804" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3804" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3805">
+      <c r="A3805" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3805" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3805" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3805" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3806">
+      <c r="A3806" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3806" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3806" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3806" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3807">
+      <c r="A3807" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3807" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3807" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3807" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3808">
+      <c r="A3808" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3808" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3808" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3808" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3809">
+      <c r="A3809" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3809" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3809" t="inlineStr">
+        <is>
+          <t>関東地方イオン伊勢原店 2024年1月31日(水)に閉店し建て替えへ！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3809" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36886</t>
+        </is>
+      </c>
+    </row>
+    <row r="3810">
+      <c r="A3810" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3810" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3810" t="inlineStr">
+        <is>
+          <t>中部地方能美市福島町 複合商業施設 2027年度以降開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3810" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/36955</t>
+        </is>
+      </c>
+    </row>
+    <row r="3811">
+      <c r="A3811" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3811" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3811" t="inlineStr">
+        <is>
+          <t>中国地方そよら鳥取駅南 2026年10月9日(金)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3811" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/49474</t>
+        </is>
+      </c>
+    </row>
+    <row r="3812">
+      <c r="A3812" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3812" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3812" t="inlineStr">
+        <is>
+          <t>中部地方富士駅北口第一地区市街地再開発事業 2030年初頭開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3812" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/26250</t>
+        </is>
+      </c>
+    </row>
+    <row r="3813">
+      <c r="A3813" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3813" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3813" t="inlineStr">
+        <is>
+          <t>九州地方YAEYAMA GATE 石垣市役所跡地 2030年開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3813" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/33011</t>
+        </is>
+      </c>
+    </row>
+    <row r="3814">
+      <c r="A3814" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3814" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3814" t="inlineStr">
+        <is>
+          <t>中部地方三郷駅前地区市街地再開発事業 2029年春完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3814" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/24605</t>
+        </is>
+      </c>
+    </row>
+    <row r="3815">
+      <c r="A3815" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3815" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3815" t="inlineStr">
+        <is>
+          <t>関東地方藤沢駅南口391地区市街地再開発事業 2035年完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3815" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/32666</t>
+        </is>
+      </c>
+    </row>
+    <row r="3816">
+      <c r="A3816" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3816" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3816" t="inlineStr">
+        <is>
+          <t>関東地方コトエ橋本 2026年5月29日(金)開業！全21テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3816" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/41085</t>
+        </is>
+      </c>
+    </row>
+    <row r="3817">
+      <c r="A3817" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3817" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3817" t="inlineStr">
+        <is>
+          <t>東北地方ニトリ気仙沼中央インター店 2026年2月27日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3817" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/46473</t>
+        </is>
+      </c>
+    </row>
+    <row r="3818">
+      <c r="A3818" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3818" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3818" t="inlineStr">
+        <is>
+          <t>関東地方フォルテさくら氏家 2026年1月28日(水)開業！テナント随時更新中！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3818" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/43900</t>
+        </is>
+      </c>
+    </row>
+    <row r="3819">
+      <c r="A3819" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3819" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3819" t="inlineStr">
+        <is>
+          <t>東北地方オルフィーカ美田園 2025年5月23日(金)より順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3819" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/39130</t>
+        </is>
+      </c>
+    </row>
+    <row r="3820">
+      <c r="A3820" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3820" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3820" t="inlineStr">
+        <is>
+          <t>関東地方TAIRAYA与野店 与野フード建て替え 2025年4月24日(木)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3820" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/37854</t>
+        </is>
+      </c>
+    </row>
+    <row r="3821">
+      <c r="A3821" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3821" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3821" t="inlineStr">
+        <is>
+          <t>中部地方そよら三条須頃 2025年11月7日(金)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3821" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/36987</t>
+        </is>
+      </c>
+    </row>
+    <row r="3822">
+      <c r="A3822" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3822" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3822" t="inlineStr">
+        <is>
+          <t>関西地方グラングリーン大阪 2025年3月21日(金)南館開業！テナントは？どのような街に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3822" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/4448</t>
+        </is>
+      </c>
+    </row>
+    <row r="3823">
+      <c r="A3823" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3823" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3823" t="inlineStr">
+        <is>
+          <t>九州地方スーパーセンタートライアルうきは店 2026年11月下旬に開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3823" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/49325</t>
+        </is>
+      </c>
+    </row>
+    <row r="3824">
+      <c r="A3824" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3824" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3824" t="inlineStr">
+        <is>
+          <t>中部地方イオンタウン沼津 2027年夏以降開業！イシバシプラザ跡地に50店舗が出店へ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3824" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/39611</t>
+        </is>
+      </c>
+    </row>
+    <row r="3825">
+      <c r="A3825" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3825" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3825" t="inlineStr">
+        <is>
+          <t>中部地方トライアルスマート西尾一色店 2026年3月25日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3825" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/44433</t>
+        </is>
+      </c>
+    </row>
+    <row r="3826">
+      <c r="A3826" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3826" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3826" t="inlineStr">
+        <is>
+          <t>関東地方前橋市野中町SC計画 2028年春開業！ベルクが出店へ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3826" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49033</t>
+        </is>
+      </c>
+    </row>
+    <row r="3827">
+      <c r="A3827" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3827" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3827" t="inlineStr">
+        <is>
+          <t>関東地方アクアゲート千住大川端 2030年度まちびらき！テナントは？最新情報も！東京都足立区千住関屋町のアメージングスクエア跡地に、約5.2ha・約2,100戸の水辺の巨大複合都市「AQUA GATE 千住大川端（アクアゲート千住大川端）」が2030年度まちびらき！2034年度完成！タウンネームが「AQUA GATE ...2026.10.26関東地方</t>
+        </is>
+      </c>
+      <c r="D3827" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/50104</t>
+        </is>
+      </c>
+    </row>
+    <row r="3828">
+      <c r="A3828" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3828" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3828" t="inlineStr">
+        <is>
+          <t>関東地方YAESU CORE（八重洲コア） 2029年春開業！50店舗が出店！テナントは？最新情報も！東京都中央区八重洲に、東京駅前3地区再開発の集大成となる大規模複合施設「YAESU CORE（ヤエス コア）」が2029年1月末に竣工予定！「八重洲二丁目中地区第一種市街地再開発事業」の施設名称が「YAESU CORE」に正式決定！最上層4...2026.10.26関東地方</t>
+        </is>
+      </c>
+      <c r="D3828" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/22140</t>
+        </is>
+      </c>
+    </row>
+    <row r="3829">
+      <c r="A3829" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3829" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3829" t="inlineStr">
+        <is>
+          <t>ウエルシア薬局／「ハックドラッグ戸塚店」新旗艦店にリニューアル、ドラッグ＆フードで食品強化注目</t>
+        </is>
+      </c>
+      <c r="D3829" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s102614.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3830">
+      <c r="A3830" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3830" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3830" t="inlineStr">
+        <is>
+          <t>東急ほか／古民家を核とする木造SC「新綱島ミッカ」オープン、綱島の歴史を継承注目</t>
+        </is>
+      </c>
+      <c r="D3830" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s102672.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3831">
+      <c r="A3831" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3831" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3831" t="inlineStr">
+        <is>
+          <t>カインズ／群馬県前橋市「まえばし赤城モール店」10月28日オープン、道の駅に隣接</t>
+        </is>
+      </c>
+      <c r="D3831" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102647.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3832">
+      <c r="A3832" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3832" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3832" t="inlineStr">
+        <is>
+          <t>カインズ／長野県に「上田国分店」10月29日オープン、上田市に32年ぶり出店</t>
+        </is>
+      </c>
+      <c r="D3832" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102650.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3833">
+      <c r="A3833" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3833" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3833" t="inlineStr">
+        <is>
+          <t>プロント／「新小岩駅」南口から徒歩2分「PRONTO 新小岩店」11月24日オープン</t>
+        </is>
+      </c>
+      <c r="D3833" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102641.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3834">
+      <c r="A3834" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3834" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3834" t="inlineStr">
+        <is>
+          <t>俺の／大阪に「俺のフレンチ・イタリアン 梅田」11月1日オープン、関西初出店</t>
+        </is>
+      </c>
+      <c r="D3834" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102642.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3835">
+      <c r="A3835" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3835" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3835" t="inlineStr">
+        <is>
+          <t>ニラックス／新静岡セノバに「串揚げバイキング くし葉」12月15日オープン</t>
+        </is>
+      </c>
+      <c r="D3835" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102613.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3836">
+      <c r="A3836" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3836" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3836" t="inlineStr">
+        <is>
+          <t>ゴディバ／「ミナ ペルホネン」とのコラボ店舗、伊勢丹新宿にオープン</t>
+        </is>
+      </c>
+      <c r="D3836" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102643.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3837">
+      <c r="A3837" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3837" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3837" t="inlineStr">
+        <is>
+          <t>サブウェイ／神奈川県「川崎市役所前店」10月30日オープン</t>
+        </is>
+      </c>
+      <c r="D3837" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102671.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3838">
+      <c r="A3838" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3838" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3838" t="inlineStr">
+        <is>
+          <t>東洋／埼玉県「エブリデイとれトレ屋桶川店」にクレーンゲームスーパー導入</t>
+        </is>
+      </c>
+      <c r="D3838" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102612.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3839">
+      <c r="A3839" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3839" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3839" t="inlineStr">
+        <is>
+          <t>イオンリテール／茨城県牛久市に「そよらひたち野うしく」11月18日オープン</t>
+        </is>
+      </c>
+      <c r="D3839" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102342.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3840">
+      <c r="A3840" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3840" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3840" t="inlineStr">
+        <is>
+          <t>ニトリ／世界最大の旗艦店「梅田茶屋町店」10月30日オープン、梅田ロフト跡地に出店</t>
+        </is>
+      </c>
+      <c r="D3840" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102379.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3841">
+      <c r="A3841" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3841" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3841" t="inlineStr">
+        <is>
+          <t>マルエツ／東京都大田区「新糀谷店」10月30日リニューアルオープン、鮮魚を対面販売</t>
+        </is>
+      </c>
+      <c r="D3841" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102343.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3842">
+      <c r="A3842" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3842" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3842" t="inlineStr">
+        <is>
+          <t>大和ハウス／福岡市に「ボートレース福岡 天神ストリートパーク」10月30日オープン</t>
+        </is>
+      </c>
+      <c r="D3842" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102381.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3843">
+      <c r="A3843" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3843" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3843" t="inlineStr">
+        <is>
+          <t>NTT都市開発／広島市「パセーラ」11月6日リニューアル、来春までに5店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3843" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102378.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3844">
+      <c r="A3844" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3844" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3844" t="inlineStr">
+        <is>
+          <t>ヤマダデンキ／「広島本店」11月6日オープン、体験型の展示充実・トレンド商品そろう</t>
+        </is>
+      </c>
+      <c r="D3844" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102377.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3845">
+      <c r="A3845" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3845" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3845" t="inlineStr">
+        <is>
+          <t>バローグループ／大阪府高槻市に「たこ一高槻駅前店」10月30日オープン</t>
+        </is>
+      </c>
+      <c r="D3845" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102311.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3846">
+      <c r="A3846" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3846" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3846" t="inlineStr">
+        <is>
+          <t>阪急オアシスマルシェ武庫之荘店／10月30日オープン、価値訴求型店舗に転換</t>
+        </is>
+      </c>
+      <c r="D3846" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102314.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3847">
+      <c r="A3847" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3847" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3847" t="inlineStr">
+        <is>
+          <t>メガネトップ／東京都国分寺市に「眼鏡市場 セレオ国分寺店」オープン</t>
+        </is>
+      </c>
+      <c r="D3847" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102371.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3848">
+      <c r="A3848" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3848" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3848" t="inlineStr">
+        <is>
+          <t>バーガーキング／「そよらつくば学園の森店」「下丸子駅前店」10月下旬オープン</t>
+        </is>
+      </c>
+      <c r="D3848" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102376.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-27
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3848"/>
+  <dimension ref="A1:D3920"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85072,6 +85072,1590 @@
         </is>
       </c>
     </row>
+    <row r="3849">
+      <c r="A3849" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3849" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3849" t="inlineStr">
+        <is>
+          <t>10/31ビッグ・エー越谷東大沢二丁目店</t>
+        </is>
+      </c>
+      <c r="D3849" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gS6</t>
+        </is>
+      </c>
+    </row>
+    <row r="3850">
+      <c r="A3850" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3850" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3850" t="inlineStr">
+        <is>
+          <t>(10/27プレ)10/28スーパーセンタートライアル津河芸店</t>
+        </is>
+      </c>
+      <c r="D3850" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gRp</t>
+        </is>
+      </c>
+    </row>
+    <row r="3851">
+      <c r="A3851" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3851" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3851" t="inlineStr">
+        <is>
+          <t>10/27スーパーやまのぶ赤池店</t>
+        </is>
+      </c>
+      <c r="D3851" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1dGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3852">
+      <c r="A3852" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3852" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3852" t="inlineStr">
+        <is>
+          <t>10/29うな好多治見店</t>
+        </is>
+      </c>
+      <c r="D3852" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gRX</t>
+        </is>
+      </c>
+    </row>
+    <row r="3853">
+      <c r="A3853" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3853" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3853" t="inlineStr">
+        <is>
+          <t>10/23タチヤ豊田小坂店</t>
+        </is>
+      </c>
+      <c r="D3853" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1goQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3854">
+      <c r="A3854" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3854" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3854" t="inlineStr">
+        <is>
+          <t>10/23スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D3854" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="3855">
+      <c r="A3855" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3855" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3855" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D3855" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3856">
+      <c r="A3856" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3856" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3856" t="inlineStr">
+        <is>
+          <t>11/5ローソン羽島市役所南店(岐阜県羽島市)</t>
+        </is>
+      </c>
+      <c r="D3856" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gRd</t>
+        </is>
+      </c>
+    </row>
+    <row r="3857">
+      <c r="A3857" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3857" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3857" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D3857" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3858">
+      <c r="A3858" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3858" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3858" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D3858" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="3859">
+      <c r="A3859" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3859" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3859" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D3859" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="3860">
+      <c r="A3860" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3860" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3860" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D3860" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="3861">
+      <c r="A3861" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3861" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3861" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3861" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3862">
+      <c r="A3862" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3862" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3862" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3862" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3863">
+      <c r="A3863" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3863" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3863" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3863" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3864">
+      <c r="A3864" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3864" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3864" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3864" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3865">
+      <c r="A3865" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3865" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3865" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3865" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3866">
+      <c r="A3866" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3866" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3866" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3866" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3867">
+      <c r="A3867" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3867" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3867" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3867" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3868">
+      <c r="A3868" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3868" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3868" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3868" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3869">
+      <c r="A3869" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3869" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3869" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3869" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3870">
+      <c r="A3870" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3870" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3870" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3870" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3871">
+      <c r="A3871" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3871" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3871" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3871" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3872">
+      <c r="A3872" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3872" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3872" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3872" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3873">
+      <c r="A3873" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3873" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3873" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3873" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3874">
+      <c r="A3874" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3874" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3874" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3874" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3875">
+      <c r="A3875" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3875" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3875" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3875" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3876">
+      <c r="A3876" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3876" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3876" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3876" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3877">
+      <c r="A3877" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3877" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3877" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3877" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3878">
+      <c r="A3878" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3878" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3878" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3878" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3879">
+      <c r="A3879" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3879" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3879" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3879" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3880">
+      <c r="A3880" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3880" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3880" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3880" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3881">
+      <c r="A3881" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3881" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3881" t="inlineStr">
+        <is>
+          <t>中国地方スーパーセンタートライアル山口小郡店 2026年11月上旬開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3881" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/49136</t>
+        </is>
+      </c>
+    </row>
+    <row r="3882">
+      <c r="A3882" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3882" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3882" t="inlineStr">
+        <is>
+          <t>関西地方J.GRAN TOWER 京都向日町 2028年夏開業！駅ビルのテナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3882" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39560</t>
+        </is>
+      </c>
+    </row>
+    <row r="3883">
+      <c r="A3883" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3883" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3883" t="inlineStr">
+        <is>
+          <t>関東地方スーパーセンタートライアル山武成東店 2026年5月20日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3883" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/46150</t>
+        </is>
+      </c>
+    </row>
+    <row r="3884">
+      <c r="A3884" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3884" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3884" t="inlineStr">
+        <is>
+          <t>中国地方カミハチクロス 2027年度開業！アンダーズ広島が進出！商業施設も！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3884" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/27582</t>
+        </is>
+      </c>
+    </row>
+    <row r="3885">
+      <c r="A3885" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3885" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3885" t="inlineStr">
+        <is>
+          <t>関東地方銀座コア建替計画 2028年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3885" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49726</t>
+        </is>
+      </c>
+    </row>
+    <row r="3886">
+      <c r="A3886" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3886" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3886" t="inlineStr">
+        <is>
+          <t>関東地方北小金駅南口東地区市街地再開発事業 2028年度完成 テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3886" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49735</t>
+        </is>
+      </c>
+    </row>
+    <row r="3887">
+      <c r="A3887" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3887" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3887" t="inlineStr">
+        <is>
+          <t>東北地方スーパーセンタートライアル錦ケ丘店 2025年5月21日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3887" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/40364</t>
+        </is>
+      </c>
+    </row>
+    <row r="3888">
+      <c r="A3888" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3888" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3888" t="inlineStr">
+        <is>
+          <t>関西地方ケーズデンキ桜井店 2026年9月17日(木)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3888" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49275</t>
+        </is>
+      </c>
+    </row>
+    <row r="3889">
+      <c r="A3889" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3889" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3889" t="inlineStr">
+        <is>
+          <t>東北地方オルフィーカ美田園 2025年5月23日(金)より順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3889" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/39130</t>
+        </is>
+      </c>
+    </row>
+    <row r="3890">
+      <c r="A3890" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3890" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3890" t="inlineStr">
+        <is>
+          <t>中部地方イオン今池店 ブランズタワー名古屋今池 2024年2月29日(木)に閉店し建て替え！2028年以降開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3890" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/33420</t>
+        </is>
+      </c>
+    </row>
+    <row r="3891">
+      <c r="A3891" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3891" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3891" t="inlineStr">
+        <is>
+          <t>東北地方イオンモール仙台上杉 2025年10月8日(水)開業！全テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3891" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/2380</t>
+        </is>
+      </c>
+    </row>
+    <row r="3892">
+      <c r="A3892" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3892" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3892" t="inlineStr">
+        <is>
+          <t>関東地方みなとみらい21中央地区52街区開発計画 2027年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3892" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48050</t>
+        </is>
+      </c>
+    </row>
+    <row r="3893">
+      <c r="A3893" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3893" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3893" t="inlineStr">
+        <is>
+          <t>関東地方YAESU CORE（八重洲コア） 2029年春開業！50店舗が出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3893" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/22140</t>
+        </is>
+      </c>
+    </row>
+    <row r="3894">
+      <c r="A3894" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3894" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3894" t="inlineStr">
+        <is>
+          <t>関東地方逗子駅ビル 2028年春開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3894" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49835</t>
+        </is>
+      </c>
+    </row>
+    <row r="3895">
+      <c r="A3895" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3895" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3895" t="inlineStr">
+        <is>
+          <t>東北地方スーパーセンタートライアル石巻店 2026年7月1日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3895" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/44362</t>
+        </is>
+      </c>
+    </row>
+    <row r="3896">
+      <c r="A3896" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3896" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3896" t="inlineStr">
+        <is>
+          <t>関東地方セントラルガーデン月島 ザ タワー 2028年春完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3896" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26835</t>
+        </is>
+      </c>
+    </row>
+    <row r="3897">
+      <c r="A3897" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3897" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3897" t="inlineStr">
+        <is>
+          <t>中部地方カインズ岡崎美合店 2025年10月23日(木)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3897" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/39138</t>
+        </is>
+      </c>
+    </row>
+    <row r="3898">
+      <c r="A3898" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3898" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3898" t="inlineStr">
+        <is>
+          <t>関東地方TAIRAYA与野店 与野フード建て替え 2025年4月24日(木)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3898" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/37854</t>
+        </is>
+      </c>
+    </row>
+    <row r="3899">
+      <c r="A3899" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3899" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3899" t="inlineStr">
+        <is>
+          <t>関東地方つくば市上河原崎商業施設 2027年夏開業！約30店舗が出店へ！テナントは？最新情報も！茨城県つくば市の「上河原崎・中西特定土地区画整理事業」区域内に、日本エスコンと新昭和が共同開発する大型商業施設「（仮称）つくば市上河原崎商業施設」が2027年夏に開業予定！敷地面積は約8.9万㎡（約8.9ha）！大店立地法の新設届出が行われ...2026.10.27関東地方</t>
+        </is>
+      </c>
+      <c r="D3899" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48117</t>
+        </is>
+      </c>
+    </row>
+    <row r="3900">
+      <c r="A3900" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3900" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3900" t="inlineStr">
+        <is>
+          <t>九州地方TABISIA(タビジア) 福岡空港国内線ターミナルに2027年夏開業！180店舗が出店！テナントは？最新情報も！福岡県福岡市博多区の福岡空港国内線ターミナル直結の大型複合施設「TABISIA（タビジア）」が2027年夏グランドオープン！正式施設名称が「TABISIA（タビジア）」に決定！国内線ターミナルと直結する地上11階建て・総事業費約450億円の...2026.10.27九州地方</t>
+        </is>
+      </c>
+      <c r="D3900" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/43493</t>
+        </is>
+      </c>
+    </row>
+    <row r="3901">
+      <c r="A3901" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3901" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3901" t="inlineStr">
+        <is>
+          <t>ハックドラッグ戸塚店／コスメ・キャンドゥ充実、予防・介護相談まで担う「ライフストア」へ</t>
+        </is>
+      </c>
+      <c r="D3901" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s102714.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3902">
+      <c r="A3902" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3902" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3902" t="inlineStr">
+        <is>
+          <t>福岡空港／複合施設「タビジア」27年夏開業、日本初上陸の飲食7店舗オープン決定</t>
+        </is>
+      </c>
+      <c r="D3902" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102777.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3903">
+      <c r="A3903" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3903" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3903" t="inlineStr">
+        <is>
+          <t>ドリームオン／「新綱島ミッカ」にベーカリービストロとベーグル専門店10月28日オープン</t>
+        </is>
+      </c>
+      <c r="D3903" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102776.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3904">
+      <c r="A3904" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3904" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3904" t="inlineStr">
+        <is>
+          <t>新綱島ミッカ／季節で主役が変わる洋菓子店「ラトリエ ドゥ アンティーク」10月28日オープン</t>
+        </is>
+      </c>
+      <c r="D3904" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102774.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3905">
+      <c r="A3905" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3905" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3905" t="inlineStr">
+        <is>
+          <t>新綱島ミッカ／海鮮酒場と鮮魚専門店の複合店舗10月28日オープン</t>
+        </is>
+      </c>
+      <c r="D3905" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102775.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3906">
+      <c r="A3906" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3906" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3906" t="inlineStr">
+        <is>
+          <t>ドンキ／山形県東根市に初出店、11月17日オープン</t>
+        </is>
+      </c>
+      <c r="D3906" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102713.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3907">
+      <c r="A3907" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3907" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3907" t="inlineStr">
+        <is>
+          <t>トライアル／茨城県土浦市に「スーパーセンタートライアル荒川沖店（店舗面積4200m2）」27年5月25日新設</t>
+        </is>
+      </c>
+      <c r="D3907" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1027011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3908">
+      <c r="A3908" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3908" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3908" t="inlineStr">
+        <is>
+          <t>ミスターマックスほか／茨城県つくば市に「（仮称）つくば市上河原崎商業施設（店舗面積1万4854m2）」27年6月1日新設</t>
+        </is>
+      </c>
+      <c r="D3908" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1027012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3909">
+      <c r="A3909" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3909" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3909" t="inlineStr">
+        <is>
+          <t>ゴンチャ／東京都港区「ルミネ町田店」10月30日オープン</t>
+        </is>
+      </c>
+      <c r="D3909" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102771.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3910">
+      <c r="A3910" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3910" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3910" t="inlineStr">
+        <is>
+          <t>物語コーポレーション／北海道に「丸源ラーメン 旭川永山店」10月31日オープン</t>
+        </is>
+      </c>
+      <c r="D3910" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102778.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3911">
+      <c r="A3911" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3911" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3911" t="inlineStr">
+        <is>
+          <t>HMV／大阪・ららぽーと堺に11月17日新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3911" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102712.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3912">
+      <c r="A3912" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3912" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3912" t="inlineStr">
+        <is>
+          <t>ウエルシア薬局／「ハックドラッグ戸塚店」新旗艦店にリニューアル、ドラッグ＆フードで食品強化注目</t>
+        </is>
+      </c>
+      <c r="D3912" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s102614.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3913">
+      <c r="A3913" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3913" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3913" t="inlineStr">
+        <is>
+          <t>東急ほか／古民家を核とする木造SC「新綱島ミッカ」オープン、綱島の歴史を継承注目</t>
+        </is>
+      </c>
+      <c r="D3913" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s102672.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3914">
+      <c r="A3914" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3914" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3914" t="inlineStr">
+        <is>
+          <t>カインズ／群馬県前橋市「まえばし赤城モール店」10月28日オープン、道の駅に隣接</t>
+        </is>
+      </c>
+      <c r="D3914" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102647.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3915">
+      <c r="A3915" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3915" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3915" t="inlineStr">
+        <is>
+          <t>カインズ／長野県に「上田国分店」10月29日オープン、上田市に32年ぶり出店</t>
+        </is>
+      </c>
+      <c r="D3915" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102650.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3916">
+      <c r="A3916" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3916" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3916" t="inlineStr">
+        <is>
+          <t>プロント／「新小岩駅」南口から徒歩2分「PRONTO 新小岩店」11月24日オープン</t>
+        </is>
+      </c>
+      <c r="D3916" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102641.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3917">
+      <c r="A3917" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3917" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3917" t="inlineStr">
+        <is>
+          <t>俺の／大阪に「俺のフレンチ・イタリアン 梅田」11月1日オープン、関西初出店</t>
+        </is>
+      </c>
+      <c r="D3917" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102642.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3918">
+      <c r="A3918" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3918" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3918" t="inlineStr">
+        <is>
+          <t>ニラックス／新静岡セノバに「串揚げバイキング くし葉」12月15日オープン</t>
+        </is>
+      </c>
+      <c r="D3918" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102613.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3919">
+      <c r="A3919" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3919" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3919" t="inlineStr">
+        <is>
+          <t>ゴディバ／「ミナ ペルホネン」とのコラボ店舗、伊勢丹新宿にオープン</t>
+        </is>
+      </c>
+      <c r="D3919" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102643.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3920">
+      <c r="A3920" t="inlineStr">
+        <is>
+          <t>2026年10月27日</t>
+        </is>
+      </c>
+      <c r="B3920" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3920" t="inlineStr">
+        <is>
+          <t>サブウェイ／神奈川県「川崎市役所前店」10月30日オープン</t>
+        </is>
+      </c>
+      <c r="D3920" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102671.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-10-28
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3920"/>
+  <dimension ref="A1:D3992"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -86656,6 +86656,1590 @@
         </is>
       </c>
     </row>
+    <row r="3921">
+      <c r="A3921" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3921" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3921" t="inlineStr">
+        <is>
+          <t>11/5まちのパン屋さんマルイチ( 岐阜県美濃加茂市)</t>
+        </is>
+      </c>
+      <c r="D3921" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3922">
+      <c r="A3922" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3922" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3922" t="inlineStr">
+        <is>
+          <t>10/28厚切りとんかつ よし平 各務原店</t>
+        </is>
+      </c>
+      <c r="D3922" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3923">
+      <c r="A3923" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3923" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3923" t="inlineStr">
+        <is>
+          <t>10/28 (10/27プレ)  スーパーセンタートライアル津河芸店</t>
+        </is>
+      </c>
+      <c r="D3923" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gRp</t>
+        </is>
+      </c>
+    </row>
+    <row r="3924">
+      <c r="A3924" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3924" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3924" t="inlineStr">
+        <is>
+          <t>10/23タチヤ豊田小坂店</t>
+        </is>
+      </c>
+      <c r="D3924" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1goQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3925">
+      <c r="A3925" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3925" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3925" t="inlineStr">
+        <is>
+          <t>10/23スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D3925" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="3926">
+      <c r="A3926" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3926" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3926" t="inlineStr">
+        <is>
+          <t>10/27やまのぶ赤池店(愛知県日進市)</t>
+        </is>
+      </c>
+      <c r="D3926" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1dGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3927">
+      <c r="A3927" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3927" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3927" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D3927" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3928">
+      <c r="A3928" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3928" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3928" t="inlineStr">
+        <is>
+          <t>11/5ローソン羽島市役所南店(岐阜県羽島市)</t>
+        </is>
+      </c>
+      <c r="D3928" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gRd</t>
+        </is>
+      </c>
+    </row>
+    <row r="3929">
+      <c r="A3929" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3929" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3929" t="inlineStr">
+        <is>
+          <t>11/27イオンモール伊達(福島県伊達市)</t>
+        </is>
+      </c>
+      <c r="D3929" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gq8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3930">
+      <c r="A3930" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3930" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3930" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D3930" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="3931">
+      <c r="A3931" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3931" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3931" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D3931" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="3932">
+      <c r="A3932" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3932" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C3932" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D3932" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="3933">
+      <c r="A3933" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3933" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3933" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3933" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3934">
+      <c r="A3934" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3934" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3934" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3934" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3935">
+      <c r="A3935" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3935" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3935" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3935" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3936">
+      <c r="A3936" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3936" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3936" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3936" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3937">
+      <c r="A3937" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3937" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3937" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3937" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3938">
+      <c r="A3938" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3938" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3938" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3938" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3939">
+      <c r="A3939" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3939" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3939" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3939" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3940">
+      <c r="A3940" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3940" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3940" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3940" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3941">
+      <c r="A3941" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3941" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3941" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3941" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3942">
+      <c r="A3942" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3942" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3942" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3942" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3943">
+      <c r="A3943" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3943" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3943" t="inlineStr">
+        <is>
+          <t>埼玉県上尾市に登場！ナポリタン専門店「スパゲッティーのパンチョ 上尾店」が10月22日（木）に新規開店、3つのオープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3943" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000115.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3944">
+      <c r="A3944" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3944" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3944" t="inlineStr">
+        <is>
+          <t>10月2日（金）よりオープニングキャンペーン！パンチョ発の新ブランド「ごちそうスープパスタ」、東京・代々木に1号店オープン</t>
+        </is>
+      </c>
+      <c r="D3944" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000114.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3945">
+      <c r="A3945" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3945" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3945" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D3945" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3946">
+      <c r="A3946" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3946" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3946" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D3946" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3947">
+      <c r="A3947" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3947" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3947" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D3947" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3948">
+      <c r="A3948" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3948" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3948" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D3948" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3949">
+      <c r="A3949" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3949" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3949" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3949" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3950">
+      <c r="A3950" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3950" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3950" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D3950" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3951">
+      <c r="A3951" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3951" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3951" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D3951" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3952">
+      <c r="A3952" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3952" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C3952" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D3952" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3953">
+      <c r="A3953" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3953" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3953" t="inlineStr">
+        <is>
+          <t>中部地方M20 cosa（コーサ）静岡駅北口 2024年10月28日(月)開業！全13テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3953" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/26298</t>
+        </is>
+      </c>
+    </row>
+    <row r="3954">
+      <c r="A3954" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3954" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3954" t="inlineStr">
+        <is>
+          <t>関西地方金剛駅周辺地区再整備事業 (駅ビル) 2031年度開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3954" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49715</t>
+        </is>
+      </c>
+    </row>
+    <row r="3955">
+      <c r="A3955" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3955" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3955" t="inlineStr">
+        <is>
+          <t>九州地方イオン鹿児島鴨池店 2024年8月31日(土)に閉店し建て替えへ！イオンモールが取得！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3955" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/36900</t>
+        </is>
+      </c>
+    </row>
+    <row r="3956">
+      <c r="A3956" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3956" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3956" t="inlineStr">
+        <is>
+          <t>関東地方登戸駅前地区市街地再開発事業 2029年竣工！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3956" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/24273</t>
+        </is>
+      </c>
+    </row>
+    <row r="3957">
+      <c r="A3957" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3957" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3957" t="inlineStr">
+        <is>
+          <t>東北地方ヨークベニマル岩沼店 リニューアルオープン 2025年11月28日(金)9時~開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3957" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/38131</t>
+        </is>
+      </c>
+    </row>
+    <row r="3958">
+      <c r="A3958" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3958" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3958" t="inlineStr">
+        <is>
+          <t>関東地方藍テラス（あおてらす）青梅駅前に2026年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3958" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26304</t>
+        </is>
+      </c>
+    </row>
+    <row r="3959">
+      <c r="A3959" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3959" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3959" t="inlineStr">
+        <is>
+          <t>中部地方コメリパワー亀山店 2027年3月開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3959" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48442</t>
+        </is>
+      </c>
+    </row>
+    <row r="3960">
+      <c r="A3960" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3960" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3960" t="inlineStr">
+        <is>
+          <t>東北地方鶴岡茅原に無印良品・ワークマン 2025年4月24日(木)より順次開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3960" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/42243</t>
+        </is>
+      </c>
+    </row>
+    <row r="3961">
+      <c r="A3961" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3961" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3961" t="inlineStr">
+        <is>
+          <t>関東地方パークタワー川口本町 2026年冬から順次開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3961" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26762</t>
+        </is>
+      </c>
+    </row>
+    <row r="3962">
+      <c r="A3962" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3962" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3962" t="inlineStr">
+        <is>
+          <t>関東地方イオン伊勢原店 2024年1月31日(水)に閉店し建て替えへ！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3962" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36886</t>
+        </is>
+      </c>
+    </row>
+    <row r="3963">
+      <c r="A3963" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3963" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3963" t="inlineStr">
+        <is>
+          <t>関東地方イオン石岡店が建て替えへ！2028年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3963" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/45661</t>
+        </is>
+      </c>
+    </row>
+    <row r="3964">
+      <c r="A3964" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3964" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3964" t="inlineStr">
+        <is>
+          <t>関東地方ヤオコーまるひろ上尾SC 2025年9月12日(金)開業！全テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3964" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42379</t>
+        </is>
+      </c>
+    </row>
+    <row r="3965">
+      <c r="A3965" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3965" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3965" t="inlineStr">
+        <is>
+          <t>関東地方東京科学大学田町キャンパス土地活用事業 2030年頃開業！どのような建物に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3965" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/19257</t>
+        </is>
+      </c>
+    </row>
+    <row r="3966">
+      <c r="A3966" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3966" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3966" t="inlineStr">
+        <is>
+          <t>関東地方逗子駅ビル 2028年春開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3966" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49835</t>
+        </is>
+      </c>
+    </row>
+    <row r="3967">
+      <c r="A3967" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3967" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3967" t="inlineStr">
+        <is>
+          <t>関東地方アクロスプラザ北柏 2026年4月1日(水)より順次開業！全19テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3967" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/35911</t>
+        </is>
+      </c>
+    </row>
+    <row r="3968">
+      <c r="A3968" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3968" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3968" t="inlineStr">
+        <is>
+          <t>中部地方イオンモール須坂 2025年10月3日(金)開業！全テナント166店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3968" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/11811</t>
+        </is>
+      </c>
+    </row>
+    <row r="3969">
+      <c r="A3969" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3969" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3969" t="inlineStr">
+        <is>
+          <t>関東地方ekubo京成 新鎌ヶ谷 2026年9月10日(木)開業！全15テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3969" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/30880</t>
+        </is>
+      </c>
+    </row>
+    <row r="3970">
+      <c r="A3970" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3970" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3970" t="inlineStr">
+        <is>
+          <t>関東地方川崎アリーナシティプロジェクト 2030年10月開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D3970" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/33041</t>
+        </is>
+      </c>
+    </row>
+    <row r="3971">
+      <c r="A3971" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3971" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3971" t="inlineStr">
+        <is>
+          <t>関東地方明治安田新宿ビル 2026年11月28日(土)開業！全テナント一覧！東京都新宿区の新宿駅西口前における大型建て替え事業「明治安田新宿ビル」の商業エリアが2026年11月28日(土)グランドオープン！2026年8月31日に竣工した地上23階・地下4階の超高層複合オフィスビル！低層階（1階・地下1階）の商業エリ...2026.10.28関東地方</t>
+        </is>
+      </c>
+      <c r="D3971" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26240</t>
+        </is>
+      </c>
+    </row>
+    <row r="3972">
+      <c r="A3972" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3972" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C3972" t="inlineStr">
+        <is>
+          <t>関西地方アクロスプラザ和泉観音寺 2026年11月開業！テナントは？最新情報も！大阪府和泉市観音寺町のTSUTAYA観音寺店跡地一帯に、大和ハウスリアルティマネジメントの複合商業施設「アクロスプラザ和泉観音寺」が2026年11月頃に開業予定！アクロスプラザ和泉観音寺は、食品スーパーマーケット「万代」を核店舗として、複数...2026.10.28関西地方</t>
+        </is>
+      </c>
+      <c r="D3972" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/47867</t>
+        </is>
+      </c>
+    </row>
+    <row r="3973">
+      <c r="A3973" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3973" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3973" t="inlineStr">
+        <is>
+          <t>コメリ／上期出店は5店舗のみ、改装は82店舗</t>
+        </is>
+      </c>
+      <c r="D3973" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102817.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3974">
+      <c r="A3974" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3974" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3974" t="inlineStr">
+        <is>
+          <t>ベイシア／千葉・幕張「Beisia Foods Park 幕張店」オープン、鮮魚売場に魚耕が出店</t>
+        </is>
+      </c>
+      <c r="D3974" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102842.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3975">
+      <c r="A3975" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3975" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3975" t="inlineStr">
+        <is>
+          <t>サンシティ池田／「イケディア」に新規4店舗11月20日オープン、カルディなど出店</t>
+        </is>
+      </c>
+      <c r="D3975" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102877.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3976">
+      <c r="A3976" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3976" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3976" t="inlineStr">
+        <is>
+          <t>オアシス21／27年春リニューアル、サンエース・天ぷら定食まきのがオープン</t>
+        </is>
+      </c>
+      <c r="D3976" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102813.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3977">
+      <c r="A3977" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3977" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3977" t="inlineStr">
+        <is>
+          <t>あみプレミアム・アウトレット／10～12月アウトドアブランドなど6店舗オープン</t>
+        </is>
+      </c>
+      <c r="D3977" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102876.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3978">
+      <c r="A3978" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3978" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3978" t="inlineStr">
+        <is>
+          <t>シェアグリーン南青山／27年新春に拡大、ホンダのブランド施設や商業施設オープン</t>
+        </is>
+      </c>
+      <c r="D3978" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102811.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3979">
+      <c r="A3979" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3979" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3979" t="inlineStr">
+        <is>
+          <t>アルビス／富山県高岡市「福岡駅前店」オープン「タピス店」改装で年商14億円目指す</t>
+        </is>
+      </c>
+      <c r="D3979" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102844.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3980">
+      <c r="A3980" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3980" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3980" t="inlineStr">
+        <is>
+          <t>うちだ屋うどん／関東初進出、横浜市の商業施設「港北みなも」に11月26日オープン</t>
+        </is>
+      </c>
+      <c r="D3980" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102812.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3981">
+      <c r="A3981" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3981" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3981" t="inlineStr">
+        <is>
+          <t>ピソラ／千葉市中央区に初の公園内店舗「PISOLA千葉公園店」11月11日オープン</t>
+        </is>
+      </c>
+      <c r="D3981" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102875.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3982">
+      <c r="A3982" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3982" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3982" t="inlineStr">
+        <is>
+          <t>がってん寿司／「イオンレイクタウンkaze」に初のフードコート業態オープン</t>
+        </is>
+      </c>
+      <c r="D3982" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102872.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3983">
+      <c r="A3983" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3983" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3983" t="inlineStr">
+        <is>
+          <t>アリオ八尾／「鳥〇食堂×タニタカフェ」10月29日オープン</t>
+        </is>
+      </c>
+      <c r="D3983" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102873.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3984">
+      <c r="A3984" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3984" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3984" t="inlineStr">
+        <is>
+          <t>オリジン東秀／東京都昭島市に「れんげ食堂Toshu 中神店」10月30日オープン</t>
+        </is>
+      </c>
+      <c r="D3984" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102874.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3985">
+      <c r="A3985" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3985" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3985" t="inlineStr">
+        <is>
+          <t>ハックドラッグ戸塚店／コスメ・キャンドゥ充実、予防・介護相談まで担う「ライフストア」へ</t>
+        </is>
+      </c>
+      <c r="D3985" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s102714.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3986">
+      <c r="A3986" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3986" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3986" t="inlineStr">
+        <is>
+          <t>福岡空港／複合施設「タビジア」27年夏開業、日本初上陸の飲食7店舗オープン決定</t>
+        </is>
+      </c>
+      <c r="D3986" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102777.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3987">
+      <c r="A3987" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3987" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3987" t="inlineStr">
+        <is>
+          <t>ドリームオン／「新綱島ミッカ」にベーカリービストロとベーグル専門店10月28日オープン</t>
+        </is>
+      </c>
+      <c r="D3987" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102776.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3988">
+      <c r="A3988" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3988" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3988" t="inlineStr">
+        <is>
+          <t>新綱島ミッカ／季節で主役が変わる洋菓子店「ラトリエ ドゥ アンティーク」10月28日オープン</t>
+        </is>
+      </c>
+      <c r="D3988" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102774.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3989">
+      <c r="A3989" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3989" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3989" t="inlineStr">
+        <is>
+          <t>新綱島ミッカ／海鮮酒場と鮮魚専門店の複合店舗10月28日オープン</t>
+        </is>
+      </c>
+      <c r="D3989" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102775.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3990">
+      <c r="A3990" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3990" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3990" t="inlineStr">
+        <is>
+          <t>ドンキ／山形県東根市に初出店、11月17日オープン</t>
+        </is>
+      </c>
+      <c r="D3990" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s102713.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3991">
+      <c r="A3991" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3991" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3991" t="inlineStr">
+        <is>
+          <t>トライアル／茨城県土浦市に「スーパーセンタートライアル荒川沖店（店舗面積4200m2）」27年5月25日新設</t>
+        </is>
+      </c>
+      <c r="D3991" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1027011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3992">
+      <c r="A3992" t="inlineStr">
+        <is>
+          <t>2026年10月28日</t>
+        </is>
+      </c>
+      <c r="B3992" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C3992" t="inlineStr">
+        <is>
+          <t>ミスターマックスほか／茨城県つくば市に「（仮称）つくば市上河原崎商業施設（店舗面積1万4854m2）」27年6月1日新設</t>
+        </is>
+      </c>
+      <c r="D3992" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s1027012.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>